<commit_message>
docs: record P1 QA kickoff
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R4bc6b3db5a6c428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R7d23391e7ec4457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd91f3f228da142f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9266a6f58d1d4f07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rd0ead783931f4b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc5abaaf79c794b77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R61e0ec20a7744657"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1a1ad79ad8cc45b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc35971d6321c4257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd929620dfeb54441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8fb7f25bbe2b43e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb7577743949e427d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations applied to linked remote and production smoke/security smoke passed.</x:v>
+        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations applied to linked remote; production smoke/security smoke and P1 focused automated QA passed. Live Telegram media/private-group and Admin Operator UX remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7578,6 +7578,32 @@
         <x:v>Decide whether to move embed/check to a separate origin/subdomain or add explicit CORS support before changing sandbox.</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>QA-2026-06-30-001</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>P1 automated user-story QA kickoff</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>npm run test:run -- bot QA matrix, follow-up routing, voice, report scenario, webhook dedup/integration, AI safety, URL/contact/rules, admin/migration/security env tests</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Passed: 16 files / 323 tests</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>TG-001, TG-005, TG-010, TG-014, TG-027, TG-028, WEB/Admin/Core security regressions</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Focused P1 suite passed after commit series. Production smoke and production security smoke also passed after linked Supabase migrations.</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Live Telegram image/QR, real voice/private/group chat scoping and Admin Operator UX walkthrough remain manual P1 QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record live QA blockers
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R61e0ec20a7744657"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1a1ad79ad8cc45b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc35971d6321c4257"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd929620dfeb54441"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8fb7f25bbe2b43e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb7577743949e427d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re1586bd0164e48e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rec51e313b72848d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R315addeb8d674240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R67120692ffc34538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rdc710a48255f429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc1d9a20e420a44b1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations applied to linked remote; production smoke/security smoke and P1 focused automated QA passed. Live Telegram media/private-group and Admin Operator UX remain.</x:v>
+        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations are applied to linked remote; production, security, TTS and P1 focused automated QA passed. Live Telegram text webhook passed. Live Telegram image/QR/voice private-group QA is blocked until a QA private chat/group and real media fixtures are provisioned; full Admin Operator UX is blocked until admin test credentials are available.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7578,30 +7578,56 @@
         <x:v>Decide whether to move embed/check to a separate origin/subdomain or add explicit CORS support before changing sandbox.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
+    <x:row r="10" ht="78" customHeight="1">
+      <x:c r="A10" s="4" t="str">
         <x:v>QA-2026-06-30-001</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B10" s="4" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C10" s="4" t="str">
         <x:v>P1 automated user-story QA kickoff</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" s="4" t="str">
         <x:v>npm run test:run -- bot QA matrix, follow-up routing, voice, report scenario, webhook dedup/integration, AI safety, URL/contact/rules, admin/migration/security env tests</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E10" s="4" t="str">
         <x:v>Passed: 16 files / 323 tests</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="F10" s="4" t="str">
         <x:v>TG-001, TG-005, TG-010, TG-014, TG-027, TG-028, WEB/Admin/Core security regressions</x:v>
       </x:c>
-      <x:c r="G10" t="str">
+      <x:c r="G10" s="4" t="str">
         <x:v>Focused P1 suite passed after commit series. Production smoke and production security smoke also passed after linked Supabase migrations.</x:v>
       </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="H10" s="4" t="str">
         <x:v>Live Telegram image/QR, real voice/private/group chat scoping and Admin Operator UX walkthrough remain manual P1 QA.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="78" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>QA-2026-06-30-002</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>P1 live Telegram/admin manual QA residue</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>railway run npm run tts:smoke; railway run npx vite-node scripts/prod-smoke.ts https://scam-guard-main-production.up.railway.app --live-telegram; Playwright /admin</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>Partial: automated live checks passed; manual media/admin flows blocked</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>TG-010, TG-014, TG-017, TG-022, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>TTS smoke passed with Gemini audio bytes; production smoke passed with live Telegram synthetic text update status=200 and pending=0. Playwright verified /admin redirects to /login, login form is visible and console/page errors=0.</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>Provision TELEGRAM_QA_CHAT_ID/private QA chat, QA group, image/QR and voice fixtures, plus ADMIN_EMAIL/ADMIN_PASSWORD or a disposable admin test account; then run real Telegram media/private-group and full Admin Operator moderation walkthrough.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record live Telegram and admin QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re1586bd0164e48e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rec51e313b72848d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R315addeb8d674240"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R67120692ffc34538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rdc710a48255f429f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc1d9a20e420a44b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R21c068ef070a4575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R552b2206c49a48f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8c4be6a184454cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R189d982335444a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R788667f0e8d44117"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rdc38bf376ab84dab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations are applied to linked remote; production, security, TTS and P1 focused automated QA passed. Live Telegram text webhook passed. Live Telegram image/QR/voice private-group QA is blocked until a QA private chat/group and real media fixtures are provisioned; full Admin Operator UX is blocked until admin test credentials are available.</x:v>
+        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations are applied to linked remote; production, security, TTS, P1 focused automated QA, live Telegram text/image/audio/private-group checks, and Admin Operator read-only walkthrough passed. No open P1 live blocker remains; next phase is UX/logistics fixes plus optional cleanup/rejection of old QA smoke report and appeal records.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7630,6 +7630,32 @@
         <x:v>Provision TELEGRAM_QA_CHAT_ID/private QA chat, QA group, image/QR and voice fixtures, plus ADMIN_EMAIL/ADMIN_PASSWORD or a disposable admin test account; then run real Telegram media/private-group and full Admin Operator moderation walkthrough.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="78" customHeight="1">
+      <x:c r="A12" s="4" t="str">
+        <x:v>QA-2026-06-30-003</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>P1 live Telegram media/admin QA closure</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>railway run npx vite-node .codex-tmp/live-telegram-qa/live-telegram-media-qa.ts; Playwright disposable admin login/details walkthrough; Supabase cleanup sanity SQL</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>Passed: live blockers cleared; admin mutation intentionally not performed</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>TG-010, TG-014, TG-017, TG-022, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>Bot uploaded synthetic QR photo/audio fixtures to moderation chat. Private image QR webhook, private audio/STT webhook, group-scoped /check and private follow-up after group scope all returned 200. Disposable admin login loaded stats, operator guide, reports, appeals, entities and details modal; cleanup left 0 QA admin auth/role/allowlist rows.</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>Proceed to UX/logistics fixes. Optional: reject/resolve old QA smoke report/appeal records or add dedicated staging fixtures for moderation mutation tests.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record QA smoke cleanup
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R21c068ef070a4575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R552b2206c49a48f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8c4be6a184454cc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R189d982335444a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R788667f0e8d44117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rdc38bf376ab84dab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcc328e49a9044034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R083f9edfb0ba4031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R86b8efee7d554767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R7db5e77f14054274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R81e420df4b2f4d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rabe0734a9c6949ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations are applied to linked remote; production, security, TTS, P1 focused automated QA, live Telegram text/image/audio/private-group checks, and Admin Operator read-only walkthrough passed. No open P1 live blocker remains; next phase is UX/logistics fixes plus optional cleanup/rejection of old QA smoke report and appeal records.</x:v>
+        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations are applied to linked remote; production, security, TTS, P1 focused automated QA, live Telegram text/image/audio/private-group checks, Admin Operator read-only walkthrough and QA smoke queue cleanup passed. No open P1 live blocker remains; next phase is UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7656,6 +7656,32 @@
         <x:v>Proceed to UX/logistics fixes. Optional: reject/resolve old QA smoke report/appeal records or add dedicated staging fixtures for moderation mutation tests.</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="78" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(web): polish quick report feedback
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcc328e49a9044034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R083f9edfb0ba4031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R86b8efee7d554767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R7db5e77f14054274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R81e420df4b2f4d62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rabe0734a9c6949ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R532d88887e484bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re567402d77d8416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R0e45abf7e0f04f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1eb073f05a7d4154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb4234ee56c764ff3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf1feff437ff04f40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog is closed; browser QA has 8 closed issues and 0 open embed sandbox architecture notes. Supabase migrations are applied to linked remote; production, security, TTS, P1 focused automated QA, live Telegram text/image/audio/private-group checks, Admin Operator read-only walkthrough and QA smoke queue cleanup passed. No open P1 live blocker remains; next phase is UX/logistics fixes.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, and QA smoke queue cleanup passed. WEB-003 quick-report UX/logistics first slice shipped: rate-limit errors are user-safe and success copy states manual moderation. Next phase: continue ROAD-002 Telegram report-flow polish and remaining UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4109,19 +4109,19 @@
         <x:v>.kiro/specs/report-flow-reputation-boundary-v1</x:v>
       </x:c>
       <x:c r="H32" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I32" s="8" t="str">
         <x:v>Unit tests</x:v>
       </x:c>
       <x:c r="J32" s="8" t="str">
-        <x:v>Other agent is editing this area; verify no-target incident handling and redaction after merge.</x:v>
+        <x:v>Re-run browser smoke for homepage quick report after deploy; include rate-limit path if a low-risk staging/prod bucket is available.</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L32" s="8" t="str">
-        <x:v>Do not let no-target quick reports suppress unrelated target reports.</x:v>
+        <x:v>2026-06-30: QuickReportForm now maps report rate limits to localized user copy, no longer exposes internal error codes, announces success accessibly, and states that public labels appear only after manual moderation.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -4907,19 +4907,19 @@
         <x:v>User plan P7</x:v>
       </x:c>
       <x:c r="H53" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="I53" s="8" t="str">
         <x:v>Needs live QA</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>Implement after dashboard slice or with it if low conflict.</x:v>
+        <x:v>Continue Report Flow Polish in Telegram /report copy and duplicate reassurance; verify duplicate-count context in admin detail view.</x:v>
       </x:c>
       <x:c r="K53" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L53" s="8" t="str">
-        <x:v>Do not reveal full target in moderation Telegram chat.</x:v>
+        <x:v>2026-06-30: First web slice shipped for quick-report success/rate-limit UX; duplicate handling remains intentionally non-disclosing to reporters while moderation receives the signal.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -7682,6 +7682,32 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): clarify report confirmation copy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R532d88887e484bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re567402d77d8416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R0e45abf7e0f04f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1eb073f05a7d4154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb4234ee56c764ff3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf1feff437ff04f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcb734e7a2b254245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R97ddf3ce13b54bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rbe4c25a8fe4e4a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc1f153384afd40e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf418015164d14971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0067ccf627d14b10"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, and QA smoke queue cleanup passed. WEB-003 quick-report UX/logistics first slice shipped: rate-limit errors are user-safe and success copy states manual moderation. Next phase: continue ROAD-002 Telegram report-flow polish and remaining UX/logistics fixes.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, and QA smoke queue cleanup passed. WEB-003 quick-report UX/logistics shipped; ROAD-002 is now partial with web feedback and Telegram report-confirmation copy polished. Next phase: live /report copy smoke, then admin duplicate-count/last-report-time UX.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4910,16 +4910,16 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="I53" s="8" t="str">
-        <x:v>Needs live QA</x:v>
+        <x:v>Unit tests + build</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>Continue Report Flow Polish in Telegram /report copy and duplicate reassurance; verify duplicate-count context in admin detail view.</x:v>
+        <x:v>Run live Telegram /report smoke after deploy to verify final confirmation copy; then continue admin duplicate-count/last-report-time polish.</x:v>
       </x:c>
       <x:c r="K53" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L53" s="8" t="str">
-        <x:v>2026-06-30: First web slice shipped for quick-report success/rate-limit UX; duplicate handling remains intentionally non-disclosing to reporters while moderation receives the signal.</x:v>
+        <x:v>2026-06-30: Web quick-report success/rate-limit UX shipped. Telegram /report confirmation now says similar prior signals can raise review priority without disclosing whether the current report is a duplicate; moderator still receives only safe summary.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -7708,6 +7708,32 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: close report flow polish tracker
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcb734e7a2b254245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R97ddf3ce13b54bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rbe4c25a8fe4e4a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc1f153384afd40e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf418015164d14971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0067ccf627d14b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcb33caa6b88e42db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc0a4a47d961e4a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8da83c1974ee4e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R18544c91f1aa48b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2b9e2d3e3fe44f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R30764c86392f445c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, and QA smoke queue cleanup passed. WEB-003 quick-report UX/logistics shipped; ROAD-002 is now partial with web feedback and Telegram report-confirmation copy polished. Next phase: live /report copy smoke, then admin duplicate-count/last-report-time UX.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, and QA smoke queue cleanup passed. WEB-003 and ROAD-002 UX/logistics slices are implemented and tested; live /report confirmation remains a release smoke, not an implementation blocker. Next phase: pick next P1 item from TG-005/TG-010/TG-014 or ADM-001.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4907,19 +4907,19 @@
         <x:v>User plan P7</x:v>
       </x:c>
       <x:c r="H53" s="15" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I53" s="8" t="str">
-        <x:v>Unit tests + build</x:v>
+        <x:v>Unit tests + build + admin live QA evidence</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>Run live Telegram /report smoke after deploy to verify final confirmation copy; then continue admin duplicate-count/last-report-time polish.</x:v>
+        <x:v>Keep live Telegram /report confirmation smoke in release checklist after deploy; no implementation blocker remains for Report Flow Polish.</x:v>
       </x:c>
       <x:c r="K53" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L53" s="8" t="str">
-        <x:v>2026-06-30: Web quick-report success/rate-limit UX shipped. Telegram /report confirmation now says similar prior signals can raise review priority without disclosing whether the current report is a duplicate; moderator still receives only safe summary.</x:v>
+        <x:v>2026-06-30: ROAD-002 implemented. Web quick report uses safe rate-limit feedback and manual-moderation success copy; Telegram /report confirms repeated similar signals can raise review priority without disclosing duplicates; admin cards/detail already show duplicate signal strength and latest signal time.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -7734,6 +7734,32 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: verify admin login allowlist
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcb33caa6b88e42db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc0a4a47d961e4a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8da83c1974ee4e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R18544c91f1aa48b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2b9e2d3e3fe44f16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R30764c86392f445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc51b94a9b43345c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb58833a1b0e247fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R33718ecbfe7c41ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5e31bb6cd9064746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rbebb184ae8c04f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5fa9b2bac65c452e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, and QA smoke queue cleanup passed. WEB-003 and ROAD-002 UX/logistics slices are implemented and tested; live /report confirmation remains a release smoke, not an implementation blocker. Next phase: pick next P1 item from TG-005/TG-010/TG-014 or ADM-001.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke queue cleanup, WEB-003, ROAD-002, and ADM-001 are implemented/verified. Admin access is allowlist + email-confirmation gated with no unconfirmed or non-allowlisted admin roles in linked Supabase. Next phase: TG-005 conversational follow-up router.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4293,25 +4293,25 @@
         <x:v>Only allowlisted admin accounts can access moderation dashboard; first-user/admin behavior must be controlled.</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
-        <x:v>src/lib/auth.server.ts; src/routes/admin.tsx</x:v>
+        <x:v>src/integrations/supabase/auth-middleware.ts; src/integrations/supabase/auth-attacher.ts; src/lib/auth-context.tsx; src/routes/login.tsx; src/routes/admin.tsx; supabase/migrations/20260629085533_gate_admin_allowlist_on_email_confirmation.sql</x:v>
       </x:c>
       <x:c r="G37" s="8" t="str">
         <x:v>ai_docs/MODERATION_GUIDELINES.md</x:v>
       </x:c>
       <x:c r="H37" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I37" s="8" t="str">
-        <x:v>Manual QA</x:v>
+        <x:v>Unit tests + linked Supabase read-only verification</x:v>
       </x:c>
       <x:c r="J37" s="8" t="str">
-        <x:v>Security scan: allowlisted email signup can grant admin before mailbox ownership verified.</x:v>
+        <x:v>Keep admin sign-in/no-access browser smoke in release checklist after auth or Supabase Auth setting changes.</x:v>
       </x:c>
       <x:c r="K37" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L37" s="8" t="str">
-        <x:v>Require proven mailbox/session ownership before admin grant.</x:v>
+        <x:v>2026-06-30: ADM-001 verified. Server functions require bearer token and user_roles.role='admin'; client admin page gates on isAdmin for UX. Linked Supabase check: trigger functions not executable by anon/authenticated, auth.users triggers enabled, no first-user bootstrap, 0 unconfirmed allowlisted admins, 0 admin roles outside allowlist, 1 confirmed allowlisted admin.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -7760,6 +7760,58 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): route code follow-ups through checks
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc51b94a9b43345c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb58833a1b0e247fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R33718ecbfe7c41ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5e31bb6cd9064746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rbebb184ae8c04f38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5fa9b2bac65c452e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R83d251d8515c418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2582ee7f53b443c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb044e79d56da4302"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R569e9b73f45b4d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re92706cb6de246fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R22fbd854eb814a7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke queue cleanup, WEB-003, ROAD-002, and ADM-001 are implemented/verified. Admin access is allowlist + email-confirmation gated with no unconfirmed or non-allowlisted admin roles in linked Supabase. Next phase: TG-005 conversational follow-up router.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke queue cleanup, WEB-003, ROAD-002, ADM-001, and TG-005 are implemented/verified. TG-005 now keeps secret-code/kod/code payloads in the risk pipeline instead of treating them as generic follow-ups. Next phase: TG-010 image/OCR/QR intelligence tuning.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3121,19 +3121,19 @@
         <x:v>.kiro/specs/telegram-context-router-v2; .kiro/specs/telegram-followup-memory-v1</x:v>
       </x:c>
       <x:c r="H6" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I6" s="8" t="str">
-        <x:v>Unit tests for known follow-ups</x:v>
+        <x:v>Unit tests</x:v>
       </x:c>
       <x:c r="J6" s="8" t="str">
-        <x:v>Implement narrow AI conversational layer over last check for unsupported clarifying questions.</x:v>
+        <x:v>Keep live Telegram smoke for RU/UZ/EN follow-ups after deploy; extend phrase list only from real transcripts.</x:v>
       </x:c>
       <x:c r="K6" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L6" s="8" t="str">
-        <x:v>AI follow-up must pass output-safety firewall and never upgrade/downgrade verdict.</x:v>
+        <x:v>2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -7812,6 +7812,32 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(risk): preserve private invite image signals
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R83d251d8515c418c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2582ee7f53b443c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb044e79d56da4302"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R569e9b73f45b4d49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re92706cb6de246fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R22fbd854eb814a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6820742b1e7440a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc17181d0030749c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd3f9f1bb0aac43d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R20288e075c664068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R420b1ea118eb4b9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rae803fd94d3e4129"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke queue cleanup, WEB-003, ROAD-002, ADM-001, and TG-005 are implemented/verified. TG-005 now keeps secret-code/kod/code payloads in the risk pipeline instead of treating them as generic follow-ups. Next phase: TG-010 image/OCR/QR intelligence tuning.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005 and TG-010 are implemented/verified. TG-010 now preserves private invite risk while redacting real invite codes. Next recommended P1: TG-014 voice STT false-positive/hook phrase tuning, then ADM-002 Dashboard Operator UX v2.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3311,19 +3311,19 @@
         <x:v>.kiro/specs/telegram-image-intelligence-v2; .kiro/specs/telegram-image-intelligence-v3; .kiro/specs/telegram-qr-decoder-v1</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I11" s="8" t="str">
-        <x:v>Unit tests + live QA</x:v>
+        <x:v>Unit tests + integration tests + live QA</x:v>
       </x:c>
       <x:c r="J11" s="8" t="str">
-        <x:v>P3: QR/Image Precision v2 must separate menu, Telegram login, payment, invite, bot/captcha, unreadable.</x:v>
+        <x:v>Keep live Telegram image/QR fixture smoke after image-copy or parser changes; continue production timing tuning from logs.</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L11" s="8" t="str">
-        <x:v>Do not assert model-guessed visibleUrl as decoded QR URL unless QR pixels were decoded.</x:v>
+        <x:v>2026-06-30: TG-010 implemented/verified. QR/image precision now separates menu/info QR, Telegram login/device/2FA QR, payment QR, private invite links, bot/captcha/giveaway screenshots, wallet/DeFi urgency and unreadable images. Added regression that private Telegram invite OCR is scored as suspicious_invite_link while the real invite code is redacted and not stored in image check input.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -7838,6 +7838,32 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>QA-2026-06-30-004</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Production QA smoke queue cleanup</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Passed: synthetic QA queue records closed</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): surface voice transcript hooks
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6820742b1e7440a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc17181d0030749c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd3f9f1bb0aac43d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R20288e075c664068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R420b1ea118eb4b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rae803fd94d3e4129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R961e0bdb50674e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R785d9f30922d48fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7faec1a2c77149c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R30653bb1d5204855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0c2c0c5a20fb478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R9498b1c4997946e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005 and TG-010 are implemented/verified. TG-010 now preserves private invite risk while redacting real invite codes. Next recommended P1: TG-014 voice STT false-positive/hook phrase tuning, then ADM-002 Dashboard Operator UX v2.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005, TG-010 and TG-014 are implemented/verified. TG-014 now surfaces a sanitized voice hook phrase while preserving delivery/card false-positive guards and STT privacy limits. Next recommended P1: ADM-002 Dashboard Operator UX v2 / ROAD-001.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2649,7 +2649,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>27</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2662,7 +2662,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -2675,7 +2675,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -3463,19 +3463,19 @@
         <x:v>.kiro/specs/telegram-voice-stt-v1; .kiro/specs/telegram-voice-in-v2</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
-        <x:v>Live QA + unit tests</x:v>
+        <x:v>Unit tests + integration tests + live QA</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>P1/P3: fix false-positive reasons for friendly delivery/card voice and extract concrete hook phrase.</x:v>
+        <x:v>Closed 2026-06-30: friendly delivery/card voice stays below high-risk; sanitized hook phrase is shown for concrete risk triggers. Keep real-audio STT corpus/timing watch after provider/model changes.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L15" s="8" t="str">
-        <x:v>Rate-limit before expensive STT; never transcribe long/unsupported media silently.</x:v>
+        <x:v>2026-06-30 verified: voice hook phrase is derived from sanitized transcript preview, so raw URLs, @handles and long digit runs remain hidden; long/unsupported/over-budget voice guard remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6373,13 +6373,13 @@
         <x:v>Short voice is transcribed, shown back to the user, and then checked; uncertain transcription should avoid hard verdicts.</x:v>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>P1/P3: fix false-positive reasons for friendly delivery/card voice and extract concrete hook phrase.</x:v>
+        <x:v>Closed 2026-06-30: friendly delivery/card false positives covered; concrete voice hook phrase is extracted from sanitized transcript preview.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-06-30; live voice/STT QA covered 2026-06-30; regression watch</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
@@ -7864,6 +7864,32 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>QA-2026-06-30-005</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>TG-014 Voice STT / Voice-in tuning</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/format.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/risk/voice-transcription.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/router.test.ts src/lib/telegram/bot-qa-matrix.test.ts</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>Passed: 7 files / 332 tests</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>TG-014</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Voice result surfaces a sanitized hook phrase from transcript preview; raw URLs, @handles and long digit runs stay hidden; high-risk cards show the hook; Telegram voice, formatter, risk voice/rule, webhook, router and bot QA matrix suites passed.</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Proceed to ADM-002 Dashboard Operator UX v2 / ROAD-001; keep real-audio STT corpus/timing watch after provider/model changes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(admin): show report reason summaries
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R961e0bdb50674e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R785d9f30922d48fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7faec1a2c77149c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R30653bb1d5204855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0c2c0c5a20fb478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R9498b1c4997946e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1a0bd4f915cb4dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R764f2920f5ec4925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9c35f350cb614bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb97f3197ada74ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R69a397b234de4796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8a66c8ee28bf4002"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005, TG-010 and TG-014 are implemented/verified. TG-014 now surfaces a sanitized voice hook phrase while preserving delivery/card false-positive guards and STT privacy limits. Next recommended P1: ADM-002 Dashboard Operator UX v2 / ROAD-001.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified. ROAD-001 Dashboard Operator UX v2 is partial: cards/details now show latest-check reason summaries and legal-safe decision context. Next recommended P1: full admin mutation QA, then ROAD-001 queue ergonomics polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2649,7 +2649,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2675,7 +2675,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -4337,19 +4337,19 @@
         <x:v>Roadmap P6; ai_docs/EXECUTION_PLAN_2026-06-21.md</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>Unit + manual QA</x:v>
+        <x:v>Unit tests + production build + prior live admin read-only QA</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>P6 v2: detail view, duplicate count, role of Telegram chat, human decision passport.</x:v>
+        <x:v>Closed 2026-06-30: report cards/detail view now show latest target check reason summary, score, duplicate signal and human decision passport. Next: disposable live moderation mutation walkthrough.</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L38" s="8" t="str">
-        <x:v>Moderation state changes need durable admin_actions audit records.</x:v>
+        <x:v>Admin decision audit remains in admin_actions; latest-check summary is read-only service-role admin context and shows only reason codes/score, not raw input.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -4869,19 +4869,19 @@
         <x:v>User plan; ai_docs/EXECUTION_PLAN_2026-06-21.md</x:v>
       </x:c>
       <x:c r="H52" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>Needs UX tests</x:v>
+        <x:v>Unit tests + production build</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>Start after PR #66/#67 review/deploy if they exist in current workflow.</x:v>
+        <x:v>V2 started 2026-06-30 with operator reason-summary cards/details. Remaining: full browser QA with seeded disposable report/appeal mutation and queue ergonomics polish.</x:v>
       </x:c>
       <x:c r="K52" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L52" s="8" t="str">
-        <x:v>Audit log every moderation decision.</x:v>
+        <x:v>Operator console continues to rely on admin-only server functions and durable admin_actions for state changes.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -6603,13 +6603,13 @@
         <x:v>Dashboard shows incoming reports, masked targets, reason summary, duplicate strength, and clear actions like confirm risk/reject.</x:v>
       </x:c>
       <x:c r="E21" s="50" t="str">
-        <x:v>P6 v2: detail view, duplicate count, role of Telegram chat, human decision passport.</x:v>
+        <x:v>Closed 2026-06-30: cards/details show latest-check reason summary, score, duplicate strength, privacy and human decision passport.</x:v>
       </x:c>
       <x:c r="F21" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G21" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-06-30: admin helper tests + production build; disposable live mutation walkthrough pending</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="76" customHeight="1">
@@ -6902,13 +6902,13 @@
         <x:v>Cards show target, user story, duplicate signal, reasons, full detail view, privacy explanation, and clear legal-safe decisions.</x:v>
       </x:c>
       <x:c r="E34" s="50" t="str">
-        <x:v>Start after PR #66/#67 review/deploy if they exist in current workflow.</x:v>
+        <x:v>Partial 2026-06-30: reason-summary operator console slice implemented; queue ergonomics and live mutation QA remain.</x:v>
       </x:c>
       <x:c r="F34" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G34" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Partial 2026-06-30: production build passed; full browser/mutation QA pending</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="76" customHeight="1">
@@ -7890,6 +7890,32 @@
         <x:v>Proceed to ADM-002 Dashboard Operator UX v2 / ROAD-001; keep real-audio STT corpus/timing watch after provider/model changes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>QA-2026-06-30-006</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>ADM-002 / ROAD-001 Dashboard Operator UX v2 reason summaries</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>npm run test:run -- src/lib/admin.functions.test.ts; npm run build</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Passed: 1 file / 10 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>ADM-002, ROAD-001</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>Admin listReports now attaches latest target check context from checks by entity_hash. Report cards and detail modal show risk level, score, reason-code labels, check timestamp, AI/rules source and existing duplicate/privacy decision context. No moderation mutation was performed.</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Run disposable live admin mutation walkthrough and continue ROAD-001 queue ergonomics polish.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record admin mutation QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1a0bd4f915cb4dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R764f2920f5ec4925"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9c35f350cb614bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb97f3197ada74ea0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R69a397b234de4796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8a66c8ee28bf4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R85e5ecd8c52a4aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf839a0dcd8574512"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7a0bbe21516748da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0a9e6e3065274ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R81a8f52ad67f40c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rea97ff162c4b44d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>User-story QA in progress: P1 web/Telegram flows, then UX/logistics fixes</x:v>
+        <x:v>ROAD-001 queue ergonomics polish next; then P1/P2 user-story QA and UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified. ROAD-001 Dashboard Operator UX v2 is partial: cards/details now show latest-check reason summaries and legal-safe decision context. Next recommended P1: full admin mutation QA, then ROAD-001 queue ergonomics polish.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, disposable live admin mutation QA, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified. ROAD-001 Dashboard Operator UX v2 is partial: cards/details show latest-check reason summaries and legal-safe decision context; live admin mutations now verify report confirm/reject, appeal remove/keep, audit rows and entity counters. Next recommended P1: ROAD-001 queue ergonomics polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4340,10 +4340,10 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I38" s="8" t="str">
-        <x:v>Unit tests + production build + prior live admin read-only QA</x:v>
+        <x:v>Unit tests + production build + live admin read-only QA + disposable live mutation QA</x:v>
       </x:c>
       <x:c r="J38" s="8" t="str">
-        <x:v>Closed 2026-06-30: report cards/detail view now show latest target check reason summary, score, duplicate signal and human decision passport. Next: disposable live moderation mutation walkthrough.</x:v>
+        <x:v>Closed 2026-06-30: report cards/detail view now show latest target check reason summary, score, duplicate signal and human decision passport. Disposable live mutation QA also passed for report confirm/reject and appeal remove/keep with audit/entity checks.</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str">
         <x:v>P1</x:v>
@@ -4872,10 +4872,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>Unit tests + production build</x:v>
+        <x:v>Unit tests + production build + live disposable admin mutation QA</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>V2 started 2026-06-30 with operator reason-summary cards/details. Remaining: full browser QA with seeded disposable report/appeal mutation and queue ergonomics polish.</x:v>
+        <x:v>V2 started 2026-06-30 with operator reason-summary cards/details. Live admin mutation QA is complete. Remaining: queue ergonomics polish and a fresh browser pass after the queue UI changes.</x:v>
       </x:c>
       <x:c r="K52" s="12" t="str">
         <x:v>P1</x:v>
@@ -6603,13 +6603,13 @@
         <x:v>Dashboard shows incoming reports, masked targets, reason summary, duplicate strength, and clear actions like confirm risk/reject.</x:v>
       </x:c>
       <x:c r="E21" s="50" t="str">
-        <x:v>Closed 2026-06-30: cards/details show latest-check reason summary, score, duplicate strength, privacy and human decision passport.</x:v>
+        <x:v>Closed 2026-06-30: cards/details show latest-check reason summary, score, duplicate strength, privacy and human decision passport; disposable mutation QA passed.</x:v>
       </x:c>
       <x:c r="F21" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G21" s="50" t="str">
-        <x:v>Automated pass 2026-06-30: admin helper tests + production build; disposable live mutation walkthrough pending</x:v>
+        <x:v>Verified 2026-06-30: admin helper tests, production build, read-only admin walkthrough and live disposable mutation QA all passed; cleanup_remaining=0.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="76" customHeight="1">
@@ -6856,13 +6856,13 @@
         <x:v>Main site avoids unnecessary unsafe-inline; embed CSP is documented and intentionally allows partner framing.</x:v>
       </x:c>
       <x:c r="E32" s="50" t="str">
-        <x:v>Remove/soften unsafe-inline where possible and document embed frame-ancestor policy.</x:v>
+        <x:v>Closed 2026-06-30: default embed snippet/preview no longer uses iframe sandbox; /embed/check framing remains controlled by CSP frame-ancestors.</x:v>
       </x:c>
       <x:c r="F32" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G32" s="50" t="str">
-        <x:v>Open 2026-06-29: embed preview sandbox warning needs separate embed-origin/CORS hardening decision</x:v>
+        <x:v>Verified 2026-06-30: ERR-2026-06-29-003 is closed. Keep CSP allowlist checks in release checklist after embed deployment changes.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="76" customHeight="1">
@@ -6902,13 +6902,13 @@
         <x:v>Cards show target, user story, duplicate signal, reasons, full detail view, privacy explanation, and clear legal-safe decisions.</x:v>
       </x:c>
       <x:c r="E34" s="50" t="str">
-        <x:v>Partial 2026-06-30: reason-summary operator console slice implemented; queue ergonomics and live mutation QA remain.</x:v>
+        <x:v>Partial 2026-06-30: reason-summary operator console slice implemented and live admin mutation QA passed; queue ergonomics remain.</x:v>
       </x:c>
       <x:c r="F34" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G34" s="50" t="str">
-        <x:v>Partial 2026-06-30: production build passed; full browser/mutation QA pending</x:v>
+        <x:v>Partial 2026-06-30: production build and live mutation QA passed; browser pass should be repeated after queue ergonomics polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="76" customHeight="1">
@@ -7682,239 +7682,143 @@
         <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>QA-2026-06-30-005</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
-      <x:c r="C14" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H14" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
+      <x:c r="C14" s="4" t="str">
+        <x:v>TG-014 Voice STT / Voice-in tuning</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/format.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/risk/voice-transcription.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/router.test.ts src/lib/telegram/bot-qa-matrix.test.ts</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>Passed: 7 files / 332 tests</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>TG-014</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>Voice result surfaces a sanitized hook phrase from transcript preview; raw URLs, @handles and long digit runs stay hidden; high-risk cards show the hook; Telegram voice, formatter, risk voice/rule, webhook, router and bot QA matrix suites passed.</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>Proceed to ADM-002 Dashboard Operator UX v2 / ROAD-001; keep real-audio STT corpus/timing watch after provider/model changes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="4" t="str">
+        <x:v>QA-2026-06-30-006</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
-      <x:c r="C15" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H15" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="C15" s="4" t="str">
+        <x:v>ADM-002 / ROAD-001 Dashboard Operator UX v2 reason summaries</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>npm run test:run -- src/lib/admin.functions.test.ts; npm run build</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>Passed: 1 file / 10 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>ADM-002, ROAD-001</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>Admin listReports now attaches latest target check context from checks by entity_hash. Report cards and detail modal show risk level, score, reason-code labels, check timestamp, AI/rules source and existing duplicate/privacy decision context. No moderation mutation was performed.</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>Completed by QA-2026-06-30-007; continue ROAD-001 queue ergonomics polish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="54" customHeight="1">
+      <x:c r="A16" s="4" t="str">
+        <x:v>QA-2026-06-30-007</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
         <x:v>2026-06-30</x:v>
       </x:c>
-      <x:c r="C16" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H16" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Disposable live admin mutation QA</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>railway run npm exec vite-node -- .codex-tmp/admin-mutation-qa/admin-mutation-qa.ts</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>Passed: live disposable rows mutated and cleaned</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>ADM-002, ROAD-001, WEB-Admin, CORE-009</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>Production service-role QA used existing admin audit FK and synthetic URL targets only. Covered report confirm/reject, appeal remove/keep, admin_actions audit rows, entity moderation status/risk/report_count; cleanup_remaining=0 and no secrets were printed.</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>Proceed to ROAD-001 queue ergonomics polish; keep mutation QA disposable or port it to a guarded reusable smoke later.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H17" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
-      </x:c>
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F18" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G18" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H18" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
-      </x:c>
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E19" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F19" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G19" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H19" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
-      </x:c>
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>QA-2026-06-30-004</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>Production QA smoke queue cleanup</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>Guarded Supabase service-role SQL cleanup for qa-*smoke-2026-06-30.invalid reports/appeals/entities; railway run npm run prod:smoke</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Passed: synthetic QA queue records closed</x:v>
-      </x:c>
-      <x:c r="F20" t="str">
-        <x:v>WEB-003, WEB-007, WEB-Admin, Operator UX</x:v>
-      </x:c>
-      <x:c r="G20" t="str">
-        <x:v>Guard required exactly 2 QA reports, 2 QA appeals and 2 QA entities before mutation. Cleanup marked QA reports rejected, QA appeals rejected, QA entities rejected/unknown/report_count=0. Post-check: QA new reports=0, QA open appeals=0, QA new entities=0; production smoke passed.</x:v>
-      </x:c>
-      <x:c r="H20" t="str">
-        <x:v>Proceed to UX/logistics fixes. Remaining new reports are non-QA operator queue items.</x:v>
-      </x:c>
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" t="str">
-        <x:v>QA-2026-06-30-005</x:v>
-      </x:c>
-      <x:c r="B21" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="C21" t="str">
-        <x:v>TG-014 Voice STT / Voice-in tuning</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
-        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/format.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/risk/voice-transcription.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/router.test.ts src/lib/telegram/bot-qa-matrix.test.ts</x:v>
-      </x:c>
-      <x:c r="E21" t="str">
-        <x:v>Passed: 7 files / 332 tests</x:v>
-      </x:c>
-      <x:c r="F21" t="str">
-        <x:v>TG-014</x:v>
-      </x:c>
-      <x:c r="G21" t="str">
-        <x:v>Voice result surfaces a sanitized hook phrase from transcript preview; raw URLs, @handles and long digit runs stay hidden; high-risk cards show the hook; Telegram voice, formatter, risk voice/rule, webhook, router and bot QA matrix suites passed.</x:v>
-      </x:c>
-      <x:c r="H21" t="str">
-        <x:v>Proceed to ADM-002 Dashboard Operator UX v2 / ROAD-001; keep real-audio STT corpus/timing watch after provider/model changes.</x:v>
-      </x:c>
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" t="str">
-        <x:v>QA-2026-06-30-006</x:v>
-      </x:c>
-      <x:c r="B22" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="C22" t="str">
-        <x:v>ADM-002 / ROAD-001 Dashboard Operator UX v2 reason summaries</x:v>
-      </x:c>
-      <x:c r="D22" t="str">
-        <x:v>npm run test:run -- src/lib/admin.functions.test.ts; npm run build</x:v>
-      </x:c>
-      <x:c r="E22" t="str">
-        <x:v>Passed: 1 file / 10 tests; production build passed</x:v>
-      </x:c>
-      <x:c r="F22" t="str">
-        <x:v>ADM-002, ROAD-001</x:v>
-      </x:c>
-      <x:c r="G22" t="str">
-        <x:v>Admin listReports now attaches latest target check context from checks by entity_hash. Report cards and detail modal show risk level, score, reason-code labels, check timestamp, AI/rules source and existing duplicate/privacy decision context. No moderation mutation was performed.</x:v>
-      </x:c>
-      <x:c r="H22" t="str">
-        <x:v>Run disposable live admin mutation walkthrough and continue ROAD-001 queue ergonomics polish.</x:v>
-      </x:c>
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(admin): prioritize operator queue
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R85e5ecd8c52a4aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf839a0dcd8574512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7a0bbe21516748da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0a9e6e3065274ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R81a8f52ad67f40c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rea97ff162c4b44d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1f30309e8f9d4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbd886c2764be481b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5352f23196a24bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rcb7856541aa04d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0186fc9c8fda49d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rae1d5d0246044b9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>ROAD-001 queue ergonomics polish next; then P1/P2 user-story QA and UX/logistics fixes</x:v>
+        <x:v>ROAD-001 browser/live admin queue QA; then P1/P2 user-story QA and UX/logistics fixes</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, disposable live admin mutation QA, QA smoke cleanup, WEB-003, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified. ROAD-001 Dashboard Operator UX v2 is partial: cards/details show latest-check reason summaries and legal-safe decision context; live admin mutations now verify report confirm/reject, appeal remove/keep, audit rows and entity counters. Next recommended P1: ROAD-001 queue ergonomics polish.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, disposable live admin mutation QA, queue ergonomics, QA smoke cleanup, WEB-003, ROAD-001, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified in code. ROAD-001 still needs browser/live queue QA with seeded reports. Next recommended P1: browser/live admin queue pass, then continue P1/P2 user-story QA and UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2649,7 +2649,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2662,7 +2662,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4869,19 +4869,19 @@
         <x:v>User plan; ai_docs/EXECUTION_PLAN_2026-06-21.md</x:v>
       </x:c>
       <x:c r="H52" s="15" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>Unit tests + production build + live disposable admin mutation QA</x:v>
+        <x:v>Unit tests + production build + scoped eslint + live disposable admin mutation QA</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>V2 started 2026-06-30 with operator reason-summary cards/details. Live admin mutation QA is complete. Remaining: queue ergonomics polish and a fresh browser pass after the queue UI changes.</x:v>
+        <x:v>Implemented 2026-06-30: queue priority model, priority/newest sorting, queue summary counts and review-next/needs-context badges are live in the admin report list. Next: browser/live admin queue QA with seeded reports after deploy.</x:v>
       </x:c>
       <x:c r="K52" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L52" s="8" t="str">
-        <x:v>Operator console continues to rely on admin-only server functions and durable admin_actions for state changes.</x:v>
+        <x:v>Queue priority uses only admin-only redacted report context, latest-check score/reason metadata and confirmed report counts; it adds no new public exposure or moderation mutation path.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -6902,13 +6902,13 @@
         <x:v>Cards show target, user story, duplicate signal, reasons, full detail view, privacy explanation, and clear legal-safe decisions.</x:v>
       </x:c>
       <x:c r="E34" s="50" t="str">
-        <x:v>Partial 2026-06-30: reason-summary operator console slice implemented and live admin mutation QA passed; queue ergonomics remain.</x:v>
+        <x:v>Implemented 2026-06-30: reason-summary operator console plus queue priority/sort/summary badges are in code; browser/live queue QA remains.</x:v>
       </x:c>
       <x:c r="F34" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G34" s="50" t="str">
-        <x:v>Partial 2026-06-30: production build and live mutation QA passed; browser pass should be repeated after queue ergonomics polish.</x:v>
+        <x:v>Automated pass 2026-06-30: queue helper tests, admin helper tests, production build and scoped eslint passed. Browser/live queue pass pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="76" customHeight="1">
@@ -7760,15 +7760,31 @@
         <x:v>Proceed to ROAD-001 queue ergonomics polish; keep mutation QA disposable or port it to a guarded reusable smoke later.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17"/>
-      <x:c r="B17"/>
-      <x:c r="C17"/>
-      <x:c r="D17"/>
-      <x:c r="E17"/>
-      <x:c r="F17"/>
-      <x:c r="G17"/>
-      <x:c r="H17"/>
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" s="4" t="str">
+        <x:v>QA-2026-06-30-008</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>ROAD-001 queue ergonomics polish</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>npm run test:run -- src/lib/admin-operator-queue.test.ts src/lib/admin.functions.test.ts; npm run build; npx eslint src/routes/admin.tsx src/lib/admin-operator-queue.ts src/lib/admin-operator-queue.test.ts</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>Passed: 2 files / 17 tests; production build passed; scoped eslint passed</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>ROAD-001, ADM-002, WEB-Admin</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>Admin queue now has priority/newest sorting, queue summary counts, review-next/needs-context badges and pure priority helper coverage, including null risk-score handling. `npm run lint -- ...` was not usable because the repo script expands to eslint . and hit unrelated existing CRLF/prettier issues.</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>Run browser/live admin queue QA with seeded reports after deploy; keep full repo lint cleanup separate from this feature slice.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18"/>

</xml_diff>

<commit_message>
docs: record operator queue live QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1f30309e8f9d4310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbd886c2764be481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5352f23196a24bf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rcb7856541aa04d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0186fc9c8fda49d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rae1d5d0246044b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R373a401114534c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra6d3a7f1744e432a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6d633ecbcd8f4830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ref273b6dcaa9474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R4449c10ac6f84dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R28542bc98f964ca6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>ROAD-001 browser/live admin queue QA; then P1/P2 user-story QA and UX/logistics fixes</x:v>
+        <x:v>P1/P2 user-story QA and UX/logistics fixes; embed sandbox architecture decision remains open</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, disposable live admin mutation QA, queue ergonomics, QA smoke cleanup, WEB-003, ROAD-001, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified in code. ROAD-001 still needs browser/live queue QA with seeded reports. Next recommended P1: browser/live admin queue pass, then continue P1/P2 user-story QA and UX/logistics fixes.</x:v>
+        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, disposable live admin mutation QA, queue ergonomics, QA smoke cleanup, WEB-003, ROAD-001, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified in code. ROAD-001 browser/live queue QA passed 2026-06-30 with disposable admin and seeded reports; cleanupRemainingReports=0. Next recommended P1: continue web/Telegram user-story QA, then UX/logistics fixes; keep embed sandbox architecture note as a separate product/security decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4872,16 +4872,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>Unit tests + production build + scoped eslint + live disposable admin mutation QA</x:v>
+        <x:v>Unit tests + production build + scoped eslint + live disposable admin mutation QA + browser/live seeded queue QA</x:v>
       </x:c>
       <x:c r="J52" s="8" t="str">
-        <x:v>Implemented 2026-06-30: queue priority model, priority/newest sorting, queue summary counts and review-next/needs-context badges are live in the admin report list. Next: browser/live admin queue QA with seeded reports after deploy.</x:v>
+        <x:v>Closed browser/live queue QA 2026-06-30: disposable admin and seeded production reports verified priority/newest sorting, summary counts, review-next/needs-context badges and detail modal. cleanupRemainingReports=0.</x:v>
       </x:c>
       <x:c r="K52" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L52" s="8" t="str">
-        <x:v>Queue priority uses only admin-only redacted report context, latest-check score/reason metadata and confirmed report counts; it adds no new public exposure or moderation mutation path.</x:v>
+        <x:v>Queue priority uses only admin-only redacted report context, latest-check score/reason metadata and confirmed report counts; disposable browser QA rows and auth user were cleaned after verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -6902,13 +6902,13 @@
         <x:v>Cards show target, user story, duplicate signal, reasons, full detail view, privacy explanation, and clear legal-safe decisions.</x:v>
       </x:c>
       <x:c r="E34" s="50" t="str">
-        <x:v>Implemented 2026-06-30: reason-summary operator console plus queue priority/sort/summary badges are in code; browser/live queue QA remains.</x:v>
+        <x:v>Implemented + browser/live verified 2026-06-30: reason-summary console and queue priority/sort/summary badges passed seeded admin QA.</x:v>
       </x:c>
       <x:c r="F34" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G34" s="50" t="str">
-        <x:v>Automated pass 2026-06-30: queue helper tests, admin helper tests, production build and scoped eslint passed. Browser/live queue pass pending.</x:v>
+        <x:v>Automated pass 2026-06-30: queue helper tests, admin helper tests, production build and scoped eslint passed. Browser/live pass 2026-06-30: disposable admin login, seeded reports, priority/newest sorting, summary counters, badges, detail modal and console errors=0; cleanupRemainingReports=0.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="76" customHeight="1">
@@ -7787,14 +7787,30 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
-      <x:c r="C18"/>
-      <x:c r="D18"/>
-      <x:c r="E18"/>
-      <x:c r="F18"/>
-      <x:c r="G18"/>
-      <x:c r="H18"/>
+      <x:c r="A18" s="4" t="str">
+        <x:v>QA-2026-06-30-009</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="str">
+        <x:v>ROAD-001 browser/live admin queue QA with seeded reports</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="str">
+        <x:v>railway run node .codex-tmp/road001-live-qa/road001-live-qa.mjs seed; railway run npm run dev -- --host 127.0.0.1 --port 4173; Playwright CLI login/admin queue pass; railway run node .codex-tmp/road001-live-qa/road001-live-qa.mjs cleanup</x:v>
+      </x:c>
+      <x:c r="E18" s="4" t="str">
+        <x:v>Passed: disposable admin login, priority/newest sorting, summary badges, detail modal, console errors=0; cleanupRemainingReports=0</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>ROAD-001, ADM-002, WEB-Admin</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>Seeded 4 production disposable reports. Priority mode put high-risk older report first and repeated suspicious report second; newest mode put context-gap report first. Summary showed total 6, review-next 2, needs-context 1, repeats 1. Detail modal showed passport, target signals and reason timeline. Screenshot: output/playwright/road001-admin-queue-live.png.</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>Proceed to P1/P2 user-story QA and UX/logistics fixes; keep embed sandbox architecture note separate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19"/>

</xml_diff>

<commit_message>
test(web): record production user-story qa
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R373a401114534c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra6d3a7f1744e432a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6d633ecbcd8f4830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ref273b6dcaa9474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R4449c10ac6f84dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R28542bc98f964ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7832be319be74d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2122d7fd742941db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcce34b1cf8d74b47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R038eff48a27b4957"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2124310edce34dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R73b294f50dd9487a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>P1/P2 user-story QA and UX/logistics fixes; embed sandbox architecture decision remains open</x:v>
+        <x:v>P1 Telegram/private-group user-story QA and UX/logistics fixes; Voice-out human audio review/compression remains follow-up</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog, live Telegram, Admin Operator read-only walkthrough, disposable live admin mutation QA, queue ergonomics, QA smoke cleanup, WEB-003, ROAD-001, ROAD-002, ADM-001, TG-005, TG-010, TG-014 and ADM-002 are implemented/verified in code. ROAD-001 browser/live queue QA passed 2026-06-30 with disposable admin and seeded reports; cleanupRemainingReports=0. Next recommended P1: continue web/Telegram user-story QA, then UX/logistics fixes; keep embed sandbox architecture note as a separate product/security decision.</x:v>
+        <x:v>Security backlog closed. Live production smoke, live Telegram synthetic update, P1 web homepage high-risk result, report success path, appeal success path and admin moderation smoke passed 2026-06-30. QA marker QA-P1-WEB-20260630111649 was cleaned from reports, appeals, entities, audit actions and checks. Next recommended P1: Telegram/private-group user-story QA or UX/logistics fixes; keep Voice-out human audio review/compression as a separate follow-up.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6517,7 +6517,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G17" s="50" t="str">
-        <x:v>Browser QA 2026-06-29: graceful unavailable fallback + sanitized console verified; full live result pending configured env</x:v>
+        <x:v>Production browser pass 2026-06-30: homepage high-risk result passed against configured env.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="76" customHeight="1">
@@ -6540,7 +6540,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G18" s="50" t="str">
-        <x:v>Browser QA 2026-06-29: report fallback + sanitized console verified; full live submit pending configured env</x:v>
+        <x:v>Production browser pass 2026-06-30: report success path passed; synthetic report moderated/rejected and cleaned.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="76" customHeight="1">
@@ -6563,7 +6563,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G19" s="50" t="str">
-        <x:v>Browser QA 2026-06-29: appeal fallback + sanitized console verified; admin QA pending</x:v>
+        <x:v>Production browser pass 2026-06-30: appeal success path plus admin keep-reputation moderation passed; synthetic appeal/audit cleaned.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="76" customHeight="1">
@@ -7813,14 +7813,30 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
-      <x:c r="C19"/>
-      <x:c r="D19"/>
-      <x:c r="E19"/>
-      <x:c r="F19"/>
-      <x:c r="G19"/>
-      <x:c r="H19"/>
+      <x:c r="A19" t="str">
+        <x:v>QA-2026-06-30-010</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>P1 production web user-story smoke</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Playwright browser against production homepage, /report and /appeal; railway run npx vite-node scripts/prod-admin-moderation-smoke.ts --marker QA-P1-WEB-20260630111649; targeted service-role check cleanup</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Passed: production web flows and admin moderation smoke; QA rows cleaned</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>WEB-002, WEB-003, WEB-007, ADM-002, CORE-008</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>Marker QA-P1-WEB-20260630111649. Homepage showed high-risk result; report and appeal success pages rendered. Admin smoke rejected the synthetic report, kept/rejected the synthetic appeal, verified audit actions, and cleaned synthetic rows; remaining synthetic check row was deleted.</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Next P1: Telegram/private-group user-story QA or UX/logistics fixes; keep Voice-out human audio review/compression as follow-up.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20"/>

</xml_diff>

<commit_message>
test(telegram): add production scope smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7832be319be74d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2122d7fd742941db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcce34b1cf8d74b47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R038eff48a27b4957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2124310edce34dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R73b294f50dd9487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re9bf55f89e9e4c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb4e63c526c8741d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R523b6b47cc884eee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R55448c989b324fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R65ab792409154c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra989ec2834b74141"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>P1 Telegram/private-group user-story QA and UX/logistics fixes; Voice-out human audio review/compression remains follow-up</x:v>
+        <x:v>Continue remaining P1 Telegram live QA: image/QR, high-risk Guardian Angel, conversational follow-ups; then UX/logistics fixes. Voice-out human audio review/compression remains follow-up</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed. Live production smoke, live Telegram synthetic update, P1 web homepage high-risk result, report success path, appeal success path and admin moderation smoke passed 2026-06-30. QA marker QA-P1-WEB-20260630111649 was cleaned from reports, appeals, entities, audit actions and checks. Next recommended P1: Telegram/private-group user-story QA or UX/logistics fixes; keep Voice-out human audio review/compression as a separate follow-up.</x:v>
+        <x:v>Security backlog closed. Production was redeployed on 2026-06-30 (Railway deployment 53f77ca3...) after the previous production app lagged behind current session chatScope code. New prod:telegram-scope-smoke verifies private /report session scope and supergroup callback reset without reusing private state; synthetic telegram_sessions and telegram_webhook_updates rows were cleaned. General prod:smoke also passed. Next recommended P1: live Telegram image/QR and high-risk Guardian Angel flows, then UX/logistics fixes; keep Voice-out human audio review/compression separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6465,13 +6465,13 @@
         <x:v>Webhook secret is checked, updates are deduped, and failures degrade safely.</x:v>
       </x:c>
       <x:c r="E15" s="50" t="str">
-        <x:v>Address deep-scan finding: dedupe fails open when shared claim storage unavailable.</x:v>
+        <x:v>Closed 2026-06-30: production initially lagged current chatScope code; redeployed current app and verified private/group session scoping with synthetic webhook updates.</x:v>
       </x:c>
       <x:c r="F15" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G15" s="50" t="str">
-        <x:v>Automated pass 2026-06-29; production webhook smoke pending</x:v>
+        <x:v>Production pass 2026-06-30: prod:telegram-scope-smoke passed after Railway deployment 53f77ca3; general prod:smoke passed; synthetic session/dedup rows cleaned.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="76" customHeight="1">

</xml_diff>

<commit_message>
test(telegram): add live qr guardian smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re9bf55f89e9e4c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb4e63c526c8741d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R523b6b47cc884eee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R55448c989b324fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R65ab792409154c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra989ec2834b74141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Raaba41f9074144c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R35ae6fb7ca3f4b1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rdcd5ce4b2a464a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R39556be3f69e4bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf2c3dc4f2fbb4604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R62420eff32aa42b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1 Telegram live QA: image/QR, high-risk Guardian Angel, conversational follow-ups; then UX/logistics fixes. Voice-out human audio review/compression remains follow-up</x:v>
+        <x:v>Continue remaining P1 Telegram user-story QA: start/check/passport/conversational live RU/UZ/EN and false-positive flows; then UX/logistics fixes. Voice-out human audio review/compression remains follow-up.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed. Production was redeployed on 2026-06-30 (Railway deployment 53f77ca3...) after the previous production app lagged behind current session chatScope code. New prod:telegram-scope-smoke verifies private /report session scope and supergroup callback reset without reusing private state; synthetic telegram_sessions and telegram_webhook_updates rows were cleaned. General prod:smoke also passed. Next recommended P1: live Telegram image/QR and high-risk Guardian Angel flows, then UX/logistics fixes; keep Voice-out human audio review/compression separate.</x:v>
+        <x:v>Security backlog closed. Production was redeployed on 2026-06-30 (Railway deployment 53f77ca3...) after the previous production app lagged behind current session chatScope code. prod:telegram-scope-smoke verifies private/group session scope; prod:telegram-live-qa-smoke now verifies high-risk Guardian text and real Telegram QR photo/file_id decode through the moderation chat, with synthetic checks/sessions/dedup rows and uploaded QA photo cleaned. General prod:smoke also passed. Remaining P1 is conversation/start/check/passport/false-positive user-story QA before UX/logistics fixes; keep Voice-out human audio review/compression separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3133,7 +3133,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L6" s="8" t="str">
-        <x:v>2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups.</x:v>
+        <x:v>2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups. 2026-06-30: .claude QA feedback rechecked in focused suite: acknowledgement replies, confirmation-request follow-ups and word-boundary voice transcript previews are covered; `npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/check-followup.test.ts` passed 4 files / 127 tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3317,13 +3317,13 @@
         <x:v>Unit tests + integration tests + live QA</x:v>
       </x:c>
       <x:c r="J11" s="8" t="str">
-        <x:v>Keep live Telegram image/QR fixture smoke after image-copy or parser changes; continue production timing tuning from logs.</x:v>
+        <x:v>Keep prod:telegram-live-qa-smoke in release checklist after image-copy, QR parser or Telegram file API changes; continue production timing tuning from logs.</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L11" s="8" t="str">
-        <x:v>2026-06-30: TG-010 implemented/verified. QR/image precision now separates menu/info QR, Telegram login/device/2FA QR, payment QR, private invite links, bot/captcha/giveaway screenshots, wallet/DeFi urgency and unreadable images. Added regression that private Telegram invite OCR is scored as suspicious_invite_link while the real invite code is redacted and not stored in image check input.</x:v>
+        <x:v>2026-06-30: TG-010 implemented/verified. QR/image precision now separates menu/info QR, Telegram login/device/2FA QR, payment QR, private invite links, bot/captcha/giveaway screenshots, wallet/DeFi urgency and unreadable images. Added regression that private Telegram invite OCR is scored as suspicious_invite_link while the real invite code is redacted and not stored in image check input. 2026-06-30 production pass: prod:telegram-live-qa-smoke uploaded a synthetic QR photo to the moderation chat, processed the real Telegram file_id through download + pixel QR decode, verified asks_to_scan_qr high-risk safe session metadata, and cleaned synthetic checks/session/dedup/message artifacts.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -3770,16 +3770,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I23" s="8" t="str">
-        <x:v>Manual QA</x:v>
+        <x:v>Unit + live QA</x:v>
       </x:c>
       <x:c r="J23" s="8" t="str">
-        <x:v>Strengthen stop-card with one primary action and optional timed pause.</x:v>
+        <x:v>Production high-risk Guardian text smoke passed; continue copy polish for one-primary-action stop-card.</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="L23" s="8" t="str">
-        <x:v>Auto-prompt should be clearly labeled as not a new check.</x:v>
+        <x:v>Auto-prompt should be clearly labeled as not a new check. 2026-06-30 production pass: prod:telegram-live-qa-smoke sent a synthetic verification-code/CVV text through webhook, verified high-risk lastCheck + Guardian safe metadata in session, and cleaned synthetic rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6212,13 +6212,13 @@
         <x:v>Known follow-up intents reuse last result/session context and answer without changing the verdict.</x:v>
       </x:c>
       <x:c r="E4" s="50" t="str">
-        <x:v>Implement narrow AI conversational layer over last check for unsupported clarifying questions.</x:v>
+        <x:v>Keep live RU/UZ/EN phrase QA and open-ended conversational layer as follow-up; current .claude acknowledgement/confirmation/voice-preview gaps are covered by focused tests.</x:v>
       </x:c>
       <x:c r="F4" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G4" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-06-30: acknowledgements, confirmation requests, orphan follow-ups and voice transcript preview trimming covered; live conversational follow-up QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="76" customHeight="1">
@@ -6327,13 +6327,13 @@
         <x:v>Images are OCRed/decoded in memory, classified into visual categories, and only dangerous QR/login/payment/APK/coded flows raise risk.</x:v>
       </x:c>
       <x:c r="E9" s="50" t="str">
-        <x:v>P3: QR/Image Precision v2 must separate menu, Telegram login, payment, invite, bot/captcha, unreadable.</x:v>
+        <x:v>Closed 2026-06-30: production live QR image smoke covered real Telegram sendPhoto/file_id download + pixel QR decode; keep smoke in release checklist.</x:v>
       </x:c>
       <x:c r="F9" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G9" s="50" t="str">
-        <x:v>Automated pass 2026-06-29; live Telegram image/QR QA pending</x:v>
+        <x:v>Production pass 2026-06-30: prod:telegram-live-qa-smoke uploaded synthetic QR photo to moderation chat, verified high-risk QR session/guardian safe metadata, and cleaned checks/session/dedup/message artifacts.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="76" customHeight="1">
@@ -7238,7 +7238,7 @@
         <x:v>After high risk, the bot should guide the user to one safe next step; missing the follow-up weakens emergency UX.</x:v>
       </x:c>
       <x:c r="F6" s="50" t="str">
-        <x:v>Verified 2026-06-29: `webhook.integration.test.ts -t decoded QR|Guardian Angel|forwarded image-post` passed, plus Guardian Angel/follow-up suites passed 2 files / 13 tests.</x:v>
+        <x:v>Verified 2026-06-29: `webhook.integration.test.ts -t decoded QR|Guardian Angel|forwarded image-post` passed, plus Guardian Angel/follow-up suites passed 2 files / 13 tests. Production re-verified 2026-06-30: prod:telegram-live-qa-smoke passed the high-risk Guardian text path and cleanup.</x:v>
       </x:c>
       <x:c r="G6" s="566" t="str">
         <x:v>P1</x:v>
@@ -7839,14 +7839,30 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20"/>
-      <x:c r="B20"/>
-      <x:c r="C20"/>
-      <x:c r="D20"/>
-      <x:c r="E20"/>
-      <x:c r="F20"/>
-      <x:c r="G20"/>
-      <x:c r="H20"/>
+      <x:c r="A20" t="str">
+        <x:v>QA-2026-06-30-011</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>P1 production Telegram QR + Guardian live smoke</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>npx eslint scripts/prod-telegram-live-qa-smoke.ts --quiet; npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/check-followup.test.ts; railway run npm run prod:telegram-live-qa-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Passed: scoped eslint; 4 files / 127 tests; production Telegram live QA smoke; general prod:smoke</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>TG-005, TG-010, TG-014, TG-022, CORE-008</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Live smoke used synthetic Telegram users and TELEGRAM_MODERATION_CHAT_ID. High-risk verification-code/CVV text produced safe lastCheck + Guardian metadata. Synthetic payme QR photo went through real Telegram sendPhoto/file_id download and pixel QR decode, then cleanup removed checks, sessions, dedup rows and uploaded QA message.</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Continue remaining P1 Telegram user-story QA: start/check/passport/conversational live RU/UZ/EN and false-positive flows; keep Voice-out audio review/compression separate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21"/>

</xml_diff>

<commit_message>
test(telegram): add user story smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Raaba41f9074144c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R35ae6fb7ca3f4b1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rdcd5ce4b2a464a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R39556be3f69e4bb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf2c3dc4f2fbb4604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R62420eff32aa42b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R8854a106d5354f10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R969dc35f1fc54758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcebe66460a1943e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6508a299792a4b55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R20f5e79d6328405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rae2dbf5e85e54907"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1 Telegram user-story QA: start/check/passport/conversational live RU/UZ/EN and false-positive flows; then UX/logistics fixes. Voice-out human audio review/compression remains follow-up.</x:v>
+        <x:v>Proceed to UX/logistics fixes; Voice-out real RU/UZ/EN .ogg SOS assets/audio compression remain separate follow-up.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed. Production was redeployed on 2026-06-30 (Railway deployment 53f77ca3...) after the previous production app lagged behind current session chatScope code. prod:telegram-scope-smoke verifies private/group session scope; prod:telegram-live-qa-smoke now verifies high-risk Guardian text and real Telegram QR photo/file_id decode through the moderation chat, with synthetic checks/sessions/dedup rows and uploaded QA photo cleaned. General prod:smoke also passed. Remaining P1 is conversation/start/check/passport/false-positive user-story QA before UX/logistics fixes; keep Voice-out human audio review/compression separate.</x:v>
+        <x:v>Security backlog closed. Production was redeployed on 2026-06-30 (Railway deployment 53f77ca3...) after the previous production app lagged behind current session chatScope code. prod:telegram-scope-smoke verifies private/group session scope; prod:telegram-live-qa-smoke now verifies high-risk Guardian text and real Telegram QR photo/file_id decode through the moderation chat, with synthetic checks/sessions/dedup rows and uploaded QA photo cleaned. General prod:smoke also passed. Remaining P1 is conversation/start/check/passport/false-positive user-story QA before UX/logistics fixes; keep Voice-out human audio review/compression separate. 2026-06-30: prod:telegram-user-story-smoke added and passed. It covers /start, RU/UZ/EN language callbacks, phone passport, benign delivery false-positive and RU/UZ/EN acknowledgement/confirmation follow-ups, with synthetic checks/sessions/dedup cleanup. General prod:smoke also passed after the run.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2972,16 +2972,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I2" s="8" t="str">
-        <x:v>Unit + live bot QA evidence</x:v>
+        <x:v>Unit + live production smoke</x:v>
       </x:c>
       <x:c r="J2" s="8" t="str">
-        <x:v>Re-test that /call or urgent help remains the most visible path on mobile.</x:v>
+        <x:v>Live /start and RU/UZ/EN language callback smoke passed; keep /call/urgent-help prominence on mobile in UX polish.</x:v>
       </x:c>
       <x:c r="K2" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L2" s="8" t="str">
-        <x:v>Do not expose secrets or internal admin links in public menu text.</x:v>
+        <x:v>Do not expose secrets or internal admin links in public menu text. 2026-06-30 production pass: prod:telegram-user-story-smoke accepted /start and persisted ru/uz/en language callbacks with synthetic sessions cleaned.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3010,16 +3010,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I3" s="8" t="str">
-        <x:v>Broad unit/property tests</x:v>
+        <x:v>Broad unit/property tests + live production smoke</x:v>
       </x:c>
       <x:c r="J3" s="8" t="str">
-        <x:v>Regression test friendly delivery voice text and crypto/investment false positives.</x:v>
+        <x:v>Friendly delivery false-positive production smoke passed in RU/UZ/EN sessions; keep crypto/investment false positives in regression list.</x:v>
       </x:c>
       <x:c r="K3" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L3" s="8" t="str">
-        <x:v>Never ask for or echo SMS codes, card details, passwords, seed phrases.</x:v>
+        <x:v>Never ask for or echo SMS codes, card details, passwords, seed phrases. 2026-06-30 production pass: phone passport and benign delivery user-story smoke stayed non-high-risk and cleaned synthetic rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3124,16 +3124,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I6" s="8" t="str">
-        <x:v>Unit tests</x:v>
+        <x:v>Unit tests + live production smoke</x:v>
       </x:c>
       <x:c r="J6" s="8" t="str">
-        <x:v>Keep live Telegram smoke for RU/UZ/EN follow-ups after deploy; extend phrase list only from real transcripts.</x:v>
+        <x:v>RU/UZ/EN acknowledgement and confirmation-request follow-ups passed live smoke; extend phrase list only from real transcripts.</x:v>
       </x:c>
       <x:c r="K6" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L6" s="8" t="str">
-        <x:v>2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups. 2026-06-30: .claude QA feedback rechecked in focused suite: acknowledgement replies, confirmation-request follow-ups and word-boundary voice transcript previews are covered; `npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/check-followup.test.ts` passed 4 files / 127 tests.</x:v>
+        <x:v>2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups. 2026-06-30: .claude QA feedback rechecked in focused suite: acknowledgement replies, confirmation-request follow-ups and word-boundary voice transcript previews are covered; `npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/check-followup.test.ts` passed 4 files / 127 tests. 2026-06-30 production pass: prod:telegram-user-story-smoke verified thanks/confirmation follow-ups after a last delivery check did not create checks in RU/UZ/EN sessions.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3162,16 +3162,16 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="I7" s="8" t="str">
-        <x:v>Unit + live QA</x:v>
+        <x:v>Unit + live phone passport QA</x:v>
       </x:c>
       <x:c r="J7" s="8" t="str">
-        <x:v>P8.1/P8.2: add Telegram Native Passport Coach and username risk heuristics.</x:v>
+        <x:v>Phone passport production smoke passed for a synthetic UZ mobile number; P8.1/P8.2 username coach/heuristics remain.</x:v>
       </x:c>
       <x:c r="K7" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L7" s="8" t="str">
-        <x:v>Do not invent Telegram account age, hidden scam labels, or Telegram complaint history.</x:v>
+        <x:v>Do not invent Telegram account age, hidden scam labels, or Telegram complaint history. 2026-06-30 production pass: synthetic +998 mobile persisted phone lastCheck with valid_uz_phone and no Guardian/high-risk.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6166,13 +6166,13 @@
         <x:v>The bot shows a short calm intro, a prominent urgent-help entry, check/report/family/rules/digest/language actions, and localized command labels.</x:v>
       </x:c>
       <x:c r="E2" s="50" t="str">
-        <x:v>Re-test that /call or urgent help remains the most visible path on mobile.</x:v>
+        <x:v>Closed 2026-06-30: /start accepted and RU/UZ/EN language callbacks persisted in prod smoke; still check /call prominence in mobile UX polish.</x:v>
       </x:c>
       <x:c r="F2" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G2" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Production pass 2026-06-30: prod:telegram-user-story-smoke covered /start and language callbacks with synthetic session cleanup.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="76" customHeight="1">
@@ -6189,13 +6189,13 @@
         <x:v>Input is normalized, redacted where needed, passed through deterministic rules, optionally enriched, and returned as a short risk card with next action.</x:v>
       </x:c>
       <x:c r="E3" s="50" t="str">
-        <x:v>Regression test friendly delivery voice text and crypto/investment false positives.</x:v>
+        <x:v>Closed 2026-06-30 for friendly delivery false-positive live smoke; crypto/investment false-positive regression remains follow-up.</x:v>
       </x:c>
       <x:c r="F3" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G3" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Production pass 2026-06-30: benign delivery checks stayed non-high-risk in RU/UZ/EN sessions; synthetic checks/sessions/dedup rows cleaned.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="76" customHeight="1">
@@ -6212,13 +6212,13 @@
         <x:v>Known follow-up intents reuse last result/session context and answer without changing the verdict.</x:v>
       </x:c>
       <x:c r="E4" s="50" t="str">
-        <x:v>Keep live RU/UZ/EN phrase QA and open-ended conversational layer as follow-up; current .claude acknowledgement/confirmation/voice-preview gaps are covered by focused tests.</x:v>
+        <x:v>Closed 2026-06-30 for acknowledgement/confirmation live smoke; broader open-ended conversational AI layer remains product follow-up.</x:v>
       </x:c>
       <x:c r="F4" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G4" s="50" t="str">
-        <x:v>Automated pass 2026-06-30: acknowledgements, confirmation requests, orphan follow-ups and voice transcript preview trimming covered; live conversational follow-up QA pending.</x:v>
+        <x:v>Automated + production pass 2026-06-30: focused follow-up tests passed and prod:telegram-user-story-smoke verified RU/UZ/EN thanks/confirmation follow-ups created no checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="76" customHeight="1">
@@ -6235,13 +6235,13 @@
         <x:v>The bot shows what is visible, what is unavailable through Bot API, local reputation, official contact matches, and what evidence to send next.</x:v>
       </x:c>
       <x:c r="E5" s="50" t="str">
-        <x:v>P8.1/P8.2: add Telegram Native Passport Coach and username risk heuristics.</x:v>
+        <x:v>Phone passport production smoke passed 2026-06-30; username Native Passport Coach / heuristics remain P2 follow-up.</x:v>
       </x:c>
       <x:c r="F5" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G5" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Production pass 2026-06-30: synthetic +998 mobile produced non-high-risk phone passport with valid_uz_phone and safe session metadata.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="76" customHeight="1">
@@ -7865,14 +7865,30 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21"/>
-      <x:c r="B21"/>
-      <x:c r="C21"/>
-      <x:c r="D21"/>
-      <x:c r="E21"/>
-      <x:c r="F21"/>
-      <x:c r="G21"/>
-      <x:c r="H21"/>
+      <x:c r="A21" t="str">
+        <x:v>QA-2026-06-30-012</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>P1 production Telegram user-story smoke</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>npx eslint scripts/prod-telegram-user-story-smoke.ts --quiet; npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/check-followup.test.ts src/lib/telegram/router.test.ts src/lib/risk/check-core.property.test.ts; railway run npm run prod:telegram-user-story-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>Passed: scoped eslint; 5 files / 198 tests; production Telegram user-story smoke; general prod:smoke</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>TG-001, TG-002, TG-005, TG-006, CORE-008</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Live smoke used synthetic Telegram users and TELEGRAM_MODERATION_CHAT_ID. /start accepted; ru/uz/en language callbacks persisted; synthetic +998 phone produced non-high-risk phone passport; RU/UZ/EN benign delivery checks stayed non-high-risk and thanks/confirmation follow-ups created no checks; cleanup removed checks, sessions and dedup rows.</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Proceed to UX/logistics fixes. Voice-out real RU/UZ/EN .ogg assets for SOS scenarios remain separate follow-up.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22"/>

</xml_diff>

<commit_message>
feat(report): surface duplicate signals to operators
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R8854a106d5354f10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R969dc35f1fc54758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcebe66460a1943e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6508a299792a4b55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R20f5e79d6328405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rae2dbf5e85e54907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdb894b5f97864f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R00748ecac8ec4e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R06da55d1f87c4628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R4c2951cbc099459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R3ec0400bf218440c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R886c9c458d0943ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2609,7 +2609,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
-        <x:v>2026-06-30</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
         <x:v>58</x:v>
@@ -2618,10 +2618,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Proceed to UX/logistics fixes; Voice-out real RU/UZ/EN .ogg SOS assets/audio compression remain separate follow-up.</x:v>
+        <x:v>Continue UX/logistics fixes; next P2 Telegram username/native-passport heuristics or Voice-out human audio review/compression. Report duplicate-signal polish has automated pass; run production/live report smoke after deploy.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed. Production was redeployed on 2026-06-30 (Railway deployment 53f77ca3...) after the previous production app lagged behind current session chatScope code. prod:telegram-scope-smoke verifies private/group session scope; prod:telegram-live-qa-smoke now verifies high-risk Guardian text and real Telegram QR photo/file_id decode through the moderation chat, with synthetic checks/sessions/dedup rows and uploaded QA photo cleaned. General prod:smoke also passed. Remaining P1 is conversation/start/check/passport/false-positive user-story QA before UX/logistics fixes; keep Voice-out human audio review/compression separate. 2026-06-30: prod:telegram-user-story-smoke added and passed. It covers /start, RU/UZ/EN language callbacks, phone passport, benign delivery false-positive and RU/UZ/EN acknowledgement/confirmation follow-ups, with synthetic checks/sessions/dedup cleanup. General prod:smoke also passed after the run.</x:v>
+        <x:v>Security backlog closed. Production P1 Telegram/web smokes passed on 2026-06-30. 2026-07-01: TG-019 / ROAD-002 report-flow polish refreshed: web success copy is warmer, admin listReports attaches operator-only active target_signal_count and target_last_report_at from reports, and queue priority uses that signal without changing public confirmed target_report_count. Verification passed: scoped eslint, focused admin/report tests and npm run build.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2649,7 +2649,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2662,7 +2662,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -3653,19 +3653,19 @@
         <x:v>.kiro/specs/report-flow-reputation-boundary-v1; .kiro/specs/report-screenshot-evidence-v1</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I20" s="8" t="str">
-        <x:v>Unit + live QA</x:v>
+        <x:v>Unit + focused admin/report tests + build; live Telegram report smoke recommended</x:v>
       </x:c>
       <x:c r="J20" s="8" t="str">
-        <x:v>P7: friendlier final copy, duplicate-as-signal language, show duplicate count in admin.</x:v>
+        <x:v>2026-07-01: P7 polish closed. Web final copy is warmer; duplicate-as-signal language stays non-disclosing; admin uses active target_signal_count and target_last_report_at. Run live Telegram /report smoke after deploy.</x:v>
       </x:c>
       <x:c r="K20" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L20" s="8" t="str">
-        <x:v>Never send raw report text, screenshots, codes, full numbers, or URLs to Telegram moderation chat.</x:v>
+        <x:v>Never send raw report text, screenshots, codes, full numbers, or URLs to Telegram moderation chat. Active raw signal count is operator-only and separate from public confirmed report_count.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -4910,16 +4910,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I53" s="8" t="str">
-        <x:v>Unit tests + build + admin live QA evidence</x:v>
+        <x:v>Unit tests + production build + scoped eslint + admin live QA evidence</x:v>
       </x:c>
       <x:c r="J53" s="8" t="str">
-        <x:v>Keep live Telegram /report confirmation smoke in release checklist after deploy; no implementation blocker remains for Report Flow Polish.</x:v>
+        <x:v>2026-07-01 automated-pass refresh: active duplicate-signal count now comes from report rows for admin priority and latest-signal time; production/live report smoke remains release-check follow-up.</x:v>
       </x:c>
       <x:c r="K53" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L53" s="8" t="str">
-        <x:v>2026-06-30: ROAD-002 implemented. Web quick report uses safe rate-limit feedback and manual-moderation success copy; Telegram /report confirms repeated similar signals can raise review priority without disclosing duplicates; admin cards/detail already show duplicate signal strength and latest signal time.</x:v>
+        <x:v>2026-06-30: ROAD-002 implemented. 2026-07-01: target_signal_count is operator-only, while public target_report_count remains confirmed-only to avoid exposing or inflating unmoderated duplicates.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -6419,13 +6419,13 @@
         <x:v>The flow validates target, description, type, city, loss; accepts 'none'; stores moderated report and masks public alerts.</x:v>
       </x:c>
       <x:c r="E13" s="50" t="str">
-        <x:v>P7: friendlier final copy, duplicate-as-signal language, show duplicate count in admin.</x:v>
+        <x:v>Closed 2026-07-01: warmer final copy, duplicate-as-signal language and admin active signal count/latest report time implemented; live report smoke after deploy remains release check.</x:v>
       </x:c>
       <x:c r="F13" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G13" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: focused admin/report tests passed 3 files / 28 tests; scoped eslint and npm run build passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="76" customHeight="1">
@@ -6925,13 +6925,13 @@
         <x:v>Final copy is warm; duplicate reports say they strengthen signal; admin shows duplicate count and last report time.</x:v>
       </x:c>
       <x:c r="E35" s="50" t="str">
-        <x:v>Implement after dashboard slice or with it if low conflict.</x:v>
+        <x:v>Closed 2026-07-01: web final copy is warm; duplicate reports strengthen operator signal without public disclosure; admin shows active signal count and latest report time.</x:v>
       </x:c>
       <x:c r="F35" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G35" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: focused admin/report tests passed 3 files / 28 tests; scoped eslint and npm run build passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="76" customHeight="1">
@@ -7891,14 +7891,30 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22"/>
-      <x:c r="B22"/>
-      <x:c r="C22"/>
-      <x:c r="D22"/>
-      <x:c r="E22"/>
-      <x:c r="F22"/>
-      <x:c r="G22"/>
-      <x:c r="H22"/>
+      <x:c r="A22" t="str">
+        <x:v>QA-2026-07-01-001</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>ROAD-002 / TG-019 report duplicate-signal UX polish</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>npx eslint src/lib/admin.functions.ts src/lib/admin-operator-queue.ts src/routes/admin.tsx src/routes/report.tsx src/lib/admin.functions.test.ts src/lib/admin-operator-queue.test.ts --quiet; npm run test:run -- src/lib/admin.functions.test.ts src/lib/admin-operator-queue.test.ts src/lib/report.functions.test.ts; npm run build</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Passed: scoped eslint; 3 files / 28 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>TG-019, ROAD-002, WEB-003, ADM-002</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>Web /report success copy now thanks the reporter, explains manual moderation and non-disclosing duplicate-signal value. Admin listReports attaches target_signal_count/target_last_report_at from active reports; operator queue uses target_signal_count for priority while public target_report_count stays confirmed-only.</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Run production/live report submit plus Telegram /report confirmation smoke after deploy; continue next UX/logistics slice or Voice-out audio review/compression.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(telegram): keep username passport coach visible
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdb894b5f97864f27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R00748ecac8ec4e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R06da55d1f87c4628"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R4c2951cbc099459a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R3ec0400bf218440c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R886c9c458d0943ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd91f70924f3d412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R68df5757e8cc4106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3472d01239004dd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R623d2425c9a243b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb3b856a173b244b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2ca4c9674f55490c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2431,9 +2431,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2606,6 +2606,9 @@
       <x:c r="E1" s="588" t="str">
         <x:v>Owner note</x:v>
       </x:c>
+      <x:c r="F1" t="str">
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-007/TG-008 final username passport now preserves Native Passport Coach; QA report regenerated; scoped eslint, 5 files / 83 tests, qa:telegram-report and qa:telegram-visual passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
@@ -2618,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue UX/logistics fixes; next P2 Telegram username/native-passport heuristics or Voice-out human audio review/compression. Report duplicate-signal polish has automated pass; run production/live report smoke after deploy.</x:v>
+        <x:v>Continue UX/logistics fixes; next Profile Screenshot Intelligence (T-007/TG-009) or Voice-out human audio review/compression.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed. Production P1 Telegram/web smokes passed on 2026-06-30. 2026-07-01: TG-019 / ROAD-002 report-flow polish refreshed: web success copy is warmer, admin listReports attaches operator-only active target_signal_count and target_last_report_at from reports, and queue priority uses that signal without changing public confirmed target_report_count. Verification passed: scoped eslint, focused admin/report tests and npm run build.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-007/TG-008 final username passport now preserves Native Passport Coach; QA report regenerated; scoped eslint, 5 files / 83 tests, qa:telegram-report and qa:telegram-visual passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2649,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2675,7 +2678,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -3197,19 +3200,19 @@
         <x:v>Roadmap P8.1 from user feedback</x:v>
       </x:c>
       <x:c r="H8" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I8" s="8" t="str">
-        <x:v>Needs tests</x:v>
+        <x:v>Unit tests + formatter regression + Telegram QA report</x:v>
       </x:c>
       <x:c r="J8" s="8" t="str">
-        <x:v>Design and implement checklist copy for RU/UZ/EN.</x:v>
+        <x:v>2026-07-01: Native Passport Coach is visible in the final formatted username passport: phone country, registration month, not-official label and recent name/photo changes are framed as user-visible Telegram-client checks. Live username smoke remains a release check.</x:v>
       </x:c>
       <x:c r="K8" s="13" t="str">
-        <x:v>P2</x:v>
+        <x:v>Bot still avoids hidden Telegram claims: no SCAM labels, account age, or report-count claims are invented.</x:v>
       </x:c>
       <x:c r="L8" s="8" t="str">
-        <x:v>Must say 'Telegram may show...' not 'I know...'.</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3235,19 +3238,19 @@
         <x:v>Roadmap P8.2</x:v>
       </x:c>
       <x:c r="H9" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I9" s="8" t="str">
-        <x:v>Needs tests</x:v>
+        <x:v>Unit tests + formatter regression + Telegram QA report</x:v>
       </x:c>
       <x:c r="J9" s="8" t="str">
-        <x:v>Add entropy/lookalike tests and ensure weak signals alone do not make high risk.</x:v>
+        <x:v>2026-07-01: Conservative random/generated, brand/support-lookalike and promo wording hints are covered; weak username signs remain visible clues only and do not change the verdict by themselves.</x:v>
       </x:c>
       <x:c r="K9" s="13" t="str">
-        <x:v>P2</x:v>
+        <x:v>Heuristics are presentation-only, source-backed and non-accusatory.</x:v>
       </x:c>
       <x:c r="L9" s="8" t="str">
-        <x:v>False accusation risk: phrase as 'looks unusual', not 'scammer'.</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6258,13 +6261,13 @@
         <x:v>For username checks, the bot tells the user to inspect native Telegram fields and explains risky combinations without claiming hidden access.</x:v>
       </x:c>
       <x:c r="E6" s="50" t="str">
-        <x:v>Design and implement checklist copy for RU/UZ/EN.</x:v>
+        <x:v>Closed 2026-07-01: final Telegram username passport now preserves Native Passport Coach in the user-facing formatted card; live username smoke after deploy remains release check.</x:v>
       </x:c>
       <x:c r="F6" s="567" t="str">
-        <x:v>P2</x:v>
+        <x:v>Automated pass 2026-07-01: public-metadata, formatter, bot QA matrix, Telegram metadata handler and public-post suites passed 5 files / 83 tests; qa:telegram-report and qa:telegram-visual regenerated.</x:v>
       </x:c>
       <x:c r="G6" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>TG-007/TG-008</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="76" customHeight="1">
@@ -6281,13 +6284,13 @@
         <x:v>The passport flags gibberish-like names, brand lookalikes, support/bank impersonation words, and local complaint counts as weak signals.</x:v>
       </x:c>
       <x:c r="E7" s="50" t="str">
-        <x:v>Add entropy/lookalike tests and ensure weak signals alone do not make high risk.</x:v>
+        <x:v>Closed 2026-07-01: username heuristics for random/generated, brand/support lookalikes and promo wording are covered; weak signals remain non-accusatory.</x:v>
       </x:c>
       <x:c r="F7" s="567" t="str">
-        <x:v>P2</x:v>
+        <x:v>Automated pass 2026-07-01: public-metadata, formatter, bot QA matrix, Telegram metadata handler and public-post suites passed 5 files / 83 tests; qa:telegram-report and qa:telegram-visual regenerated.</x:v>
       </x:c>
       <x:c r="G7" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>TG-008</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="76" customHeight="1">
@@ -7916,6 +7919,32 @@
         <x:v>Run production/live report submit plus Telegram /report confirmation smoke after deploy; continue next UX/logistics slice or Voice-out audio review/compression.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>QA-2026-07-01-002</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>TG-007/TG-008 Telegram username/native passport</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>npx eslint src/lib/telegram/format.ts src/lib/telegram/format.test.ts scripts/telegram-bot-qa-report.ts src/lib/telegram/public-metadata.server.test.ts --quiet; npm run test:run -- src/lib/telegram/format.test.ts src/lib/telegram/public-metadata.server.test.ts src/lib/telegram/bot-qa-matrix.test.ts src/lib/telegram/handlers/check.telegram-metadata.test.ts src/lib/telegram/public-post.server.test.ts; npm run qa:telegram-report; npm run qa:telegram-visual</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Passed: scoped eslint; 5 files / 83 tests; Telegram QA report and visual board regenerated</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>TG-007, TG-008, T-005, T-006</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Final formatted username passport now includes Native Passport Coach instead of truncating it. QA report shows phone-country/registration-month/not-official/recent-change guidance; conservative username clues remain unit-covered without hidden Telegram claims.</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Run live username smoke after deploy; next UX/logistics slice: Profile Screenshot Intelligence (T-007/TG-009) or Voice-out audio review/compression.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): preserve profile screenshot passport
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd91f70924f3d412b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R68df5757e8cc4106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3472d01239004dd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R623d2425c9a243b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb3b856a173b244b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2ca4c9674f55490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R86ca606eba6744e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R003e0d4ee10b40e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1f11e4c3cd0b4ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rca81b29ee1d54288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6887bea5bac4465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rcc36c4ec1f814a2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue UX/logistics fixes; next Profile Screenshot Intelligence (T-007/TG-009) or Voice-out human audio review/compression.</x:v>
+        <x:v>Continue UX/logistics fixes; next Voice-out human audio review/compression or live username/profile screenshot smoke after deploy.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-007/TG-008 final username passport now preserves Native Passport Coach; QA report regenerated; scoped eslint, 5 files / 83 tests, qa:telegram-report and qa:telegram-visual passed.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-009 profile screenshot intelligence now has final Telegram card and QA report coverage; scoped eslint, image/formatter tests, qa:telegram-report and qa:telegram-visual passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2678,7 +2678,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -3276,19 +3276,19 @@
         <x:v>Roadmap P8.5</x:v>
       </x:c>
       <x:c r="H10" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I10" s="8" t="str">
-        <x:v>Needs fixtures</x:v>
+        <x:v>Image-intelligence unit tests + formatter regression + Telegram QA report</x:v>
       </x:c>
       <x:c r="J10" s="8" t="str">
-        <x:v>Add category telegram_profile_card and tests with fakeable/privacy caveats.</x:v>
+        <x:v>2026-07-01: telegram_profile_card evidence extracts visible phone country, registration month, not-official and recent profile-change fields; final Telegram card preserves fakeable-screenshot caveat and quick asked-context buttons.</x:v>
       </x:c>
       <x:c r="K10" s="14" t="str">
-        <x:v>P3</x:v>
+        <x:v>Live profile screenshot smoke after deploy remains release check; profile card alone must never create high-risk without a visible dangerous request.</x:v>
       </x:c>
       <x:c r="L10" s="8" t="str">
-        <x:v>Screenshots can be forged; never treat profile card alone as high risk.</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6307,13 +6307,13 @@
         <x:v>OCR extracts visible fields like country, registration month, unofficial-account notice, recent name/photo changes, then explains them as screenshot evidence.</x:v>
       </x:c>
       <x:c r="E8" s="50" t="str">
-        <x:v>Add category telegram_profile_card and tests with fakeable/privacy caveats.</x:v>
+        <x:v>Closed 2026-07-01: profile screenshot intelligence has category/tests, fakeable/privacy caveat, final-card formatter regression and QA report fixture.</x:v>
       </x:c>
       <x:c r="F8" s="568" t="str">
-        <x:v>P3</x:v>
+        <x:v>Automated pass 2026-07-01: format + image-intelligence suites passed 2 files / 70 tests; qa:telegram-report and qa:telegram-visual regenerated.</x:v>
       </x:c>
       <x:c r="G8" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>TG-009</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="76" customHeight="1">
@@ -7945,6 +7945,32 @@
         <x:v>Run live username smoke after deploy; next UX/logistics slice: Profile Screenshot Intelligence (T-007/TG-009) or Voice-out audio review/compression.</x:v>
       </x:c>
     </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>QA-2026-07-01-003</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>TG-009 Telegram profile screenshot intelligence</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>npx eslint src/lib/telegram/format.ts src/lib/telegram/format.test.ts scripts/telegram-bot-qa-report.ts --quiet; npm run test:run -- src/lib/telegram/format.test.ts src/lib/risk/image-intelligence.test.ts; npm run qa:telegram-report; npm run qa:telegram-visual; npm run build</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>Passed: scoped eslint for touched TS files; 2 files / 70 tests; Telegram QA report and visual board regenerated; production build passed</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>TG-009, T-007</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Final Telegram card now keeps profile screenshot fields and fakeable-screenshot caveat. QA report includes synthetic Telegram profile screenshot with phone country, registration month, not-official notice, contact status and recent name/photo changes plus asked-context buttons.</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Run live profile screenshot smoke after deploy; next UX/logistics slice: Voice-out human audio review/compression or remaining live web/Telegram QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): add voice-out ogg assets
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R86ca606eba6744e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R003e0d4ee10b40e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1f11e4c3cd0b4ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rca81b29ee1d54288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6887bea5bac4465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rcc36c4ec1f814a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3e0ad4f3d5b54615"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ree9778f6c6ff45d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5da55990c96144cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rda985cf7764140a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re20268d43ac74d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5430b6974ce14065"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue UX/logistics fixes; next Voice-out human audio review/compression or live username/profile screenshot smoke after deploy.</x:v>
+        <x:v>Continue Voice-out live Telegram playback smoke and provider-limit UX, or move to remaining web/Telegram live QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-009 profile screenshot intelligence now has final Telegram card and QA report coverage; scoped eslint, image/formatter tests, qa:telegram-report and qa:telegram-visual passed.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 Voice-out SOS static OGG slice shipped: 45 panic RU/UZ/EN Opus assets validated, OGG is preferred before WAV/TTS, scoped unit tests and asset audit passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3507,16 +3507,16 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>Live QA</x:v>
+        <x:v>Unit tests + static asset audit</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>Move frequent SOS to pre-generated audio; hide/soft-disable button when limit is exhausted.</x:v>
+        <x:v>2026-07-01: 45 pre-generated SOS OGG/Opus assets committed for panic-1..15 in RU/UZ/EN; validator checks Ogg/Opus headers, durations, size limits and safe short scripts. Server regression confirms OGG is selected before WAV/TTS budget/provider.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="str">
-        <x:v>P2</x:v>
+        <x:v>Remaining: live Telegram playback smoke after deploy; decide whether to hide/soft-disable provider-only voice buttons when daily limit is exhausted.</x:v>
       </x:c>
       <x:c r="L16" s="8" t="str">
-        <x:v>Never voice codes, card data, passwords, phone numbers, URLs, or sensitive identifiers.</x:v>
+        <x:v>2026-07-01</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6399,13 +6399,13 @@
         <x:v>The button voices only a short safe script, with text caption, cache/cooldown, and graceful daily-limit messaging.</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
-        <x:v>Move frequent SOS to pre-generated audio; hide/soft-disable button when limit is exhausted.</x:v>
+        <x:v>Automated pass 2026-07-01 for static SOS assets: all 15 SOS scenarios now have RU/UZ/EN OGG assets under the Telegram size limit; WAV fallback/source files remain.</x:v>
       </x:c>
       <x:c r="F12" s="567" t="str">
-        <x:v>P2</x:v>
+        <x:v>Passed: voice-out unit suite 1 file / 13 tests; npm run tts:validate-assets verified 45 OGG assets, total 1,683,698 bytes, duration range 7.73s-14.05s; build pending in final verification.</x:v>
       </x:c>
       <x:c r="G12" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>TG-015</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
@@ -7971,6 +7971,32 @@
         <x:v>Run live profile screenshot smoke after deploy; next UX/logistics slice: Voice-out human audio review/compression or remaining live web/Telegram QA.</x:v>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>QA-2026-07-01-004</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>TG-015 Voice-out static SOS OGG assets</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>npx eslint src/lib/telegram/voice-out.server.test.ts scripts/validate-voice-out-assets.ts --quiet; npm run test:run -- src/lib/telegram/voice-out.server.test.ts; npm run tts:validate-assets; npm run build</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>Passed: scoped eslint; 1 file / 13 tests; 45 OGG assets validated; production build passed</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>TG-015, T-011</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>Committed panic-1..15 RU/UZ/EN OGG/Opus files. Validator confirmed 45 assets, total 1,683,698 bytes, smallest panic-3-uz.ogg 27,662 bytes / 7.73s, largest panic-12-ru.ogg 48,611 bytes / 14.05s. Unit regression confirms OGG is preferred before WAV, TTS budget and provider calls.</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>Run live Telegram playback smoke after deploy; decide provider-limit button soft-disable for Guardian/follow-up voice buttons.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(telegram): add voice-out ogg smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3e0ad4f3d5b54615"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ree9778f6c6ff45d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5da55990c96144cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rda985cf7764140a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re20268d43ac74d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5430b6974ce14065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb6e918aa12be4930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R56ada30de9464144"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb0d44db12a2f472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rfd81937907d94de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc4f4c4d9e97143f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd9fbce3bf29148dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue Voice-out live Telegram playback smoke and provider-limit UX, or move to remaining web/Telegram live QA.</x:v>
+        <x:v>Deploy Voice-out OGG assets, run full production voice-out webhook playback smoke, then decide provider-limit UX or continue remaining web/Telegram live QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 Voice-out SOS static OGG slice shipped: 45 panic RU/UZ/EN Opus assets validated, OGG is preferred before WAV/TTS, scoped unit tests and asset audit passed.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 Voice-out SOS static OGG slice shipped and Telegram Bot API accepted panic-6 RU/UZ/EN OGG via Railway smoke; full app webhook playback waits for deployment.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3507,16 +3507,16 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>Unit tests + static asset audit</x:v>
+        <x:v>Unit tests + static asset audit + Telegram Bot API OGG acceptance</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>2026-07-01: 45 pre-generated SOS OGG/Opus assets committed for panic-1..15 in RU/UZ/EN; validator checks Ogg/Opus headers, durations, size limits and safe short scripts. Server regression confirms OGG is selected before WAV/TTS budget/provider.</x:v>
+        <x:v>2026-07-01: 45 pre-generated SOS OGG/Opus assets committed for panic-1..15 in RU/UZ/EN; validator checks Ogg/Opus headers, durations, size limits and safe short scripts. Server regression confirms OGG is selected before WAV/TTS budget/provider. Direct Railway smoke confirmed Telegram sendAudio accepts panic-6 RU/UZ/EN OGG and cleanup deletes those direct test messages. Remaining: deploy assets, run full production webhook voice-out callback playback smoke; decide provider-limit button soft-disable for Guardian/follow-up provider-only voice buttons.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="str">
-        <x:v>Remaining: live Telegram playback smoke after deploy; decide whether to hide/soft-disable provider-only voice buttons when daily limit is exhausted.</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="L16" s="8" t="str">
-        <x:v>2026-07-01</x:v>
+        <x:v>Never voice codes, card data, passwords, phone numbers, URLs, or sensitive identifiers.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -6399,13 +6399,13 @@
         <x:v>The button voices only a short safe script, with text caption, cache/cooldown, and graceful daily-limit messaging.</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
-        <x:v>Automated pass 2026-07-01 for static SOS assets: all 15 SOS scenarios now have RU/UZ/EN OGG assets under the Telegram size limit; WAV fallback/source files remain.</x:v>
+        <x:v>Static SOS OGG assets and direct Telegram Bot API acceptance passed for panic-6 RU/UZ/EN; full app webhook playback remains pending until deployment includes the OGG assets.</x:v>
       </x:c>
       <x:c r="F12" s="567" t="str">
-        <x:v>Passed: voice-out unit suite 1 file / 13 tests; npm run tts:validate-assets verified 45 OGG assets, total 1,683,698 bytes, duration range 7.73s-14.05s; build pending in final verification.</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="G12" s="50" t="str">
-        <x:v>TG-015</x:v>
+        <x:v>Partial pass 2026-07-01: voice-out unit suite 1 file / 13 tests, npm run tts:validate-assets verified 45 OGG assets, npm run build passed, and railway run npx vite-node scripts/prod-telegram-voice-out-smoke.ts --skip-webhook confirmed Telegram sendAudio acceptance. Full app webhook playback smoke remains post-deploy.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
@@ -7997,6 +7997,32 @@
         <x:v>Run live Telegram playback smoke after deploy; decide provider-limit button soft-disable for Guardian/follow-up voice buttons.</x:v>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>QA-2026-07-01-005</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>TG-015 Voice-out Telegram OGG acceptance smoke</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>npx eslint scripts/prod-telegram-voice-out-smoke.ts --quiet; npm run tts:validate-assets; railway run npx vite-node scripts/prod-telegram-voice-out-smoke.ts --skip-webhook</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>Passed: scoped eslint; 45 OGG assets validated; Telegram Bot API sendAudio accepted panic-6 RU/UZ/EN OGG and cleanup deleted direct test messages</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>TG-015, T-011</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>QA marker QAVOICEOUTDTFHKDAC. Direct smoke used Railway env, did not print secrets/chat id, sent only to TELEGRAM_MODERATION_CHAT_ID, and skipped production webhook because deployed app does not yet include the new OGG assets.</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Deploy commit 7487cb3 or newer, then run full prod:telegram-voice-out-smoke against https://scam-guard-main-production.up.railway.app without --skip-webhook; decide provider-limit button soft-disable.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record voice-out deployment smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb6e918aa12be4930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R56ada30de9464144"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb0d44db12a2f472d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rfd81937907d94de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc4f4c4d9e97143f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd9fbce3bf29148dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7c96a0ce86f0489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf8bcfcf867e34903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3925d96ae43e495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rdc68c8087c264fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8f7a4e8a5efc4d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R6c656d5544004538"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Deploy Voice-out OGG assets, run full production voice-out webhook playback smoke, then decide provider-limit UX or continue remaining web/Telegram live QA.</x:v>
+        <x:v>Decide Voice-out provider-limit UX for dynamic Guardian/follow-up voice buttons, or continue remaining web/Telegram live QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 Voice-out SOS static OGG slice shipped and Telegram Bot API accepted panic-6 RU/UZ/EN OGG via Railway smoke; full app webhook playback waits for deployment.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 SOS Voice-out OGG assets deployed to Railway and full Telegram webhook playback smoke passed; remaining Voice-out item is provider-limit UX decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3507,10 +3507,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>Unit tests + static asset audit + Telegram Bot API OGG acceptance</x:v>
+        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>2026-07-01: 45 pre-generated SOS OGG/Opus assets committed for panic-1..15 in RU/UZ/EN; validator checks Ogg/Opus headers, durations, size limits and safe short scripts. Server regression confirms OGG is selected before WAV/TTS budget/provider. Direct Railway smoke confirmed Telegram sendAudio accepts panic-6 RU/UZ/EN OGG and cleanup deletes those direct test messages. Remaining: deploy assets, run full production webhook voice-out callback playback smoke; decide provider-limit button soft-disable for Guardian/follow-up provider-only voice buttons.</x:v>
+        <x:v>2026-07-01: Deployed Railway build 962b98c9-b600-4c51-8e6d-98e14ebb15fd with 45 SOS OGG/Opus assets and smoke harness. Full production Voice-out smoke passed: direct Telegram sendAudio accepted panic-6 RU/UZ/EN OGG, and production webhook accepted voiceout:panic:6 callback against https://scam-guard-main-production.up.railway.app. General prod:smoke also passed. Remaining P2 product decision: provider-limit button soft-disable for Guardian/follow-up provider-only voice buttons.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="str">
         <x:v>P2</x:v>
@@ -6399,13 +6399,13 @@
         <x:v>The button voices only a short safe script, with text caption, cache/cooldown, and graceful daily-limit messaging.</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
-        <x:v>Static SOS OGG assets and direct Telegram Bot API acceptance passed for panic-6 RU/UZ/EN; full app webhook playback remains pending until deployment includes the OGG assets.</x:v>
+        <x:v>SOS OGG static assets and deployed production webhook playback passed for panic-6 RU/UZ/EN; remaining risk is provider-limit UX for dynamic/provider-only voice buttons.</x:v>
       </x:c>
       <x:c r="F12" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G12" s="50" t="str">
-        <x:v>Partial pass 2026-07-01: voice-out unit suite 1 file / 13 tests, npm run tts:validate-assets verified 45 OGG assets, npm run build passed, and railway run npx vite-node scripts/prod-telegram-voice-out-smoke.ts --skip-webhook confirmed Telegram sendAudio acceptance. Full app webhook playback smoke remains post-deploy.</x:v>
+        <x:v>Passed for SOS OGG playback 2026-07-01: voice-out unit suite 1 file / 13 tests, asset validator 45 files, build, deploy 962b98c9-b600-4c51-8e6d-98e14ebb15fd, full prod:telegram-voice-out-smoke and prod:smoke passed. Provider-limit UX remains a P2 follow-up.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
@@ -8023,6 +8023,32 @@
         <x:v>Deploy commit 7487cb3 or newer, then run full prod:telegram-voice-out-smoke against https://scam-guard-main-production.up.railway.app without --skip-webhook; decide provider-limit button soft-disable.</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>QA-2026-07-01-006</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>TG-015 Voice-out deployed Telegram webhook playback smoke</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>railway up --message "Deploy Voice-out OGG assets and smoke harness"; railway run npm run prod:telegram-voice-out-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>Passed after lockfile fix: deployment 962b98c9-b600-4c51-8e6d-98e14ebb15fd succeeded; full Voice-out smoke passed; general production smoke passed</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>TG-015, T-011</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>First deploy 90f56ca4-7172-438d-b00e-574c91a1394c failed at bun install --frozen-lockfile because bun.lock was stale after script additions; fixed by commit 298babb. Full smoke marker QAVOICEOUTAMGAHXBB: direct sendAudio accepted panic-6 RU/UZ/EN OGG, production webhook accepted voiceout:panic:6 callback, cleanup removed direct test messages and synthetic DB rows. prod:smoke returned home 200, healthz 200, webhook auth checks 401/200, pending=0, AI provider 200.</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Decide provider-limit soft-disable UX for dynamic Guardian/follow-up voice buttons, or resume remaining P1/P2 web/Telegram live QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): soften voice-out limit fallback
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7c96a0ce86f0489d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf8bcfcf867e34903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3925d96ae43e495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rdc68c8087c264fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8f7a4e8a5efc4d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R6c656d5544004538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R84cc94561470428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Raf9c78f04d224036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6aaf33b4f44941b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R3dc87c7910eb432c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0a38770f898849e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb6b0723da52340c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Decide Voice-out provider-limit UX for dynamic Guardian/follow-up voice buttons, or continue remaining web/Telegram live QA.</x:v>
+        <x:v>Continue remaining P1/P2 web/Telegram live QA flows; then UX/logistics fixes.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 SOS Voice-out OGG assets deployed to Railway and full Telegram webhook playback smoke passed; remaining Voice-out item is provider-limit UX decision.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 Voice-out OGG assets deployed and provider-limit fallback keyboard UX fixed; next is remaining P1/P2 web/Telegram live QA.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -3504,13 +3504,13 @@
         <x:v>.kiro/specs/telegram-voice-out-tts-v1</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke</x:v>
+        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke + provider-limit fallback regression</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>2026-07-01: Deployed Railway build 962b98c9-b600-4c51-8e6d-98e14ebb15fd with 45 SOS OGG/Opus assets and smoke harness. Full production Voice-out smoke passed: direct Telegram sendAudio accepted panic-6 RU/UZ/EN OGG, and production webhook accepted voiceout:panic:6 callback against https://scam-guard-main-production.up.railway.app. General prod:smoke also passed. Remaining P2 product decision: provider-limit button soft-disable for Guardian/follow-up provider-only voice buttons.</x:v>
+        <x:v>2026-07-01: Deployed Railway build 962b98c9-b600-4c51-8e6d-98e14ebb15fd with 45 SOS OGG/Opus assets and smoke harness. Full production Voice-out smoke passed: direct Telegram sendAudio accepted panic-6 RU/UZ/EN OGG, and production webhook accepted voiceout:panic:6 callback against https://scam-guard-main-production.up.railway.app. General prod:smoke also passed. Provider-limit UX fixed: rate-limit fallback now removes Guardian/follow-up provider-only voice buttons while preserving static SOS voice and normal action buttons.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="str">
         <x:v>P2</x:v>
@@ -6399,13 +6399,13 @@
         <x:v>The button voices only a short safe script, with text caption, cache/cooldown, and graceful daily-limit messaging.</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
-        <x:v>SOS OGG static assets and deployed production webhook playback passed for panic-6 RU/UZ/EN; remaining risk is provider-limit UX for dynamic/provider-only voice buttons.</x:v>
+        <x:v>Closed 2026-07-01: SOS OGG static assets and deployed production webhook playback passed; provider-limit fallback now removes dynamic/provider-only voice buttons while preserving static SOS voice buttons.</x:v>
       </x:c>
       <x:c r="F12" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G12" s="50" t="str">
-        <x:v>Passed for SOS OGG playback 2026-07-01: voice-out unit suite 1 file / 13 tests, asset validator 45 files, build, deploy 962b98c9-b600-4c51-8e6d-98e14ebb15fd, full prod:telegram-voice-out-smoke and prod:smoke passed. Provider-limit UX remains a P2 follow-up.</x:v>
+        <x:v>Passed 2026-07-01: voice-out unit suite 14 tests, asset validator 45 files, build, deploy/full production smokes, and provider-limit keyboard regression passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
@@ -8046,7 +8046,33 @@
         <x:v>First deploy 90f56ca4-7172-438d-b00e-574c91a1394c failed at bun install --frozen-lockfile because bun.lock was stale after script additions; fixed by commit 298babb. Full smoke marker QAVOICEOUTAMGAHXBB: direct sendAudio accepted panic-6 RU/UZ/EN OGG, production webhook accepted voiceout:panic:6 callback, cleanup removed direct test messages and synthetic DB rows. prod:smoke returned home 200, healthz 200, webhook auth checks 401/200, pending=0, AI provider 200.</x:v>
       </x:c>
       <x:c r="H27" t="str">
-        <x:v>Decide provider-limit soft-disable UX for dynamic Guardian/follow-up voice buttons, or resume remaining P1/P2 web/Telegram live QA.</x:v>
+        <x:v>Completed by QA-2026-07-01-007; resume remaining P1/P2 web/Telegram live QA.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>QA-2026-07-01-007</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>TG-015 Voice-out provider-limit fallback UX</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>npx eslint src/lib/telegram/voice-out.server.ts src/lib/telegram/voice-out.server.test.ts --quiet; npm run test:run -- src/lib/telegram/voice-out.server.test.ts; npm run build</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Passed: scoped eslint; 1 file / 14 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>TG-015, T-011</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>Rate-limit fallback now strips provider-only voice buttons (`voiceout:guardian`, contextual `voiceout:panic:&lt;id&gt;:&lt;action&gt;`) so users do not tap into the same limit loop; static SOS `voiceout:panic:&lt;id&gt;` and normal action buttons remain. Regression caught and fixed non-voice callback preservation.</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Proceed to remaining P1/P2 web/Telegram live QA flows; keep real-audio human review/compression as optional polish.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record post-deploy P1 live QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R84cc94561470428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Raf9c78f04d224036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6aaf33b4f44941b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R3dc87c7910eb432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0a38770f898849e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb6b0723da52340c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9fe72f34494740ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rcda77d72f0304995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Red6e36cdc8af4a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb32e2c44b512492c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf8f2565224844aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R84fc267683344203"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1/P2 web/Telegram live QA flows; then UX/logistics fixes.</x:v>
+        <x:v>Proceed to UX/logistics fixes or next product backlog; optional real-audio Voice-out review/compression.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-015 Voice-out OGG assets deployed and provider-limit fallback keyboard UX fixed; next is remaining P1/P2 web/Telegram live QA.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: deployed Voice-out provider-limit fallback and re-ran P1 web/Telegram production QA; all passed with cleanup.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -8072,7 +8072,33 @@
         <x:v>Rate-limit fallback now strips provider-only voice buttons (`voiceout:guardian`, contextual `voiceout:panic:&lt;id&gt;:&lt;action&gt;`) so users do not tap into the same limit loop; static SOS `voiceout:panic:&lt;id&gt;` and normal action buttons remain. Regression caught and fixed non-voice callback preservation.</x:v>
       </x:c>
       <x:c r="H28" t="str">
-        <x:v>Proceed to remaining P1/P2 web/Telegram live QA flows; keep real-audio human review/compression as optional polish.</x:v>
+        <x:v>Completed by QA-2026-07-01-008; proceed to UX/logistics fixes or next product backlog.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>QA-2026-07-01-008</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Post-deploy P1 web/Telegram live QA</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>railway up --message "Deploy Voice-out provider-limit fallback"; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-user-story-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-scope-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-live-qa-smoke -- https://scam-guard-main-production.up.railway.app; Playwright CLI homepage/report/appeal; railway run npx vite-node scripts/prod-admin-moderation-smoke.ts --marker QA-P1-WEB-20260701112907</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>Passed: deployment ad41dc8b-f8b6-4ca2-afb6-0016aebb24b0 succeeded; general prod smoke passed; Telegram user-story/scope/live QA passed; browser homepage/report/appeal passed; admin moderation cleanup done</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>TG-001, TG-002, TG-005, TG-010, TG-014, TG-015, TG-022, WEB-002, WEB-003, WEB-007, ADM-002, CORE-008</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>prod:smoke returned home 200, healthz 200, webhook auth 401/200, Telegram pending=0, AI provider 200. Telegram markers QAPONETGUSERSTORYRMLTKFVZ and QAPONETGLIVETXAJLRWG passed. Browser homepage returned high-risk result score 100% with console warnings/errors=0; report success showed manual moderation/duplicate-priority copy; appeal success showed accepted review copy. Admin moderation smoke marker QA-P1-WEB-20260701112907 found report/appeal, verified audit actions and cleanup=done.</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Proceed to UX/logistics fixes or next product backlog; keep real-audio human review/compression as optional polish.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(risk): cover short-code prefix lookalikes
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9fe72f34494740ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rcda77d72f0304995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Red6e36cdc8af4a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb32e2c44b512492c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf8f2565224844aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R84fc267683344203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R5c80e501a1ae41d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1f491acfe03d4d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R941843361f8743cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9fe7cc898a7440cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rcdb115bc90a54cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R61d0a80f7f944b70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Proceed to UX/logistics fixes or next product backlog; optional real-audio Voice-out review/compression.</x:v>
+        <x:v>Continue P1 core rows: CORE-007 redaction/privacy, then CORE-008 rate limits; UX/logistics after remaining P1 core checks.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: deployed Voice-out provider-limit fallback and re-ran P1 web/Telegram production QA; all passed with cleanup.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-003 official-number short-code prefix regression verified and closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4492,13 +4492,13 @@
         <x:v>.kiro/specs/official-number-lookalike-v1</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I42" s="8" t="str">
-        <x:v>Unit tests</x:v>
+        <x:v>Unit tests + check-core pipeline regression</x:v>
       </x:c>
       <x:c r="J42" s="8" t="str">
-        <x:v>Security scan: country-code prefix stripping may falsely verify short-code lookalike numbers.</x:v>
+        <x:v>2026-07-01: Existing verified-contact lookup regression confirms +998-prefixed short codes do not match official short codes; added runCheck regression for +9981340 to stay unverified/unknown with score 0.</x:v>
       </x:c>
       <x:c r="K42" s="12" t="str">
         <x:v>P1</x:v>
@@ -6675,13 +6675,13 @@
         <x:v>Phone normalization distinguishes real official short numbers from longer lookalikes and foreign/non-local numbers.</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Security scan: country-code prefix stripping may falsely verify short-code lookalike numbers.</x:v>
+        <x:v>Closed 2026-07-01: country-code-prefixed short-code lookalikes are not verified as official contacts.</x:v>
       </x:c>
       <x:c r="F24" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: scoped eslint passed; verified-contacts, phone-intelligence and check-core property suites passed 3 files / 45 tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="76" customHeight="1">
@@ -8101,6 +8101,32 @@
         <x:v>Proceed to UX/logistics fixes or next product backlog; keep real-audio human review/compression as optional polish.</x:v>
       </x:c>
     </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>QA-2026-07-01-009</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>CORE-003 official-number short-code prefix regression</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>npx eslint src/lib/risk/check-core.property.test.ts --quiet; npm run test:run -- src/lib/risk/verified-contacts.test.ts src/lib/risk/phone-intelligence.test.ts src/lib/risk/check-core.property.test.ts</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>Passed: scoped eslint; 3 files / 45 tests</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>CORE-003, T-023</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>Added a runCheck-level regression for +9981340: it must not get verifiedContact, must not have matched officialDirectoryStatus, must not receive valid_uz_phone, and must remain unknown score 0. Existing helper coverage already confirmed +9981340/+998102/+9981257 do not match official short codes.</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Continue remaining P1 core rows: CORE-007 redaction/privacy, then CORE-008 rate-limit regression watch.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(privacy): close report appeal redaction gaps
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R5c80e501a1ae41d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1f491acfe03d4d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R941843361f8743cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9fe7cc898a7440cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rcdb115bc90a54cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R61d0a80f7f944b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R88bfe301e0994680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R0bbf5210e5d14315"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8bbb794143224a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5ef1e107b1fa41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2a2e21c69b3e4981"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0624a7cd0ed244f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue P1 core rows: CORE-007 redaction/privacy, then CORE-008 rate limits; UX/logistics after remaining P1 core checks.</x:v>
+        <x:v>Continue P1 core row: CORE-008 shared rate limits; UX/logistics after remaining P1 core checks.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-003 official-number short-code prefix regression verified and closed.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-007 privacy boundary tightened; report/appeal persistence and moderation-alert redaction verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4638,25 +4638,25 @@
         <x:v>Phone/card/code/URL/email/text are masked or omitted based on destination and retention policy.</x:v>
       </x:c>
       <x:c r="F46" s="8" t="str">
-        <x:v>src/lib/privacy.ts; src/lib/report.functions.ts; src/lib/check.functions.ts; src/lib/telegram/moderation-notifier.server.ts</x:v>
+        <x:v>src/lib/risk/detect.ts; src/lib/report.functions.ts; src/lib/reputation-appeal.functions.ts; src/lib/telegram/moderation-notifier.server.ts</x:v>
       </x:c>
       <x:c r="G46" s="8" t="str">
         <x:v>ai_docs/DATABASE.md; ai_docs/MODERATION_GUIDELINES.md</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I46" s="8" t="str">
-        <x:v>Unit tests</x:v>
+        <x:v>Unit/privacy regression tests</x:v>
       </x:c>
       <x:c r="J46" s="8" t="str">
-        <x:v>Security scan: report metadata/narrative/appeal text may persist raw emails/URLs/Telegram identifiers.</x:v>
+        <x:v>Closed 2026-07-01: report narrative/metadata and appeal reason/contact normalize or redact raw emails, URLs, Telegram identifiers, and tokenized links before persistence/alerts; contact URL hash strips query tokens.</x:v>
       </x:c>
       <x:c r="K46" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L46" s="8" t="str">
-        <x:v>Minimize retained raw evidence; never send raw evidence to Telegram moderation chat.</x:v>
+        <x:v>Minimize retained raw evidence; never send raw evidence to Telegram moderation chat. 2026-07-01: contact hash normalization strips URL query/fragment before hashing.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -6767,13 +6767,13 @@
         <x:v>Phone/card/code/URL/email/text are masked or omitted based on destination and retention policy.</x:v>
       </x:c>
       <x:c r="E28" s="50" t="str">
-        <x:v>Security scan: report metadata/narrative/appeal text may persist raw emails/URLs/Telegram identifiers.</x:v>
+        <x:v>Closed 2026-07-01: report metadata/narrative and appeal text/contact no longer persist raw emails, URLs, Telegram identifiers, or tokenized contact URLs.</x:v>
       </x:c>
       <x:c r="F28" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G28" s="50" t="str">
-        <x:v>Automated pass 2026-06-29; privacy copy QA pending</x:v>
+        <x:v>Automated pass 2026-07-01: scoped eslint passed; report/appeal privacy tests passed 2 files / 13 tests; risk redaction suites passed 3 files / 42 tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="76" customHeight="1">
@@ -8124,7 +8124,33 @@
         <x:v>Added a runCheck-level regression for +9981340: it must not get verifiedContact, must not have matched officialDirectoryStatus, must not receive valid_uz_phone, and must remain unknown score 0. Existing helper coverage already confirmed +9981340/+998102/+9981257 do not match official short codes.</x:v>
       </x:c>
       <x:c r="H30" t="str">
-        <x:v>Continue remaining P1 core rows: CORE-007 redaction/privacy, then CORE-008 rate-limit regression watch.</x:v>
+        <x:v>Completed by QA-2026-07-01-010; continue CORE-008 shared rate-limit regression watch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>QA-2026-07-01-010</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>CORE-007 report/appeal redaction privacy boundary</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>npx eslint src/lib/report.functions.test.ts src/lib/reputation-appeal.functions.ts src/lib/reputation-appeal.functions.test.ts --quiet; npm run test:run -- src/lib/report.functions.test.ts src/lib/reputation-appeal.functions.test.ts; npm run test:run -- src/lib/risk/detect.test.ts src/lib/risk/phone-otp-redaction.property.test.ts src/lib/risk/__tests__/barcode-false-positive.test.ts</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>Passed: scoped eslint; report/appeal privacy 2 files / 13 tests; risk redaction 3 files / 42 tests</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>CORE-007, T-027</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>Report narrative/metadata now has alert-boundary regression coverage. Appeal reason/contact tests cover raw URLs, Telegram handles/invites, and tokenized contact URLs. Contact URL hash input now normalizes away query/fragment before hashing, while stored display remains masked.</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Continue CORE-008 shared rate-limit regression watch.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(rate-limit): verify shared quota gates
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R88bfe301e0994680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R0bbf5210e5d14315"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8bbb794143224a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5ef1e107b1fa41eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2a2e21c69b3e4981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0624a7cd0ed244f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R55f191e6866a4fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra01723de2f954efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd59c42e835e94a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0c45344d61a64253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2a5406c199424590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R285dcf8653a544a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue P1 core row: CORE-008 shared rate limits; UX/logistics after remaining P1 core checks.</x:v>
+        <x:v>Continue remaining P1 test queue, starting CORE-006 verified-contact override regression; UX/logistics after P1 checks.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-007 privacy boundary tightened; report/appeal persistence and moderation-alert redaction verified.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-008 shared rate-limit/proxy/media quota gates verified locally and in production security smoke.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4682,19 +4682,19 @@
         <x:v>.kiro/specs/shared-rate-limit-v1</x:v>
       </x:c>
       <x:c r="H47" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I47" s="8" t="str">
-        <x:v>Unit tests</x:v>
+        <x:v>Unit/integration tests + production security smoke</x:v>
       </x:c>
       <x:c r="J47" s="8" t="str">
-        <x:v>Security scan: forwarded IP keying and Telegram image download-before-limit need fixes.</x:v>
+        <x:v>Closed 2026-07-01: proxy IP trust guard, shared scopes, Telegram image pre-fetch budget, report/appeal/voice-out gates verified; prod security smoke claim_rate_limit checks passed.</x:v>
       </x:c>
       <x:c r="K47" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L47" s="8" t="str">
-        <x:v>Use trusted proxy/IP provenance; rate-limit before AI/media downloads.</x:v>
+        <x:v>Use trusted proxy IP provenance; rate-limit before AI/media downloads. 2026-07-01: image download budget runs before Telegram getFile/download.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -6790,13 +6790,13 @@
         <x:v>Public, Telegram, OCR/STT/TTS, report, and appeal paths enforce shared or scoped rate limits before expensive work.</x:v>
       </x:c>
       <x:c r="E29" s="50" t="str">
-        <x:v>Security scan: forwarded IP keying and Telegram image download-before-limit need fixes.</x:v>
+        <x:v>Closed 2026-07-01: public/web/Telegram/report/appeal/TTS rate limits verified; Telegram image budget runs before getFile/download; proxy IP trust is disabled by default and prod env checked.</x:v>
       </x:c>
       <x:c r="F29" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G29" s="50" t="str">
-        <x:v>Automated pass 2026-06-29; production load/quota QA pending</x:v>
+        <x:v>Automated + production pass 2026-07-01: scoped eslint passed; focused CORE-008 tests passed 7 files / 131 tests; railway run npm run prod:security-smoke passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="76" customHeight="1">
@@ -8150,7 +8150,33 @@
         <x:v>Report narrative/metadata now has alert-boundary regression coverage. Appeal reason/contact tests cover raw URLs, Telegram handles/invites, and tokenized contact URLs. Contact URL hash input now normalizes away query/fragment before hashing, while stored display remains masked.</x:v>
       </x:c>
       <x:c r="H31" t="str">
-        <x:v>Continue CORE-008 shared rate-limit regression watch.</x:v>
+        <x:v>Completed by QA-2026-07-01-011; continue remaining P1 test queue, starting CORE-006 verified-contact override regression.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>QA-2026-07-01-011</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>CORE-008 shared rate-limit/proxy/media quota gates</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>npx eslint src/lib/risk/shared-rate-limit.server.test.ts src/lib/check.functions.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/voice-out.server.test.ts src/lib/report.functions.test.ts src/lib/reputation-appeal.functions.test.ts src/lib/prod-security-smoke-env.test.ts scripts/security-smoke-env.ts --quiet; npm run test:run -- src/lib/risk/shared-rate-limit.server.test.ts src/lib/check.functions.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/voice-out.server.test.ts src/lib/report.functions.test.ts src/lib/reputation-appeal.functions.test.ts src/lib/prod-security-smoke-env.test.ts; railway run npm run prod:security-smoke</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>Passed: scoped eslint; focused tests 7 files / 131 tests; production security smoke passed</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>CORE-008, T-028, WEB-002, WEB-003, WEB-007, TG-010, TG-015, SEC-001</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>Shared limiter now has explicit telegram_public_post scope regression. Existing web wrapper tests verify spoofable forwarding headers are ignored by default and trusted only when enabled; production smoke verifies TRUST_PROXY_IP_HEADERS unset/false. Telegram image integration verifies 11 repeated photos yield only 10 getFile/download/OCR calls, proving budget is claimed before Telegram file fetch. Voice-out prerecorded assets bypass provider budget; provider TTS fallback removes provider-only buttons.</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>Continue remaining P1 test queue, starting CORE-006 verified-contact override regression; then UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs(tracker): close verified contact override QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R55f191e6866a4fa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra01723de2f954efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd59c42e835e94a21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0c45344d61a64253"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2a5406c199424590"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R285dcf8653a544a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9887cbab51324228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R529d4b83293b4525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R41d1c1182b274c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R55c00e64e7d44cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R30a3077c38144316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0bbd11c284b642be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1 test queue, starting CORE-006 verified-contact override regression; UX/logistics after P1 checks.</x:v>
+        <x:v>Continue remaining P1 test queue, starting CORE-001 deterministic false-positive QA; then TG-028/ADM-001 checks.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-008 shared rate-limit/proxy/media quota gates verified locally and in production security smoke.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-006 verified-contact override regression re-verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4609,16 +4609,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I45" s="8" t="str">
-        <x:v>Unit tests</x:v>
+        <x:v>Unit regression tests</x:v>
       </x:c>
       <x:c r="J45" s="8" t="str">
-        <x:v>Security scan: verified contact override returns safe for confirmed high-risk reported number.</x:v>
+        <x:v>Closed 2026-07-01: confirmed high-risk entity reputation keeps known_reported/high_risk even when the input matches a verified official contact; dangerous requests also override verified contacts.</x:v>
       </x:c>
       <x:c r="K45" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L45" s="8" t="str">
-        <x:v>Official contact signal should not override confirmed abuse evidence.</x:v>
+        <x:v>Official contact signal should not override confirmed abuse evidence. 2026-07-01: T-026 regression verified in check-core property suite.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -6744,13 +6744,13 @@
         <x:v>Known official contacts produce safe evidence unless confirmed high-risk reputation or other stronger risk exists.</x:v>
       </x:c>
       <x:c r="E27" s="50" t="str">
-        <x:v>Security scan: verified contact override returns safe for confirmed high-risk reported number.</x:v>
+        <x:v>Closed 2026-07-01: verified contact override does not return safe for a confirmed high-risk reported official-looking number.</x:v>
       </x:c>
       <x:c r="F27" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G27" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: scoped eslint passed; check-core, verified-contacts, rules reason-code and phone-intelligence suites passed 4 files / 153 tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="76" customHeight="1">
@@ -8176,7 +8176,33 @@
         <x:v>Shared limiter now has explicit telegram_public_post scope regression. Existing web wrapper tests verify spoofable forwarding headers are ignored by default and trusted only when enabled; production smoke verifies TRUST_PROXY_IP_HEADERS unset/false. Telegram image integration verifies 11 repeated photos yield only 10 getFile/download/OCR calls, proving budget is claimed before Telegram file fetch. Voice-out prerecorded assets bypass provider budget; provider TTS fallback removes provider-only buttons.</x:v>
       </x:c>
       <x:c r="H32" t="str">
-        <x:v>Continue remaining P1 test queue, starting CORE-006 verified-contact override regression; then UX/logistics fixes.</x:v>
+        <x:v>Completed by QA-2026-07-01-012; continue remaining P1 test queue, starting CORE-001 deterministic false-positive QA.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>QA-2026-07-01-012</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>CORE-006 verified contact override regression</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>npx eslint src/lib/risk/check-core.property.test.ts src/lib/risk/verified-contacts.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/risk/phone-intelligence.test.ts --quiet; npm run test:run -- src/lib/risk/check-core.property.test.ts src/lib/risk/verified-contacts.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/risk/phone-intelligence.test.ts</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>Passed: scoped eslint; focused risk tests 4 files / 153 tests</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>CORE-006, T-026</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>Existing check-core regression confirms a verified official full number with a confirmed high-risk entity keeps verifiedContact metadata but also keeps known_reported and final high_risk. Dangerous SMS-code requests with official short codes also remain high_risk.</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>Continue remaining P1 test queue, starting CORE-001 deterministic false-positive QA; then TG-028/ADM-001 checks.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(telegram): add production false-positive smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9887cbab51324228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R529d4b83293b4525"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R41d1c1182b274c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R55c00e64e7d44cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R30a3077c38144316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0bbd11c284b642be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2038d9b08707423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rd1a387f244b940ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7cb0f463b71846d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2180fafb30aa4343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R5737806cc2ba4534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rdd22299d43514ef0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1 test queue, starting CORE-001 deterministic false-positive QA; then TG-028/ADM-001 checks.</x:v>
+        <x:v>Continue remaining P1 test queue: TG-028 and ADM-001 checks; then UX/logistics fixes.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-006 verified-contact override regression re-verified.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-001 false-positive boundaries re-verified locally and in production Telegram smoke.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4419,16 +4419,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>Property + unit tests</x:v>
+        <x:v>Property + unit + production smoke</x:v>
       </x:c>
       <x:c r="J40" s="8" t="str">
-        <x:v>Audit broad rules that attach unrelated reasons to voice/delivery messages.</x:v>
+        <x:v>Closed 2026-07-01: broad rule false-positive boundaries re-verified locally and in production Telegram smoke.</x:v>
       </x:c>
       <x:c r="K40" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L40" s="8" t="str">
-        <x:v>Rules must be explainable and not overfit to attacker prompt wording.</x:v>
+        <x:v>QA-2026-07-01-013 added; benign delivery, sports news and Telegram product news stayed unknown without unrelated reason codes.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -6652,13 +6652,13 @@
         <x:v>Rules assign reason codes/weights, thresholds produce verdicts, AI only explains or enriches.</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Audit broad rules that attach unrelated reasons to voice/delivery messages.</x:v>
+        <x:v>Closed 2026-07-01: local boundary suites and production Telegram false-positive smoke passed.</x:v>
       </x:c>
       <x:c r="F23" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Automated pass 2026-06-29; live false-positive QA pending</x:v>
+        <x:v>Passed 2026-07-01: scoped eslint; focused CORE-001 suites 5 files / 272 tests; production Telegram smoke 3 benign cases unknown with no forbidden reasons.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="76" customHeight="1">
@@ -8202,7 +8202,33 @@
         <x:v>Existing check-core regression confirms a verified official full number with a confirmed high-risk entity keeps verifiedContact metadata but also keeps known_reported and final high_risk. Dangerous SMS-code requests with official short codes also remain high_risk.</x:v>
       </x:c>
       <x:c r="H33" t="str">
-        <x:v>Continue remaining P1 test queue, starting CORE-001 deterministic false-positive QA; then TG-028/ADM-001 checks.</x:v>
+        <x:v>Completed by QA-2026-07-01-013; continue remaining P1 test queue: TG-028/ADM-001 checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>QA-2026-07-01-013</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>CORE-001 deterministic false-positive boundaries</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>npx eslint scripts/prod-telegram-false-positive-smoke.ts src/lib/risk/check-core.property.test.ts src/lib/risk/image-intelligence.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/telegram/format.test.ts src/lib/telegram/webhook.integration.test.ts --quiet; npm run test:run -- src/lib/risk/check-core.property.test.ts src/lib/risk/image-intelligence.test.ts src/lib/risk/rules.reason-codes.test.ts src/lib/telegram/format.test.ts src/lib/telegram/webhook.integration.test.ts; railway run npm run prod:telegram-false-positive-smoke -- https://scam-guard-main-production.up.railway.app; npm run build</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>Passed: scoped eslint; focused CORE-001 suites 5 files / 272 tests; production Telegram false-positive smoke passed for 3 benign cases; build passed.</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>CORE-001, T-022</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>Local regression coverage confirms deterministic scoring is independent of AI and broad delivery/betting/Web3 rules do not attach unrelated reason codes. Production Telegram webhook smoke persisted benign delivery, ordinary sports news and Telegram product news as unknown with empty reason lists, then cleaned its DB rows.</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>Continue remaining P1 test queue: TG-028/ADM-001 checks; then UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(ai): expand output safety adversarial coverage
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2038d9b08707423e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rd1a387f244b940ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7cb0f463b71846d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2180fafb30aa4343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R5737806cc2ba4534"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rdd22299d43514ef0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rbd841b0a6dbe448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R721c22ac51d74c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R64ccb679f9604806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1d0ce2eed66445e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb096398336764973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R165a4450a55c410d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1 test queue: TG-028 and ADM-001 checks; then UX/logistics fixes.</x:v>
+        <x:v>Continue remaining P1 test queue: ADM-001 production auth policy smoke; then UX/logistics fixes.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: CORE-001 false-positive boundaries re-verified locally and in production Telegram smoke.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-028 adversarial AI safety tests and production AI-provider smoke passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4001,16 +4001,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I29" s="8" t="str">
-        <x:v>Unit/property tests</x:v>
+        <x:v>Unit/property + production smoke</x:v>
       </x:c>
       <x:c r="J29" s="8" t="str">
-        <x:v>Add adversarial CI tests and decoy patrol for repeated blocked prompts.</x:v>
+        <x:v>Closed 2026-07-01: adversarial firewall/decoy tests added; provider degradation and production smoke re-verified.</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L29" s="8" t="str">
-        <x:v>AI must not request secrets, code, cards, password, seed phrase, or install actions.</x:v>
+        <x:v>QA-2026-07-01-014 added; AI output firewall blocks prompt leaks, secret/payment/wallet/APK action text and allows safe warnings.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -6491,13 +6491,13 @@
         <x:v>Rules remain authoritative; AI adds explanation only; provider failures have fallback; generated text passes safety firewall.</x:v>
       </x:c>
       <x:c r="E16" s="50" t="str">
-        <x:v>Add adversarial CI tests and decoy patrol for repeated blocked prompts.</x:v>
+        <x:v>Closed 2026-07-01: adversarial CI tests and production AI-provider smoke passed.</x:v>
       </x:c>
       <x:c r="F16" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G16" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-01: scoped eslint; focused AI safety/degradation suites 3 files / 29 tests; production smoke passed with AI provider healthy.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="76" customHeight="1">
@@ -8228,7 +8228,33 @@
         <x:v>Local regression coverage confirms deterministic scoring is independent of AI and broad delivery/betting/Web3 rules do not attach unrelated reason codes. Production Telegram webhook smoke persisted benign delivery, ordinary sports news and Telegram product news as unknown with empty reason lists, then cleaned its DB rows.</x:v>
       </x:c>
       <x:c r="H34" t="str">
-        <x:v>Continue remaining P1 test queue: TG-028/ADM-001 checks; then UX/logistics fixes.</x:v>
+        <x:v>Completed by QA-2026-07-01-014; continue remaining P1 test queue: ADM-001 production auth policy smoke.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>QA-2026-07-01-014</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>TG-028 AI provider resilience and output safety</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>npx eslint src/lib/risk/ai-output-safety.ts src/lib/risk/ai-output-safety.test.ts src/lib/risk/check-core.ai-output-safety.test.ts src/lib/telegram/ai-degradation.integration.test.ts --quiet; npm run test:run -- src/lib/risk/ai-output-safety.test.ts src/lib/risk/check-core.ai-output-safety.test.ts src/lib/telegram/ai-degradation.integration.test.ts; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>Passed: scoped eslint; focused AI safety/degradation tests 3 files / 29 tests; production smoke passed, including AI provider health.</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>TG-028, T-015</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>Added adversarial CI coverage for repeated prompt-injection leaks, multilingual requests for secrets/payment/wallet/APK actions, and safe-warning decoys. Existing degradation tests still prove rules-only scoring when AI is missing, failing, quota-limited, retried, or falling back.</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Continue remaining P1 test queue: ADM-001 production auth policy smoke; then UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test(admin): verify production allowlist auth policy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rbd841b0a6dbe448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R721c22ac51d74c8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R64ccb679f9604806"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1d0ce2eed66445e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb096398336764973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R165a4450a55c410d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6b0ab9ffa8424b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbaec59b5e534448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R845b0f89667a4a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R48a94e8da7a84031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2f9bc865d87146a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R556484f0fd6c4a72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Continue remaining P1 test queue: ADM-001 production auth policy smoke; then UX/logistics fixes.</x:v>
+        <x:v>P1 test queue closed; continue with UX/logistics fixes and the next product backlog.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-028 adversarial AI safety tests and production AI-provider smoke passed.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ADM-001 production auth policy smoke passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4305,16 +4305,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I37" s="8" t="str">
-        <x:v>Unit tests + linked Supabase read-only verification</x:v>
+        <x:v>Unit tests + production auth policy smoke</x:v>
       </x:c>
       <x:c r="J37" s="8" t="str">
-        <x:v>Keep admin sign-in/no-access browser smoke in release checklist after auth or Supabase Auth setting changes.</x:v>
+        <x:v>Closed 2026-07-01: production auth policy smoke verifies anon admin-table boundaries and confirmed allowlist-only admin roles.</x:v>
       </x:c>
       <x:c r="K37" s="12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L37" s="8" t="str">
-        <x:v>2026-06-30: ADM-001 verified. Server functions require bearer token and user_roles.role='admin'; client admin page gates on isAdmin for UX. Linked Supabase check: trigger functions not executable by anon/authenticated, auth.users triggers enabled, no first-user bootstrap, 0 unconfirmed allowlisted admins, 0 admin roles outside allowlist, 1 confirmed allowlisted admin.</x:v>
+        <x:v>QA-2026-07-01-015 added; prod has 1 confirmed allowlisted admin, 0 outside-allowlist admins, 0 unconfirmed allowlisted admins.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -6583,13 +6583,13 @@
         <x:v>Only allowlisted admin accounts can access moderation dashboard; first-user/admin behavior must be controlled.</x:v>
       </x:c>
       <x:c r="E20" s="50" t="str">
-        <x:v>Security scan: allowlisted email signup can grant admin before mailbox ownership verified.</x:v>
+        <x:v>Closed 2026-07-01: production auth policy smoke passed.</x:v>
       </x:c>
       <x:c r="F20" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G20" s="50" t="str">
-        <x:v>Automated pass 2026-06-29; production auth policy smoke pending</x:v>
+        <x:v>Passed 2026-07-01: scoped eslint; admin/auth/security tests 3 files / 18 tests; production security smoke passed with admin allowlist invariants.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="76" customHeight="1">
@@ -8254,7 +8254,33 @@
         <x:v>Added adversarial CI coverage for repeated prompt-injection leaks, multilingual requests for secrets/payment/wallet/APK actions, and safe-warning decoys. Existing degradation tests still prove rules-only scoring when AI is missing, failing, quota-limited, retried, or falling back.</x:v>
       </x:c>
       <x:c r="H35" t="str">
-        <x:v>Continue remaining P1 test queue: ADM-001 production auth policy smoke; then UX/logistics fixes.</x:v>
+        <x:v>Completed by QA-2026-07-01-015; P1 test queue closed, continue UX/logistics fixes and next product backlog.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>QA-2026-07-01-015</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>ADM-001 production auth policy smoke</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>npx eslint scripts/prod-security-smoke.ts src/lib/admin-allowlist-migration.test.ts src/lib/admin.functions.test.ts src/lib/prod-security-smoke-env.test.ts --quiet; npm run test:run -- src/lib/admin-allowlist-migration.test.ts src/lib/admin.functions.test.ts src/lib/prod-security-smoke-env.test.ts; railway run npm run prod:security-smoke</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>Passed: scoped eslint; focused admin/auth/security tests 3 files / 18 tests; production security smoke passed with admin allowlist invariants.</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>ADM-001, T-019</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>Production smoke now verifies anon cannot read admin_allowlist or user_roles, service can read the allowlist, and all admin roles belong to confirmed allowlisted users. Current prod counts: admins=1, confirmed_allowlisted=1, outside_allowlist=0, unconfirmed_allowlisted=0.</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>P1 test queue closed; continue with UX/logistics fixes and the next product backlog.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(telegram): clarify video thumbnail UX
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6b0ab9ffa8424b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbaec59b5e534448c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R845b0f89667a4a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R48a94e8da7a84031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2f9bc865d87146a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R556484f0fd6c4a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R776edab106e044f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R927597c150384171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rbdd4e10977954a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra8f019160d674e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R20eb986189274d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R64c6bfab3a414752"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>P1 test queue closed; continue with UX/logistics fixes and the next product backlog.</x:v>
+        <x:v>UX/logistics fixes: next T-013 / TG-025 modern scenario copy, then resume P1 web/Telegram QA flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ADM-001 production auth policy smoke passed.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-009/TG-013 video thumbnail UX closed with automated router/webhook/formatter QA and build.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -3428,13 +3428,13 @@
         <x:v>.kiro/specs/telegram-video-thumbnail-intelligence-v1</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I14" s="8" t="str">
-        <x:v>Manual QA</x:v>
+        <x:v>Router/webhook integration + QA matrix + formatter regression + build</x:v>
       </x:c>
       <x:c r="J14" s="8" t="str">
-        <x:v>Add clearer wait/unsupported video UX and avoid claiming full video analysis.</x:v>
+        <x:v>Closed 2026-07-01: video thumbnails carry video context into the result card; full video files are not fetched; fallback/help copy explicitly says only the preview frame is checked and asks for link/screenshot/text/audio when needed. Live Telegram video smoke remains a release checklist item after deploy.</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
         <x:v>P3</x:v>
@@ -6353,13 +6353,13 @@
         <x:v>The bot gives a useful fallback, asks for link/screenshot/text, and uses thumbnail intelligence where available.</x:v>
       </x:c>
       <x:c r="E10" s="50" t="str">
-        <x:v>Add clearer wait/unsupported video UX and avoid claiming full video analysis.</x:v>
+        <x:v>Closed 2026-07-01: automated coverage verifies thumbnail-only video analysis, no full-video download, and honest preview-frame/no-full-clip UX copy.</x:v>
       </x:c>
       <x:c r="F10" s="568" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="G10" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: eslint; router/webhook/bot QA matrix 3 files / 172 tests; formatter/image-intelligence 2 files / 70 tests; npm run build passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="76" customHeight="1">

</xml_diff>

<commit_message>
fix(telegram): distinguish modern sos copy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R776edab106e044f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R927597c150384171"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rbdd4e10977954a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra8f019160d674e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R20eb986189274d94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R64c6bfab3a414752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R774552f5cd0240e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rdacf5e182de84eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R703288f4629243bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc570d681f14e4ab1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R70437c2f7d294ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rfa083696fd1f472c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>UX/logistics fixes: next T-013 / TG-025 modern scenario copy, then resume P1 web/Telegram QA flows.</x:v>
+        <x:v>Next queue item: T-021 / ADM-003 phone reputation moderation signal, then remaining P2/P3 reputation/provider backlog.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-009/TG-013 video thumbnail UX closed with automated router/webhook/formatter QA and build.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-013/TG-025 modern SOS copy closed for sextortion, publication threats and minors.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -3884,13 +3884,13 @@
         <x:v>.kiro/specs/telegram-modern-sos-scenarios-v1; .kiro/specs/telegram-ai-voice-clone-sos-v1</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I26" s="8" t="str">
-        <x:v>Live QA screenshots</x:v>
+        <x:v>Unit/property/i18n tests + Telegram QA report/visual + build</x:v>
       </x:c>
       <x:c r="J26" s="8" t="str">
-        <x:v>Finish distinct copy for minors/sextortion/publication and remove duplicate generic text.</x:v>
+        <x:v>Closed 2026-07-01: first cards, detailed checklists and trusted-person follow-ups are distinct for sextortion, publication threats and minor safety; existing voice-clone and modern scenarios 12-15 remain covered. Live Telegram screenshot review remains release-check only.</x:v>
       </x:c>
       <x:c r="K26" s="14" t="str">
         <x:v>P3</x:v>
@@ -6445,13 +6445,13 @@
         <x:v>Each modern scenario has a short first card, context-specific next step, ready phrase, where-to-go, trusted-contact option, and full checklist.</x:v>
       </x:c>
       <x:c r="E14" s="50" t="str">
-        <x:v>Finish distinct copy for minors/sextortion/publication and remove duplicate generic text.</x:v>
+        <x:v>Closed 2026-07-01: distinct copy for minors, sextortion and publication threats implemented; duplicate generic trusted-person branch removed for those cases.</x:v>
       </x:c>
       <x:c r="F14" s="568" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="G14" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: eslint; emergency/panic/voice-out suite 4 files / 135 tests; emergency property/i18n/follow-up suite 5 files / 632 tests; bot QA matrix 18 tests; qa:telegram-report, qa:telegram-visual and npm run build passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">

</xml_diff>

<commit_message>
docs(tracker): close phone reputation v1
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R774552f5cd0240e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rdacf5e182de84eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R703288f4629243bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc570d681f14e4ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R70437c2f7d294ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rfa083696fd1f472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfabd182cf1644124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R300183551db14fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcc8fa3ab66374713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R293809db80f640f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc148a630f7db4c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R16c3cfc2ccf8411d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,10 +2621,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-021 / ADM-003 phone reputation moderation signal, then remaining P2/P3 reputation/provider backlog.</x:v>
+        <x:v>Next queue item: T-025 / CORE-005 URL reputation external signals, then T-029 / CORE-009 retention/audit verification and T-032 / SEC-003 adversarial safety slowdowns.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-013/TG-025 modern SOS copy closed for sextortion, publication threats and minors.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ADM-003 / CORE-004 phone reputation v1 reconciled: confirmed-only entities feed public phone reputation with source/confidence limits.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2652,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2665,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4378,19 +4378,19 @@
         <x:v>.kiro/specs/phone-reputation-v1; .kiro/specs/phone-directory-v1</x:v>
       </x:c>
       <x:c r="H39" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I39" s="8" t="str">
-        <x:v>Unit/manual QA</x:v>
+        <x:v>Admin/reputation unit tests + check-core property + formatter regression</x:v>
       </x:c>
       <x:c r="J39" s="8" t="str">
-        <x:v>Add phone reputation v1 and public confidence/source model.</x:v>
+        <x:v>Closed 2026-07-01: confirmed target moderation writes masked entities; Telegram targets sync to telegram_reputation_targets, while phone reputation uses confirmed entities rows only.</x:v>
       </x:c>
       <x:c r="K39" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L39" s="8" t="str">
-        <x:v>Confirmed label must be appealable and legally soft.</x:v>
+        <x:v>Public labels remain appealable and legally soft; incident-only reports do not create public reputation.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -4530,19 +4530,19 @@
         <x:v>.kiro/specs/phone-reputation-v1; .kiro/specs/phone-directory-v1</x:v>
       </x:c>
       <x:c r="H43" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I43" s="8" t="str">
-        <x:v>Unit tests</x:v>
+        <x:v>Phone reputation/intelligence unit tests + check-core pipeline + Telegram formatter regression</x:v>
       </x:c>
       <x:c r="J43" s="8" t="str">
-        <x:v>Build full Phone Reputation v1 after UX/security stabilization.</x:v>
+        <x:v>Closed 2026-07-01: Phone Reputation v1 combines phone passport, official contact exact-match/near-miss logic, confirmed-only moderated reports, and source/confidence labels without owner/carrier-private claims.</x:v>
       </x:c>
       <x:c r="K43" s="14" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="L43" s="8" t="str">
-        <x:v>Crowd reports need moderation before public reputation impact.</x:v>
+        <x:v>Confirmed reports only; no owner, SIM age, hidden spam label or unmoderated crowd reputation claims.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -6629,13 +6629,13 @@
         <x:v>Confirmed entities appear with masked public display, complaint count, risk, status, and last update.</x:v>
       </x:c>
       <x:c r="E22" s="50" t="str">
-        <x:v>Add phone reputation v1 and public confidence/source model.</x:v>
+        <x:v>Closed 2026-07-01: reputation entity base verified from existing code path; confirmed targeted reports become masked confirmed entities, incident-only reports do not publish reputation, and Telegram reputation sync remains confirmed/moderated only.</x:v>
       </x:c>
       <x:c r="F22" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G22" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: admin moderation boundary tests, phone reputation summary tests, check-core reputation property tests and formatter reputation regression passed locally.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="76" customHeight="1">
@@ -6698,13 +6698,13 @@
         <x:v>Number passport combines country/operator parsing, verified contacts, moderated complaints, and confidence/source labels.</x:v>
       </x:c>
       <x:c r="E25" s="50" t="str">
-        <x:v>Build full Phone Reputation v1 after UX/security stabilization.</x:v>
+        <x:v>Closed 2026-07-01: minimal Phone Reputation v1 verified; number passport shows country/operator, official directory status, confirmed Ishonch Guard report count and source/confidence limits.</x:v>
       </x:c>
       <x:c r="F25" s="568" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="G25" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Automated pass 2026-07-01: phone-intelligence, phone-reputation, check-core and Telegram formatter tests cover confirmed-only counts and no hidden owner/carrier/spam-label claims.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="76" customHeight="1">

</xml_diff>

<commit_message>
fix(risk): harden url reputation privacy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfabd182cf1644124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R300183551db14fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcc8fa3ab66374713"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R293809db80f640f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc148a630f7db4c58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R16c3cfc2ccf8411d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re5a0a84175f8434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R4d4e1d439f084be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ref38dee8a476457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0fc53a2ee07a4eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e06a7bf6f14461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re77b28b992ed4d6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2606,9 +2606,7 @@
       <x:c r="E1" s="588" t="str">
         <x:v>Owner note</x:v>
       </x:c>
-      <x:c r="F1" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: TG-007/TG-008 final username passport now preserves Native Passport Coach; QA report regenerated; scoped eslint, 5 files / 83 tests, qa:telegram-report and qa:telegram-visual passed.</x:v>
-      </x:c>
+      <x:c r="F1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
@@ -2621,10 +2619,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-025 / CORE-005 URL reputation external signals, then T-029 / CORE-009 retention/audit verification and T-032 / SEC-003 adversarial safety slowdowns.</x:v>
+        <x:v>Next queue item: T-029 / CORE-009 retention/audit verification, then T-032 / SEC-003 adversarial safety slowdowns.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ADM-003 / CORE-004 phone reputation v1 reconciled: confirmed-only entities feed public phone reputation with source/confidence limits.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-025 / CORE-005 URL reputation external signals reconciled: Safe Browsing/URLhaus/PhishTank are optional additive providers with sanitized URL-only payloads, short cache, and in-flight de-dupe.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2652,7 +2650,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2665,7 +2663,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4562,25 +4560,25 @@
         <x:v>Google Safe Browsing, URLhaus, and PhishTank signals add reason codes without replacing local rules.</x:v>
       </x:c>
       <x:c r="F44" s="8" t="str">
-        <x:v>src/lib/risk/url-reputation.server.ts; src/lib/risk/url-handling.ts</x:v>
+        <x:v>src/lib/risk/url-reputation.server.ts; src/lib/risk/check-core.ts; src/lib/risk/url-handling.ts</x:v>
       </x:c>
       <x:c r="G44" s="8" t="str">
-        <x:v>Roadmap Security Sprint</x:v>
+        <x:v>Roadmap Security Sprint; ai_docs/API.md; ai_docs/DEPLOYMENT.md</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I44" s="8" t="str">
-        <x:v>Unit tests for local URL handling</x:v>
+        <x:v>Provider unit tests + check-core privacy/cache/failure regressions + scoped eslint/tsc + full risk suite + build</x:v>
       </x:c>
       <x:c r="J44" s="8" t="str">
-        <x:v>Add providers, cache results, and redact mixed text before provider calls.</x:v>
+        <x:v>Closed 2026-07-01: Optional Safe Browsing, URLhaus, and PhishTank additive signals are wired; successful results are cached briefly, concurrent identical checks are deduped, and provider failures are not cached as clean results.</x:v>
       </x:c>
       <x:c r="K44" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L44" s="8" t="str">
-        <x:v>Security scan: mixed text URL checks can leak full user messages to external providers.</x:v>
+        <x:v>Provider calls receive only normalized http(s) URL origin/path; credentials, query, fragments, full messages, OTPs and report narratives are not sent.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -6721,13 +6719,13 @@
         <x:v>Google Safe Browsing, URLhaus, and PhishTank signals add reason codes without replacing local rules.</x:v>
       </x:c>
       <x:c r="E26" s="50" t="str">
-        <x:v>Add providers, cache results, and redact mixed text before provider calls.</x:v>
+        <x:v>Closed 2026-07-01: optional providers, URL-only privacy boundary, cache and in-flight dedupe verified.</x:v>
       </x:c>
       <x:c r="F26" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G26" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-01: tsc, scoped eslint, risk suite 29 files / 451 tests, production build.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="76" customHeight="1">
@@ -8283,6 +8281,32 @@
         <x:v>P1 test queue closed; continue with UX/logistics fixes and the next product backlog.</x:v>
       </x:c>
     </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>QA-2026-07-01-016</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>CORE-005 URL reputation external signals</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>npx tsc --noEmit --pretty false; npx eslint src/lib/risk/check-core.ts src/lib/risk/url-reputation.server.ts src/lib/risk/url-reputation.server.test.ts src/lib/risk/url-handling.test.ts; npm run test:run -- src/lib/risk; npm run build</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>Passed: tsc; scoped eslint; 29 files / 451 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>CORE-005, T-025</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>External reputation providers now receive sanitized URL-only origin/path tokens. Tests cover query/credential stripping, mixed-text redaction, payment-message URL extraction, cache reuse, concurrent de-dupe and provider failure non-cache.</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>Continue T-029 / CORE-009 retention/audit verification; keep provider API keys server-only in deployment.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(db): verify retention audit migrations
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re5a0a84175f8434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R4d4e1d439f084be8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ref38dee8a476457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0fc53a2ee07a4eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e06a7bf6f14461d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re77b28b992ed4d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1003ee7433fb411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3db32f0a5c564a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6f42dfc246114e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R83ae2059da0645e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R5c2d01edec254911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R16817fe627e743eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2619,10 +2619,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-029 / CORE-009 retention/audit verification, then T-032 / SEC-003 adversarial safety slowdowns.</x:v>
+        <x:v>Next queue item: T-032 / SEC-003 adversarial safety slowdowns, then T-035 / ROAD-003 latency/caching acknowledgements.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-025 / CORE-005 URL reputation external signals reconciled: Safe Browsing/URLhaus/PhishTank are optional additive providers with sanitized URL-only payloads, short cache, and in-flight de-dupe.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-029 / CORE-009 retention/audit verification reconciled: linked Supabase migrations match local, db lint passed, and static regressions cover retention windows, cron scheduling and admin audit RLS.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2650,7 +2650,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>48</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2663,7 +2663,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Code exists but known gaps remain.</x:v>
@@ -4718,19 +4718,19 @@
         <x:v>ai_docs/DATABASE.md; ai_docs/DEPLOYMENT.md</x:v>
       </x:c>
       <x:c r="H48" s="14" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I48" s="8" t="str">
-        <x:v>Migration/manual QA</x:v>
+        <x:v>Static migration regression + admin fail-closed tests + linked Supabase migration/lint checks + full src/lib + build</x:v>
       </x:c>
       <x:c r="J48" s="8" t="str">
-        <x:v>Verify retention cleanup and admin audit records after current dirty branch settles.</x:v>
+        <x:v>Closed 2026-07-01: retention cleanup is scheduled via pg_cron, remote migration history matches local, linked db lint passed, and tests verify retention windows plus audit/appeal preservation.</x:v>
       </x:c>
       <x:c r="K48" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L48" s="8" t="str">
-        <x:v>RLS/policies must keep service-role writes server-side only.</x:v>
+        <x:v>RLS/policies keep service-role writes server-side only; private retention helper is service-role-only and does not delete admin_actions or reputation_appeals.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -6811,13 +6811,13 @@
         <x:v>Supabase migrations create tables, constraints, indexes, privacy policies, cleanup jobs, and admin audit structures.</x:v>
       </x:c>
       <x:c r="E30" s="50" t="str">
-        <x:v>Verify retention cleanup and admin audit records after current dirty branch settles.</x:v>
+        <x:v>Closed 2026-07-01: retention cleanup and admin audit records verified by static migration tests plus linked Supabase checks.</x:v>
       </x:c>
       <x:c r="F30" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G30" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-01: focused CORE-009 tests 4 files / 20 tests; tsc; supabase db lint --linked public,private; migration list --linked; full src/lib 95 files / 1810 tests; build.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="76" customHeight="1">
@@ -8307,6 +8307,32 @@
         <x:v>Continue T-029 / CORE-009 retention/audit verification; keep provider API keys server-only in deployment.</x:v>
       </x:c>
     </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>QA-2026-07-01-017</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>CORE-009 retention and admin audit verification</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>npx eslint src/lib/retention-audit-migration.test.ts src/lib/admin.functions.test.ts src/lib/admin-allowlist-migration.test.ts src/lib/public-impact-counters-migration.test.ts --quiet; npm run test:run -- src/lib/retention-audit-migration.test.ts src/lib/admin.functions.test.ts src/lib/admin-allowlist-migration.test.ts src/lib/public-impact-counters-migration.test.ts; supabase db lint --linked --schema public,private --fail-on error; supabase migration list --linked; npx tsc --noEmit --pretty false; npm run test:run -- src/lib; npm run build</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>Passed: focused 4 files / 20 tests; linked Supabase db lint no schema errors; local/remote migrations match; tsc; full src/lib 95 files / 1810 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>CORE-009, T-029</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>Static migration coverage now verifies private service-role-only retention cleanup, documented cleanup windows, cron.schedule/cron.unschedule usage, admin_actions RLS/admin-read policy and preservation of admin_actions/reputation_appeals. Local Supabase stack was not running because Docker daemon was unavailable; linked checks were used instead.</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>Proceed to T-032 / SEC-003 adversarial safety slowdowns; local DB reset/lint can be rerun when Docker is available.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(risk): throttle repeated unsafe ai output
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1003ee7433fb411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3db32f0a5c564a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6f42dfc246114e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R83ae2059da0645e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R5c2d01edec254911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R16817fe627e743eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rabc9aec8aa1f4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R73b2b4fefbd44d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R72f5dfe207a34923"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0ae5bd2d032c4f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R43cf19112a8b4da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R56c5b7393c3e4681"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2619,7 +2619,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-032 / SEC-003 adversarial safety slowdowns, then T-035 / ROAD-003 latency/caching acknowledgements.</x:v>
+        <x:v>Next queue item: T-035 / ROAD-003 latency/caching acknowledgements, then T-036 / ROAD-004 check whole conversation.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
         <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-029 / CORE-009 retention/audit verification reconciled: linked Supabase migrations match local, db lint passed, and static regressions cover retention windows, cron scheduling and admin audit RLS.</x:v>
@@ -2650,7 +2650,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2676,7 +2676,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -4826,25 +4826,25 @@
         <x:v>CI includes red-team prompts and repeated firewall-block behavior can slow abusive probing.</x:v>
       </x:c>
       <x:c r="F51" s="8" t="str">
-        <x:v>planned: src/lib/risk/ai-output-safety.ts; tests</x:v>
+        <x:v>src/lib/risk/ai-output-safety.ts; src/lib/risk/check-core.ts; tests</x:v>
       </x:c>
       <x:c r="G51" s="8" t="str">
         <x:v>Roadmap Security Sprint</x:v>
       </x:c>
       <x:c r="H51" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I51" s="8" t="str">
-        <x:v>Needs tests</x:v>
+        <x:v>Focused tests + broad risk/Telegram tests + build</x:v>
       </x:c>
       <x:c r="J51" s="8" t="str">
-        <x:v>Add property/adversarial prompts and user-level slowdowns after repeated blocks.</x:v>
+        <x:v>Closed 2026-07-01: repeated unsafe AI provider outputs open a short per-rate-limit-key cooldown; deterministic scoring, advice and persistence continue rules-only.</x:v>
       </x:c>
       <x:c r="K51" s="13" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L51" s="8" t="str">
-        <x:v>Must avoid harming normal users who ask confused safety questions.</x:v>
+        <x:v>2026-07-01: SEC-003 implemented. AI explanation sanitization now returns blocked finding metadata; runCheck records unsafe provider output and skips subsequent AI explanations for the same key during cooldown; tests prove the third repeated adversarial response does not call AI.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -6880,13 +6880,13 @@
         <x:v>CI includes red-team prompts and repeated firewall-block behavior can slow abusive probing.</x:v>
       </x:c>
       <x:c r="E33" s="50" t="str">
-        <x:v>Add property/adversarial prompts and user-level slowdowns after repeated blocks.</x:v>
+        <x:v>Closed 2026-07-01: unsafe AI explanation blocks are counted per rate-limit key and repeated blocks open a short cooldown that skips further AI explanations without blocking deterministic checks.</x:v>
       </x:c>
       <x:c r="F33" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G33" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-01: focused AI safety/degradation tests 3 files / 31 tests; scoped eslint; tsc; broad risk/Telegram tests 32 files / 518 tests; production build.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="76" customHeight="1">
@@ -8333,6 +8333,32 @@
         <x:v>Proceed to T-032 / SEC-003 adversarial safety slowdowns; local DB reset/lint can be rerun when Docker is available.</x:v>
       </x:c>
     </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>QA-2026-07-01-018</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>SEC-003 adversarial AI-output cooldown</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>npx eslint src/lib/risk/ai-output-safety.ts src/lib/risk/ai-output-safety.test.ts src/lib/risk/check-core.ts src/lib/risk/check-core.ai-output-safety.test.ts src/lib/telegram/ai-degradation.integration.test.ts --quiet; npm run test:run -- src/lib/risk/ai-output-safety.test.ts src/lib/risk/check-core.ai-output-safety.test.ts src/lib/telegram/ai-degradation.integration.test.ts; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/risk src/lib/telegram/ai-degradation.integration.test.ts src/lib/telegram/format.test.ts src/lib/telegram/bot-qa-matrix.test.ts; npm run build</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>Passed: scoped eslint; focused 3 files / 31 tests; tsc; broad risk/Telegram 32 files / 518 tests; production build passed</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>SEC-003, T-032</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>AI-output safety now exposes sanitization findings, records repeated blocked provider responses per rate-limit key and opens a short in-memory cooldown. During cooldown runCheck keeps deterministic verdict, advice and persistence and stores ai_explanation as null.</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>Proceed to T-035 / ROAD-003 speed and cost pass; then T-036 / ROAD-004 conversation grouping design.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(tracker): close ROAD-003 speed cost pass
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rabc9aec8aa1f4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R73b2b4fefbd44d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R72f5dfe207a34923"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0ae5bd2d032c4f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R43cf19112a8b4da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R56c5b7393c3e4681"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3d29d08d20d24665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re43c660337434864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rf50095bfee5d42f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra51ea27f8afb4f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raa7363f5d9a648c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R37eeffd4a93e4ff7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2619,7 +2619,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-035 / ROAD-003 latency/caching acknowledgements, then T-036 / ROAD-004 check whole conversation.</x:v>
+        <x:v>Next queue item: T-036 / ROAD-004 check whole conversation, then T-037 / ROAD-005 explain like grandmother.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
         <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: T-029 / CORE-009 retention/audit verification reconciled: linked Supabase migrations match local, db lint passed, and static regressions cover retention windows, cron scheduling and admin audit RLS.</x:v>
@@ -2650,7 +2650,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2676,7 +2676,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -4940,25 +4940,25 @@
         <x:v>Bot sends immediate 'checking/recognizing' status, caches repeated checks/TTS, avoids AI when rules are enough, and controls quotas.</x:v>
       </x:c>
       <x:c r="F54" s="8" t="str">
-        <x:v>src/lib/risk/check-core.ts; src/lib/telegram/voice-out.server.ts; src/lib/risk/url-reputation.server.ts</x:v>
+        <x:v>src/lib/telegram/handlers/check.ts; src/lib/telegram/public-metadata.server.ts; src/lib/telegram/voice-out.server.ts; src/lib/risk/check-core.ts; src/lib/risk/url-reputation.server.ts</x:v>
       </x:c>
       <x:c r="G54" s="8" t="str">
         <x:v>User plan P9</x:v>
       </x:c>
       <x:c r="H54" s="15" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I54" s="8" t="str">
-        <x:v>Needs performance tests</x:v>
+        <x:v>Focused latency/cost tests + tsc</x:v>
       </x:c>
       <x:c r="J54" s="8" t="str">
-        <x:v>Measure 5-10s paths and add caching/early acknowledgements.</x:v>
+        <x:v>Closed 2026-07-01: Telegram checks have delayed visible checking status, per-user cache/in-flight de-dupe, public metadata soft timeout/cache, low-signal AI skip, QR fast path, URL reputation cache/de-dupe and voice/TTS budget guards.</x:v>
       </x:c>
       <x:c r="K54" s="14" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="L54" s="8" t="str">
-        <x:v>Cost guards must run before external providers.</x:v>
+        <x:v>2026-07-01: ROAD-003 reconciled/verified. Focused suite passed 7 files / 170 tests: check cache/status, metadata timeout/cache, voice STT cache/budget, Voice-out duplicate/TTS budget, QR/image fast path and URL reputation cache. Production timing-log tuning remains an operational follow-up, not a blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -6949,13 +6949,13 @@
         <x:v>Bot sends immediate 'checking/recognizing' status, caches repeated checks/TTS, avoids AI when rules are enough, and controls quotas.</x:v>
       </x:c>
       <x:c r="E36" s="50" t="str">
-        <x:v>Measure 5-10s paths and add caching/early acknowledgements.</x:v>
+        <x:v>Closed 2026-07-01: delayed checking status, repeated-check cache/in-flight de-dupe, AI skip for low-signal deterministic checks, QR fast path, URL reputation cache/de-dupe and voice/TTS budgets verified.</x:v>
       </x:c>
       <x:c r="F36" s="568" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="G36" s="50" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-01: focused latency/cost tests 7 files / 170 tests; tsc passed. Covered check.cache, public metadata timeout/cache, voice STT cache/budget, Voice-out duplicate/budget, webhook image/QR fast path and URL reputation cache.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="76" customHeight="1">
@@ -8359,6 +8359,32 @@
         <x:v>Proceed to T-035 / ROAD-003 speed and cost pass; then T-036 / ROAD-004 conversation grouping design.</x:v>
       </x:c>
     </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>QA-2026-07-01-019</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>ROAD-003 speed/cost latency guard verification</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.cache.test.ts src/lib/telegram/public-metadata.server.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/voice-out.server.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/risk/url-reputation.server.test.ts src/lib/risk/url-handling.test.ts; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>Passed: focused latency/cost suite 7 files / 170 tests; tsc passed</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>ROAD-003, T-035</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>Verified the shipped speed/cost guards: delayed checking status for slow text checks; short per-user result cache and in-flight de-duplication; Telegram metadata timeout/cache; low-signal deterministic AI skip; decoded actionable QR path that skips visual AI; URL reputation cache/de-dupe; voice STT cache/in-flight/budget and Voice-out duplicate/TTS budget guards.</x:v>
+      </x:c>
+      <x:c r="H40" t="str">
+        <x:v>Proceed to T-036 / ROAD-004 conversation grouping design; keep production telegram_timing logs for ongoing STT/image-analysis tuning.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): add conversation check mode
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2655,7 +2655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>Next queue item: T-036 / ROAD-004 implementation slice: conversation_check collector + deterministic stage/action extractor; then T-037 / ROAD-005 explain like grandmother.</t>
+          <t>Next queue item: T-037 / ROAD-005 explain like grandmother; then continue remaining P4/P5 roadmap items.</t>
         </is>
       </c>
       <c r="E2" s="20" t="inlineStr">
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>planned: src/lib/telegram/handlers/check.ts; src/lib/risk/check-core.ts; spec: .kiro/specs/telegram-conversation-check-v1</t>
+          <t>src/lib/telegram/conversation-check.ts; src/lib/telegram/handlers/conversation.ts; src/lib/telegram/session.server.ts; src/lib/telegram/handlers/index.ts; src/lib/telegram/format.ts; src/lib/telegram/bot-i18n.ts</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -6480,17 +6480,17 @@
       </c>
       <c r="H55" s="15" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>Design/spec review</t>
+          <t>Unit + Telegram integration tests</t>
         </is>
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
-          <t>Design/spec completed 2026-07-01. Implementation next: explicit conversation_check mode, bounded draft, deterministic stage/action extraction, compact RU/UZ/EN rendering.</t>
+          <t>Implemented 2026-07-01: /conversation and main-menu whole-chat action collect 2-8 text/forwarded messages, store only derived metadata, analyze stages/actions/pressure and render a compact RU/UZ/EN result.</t>
         </is>
       </c>
       <c r="K55" s="15" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="L55" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01: Privacy-first design added. Session state may store only derived stage/action/reason metadata, never raw transcripts, URLs, phone numbers, usernames, OCR, OTP/PIN/CVV, cards, passwords, seed phrases or files. T-036 remains open for implementation.</t>
+          <t>2026-07-01: ROAD-004 implemented. Session conversation draft stores message count, total chars, strongest level, stage/action/pressure/reason metadata only. Tests prove raw SMS code/URL/source text are absent from telegram_sessions and ordinary URL checks outside conversation mode still use the normal pipeline.</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="E37" s="50" t="inlineStr">
         <is>
-          <t>Design/spec completed 2026-07-01; implementation still open. Next risk: add collector without capturing ordinary single-item URL/phone/username checks and without raw transcript persistence.</t>
+          <t>Closed 2026-07-01: explicit /conversation mode implemented with privacy-safe draft, deterministic stage/action extractor, analyze/cancel callbacks and normal pipeline boundary.</t>
         </is>
       </c>
       <c r="F37" s="569" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="G37" s="50" t="inlineStr">
         <is>
-          <t>Design reviewed 2026-07-01: .kiro/specs/telegram-conversation-check-v1 created. Tests not run for implementation because code is not started.</t>
+          <t>Passed 2026-07-01: focused conversation/router/webhook/format tests 5 files / 212 tests; full Telegram suite 48 files / 1289 tests; full src/lib 96 files / 1851 tests; tsc and scoped eslint passed.</t>
         </is>
       </c>
     </row>
@@ -10245,7 +10245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11980,6 +11980,48 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>QA-2026-07-01-021</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>ROAD-004 Telegram conversation check implementation</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>npx eslint src/lib/telegram/conversation-check.ts src/lib/telegram/conversation-check.test.ts src/lib/telegram/handlers/conversation.ts src/lib/telegram/handlers/commands.ts src/lib/telegram/handlers/index.ts src/lib/telegram/handlers/misc.ts src/lib/telegram/session.server.ts src/lib/telegram/format.ts src/lib/telegram/router.ts src/lib/telegram/router.test.ts src/lib/telegram/start-language-buttons.test.ts src/lib/telegram/webhook.integration.test.ts --quiet; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Passed: scoped eslint; tsc; Telegram suite 48 files / 1289 tests; full src/lib 96 files / 1851 tests</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>ROAD-004, T-036</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Verified /conversation start, safe collection, analyze callback, compact high-risk result, no checks insert during conversation analysis, no raw SMS code/URL/source phrase in telegram_sessions, and ordinary URL checks outside explicit conversation mode still use the normal pipeline.</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>Proceed to T-037 / ROAD-005 explain-like-grandmother copy/action layer.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(telegram): add family codeword guide
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd9658a86267c46d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R5cc915cadb004fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R156835d6c7b04d91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rfec4ae4a14e14c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb1c1cff206eb4f8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R51410944e14b4f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R40a5af7c2b06454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc1907ac8f84240e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R074bdd2d35a84865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R7455ec3fde6545a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ree18e62077dc4650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd438f4d504b2441c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2701,10 +2701,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-038 / ROAD-006 family codeword; then continue remaining P4/P5 roadmap items.</x:v>
+        <x:v>Next queue item: T-039 / ROAD-007 scam-call trainer and mini-quiz; continue remaining P5 roadmap items.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ROAD-005 shipped simple explanation follow-ups/buttons for elder-friendly verdict explanations without changing risk scoring.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ROAD-006 shipped privacy-first family codeword guidance for voice-clone prevention without storing family secrets.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2740,7 +2740,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2774,7 +2774,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="8" t="inlineStr">
         <x:is>
@@ -6565,40 +6565,28 @@
           <x:t xml:space="preserve">Bot helps families set a private codeword reminder and explains how to verify voice requests through another channel.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F57" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">planned: src/lib/telegram/family-shield.server.ts; src/lib/telegram/emergency.ts</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G57" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roadmap wow features</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H57" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I57" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs privacy design</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J57" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do not store actual codeword in plaintext; consider only teaching flow without persistence.</x:t>
-        </x:is>
+      <x:c r="F57" s="8" t="str">
+        <x:v>src/lib/telegram/family-shield.server.ts; src/lib/telegram/handlers/misc.ts; src/lib/telegram/bot-i18n.ts</x:v>
+      </x:c>
+      <x:c r="G57" s="8" t="str">
+        <x:v>Roadmap wow features; ai_docs/EXECUTION_PLAN_2026-06-21.md</x:v>
+      </x:c>
+      <x:c r="H57" s="15" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I57" s="8" t="str">
+        <x:v>Unit + webhook integration tests</x:v>
+      </x:c>
+      <x:c r="J57" s="8" t="str">
+        <x:v>Closed 2026-07-01: Family Shield now exposes a privacy-first codeword guide button; callback shows RU/UZ/EN offline setup instructions and returns to Family Shield actions.</x:v>
       </x:c>
       <x:c r="K57" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P4</x:t>
         </x:is>
       </x:c>
-      <x:c r="L57" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Never ask user to send sensitive family secrets to the bot unless storage model is approved.</x:t>
-        </x:is>
+      <x:c r="L57" s="8" t="str">
+        <x:v>Does not store or request the actual family codeword; trusted-contact alerts now recommend saved-number callback plus codeword/private-question verification for suspicious voice/video requests.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -9699,20 +9687,14 @@
           <x:t xml:space="preserve">Bot helps families set a private codeword reminder and explains how to verify voice requests through another channel.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E39" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do not store actual codeword in plaintext; consider only teaching flow without persistence.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F39" s="569" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G39" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not run</x:t>
-        </x:is>
+      <x:c r="E39" s="50" t="str">
+        <x:v>Closed 2026-07-01: shipped teaching-only codeword guide in Family Shield; no plaintext or recoverable family codeword storage added.</x:v>
+      </x:c>
+      <x:c r="F39" s="569" t="str">
+        <x:v>P4</x:v>
+      </x:c>
+      <x:c r="G39" s="50" t="str">
+        <x:v>Passed 2026-07-01: focused Family Shield/webhook/i18n tests passed; final scoped eslint, tsc and Telegram suite recorded in QA-2026-07-01-023.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="76" customHeight="1">
@@ -11995,6 +11977,32 @@
         <x:v>Proceed to T-038 / ROAD-006 family codeword.</x:v>
       </x:c>
     </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>QA-2026-07-01-023</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>ROAD-006 family codeword privacy-first flow</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>npx eslint src/lib/telegram/family-shield.server.ts src/lib/telegram/family-shield.server.test.ts src/lib/telegram/bot-i18n.ts src/lib/telegram/handlers/misc.ts src/lib/telegram/webhook.integration.test.ts --quiet; npm run test:run -- src/lib/telegram/family-shield.server.test.ts; npm run test:run -- src/lib/telegram/webhook.integration.test.ts; npm run test:run -- src/lib/telegram/bot-i18n.test.ts src/lib/telegram/i18n-completeness.test.ts; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>Passed: scoped eslint; Family Shield unit 10 tests; webhook integration 86 tests; i18n completeness 644 tests; tsc; full Telegram suite 48 files / 1307 tests; full src/lib suite 96 files / 1869 tests</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>ROAD-006, T-038</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>Verified Family Shield codeword button, callback guide, no checks insert or stored family secret, no request to send a codeword to the bot, and trusted-contact alert guidance for saved-number callback plus codeword/private-question verification.</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>Proceed to T-039 / ROAD-007 scam-call trainer and mini-quiz.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): add scam-call trainer
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R40a5af7c2b06454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc1907ac8f84240e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R074bdd2d35a84865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R7455ec3fde6545a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ree18e62077dc4650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd438f4d504b2441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re9f328f59a8b4a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R60efa41607a54aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rfd57fac1e3f54e96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbc6919bd42b6447a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R7621b0181d194f2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rda35eaf1954b4885"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2689,10 +2689,8 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-01</x:t>
-        </x:is>
+      <x:c r="A2" s="20" t="str">
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
         <x:v>58</x:v>
@@ -2701,10 +2699,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-039 / ROAD-007 scam-call trainer and mini-quiz; continue remaining P5 roadmap items.</x:v>
+        <x:v>Next queue item: T-040 / ROAD-008 privacy-safe scam map/index; continue remaining P5 roadmap items.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-01: ROAD-006 shipped privacy-first family codeword guidance for voice-clone prevention without storing family secrets.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-007 shipped Telegram scam-call trainer mini-quiz with callback-only score state and defensive-only feedback.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2740,7 +2738,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2774,7 +2772,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="8" t="inlineStr">
         <x:is>
@@ -6615,40 +6613,28 @@
           <x:t xml:space="preserve">Bot/site present short simulated scenarios, feedback, streaks, and shareable safe education.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F58" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">planned: website + telegram</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G58" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roadmap wow features</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H58" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I58" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs design</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J58" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build after trust/safety backlog stabilizes.</x:t>
-        </x:is>
+      <x:c r="F58" s="8" t="str">
+        <x:v>src/lib/telegram/scam-trainer.ts; src/lib/telegram/format.ts; src/lib/telegram/handlers/commands.ts; src/lib/telegram/handlers/misc.ts; scripts/set-bot-commands.ts</x:v>
+      </x:c>
+      <x:c r="G58" s="8" t="str">
+        <x:v>Roadmap wow features; ai_docs/EXECUTION_PLAN_2026-06-21.md</x:v>
+      </x:c>
+      <x:c r="H58" s="15" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I58" s="8" t="str">
+        <x:v>Unit + webhook integration tests</x:v>
+      </x:c>
+      <x:c r="J58" s="8" t="str">
+        <x:v>Closed 2026-07-02: /trainer and main-menu trainer entry show a five-situation defensive mini-quiz; scoring is encoded in callback data and no session/check row is created.</x:v>
       </x:c>
       <x:c r="K58" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P5</x:t>
         </x:is>
       </x:c>
-      <x:c r="L58" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Trainer content must not teach attackers precise bypass scripts.</x:t>
-        </x:is>
+      <x:c r="L58" s="8" t="str">
+        <x:v>Training content stays defensive: no attacker-ready scripts, no exact scammer playbooks, no storage of user answers or sensitive evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -9718,20 +9704,14 @@
           <x:t xml:space="preserve">Bot/site present short simulated scenarios, feedback, streaks, and shareable safe education.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E40" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build after trust/safety backlog stabilizes.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F40" s="570" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G40" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not run</x:t>
-        </x:is>
+      <x:c r="E40" s="50" t="str">
+        <x:v>Closed 2026-07-02: shipped Telegram-first callback-only mini-quiz with defensive feedback and no persistence.</x:v>
+      </x:c>
+      <x:c r="F40" s="570" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="G40" s="50" t="str">
+        <x:v>Passed 2026-07-02: scoped eslint, tsc, focused trainer/menu/router/command tests, webhook integration, i18n completeness, full Telegram suite and src/lib suite all passed; final suite recorded in QA-2026-07-02-001.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="76" customHeight="1">
@@ -12003,6 +11983,32 @@
         <x:v>Proceed to T-039 / ROAD-007 scam-call trainer and mini-quiz.</x:v>
       </x:c>
     </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>QA-2026-07-02-001</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>ROAD-007 scam-call trainer mini-quiz</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>npx eslint src/lib/telegram/scam-trainer.ts src/lib/telegram/scam-trainer.test.ts src/lib/telegram/format.ts src/lib/telegram/bot-i18n.ts src/lib/telegram/router.ts src/lib/telegram/router.test.ts src/lib/telegram/handlers/commands.ts src/lib/telegram/handlers/misc.ts src/lib/telegram/bot-qa-matrix.test.ts src/lib/telegram/start-language-buttons.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/set-bot-commands.test.ts scripts/set-bot-commands.ts --quiet; npm run test:run -- src/lib/telegram/scam-trainer.test.ts src/lib/telegram/start-language-buttons.test.ts src/lib/telegram/bot-qa-matrix.test.ts src/lib/telegram/router.test.ts src/lib/telegram/set-bot-commands.test.ts; npm run test:run -- src/lib/telegram/webhook.integration.test.ts; npm run test:run -- src/lib/telegram/i18n-completeness.test.ts; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>Passed: scoped eslint 0 errors; tsc --noEmit 0 errors; focused trainer/menu/router/command suite 5 files / 120 tests; webhook integration 89 tests; i18n completeness 651 tests; full Telegram suite 49 files / 1325 tests; full src/lib suite 97 files / 1887 tests.</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>ROAD-007, T-039</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>Verified /trainer command, main-menu Trainer callback, question/answer callbacks, callback-only score state, no checks insert, and defensive-only content guards against attacker-ready scripts.</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>Proceed to T-040 / ROAD-008 privacy-safe scam map/index.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(web): add privacy-safe scam map index
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re9f328f59a8b4a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R60efa41607a54aab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rfd57fac1e3f54e96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbc6919bd42b6447a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R7621b0181d194f2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rda35eaf1954b4885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R322fd186b26c41a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R91d3e91cd93242db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3b9b19bcdcf049cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0366aa9cb4f9477d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R94ac8d393c6c4ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R505a2f64df0041f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2693,16 +2693,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-040 / ROAD-008 privacy-safe scam map/index; continue remaining P5 roadmap items.</x:v>
+        <x:v>Next queue item: T-041 / ROAD-009 Weekly Scam Digest data model; continue remaining P5 roadmap items.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-007 shipped Telegram scam-call trainer mini-quiz with callback-only score state and defensive-only feedback.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-008 shipped privacy-safe scam map/index with national/category buckets and regional suppression thresholds.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2738,7 +2738,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>55</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2900,7 +2900,7 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D14" s="8" t="n">
         <x:v>5</x:v>
@@ -6638,65 +6638,79 @@
       </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ROAD-008</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roadmap</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Public scam map/index</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">As the public, I want a privacy-safe view of current scam patterns in Uzbekistan.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Site shows aggregate trends, regions, and scheme types only when privacy thresholds are met.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">planned: src/routes/scam-trends.tsx; src/lib/scam-trends.server.ts</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roadmap differentiation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H59" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs data policy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Define aggregation thresholds and moderation rules first.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K59" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L59" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No doxxing, no raw targets, no low-count deanonymization.</x:t>
-        </x:is>
+      <x:c r="A59" s="8" t="str">
+        <x:v>ROAD-008</x:v>
+      </x:c>
+      <x:c r="B59" s="8" t="str">
+        <x:v>Roadmap</x:v>
+      </x:c>
+      <x:c r="C59" s="8" t="str">
+        <x:v>Public scam map/index</x:v>
+      </x:c>
+      <x:c r="D59" s="8" t="str">
+        <x:v>As the public, I want a privacy-safe view of current scam patterns in Uzbekistan.</x:v>
+      </x:c>
+      <x:c r="E59" s="8" t="str">
+        <x:v>Site shows aggregate trends, regions, and scheme types only when privacy thresholds are met.</x:v>
+      </x:c>
+      <x:c r="F59" s="8" t="str">
+        <x:v>src/lib/trust/scam-map-index.ts; src/components/ScamMapIndexPanel.tsx; src/routes/scam-trends.tsx</x:v>
+      </x:c>
+      <x:c r="G59" s="8" t="str">
+        <x:v>Roadmap differentiation; ai_docs/ROADMAP.md</x:v>
+      </x:c>
+      <x:c r="H59" s="15" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I59" s="8" t="str">
+        <x:v>Unit + browser build/visual tests</x:v>
+      </x:c>
+      <x:c r="J59" s="8" t="str">
+        <x:v>Closed 2026-07-02: /scam-trends now includes a national privacy-safe map/index, category buckets and a locked regional layer with explicit thresholds; no private reports are read.</x:v>
+      </x:c>
+      <x:c r="K59" s="16" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="L59" s="8" t="str">
+        <x:v>Region publication is suppressed until 5 moderated records, 3 distinct scheme types and 2 source types exist; no raw reports, screenshots, OCR, full phone numbers, usernames, URLs, cards, codes, chat ids or user ids are exposed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>ROAD-009</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>Roadmap</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>Weekly Scam Digest data model</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>As a user/operator, I want digest entries to have source, status and updated_at before automation.</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>Digest records include source, status, updated_at, manual publish and safe stale fallback before any research-feed automation.</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>planned: src/lib/telegram/digest.ts; future digest data model helper</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Roadmap wow features; ai_docs/ROADMAP.md</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>Needs data model tests</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>Define records, stale fallback and manual publish boundaries first.</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="L60" t="str">
+        <x:v>No raw reports, copied Telegram posts or unverifiable accusations; publish only curated records with source/status/updated_at and stale fallback.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9715,40 +9729,49 @@
       </x:c>
     </x:row>
     <x:row r="41" ht="76" customHeight="1">
-      <x:c r="A41" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T-040</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B41" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ROAD-008</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C41" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">As the public, I want a privacy-safe view of current scam patterns in Uzbekistan.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D41" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Site shows aggregate trends, regions, and scheme types only when privacy thresholds are met.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E41" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Define aggregation thresholds and moderation rules first.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F41" s="570" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G41" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not run</x:t>
-        </x:is>
+      <x:c r="A41" s="50" t="str">
+        <x:v>T-040</x:v>
+      </x:c>
+      <x:c r="B41" s="50" t="str">
+        <x:v>ROAD-008</x:v>
+      </x:c>
+      <x:c r="C41" s="50" t="str">
+        <x:v>As the public, I want a privacy-safe view of current scam patterns in Uzbekistan.</x:v>
+      </x:c>
+      <x:c r="D41" s="50" t="str">
+        <x:v>Site shows aggregate trends, regions, and scheme types only when privacy thresholds are met.</x:v>
+      </x:c>
+      <x:c r="E41" s="50" t="str">
+        <x:v>Closed 2026-07-02: shipped national/category privacy-safe map index and locked regional layer with explicit aggregation thresholds.</x:v>
+      </x:c>
+      <x:c r="F41" s="570" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="G41" s="50" t="str">
+        <x:v>Passed 2026-07-02: scoped eslint, trust tests, tsc, production build and Playwright desktop/mobile visual check passed; final suite recorded in QA-2026-07-02-002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>T-041</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>ROAD-009</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>As a user/operator, I want digest entries to have source, status and updated_at before automation.</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>Digest records include source, status, updated_at, manual publish and safe stale fallback before any research-feed automation.</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>Define records, stale fallback and manual publish boundaries first.</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>Not run</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12009,6 +12032,32 @@
         <x:v>Proceed to T-040 / ROAD-008 privacy-safe scam map/index.</x:v>
       </x:c>
     </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>QA-2026-07-02-002</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>ROAD-008 privacy-safe scam map/index</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>npx eslint src/lib/trust/scam-map-index.ts src/lib/trust/scam-map-index.test.ts src/components/ScamMapIndexPanel.tsx src/routes/scam-trends.tsx --quiet; npm run test:run -- src/lib/trust; npx tsc --noEmit --pretty false; npm run build; npx playwright screenshot --viewport-size=1440,1200 http://127.0.0.1:4177/scam-trends output/playwright/road008-scam-trends-desktop.png; npx playwright screenshot --viewport-size=390,1200 http://127.0.0.1:4177/scam-trends output/playwright/road008-scam-trends-mobile.png</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>Passed: scoped eslint 0 errors; trust suite 4 files / 22 tests; tsc --noEmit 0 errors; production build passed; Playwright desktop/mobile /scam-trends screenshots captured with no obvious overlap.</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>ROAD-008, T-040</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>Verified national privacy-safe map/index, category buckets, region suppression thresholds, no private-evidence shaped public fields, and desktop/mobile visual rendering.</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>Proceed to T-041 / ROAD-009 Weekly Scam Digest data model.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): add digest data model
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R322fd186b26c41a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R91d3e91cd93242db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3b9b19bcdcf049cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0366aa9cb4f9477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R94ac8d393c6c4ae5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R505a2f64df0041f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdcaa553b6a734126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra05214532fda4c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc788331f8dbd4dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R3298ecf2a76f448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R23fac298fcfc467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra8e81feb9f954d26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2693,16 +2693,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-041 / ROAD-009 Weekly Scam Digest data model; continue remaining P5 roadmap items.</x:v>
+        <x:v>Next queue item: T-042 / ROAD-010 Private moderation chat remaining workflow; finish high-signal research notifications and operator wording.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-008 shipped privacy-safe scam map/index with national/category buckets and regional suppression thresholds.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-009 shipped manual weekly digest source/status/updated-at records with stale fallback.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2738,7 +2738,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2818,10 +2818,8 @@
           <x:t xml:space="preserve">P1</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Trust/security blocker</x:t>
-        </x:is>
+      <x:c r="B10" s="8" t="str">
+        <x:v>Trust/security blocker</x:v>
       </x:c>
       <x:c r="C10" s="8" t="n">
         <x:v>19</x:v>
@@ -2837,13 +2835,11 @@
           <x:t xml:space="preserve">P2</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Near-term quality</x:t>
-        </x:is>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Near-term quality</x:v>
       </x:c>
       <x:c r="C11" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D11" s="8" t="n">
         <x:v>2</x:v>
@@ -2856,10 +2852,8 @@
           <x:t xml:space="preserve">P3</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Important product polish</x:t>
-        </x:is>
+      <x:c r="B12" s="8" t="str">
+        <x:v>Important product polish</x:v>
       </x:c>
       <x:c r="C12" s="8" t="n">
         <x:v>13</x:v>
@@ -2875,10 +2869,8 @@
           <x:t xml:space="preserve">P4</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Differentiation</x:t>
-        </x:is>
+      <x:c r="B13" s="8" t="str">
+        <x:v>Differentiation</x:v>
       </x:c>
       <x:c r="C13" s="8" t="n">
         <x:v>5</x:v>
@@ -2894,10 +2886,8 @@
           <x:t xml:space="preserve">P5</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Later growth</x:t>
-        </x:is>
+      <x:c r="B14" s="8" t="str">
+        <x:v>Later growth</x:v>
       </x:c>
       <x:c r="C14" s="8" t="n">
         <x:v>3</x:v>
@@ -6689,28 +6679,66 @@
         <x:v>As a user/operator, I want digest entries to have source, status and updated_at before automation.</x:v>
       </x:c>
       <x:c r="E60" t="str">
-        <x:v>Digest records include source, status, updated_at, manual publish and safe stale fallback before any research-feed automation.</x:v>
+        <x:v>Digest records include source, status, updatedAt, manual publish and safe stale fallback before any research-feed automation.</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>planned: src/lib/telegram/digest.ts; future digest data model helper</x:v>
+        <x:v>src/lib/telegram/digest.ts; src/lib/telegram/digest.test.ts</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>Roadmap wow features; ai_docs/ROADMAP.md</x:v>
+        <x:v>Roadmap wow features; .kiro/specs/telegram-weekly-scam-digest-v1; ai_docs/ROADMAP.md</x:v>
       </x:c>
       <x:c r="H60" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I60" t="str">
-        <x:v>Needs data model tests</x:v>
+        <x:v>Unit tests + typecheck + scoped lint</x:v>
       </x:c>
       <x:c r="J60" t="str">
-        <x:v>Define records, stale fallback and manual publish boundaries first.</x:v>
+        <x:v>Closed 2026-07-02: /digest now renders from manual source/status/updated-at records, filters drafts, stale and partial sets, and uses evergreen fallback when weekly topics are not fresh.</x:v>
       </x:c>
       <x:c r="K60" t="str">
         <x:v>P5</x:v>
       </x:c>
       <x:c r="L60" t="str">
-        <x:v>No raw reports, copied Telegram posts or unverifiable accusations; publish only curated records with source/status/updated_at and stale fallback.</x:v>
+        <x:v>No raw reports, copied Telegram posts, source labels, full URLs/phone numbers or unverifiable accusations are exposed; automation remains disabled until separate privacy review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>ROAD-010</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Roadmap</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>Private moderation chat remaining workflow</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>As an operator, I want private Telegram alerts for high-signal reports, appeals and research items without exposing user evidence.</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>Operator-only chat receives redacted summaries and admin links; high-signal research items get workflow wording and no raw evidence.</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>src/lib/telegram/moderation-notifier.server.ts; src/lib/report.functions.ts; src/lib/reputation-appeal.functions.ts; scripts/moderation-alert-smoke.ts</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>Needs unit + smoke tests</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>Finish high-signal research notifications and operator workflow wording; keep report/appeal alert slice intact.</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L61" t="str">
+        <x:v>Never send raw report text, screenshots, OCR, codes, cards, passwords, full phone numbers, URLs or user ids to moderator chat.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9762,17 +9790,46 @@
         <x:v>As a user/operator, I want digest entries to have source, status and updated_at before automation.</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Digest records include source, status, updated_at, manual publish and safe stale fallback before any research-feed automation.</x:v>
+        <x:v>Digest records include source, status, updatedAt, manual publish and safe stale fallback before any research-feed automation.</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>Define records, stale fallback and manual publish boundaries first.</x:v>
+        <x:v>Closed 2026-07-02: manual digest data model shipped with source/status/updatedAt records, draft filtering, minimum-topic freshness gate and evergreen stale fallback.</x:v>
       </x:c>
       <x:c r="F42" t="str">
         <x:v>P5</x:v>
       </x:c>
       <x:c r="G42" t="str">
+        <x:v>Passed 2026-07-02: scoped eslint for digest files, tsc 0 errors, digest unit 9 tests, full Telegram suite 49 files / 1330 tests, full src/lib suite 98 files / 1896 tests; final suite recorded in QA-2026-07-02-003.</x:v>
+      </x:c>
+      <x:c r="H42"/>
+      <x:c r="I42"/>
+      <x:c r="J42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>T-042</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>ROAD-010</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>As an operator, I want private Telegram alerts for high-signal research items without exposing user evidence.</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>Moderator chat receives redacted summaries and admin links only, including research-item workflow wording; existing report/appeal alerts stay private and sanitized.</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>Finish high-signal research notifications and operator workflow wording.</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
         <x:v>Not run</x:v>
       </x:c>
+      <x:c r="H43"/>
+      <x:c r="I43"/>
+      <x:c r="J43"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12058,6 +12115,32 @@
         <x:v>Proceed to T-041 / ROAD-009 Weekly Scam Digest data model.</x:v>
       </x:c>
     </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>QA-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>ROAD-009 weekly scam digest data model</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>npx eslint src/lib/telegram/digest.ts src/lib/telegram/digest.test.ts --quiet; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/telegram/digest.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>Passed: scoped eslint 0 errors; tsc 0 errors; digest unit 9 tests; full Telegram suite 49 files / 1330 tests; full src/lib suite 98 files / 1896 tests.</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>ROAD-009, T-041</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>Verified manual source/status/updated-at digest records, draft filtering, freshness/minimum-topic fallback, no source labels/raw report-shaped evidence in public text, and unchanged check/emergency/report keyboard.</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>Proceed to T-042 / ROAD-010 Private moderation chat remaining workflow.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(telegram): add moderation research alerts
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdcaa553b6a734126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra05214532fda4c8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc788331f8dbd4dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R3298ecf2a76f448d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R23fac298fcfc467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra8e81feb9f954d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd0c4cc38b5d94805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R260e7c8f3ab14d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R07cef81217ed43dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R8d418b2ab4ea4bb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re9d4b7d78b494338"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re1c0fe63f74e4da6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2693,16 +2693,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-042 / ROAD-010 Private moderation chat remaining workflow; finish high-signal research notifications and operator wording.</x:v>
+        <x:v>Next queue item: T-043 / ROAD-011 Web/embed Risk Passport compact reuse; reuse Telegram passport structure on web/embed without oversized partner UI.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-009 shipped manual weekly digest source/status/updated-at records with stale fallback.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-010 shipped private moderation research alerts with public scheme metadata only.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2738,7 +2738,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2890,7 +2890,7 @@
         <x:v>Later growth</x:v>
       </x:c>
       <x:c r="C14" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D14" s="8" t="n">
         <x:v>5</x:v>
@@ -6717,28 +6717,66 @@
         <x:v>As an operator, I want private Telegram alerts for high-signal reports, appeals and research items without exposing user evidence.</x:v>
       </x:c>
       <x:c r="E61" t="str">
-        <x:v>Operator-only chat receives redacted summaries and admin links; high-signal research items get workflow wording and no raw evidence.</x:v>
+        <x:v>Operator-only chat receives redacted report/appeal summaries and public-metadata research review packets with admin links only.</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>src/lib/telegram/moderation-notifier.server.ts; src/lib/report.functions.ts; src/lib/reputation-appeal.functions.ts; scripts/moderation-alert-smoke.ts</x:v>
+        <x:v>src/lib/telegram/moderation-notifier.server.ts; src/lib/telegram/moderation-notifier.server.test.ts; scripts/moderation-alert-smoke.ts</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md</x:v>
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/DEPLOYMENT.md</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I61" t="str">
-        <x:v>Needs unit + smoke tests</x:v>
+        <x:v>Unit tests + typecheck + scoped lint</x:v>
       </x:c>
       <x:c r="J61" t="str">
-        <x:v>Finish high-signal research notifications and operator workflow wording; keep report/appeal alert slice intact.</x:v>
+        <x:v>Closed 2026-07-02: high-signal research alerts now select active high/critical public scheme trends from research-feed/moderated sources, send only category/severity/source/reason-code metadata, and can be smoke-tested with --research.</x:v>
       </x:c>
       <x:c r="K61" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L61" t="str">
-        <x:v>Never send raw report text, screenshots, OCR, codes, cards, passwords, full phone numbers, URLs or user ids to moderator chat.</x:v>
+        <x:v>No raw report text, screenshots, OCR, codes, cards, passwords, full phone numbers, full URLs, raw posts or user ids are sent to moderator chat.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>ROAD-011</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>Roadmap</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>Web/embed Risk Passport compact reuse</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>As a web or partner-embed user, I want shallow phone/username checks to show the same honest passport structure as Telegram.</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>Website and iframe checks reuse compact passport sections for visible facts, local reputation boundaries and next evidence without making embeds too tall.</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>planned: src/components/RiskResultCard.tsx; src/components/EmbedCheckWidget.tsx; src/lib/risk/phone-intelligence.ts; src/lib/telegram/format.ts</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; .kiro/specs/risk-passport-v1</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>Needs web/embed UX tests</x:v>
+      </x:c>
+      <x:c r="J62" t="str">
+        <x:v>Reuse Telegram passport semantics on web/embed cards; keep partner iframe compact and avoid hidden Telegram/account-age/scam-label claims.</x:v>
+      </x:c>
+      <x:c r="K62" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="L62" t="str">
+        <x:v>No hidden Telegram facts, unmoderated report claims or raw private evidence in public/partner surfaces.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9819,17 +9857,43 @@
         <x:v>Moderator chat receives redacted summaries and admin links only, including research-item workflow wording; existing report/appeal alerts stay private and sanitized.</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>Finish high-signal research notifications and operator workflow wording.</x:v>
+        <x:v>Closed 2026-07-02: research moderation alert helper selects active high/critical public scheme trends and sends category, severity/source and reason-code ids only.</x:v>
       </x:c>
       <x:c r="F43" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G43" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-02: scoped eslint for notifier/smoke files, tsc 0 errors, moderation notifier unit 9 tests, full Telegram suite 49 files / 1333 tests, full src/lib suite 98 files / 1899 tests; final suite recorded in QA-2026-07-02-004.</x:v>
       </x:c>
       <x:c r="H43"/>
       <x:c r="I43"/>
       <x:c r="J43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>T-043</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>ROAD-011</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>As a web or partner-embed user, I want shallow phone/username checks to show the same honest passport structure as Telegram.</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>Website and iframe checks reuse compact passport sections for visible facts, local reputation boundaries and next evidence without making embeds too tall.</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>Adapt Risk Passport presentation to web and embed result cards.</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="H44"/>
+      <x:c r="I44"/>
+      <x:c r="J44"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12141,6 +12205,32 @@
         <x:v>Proceed to T-042 / ROAD-010 Private moderation chat remaining workflow.</x:v>
       </x:c>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>QA-2026-07-02-004</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>ROAD-010 private moderation chat research alerts</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>npx eslint src/lib/telegram/moderation-notifier.server.ts src/lib/telegram/moderation-notifier.server.test.ts scripts/moderation-alert-smoke.ts --quiet; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/telegram/moderation-notifier.server.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>Passed: scoped eslint 0 errors; tsc 0 errors; moderation notifier unit 9 tests; full Telegram suite 49 files / 1333 tests; full src/lib suite 98 files / 1899 tests.</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>ROAD-010, T-042</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>Verified high-signal research item selection from public scheme trends, redaction of raw report-shaped evidence, private moderator send payload, admin link only and optional --research smoke path.</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>Proceed to T-043 / ROAD-011 Web/embed Risk Passport compact reuse.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(web): reuse compact risk passports
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd0c4cc38b5d94805"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R260e7c8f3ab14d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R07cef81217ed43dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R8d418b2ab4ea4bb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re9d4b7d78b494338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re1c0fe63f74e4da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3ec7da12e6b54796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb567dee31e484fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3465c32d86c3415c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbc917a1691694367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb6520fdbe05f4178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8934a8854fe14aca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -696,7 +696,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="595">
+  <x:cellXfs count="596">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -2383,6 +2383,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="117" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2693,16 +2696,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-043 / ROAD-011 Web/embed Risk Passport compact reuse; reuse Telegram passport structure on web/embed without oversized partner UI.</x:v>
+        <x:v>Next queue item: T-044 / ROAD-012 Embed origin analytics/logging; add privacy-safe /embed/check origin telemetry before broad partner distribution.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-010 shipped private moderation research alerts with public scheme metadata only.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-011 shipped shared web/embed Risk Passport compact reuse.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2738,7 +2741,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2890,7 +2893,7 @@
         <x:v>Later growth</x:v>
       </x:c>
       <x:c r="C14" s="8" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D14" s="8" t="n">
         <x:v>5</x:v>
@@ -6741,30 +6744,30 @@
         <x:v>No raw report text, screenshots, OCR, codes, cards, passwords, full phone numbers, full URLs, raw posts or user ids are sent to moderator chat.</x:v>
       </x:c>
     </x:row>
-    <x:row r="62">
-      <x:c r="A62" t="str">
+    <x:row r="62" ht="36" customHeight="1">
+      <x:c r="A62" s="595" t="str">
         <x:v>ROAD-011</x:v>
       </x:c>
-      <x:c r="B62" t="str">
+      <x:c r="B62" s="595" t="str">
         <x:v>Roadmap</x:v>
       </x:c>
-      <x:c r="C62" t="str">
+      <x:c r="C62" s="595" t="str">
         <x:v>Web/embed Risk Passport compact reuse</x:v>
       </x:c>
-      <x:c r="D62" t="str">
+      <x:c r="D62" s="595" t="str">
         <x:v>As a web or partner-embed user, I want shallow phone/username checks to show the same honest passport structure as Telegram.</x:v>
       </x:c>
-      <x:c r="E62" t="str">
+      <x:c r="E62" s="595" t="str">
         <x:v>Website and iframe checks reuse compact passport sections for visible facts, local reputation boundaries and next evidence without making embeds too tall.</x:v>
       </x:c>
-      <x:c r="F62" t="str">
-        <x:v>planned: src/components/RiskResultCard.tsx; src/components/EmbedCheckWidget.tsx; src/lib/risk/phone-intelligence.ts; src/lib/telegram/format.ts</x:v>
-      </x:c>
-      <x:c r="G62" t="str">
+      <x:c r="F62" s="595" t="str">
+        <x:v>src/lib/risk/risk-passport.ts; src/components/RiskResultCard.tsx; src/components/EmbedCheckWidget.tsx; src/components/EmbedCheckWidget.passport.test.tsx; src/lib/risk/risk-passport.test.ts</x:v>
+      </x:c>
+      <x:c r="G62" s="595" t="str">
         <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; .kiro/specs/risk-passport-v1</x:v>
       </x:c>
-      <x:c r="H62" t="str">
-        <x:v>Planned</x:v>
+      <x:c r="H62" s="595" t="str">
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I62" t="str">
         <x:v>Needs web/embed UX tests</x:v>
@@ -6777,6 +6780,32 @@
       </x:c>
       <x:c r="L62" t="str">
         <x:v>No hidden Telegram facts, unmoderated report claims or raw private evidence in public/partner surfaces.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="36" customHeight="1">
+      <x:c r="A63" s="595" t="str">
+        <x:v>ROAD-012</x:v>
+      </x:c>
+      <x:c r="B63" s="595" t="str">
+        <x:v>Roadmap</x:v>
+      </x:c>
+      <x:c r="C63" s="595" t="str">
+        <x:v>Embed origin analytics/logging</x:v>
+      </x:c>
+      <x:c r="D63" s="595" t="str">
+        <x:v>As an operator/partner owner, I want privacy-safe visibility into where the embed is used before broad distribution.</x:v>
+      </x:c>
+      <x:c r="E63" s="595" t="str">
+        <x:v>/embed/check records privacy-safe origin usage telemetry without raw user input; partner allowlisting remains server-side.</x:v>
+      </x:c>
+      <x:c r="F63" s="595" t="str">
+        <x:v>planned: src/server.ts; src/lib/security/csp.ts; src/lib/embed-widget.ts; src/components/EmbedCheckWidget.tsx</x:v>
+      </x:c>
+      <x:c r="G63" s="595" t="str">
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/DECISIONS.md</x:v>
+      </x:c>
+      <x:c r="H63" s="595" t="str">
+        <x:v>Planned</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9869,31 +9898,55 @@
       <x:c r="I43"/>
       <x:c r="J43"/>
     </x:row>
-    <x:row r="44">
-      <x:c r="A44" t="str">
+    <x:row r="44" ht="66" customHeight="1">
+      <x:c r="A44" s="595" t="str">
         <x:v>T-043</x:v>
       </x:c>
-      <x:c r="B44" t="str">
+      <x:c r="B44" s="595" t="str">
         <x:v>ROAD-011</x:v>
       </x:c>
-      <x:c r="C44" t="str">
+      <x:c r="C44" s="595" t="str">
         <x:v>As a web or partner-embed user, I want shallow phone/username checks to show the same honest passport structure as Telegram.</x:v>
       </x:c>
-      <x:c r="D44" t="str">
+      <x:c r="D44" s="595" t="str">
         <x:v>Website and iframe checks reuse compact passport sections for visible facts, local reputation boundaries and next evidence without making embeds too tall.</x:v>
       </x:c>
-      <x:c r="E44" t="str">
-        <x:v>Adapt Risk Passport presentation to web and embed result cards.</x:v>
-      </x:c>
-      <x:c r="F44" t="str">
+      <x:c r="E44" s="595" t="str">
+        <x:v>Closed 2026-07-02: shared risk-passport presenter feeds website and embed result cards; embed passport branch stays compact and high-risk remains action-first.</x:v>
+      </x:c>
+      <x:c r="F44" s="595" t="str">
         <x:v>P5</x:v>
       </x:c>
-      <x:c r="G44" t="str">
-        <x:v>Not run</x:v>
-      </x:c>
-      <x:c r="H44"/>
+      <x:c r="G44" s="595" t="str">
+        <x:v>Passed 2026-07-02: scoped eslint, tsc 0 errors, risk-passport unit 3 tests, embed passport SSR 2 tests, full src/lib + embed component suite 100 files / 1904 tests, production build passed. Browser page load confirmed; live result submission locally blocked by missing SUPABASE_SERVICE_ROLE_KEY.</x:v>
+      </x:c>
+      <x:c r="H44" s="595"/>
       <x:c r="I44"/>
       <x:c r="J44"/>
+    </x:row>
+    <x:row r="45" ht="66" customHeight="1">
+      <x:c r="A45" s="595" t="str">
+        <x:v>T-044</x:v>
+      </x:c>
+      <x:c r="B45" s="595" t="str">
+        <x:v>ROAD-012</x:v>
+      </x:c>
+      <x:c r="C45" s="595" t="str">
+        <x:v>As an operator/partner owner, I want privacy-safe visibility into where the embed is used before broad distribution.</x:v>
+      </x:c>
+      <x:c r="D45" s="595" t="str">
+        <x:v>/embed/check records privacy-safe origin usage telemetry without raw user input; partner allowlisting remains server-side.</x:v>
+      </x:c>
+      <x:c r="E45" s="595" t="str">
+        <x:v>Add privacy-safe embed origin telemetry and operational review path.</x:v>
+      </x:c>
+      <x:c r="F45" s="595" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="G45" s="595" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="H45" s="595"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12231,6 +12284,32 @@
         <x:v>Proceed to T-043 / ROAD-011 Web/embed Risk Passport compact reuse.</x:v>
       </x:c>
     </x:row>
+    <x:row r="49" ht="72" customHeight="1">
+      <x:c r="A49" s="595" t="str">
+        <x:v>QA-2026-07-02-005</x:v>
+      </x:c>
+      <x:c r="B49" s="595" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C49" s="595" t="str">
+        <x:v>ROAD-011 web/embed Risk Passport compact reuse</x:v>
+      </x:c>
+      <x:c r="D49" s="595" t="str">
+        <x:v>npx eslint src/lib/risk/risk-passport.ts src/lib/risk/risk-passport.test.ts src/components/RiskResultCard.tsx src/components/EmbedCheckWidget.tsx src/components/EmbedCheckWidget.passport.test.tsx --quiet; npx tsc --noEmit --pretty false; npm run test:run -- src/lib src/components/EmbedCheckWidget.passport.test.tsx; npm run build; Playwright open/snapshot /embed/check</x:v>
+      </x:c>
+      <x:c r="E49" s="595" t="str">
+        <x:v>Passed: scoped eslint 0 errors; tsc 0 errors; full src/lib + embed component suite 100 files / 1904 tests; production build passed. Playwright loaded /embed/check on local dev server; live result submission requires Supabase service-role secret and was not available locally.</x:v>
+      </x:c>
+      <x:c r="F49" s="595" t="str">
+        <x:v>ROAD-011, T-043</x:v>
+      </x:c>
+      <x:c r="G49" s="595" t="str">
+        <x:v>Verified shared risk-passport presenter, phone/Telegram passport detection, no raw phone digits in embed passport SSR, compact iframe branch without generic advice duplication, and high-risk embed cards remaining action-first.</x:v>
+      </x:c>
+      <x:c r="H49" s="595" t="str">
+        <x:v>Proceed to T-044 / ROAD-012 Embed origin analytics/logging.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat(embed): log privacy-safe origin telemetry
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3ec7da12e6b54796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb567dee31e484fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3465c32d86c3415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbc917a1691694367"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb6520fdbe05f4178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8934a8854fe14aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc43346c7920246bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R03d5111d76bc490e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R92aeef99cdc94241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd4561d99600b49a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e78e1e7eb364bb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R77cbef5e40d04230"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2696,16 +2696,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-044 / ROAD-012 Embed origin analytics/logging; add privacy-safe /embed/check origin telemetry before broad partner distribution.</x:v>
+        <x:v>Next queue item: T-045 / QA-001 P1 user-story QA web/Telegram flows; rerun homepage, report, appeal/admin, live Telegram image/QR, Guardian Angel and chat-scope flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-011 shipped shared web/embed Risk Passport compact reuse.</x:v>
+        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-012 shipped privacy-safe embed origin analytics/logging.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2741,7 +2741,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2825,7 +2825,7 @@
         <x:v>Trust/security blocker</x:v>
       </x:c>
       <x:c r="C10" s="8" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D10" s="8" t="n">
         <x:v>1</x:v>
@@ -6782,7 +6782,7 @@
         <x:v>No hidden Telegram facts, unmoderated report claims or raw private evidence in public/partner surfaces.</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="36" customHeight="1">
+    <x:row r="63" ht="42" customHeight="1">
       <x:c r="A63" s="595" t="str">
         <x:v>ROAD-012</x:v>
       </x:c>
@@ -6799,12 +6799,38 @@
         <x:v>/embed/check records privacy-safe origin usage telemetry without raw user input; partner allowlisting remains server-side.</x:v>
       </x:c>
       <x:c r="F63" s="595" t="str">
-        <x:v>planned: src/server.ts; src/lib/security/csp.ts; src/lib/embed-widget.ts; src/components/EmbedCheckWidget.tsx</x:v>
+        <x:v>src/lib/embed-origin-analytics.server.ts; src/lib/check.functions.ts; src/components/EmbedCheckWidget.tsx; supabase/migrations/20260702063847_embed_origin_analytics_v1.sql; scripts/prod-security-smoke.ts</x:v>
       </x:c>
       <x:c r="G63" s="595" t="str">
-        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/DECISIONS.md</x:v>
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/DATABASE.md; ai_docs/DEPLOYMENT.md</x:v>
       </x:c>
       <x:c r="H63" s="595" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="42" customHeight="1">
+      <x:c r="A64" s="595" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="B64" s="595" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="C64" s="595" t="str">
+        <x:v>P1 web/Telegram user-story QA flows</x:v>
+      </x:c>
+      <x:c r="D64" s="595" t="str">
+        <x:v>As the product owner, I want the critical web and Telegram user stories re-run end to end after the roadmap/security work.</x:v>
+      </x:c>
+      <x:c r="E64" s="595" t="str">
+        <x:v>Homepage high-risk, report success, appeal/admin moderation, live Telegram image/QR, Guardian Angel high-risk and private/group Telegram session scoping are verified against the configured environment.</x:v>
+      </x:c>
+      <x:c r="F64" s="595" t="str">
+        <x:v>planned: src/routes/index.tsx; src/routes/report.tsx; src/routes/appeal.tsx; src/lib/telegram/handlers/check.ts; src/lib/telegram/guardian-angel.ts; src/lib/telegram/session.server.ts</x:v>
+      </x:c>
+      <x:c r="G64" s="595" t="str">
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; user-story QA plan</x:v>
+      </x:c>
+      <x:c r="H64" s="595" t="str">
         <x:v>Planned</x:v>
       </x:c>
     </x:row>
@@ -9924,7 +9950,7 @@
       <x:c r="I44"/>
       <x:c r="J44"/>
     </x:row>
-    <x:row r="45" ht="66" customHeight="1">
+    <x:row r="45" ht="69" customHeight="1">
       <x:c r="A45" s="595" t="str">
         <x:v>T-044</x:v>
       </x:c>
@@ -9938,15 +9964,39 @@
         <x:v>/embed/check records privacy-safe origin usage telemetry without raw user input; partner allowlisting remains server-side.</x:v>
       </x:c>
       <x:c r="E45" s="595" t="str">
-        <x:v>Add privacy-safe embed origin telemetry and operational review path.</x:v>
+        <x:v>Closed 2026-07-02: service-role-only embed_origin_events stores partner/referrer origin metadata and aggregate result shape only, with RLS, public grants revoked and retention pruning.</x:v>
       </x:c>
       <x:c r="F45" s="595" t="str">
         <x:v>P5</x:v>
       </x:c>
       <x:c r="G45" s="595" t="str">
+        <x:v>Passed 2026-07-02: focused telemetry/check/migration tests 3 files / 25 tests; scoped eslint and tsc 0 errors; full src/lib + embed component suite 102 files / 1914 tests; production build passed. Supabase local db lint/advisors attempted but blocked because local Postgres 127.0.0.1:54322 was not running.</x:v>
+      </x:c>
+      <x:c r="H45" s="595"/>
+    </x:row>
+    <x:row r="46" ht="69" customHeight="1">
+      <x:c r="A46" s="595" t="str">
+        <x:v>T-045</x:v>
+      </x:c>
+      <x:c r="B46" s="595" t="str">
+        <x:v>QA-001</x:v>
+      </x:c>
+      <x:c r="C46" s="595" t="str">
+        <x:v>As the product owner, I want the critical web and Telegram user stories re-run end to end after the roadmap/security work.</x:v>
+      </x:c>
+      <x:c r="D46" s="595" t="str">
+        <x:v>Homepage high-risk, report success, appeal/admin moderation, live Telegram image/QR, Guardian Angel high-risk and private/group Telegram session scoping are verified against the configured environment.</x:v>
+      </x:c>
+      <x:c r="E46" s="595" t="str">
+        <x:v>Run P1 user-story QA flows and update live/production notes.</x:v>
+      </x:c>
+      <x:c r="F46" s="595" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="G46" s="595" t="str">
         <x:v>Not run</x:v>
       </x:c>
-      <x:c r="H45" s="595"/>
+      <x:c r="H46" s="595"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12310,6 +12360,32 @@
         <x:v>Proceed to T-044 / ROAD-012 Embed origin analytics/logging.</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" ht="78" customHeight="1">
+      <x:c r="A50" s="595" t="str">
+        <x:v>QA-2026-07-02-006</x:v>
+      </x:c>
+      <x:c r="B50" s="595" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C50" s="595" t="str">
+        <x:v>ROAD-012 embed origin analytics/logging</x:v>
+      </x:c>
+      <x:c r="D50" s="595" t="str">
+        <x:v>npx eslint src/lib/embed-origin-analytics.server.ts src/lib/embed-origin-analytics.server.test.ts src/lib/embed-origin-analytics-migration.test.ts src/lib/check.functions.ts src/lib/check.functions.test.ts src/components/EmbedCheckWidget.tsx src/integrations/supabase/types.ts scripts/prod-security-smoke.ts --quiet; npx tsc --noEmit --pretty false; npm run test:run -- src/lib/embed-origin-analytics.server.test.ts src/lib/embed-origin-analytics-migration.test.ts src/lib/check.functions.test.ts; npm run test:run -- src/lib src/components/EmbedCheckWidget.passport.test.tsx; npm run build; supabase db advisors/lint --local</x:v>
+      </x:c>
+      <x:c r="E50" s="595" t="str">
+        <x:v>Passed: focused telemetry/check/migration suite 3 files / 25 tests; scoped eslint 0 errors; tsc 0 errors; full src/lib + embed component suite 102 files / 1914 tests; production build passed. Supabase local db advisors/lint were attempted and blocked by no local DB on 127.0.0.1:54322.</x:v>
+      </x:c>
+      <x:c r="F50" s="595" t="str">
+        <x:v>ROAD-012, T-044</x:v>
+      </x:c>
+      <x:c r="G50" s="595" t="str">
+        <x:v>Verified RLS/service-role-only migration text, no raw input/full URL/path/query/hash fields, 180-day telemetry retention, checkInput embed telemetry for check and meta-intent paths, helper failure isolation and prod security smoke coverage for embed_origin_events.</x:v>
+      </x:c>
+      <x:c r="H50" s="595" t="str">
+        <x:v>Proceed to T-045 / QA-001 P1 web/Telegram user-story QA flows.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(prod): close p1 user-story qa
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc43346c7920246bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R03d5111d76bc490e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R92aeef99cdc94241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd4561d99600b49a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e78e1e7eb364bb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R77cbef5e40d04230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2c76628413ef4686"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2ff129ad1dba4925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Re24fa31e5e9345c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6bfa4817e4464a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raaab071bc81d4903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5a5018a6a43947f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -696,7 +696,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="596">
+  <x:cellXfs count="597">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -2386,6 +2386,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2702,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-045 / QA-001 P1 user-story QA web/Telegram flows; rerun homepage, report, appeal/admin, live Telegram image/QR, Guardian Angel and chat-scope flows.</x:v>
+        <x:v>Next queue item: T-046 / SEC-002 CSP/security headers final reconciliation, then UX/logistics fixes.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 smokes passed. 2026-07-02: ROAD-012 shipped privacy-safe embed origin analytics/logging.</x:v>
+        <x:v>Security backlog closed; production P1 web/Telegram user-story QA passed. 2026-07-02: QA-001 closed; prod-security-smoke accepts PGRST205 as anon-denied for service-role-only embed telemetry.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2741,7 +2744,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2775,7 +2778,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="8" t="inlineStr">
         <x:is>
@@ -6808,30 +6811,42 @@
         <x:v>Implemented</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" ht="42" customHeight="1">
-      <x:c r="A64" s="595" t="str">
+    <x:row r="64" ht="112" customHeight="1">
+      <x:c r="A64" s="596" t="str">
         <x:v>QA-001</x:v>
       </x:c>
-      <x:c r="B64" s="595" t="str">
+      <x:c r="B64" s="596" t="str">
         <x:v>QA</x:v>
       </x:c>
-      <x:c r="C64" s="595" t="str">
+      <x:c r="C64" s="596" t="str">
         <x:v>P1 web/Telegram user-story QA flows</x:v>
       </x:c>
-      <x:c r="D64" s="595" t="str">
+      <x:c r="D64" s="596" t="str">
         <x:v>As the product owner, I want the critical web and Telegram user stories re-run end to end after the roadmap/security work.</x:v>
       </x:c>
-      <x:c r="E64" s="595" t="str">
-        <x:v>Homepage high-risk, report success, appeal/admin moderation, live Telegram image/QR, Guardian Angel high-risk and private/group Telegram session scoping are verified against the configured environment.</x:v>
-      </x:c>
-      <x:c r="F64" s="595" t="str">
-        <x:v>planned: src/routes/index.tsx; src/routes/report.tsx; src/routes/appeal.tsx; src/lib/telegram/handlers/check.ts; src/lib/telegram/guardian-angel.ts; src/lib/telegram/session.server.ts</x:v>
-      </x:c>
-      <x:c r="G64" s="595" t="str">
-        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; user-story QA plan</x:v>
-      </x:c>
-      <x:c r="H64" s="595" t="str">
-        <x:v>Planned</x:v>
+      <x:c r="E64" s="596" t="str">
+        <x:v>Homepage high-risk, report success, appeal/admin moderation, live Telegram image/QR, Guardian Angel high-risk and private/group Telegram session scoping are verified against the configured production environment.</x:v>
+      </x:c>
+      <x:c r="F64" s="596" t="str">
+        <x:v>src/routes/index.tsx; src/routes/report.tsx; src/routes/appeal.tsx; scripts/prod-admin-moderation-smoke.ts; scripts/prod-telegram-user-story-smoke.ts; scripts/prod-telegram-live-qa-smoke.ts; scripts/prod-telegram-scope-smoke.ts; scripts/prod-security-smoke.ts</x:v>
+      </x:c>
+      <x:c r="G64" s="596" t="str">
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/CHANGELOG_AI.md; production smoke notes</x:v>
+      </x:c>
+      <x:c r="H64" s="596" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I64" s="596" t="str">
+        <x:v>Production web/Telegram/admin/security smoke</x:v>
+      </x:c>
+      <x:c r="J64" s="596" t="str">
+        <x:v>Closed 2026-07-02: Playwright production web smoke verified homepage high-risk result, report success and appeal success; admin moderation smoke verified report reject + appeal keep-reputation audit and cleanup. Telegram production user-story, live QR/Guardian, private/group scope smokes passed. prod-security-smoke passed after accepting PGRST205 as anon-denied for service-role-only embed_origin_events.</x:v>
+      </x:c>
+      <x:c r="K64" s="596" t="str">
+        <x:v>Proceed to T-046 / SEC-002 CSP/security headers final reconciliation and UX/logistics cleanup.</x:v>
+      </x:c>
+      <x:c r="L64" s="596" t="str">
+        <x:v>2026-07-02</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9974,29 +9989,53 @@
       </x:c>
       <x:c r="H45" s="595"/>
     </x:row>
-    <x:row r="46" ht="69" customHeight="1">
-      <x:c r="A46" s="595" t="str">
+    <x:row r="46" ht="124" customHeight="1">
+      <x:c r="A46" s="596" t="str">
         <x:v>T-045</x:v>
       </x:c>
-      <x:c r="B46" s="595" t="str">
+      <x:c r="B46" s="596" t="str">
         <x:v>QA-001</x:v>
       </x:c>
-      <x:c r="C46" s="595" t="str">
+      <x:c r="C46" s="596" t="str">
         <x:v>As the product owner, I want the critical web and Telegram user stories re-run end to end after the roadmap/security work.</x:v>
       </x:c>
-      <x:c r="D46" s="595" t="str">
+      <x:c r="D46" s="596" t="str">
         <x:v>Homepage high-risk, report success, appeal/admin moderation, live Telegram image/QR, Guardian Angel high-risk and private/group Telegram session scoping are verified against the configured environment.</x:v>
       </x:c>
-      <x:c r="E46" s="595" t="str">
-        <x:v>Run P1 user-story QA flows and update live/production notes.</x:v>
-      </x:c>
-      <x:c r="F46" s="595" t="str">
+      <x:c r="E46" s="596" t="str">
+        <x:v>Closed 2026-07-02: production web, admin moderation, Telegram user-story, live Telegram QR/Guardian and private/group scope flows all passed; synthetic production rows were cleaned.</x:v>
+      </x:c>
+      <x:c r="F46" s="596" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G46" s="595" t="str">
+      <x:c r="G46" s="596" t="str">
+        <x:v>Passed 2026-07-02: Playwright production web smoke marker QA-P1-WEB-20260702071934; prod:admin-moderation-smoke cleanup=done; prod Telegram user-story/live-qa/scope smokes; prod:security-smoke.</x:v>
+      </x:c>
+      <x:c r="H46" s="596"/>
+    </x:row>
+    <x:row r="47" ht="124" customHeight="1">
+      <x:c r="A47" s="596" t="str">
+        <x:v>T-046</x:v>
+      </x:c>
+      <x:c r="B47" s="596" t="str">
+        <x:v>SEC-002</x:v>
+      </x:c>
+      <x:c r="C47" s="596" t="str">
+        <x:v>As the site owner, I want CSP/security-header tracker state reconciled with the shipped nonce and embed allowlist work.</x:v>
+      </x:c>
+      <x:c r="D47" s="596" t="str">
+        <x:v>SEC-002 either becomes Implemented with current production smoke evidence or gets a narrow remaining task for any real header gap.</x:v>
+      </x:c>
+      <x:c r="E47" s="596" t="str">
+        <x:v>Review current server CSP/header code, docs and production headers; update tracker/docs so the Partial row reflects reality.</x:v>
+      </x:c>
+      <x:c r="F47" s="596" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="G47" s="596" t="str">
         <x:v>Not run</x:v>
       </x:c>
-      <x:c r="H46" s="595"/>
+      <x:c r="H47" s="596"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12386,6 +12425,32 @@
         <x:v>Proceed to T-045 / QA-001 P1 web/Telegram user-story QA flows.</x:v>
       </x:c>
     </x:row>
+    <x:row r="51" ht="132" customHeight="1">
+      <x:c r="A51" s="596" t="str">
+        <x:v>QA-2026-07-02-007</x:v>
+      </x:c>
+      <x:c r="B51" s="596" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C51" s="596" t="str">
+        <x:v>QA-001 P1 web/Telegram user-story QA flows</x:v>
+      </x:c>
+      <x:c r="D51" s="596" t="str">
+        <x:v>Playwright production web smoke for homepage high-risk/report/appeal; railway run npm run prod:admin-moderation-smoke; railway run npm run prod:telegram-user-story-smoke; railway run npm run prod:telegram-live-qa-smoke; railway run npm run prod:telegram-scope-smoke; railway run npm run prod:security-smoke</x:v>
+      </x:c>
+      <x:c r="E51" s="596" t="str">
+        <x:v>Passed: homepage high-risk web result, report success, appeal success, admin report/appeal moderation with audit and cleanup, Telegram /start/language/phone passport/benign follow-ups, live QR photo + Guardian high-risk, private/group scoping and production security smoke.</x:v>
+      </x:c>
+      <x:c r="F51" s="596" t="str">
+        <x:v>QA-001, T-045</x:v>
+      </x:c>
+      <x:c r="G51" s="596" t="str">
+        <x:v>Verified synthetic production rows were cleaned. Confirmed user-facing Telegram smokes use a private non-moderation QA chat, not the moderator chat. prod-security-smoke now treats PGRST205 as anon-denied for service-role-only embed_origin_events while service-role count still proves the table exists.</x:v>
+      </x:c>
+      <x:c r="H51" s="596" t="str">
+        <x:v>Proceed to T-046 / SEC-002 CSP/security headers final reconciliation, then UX/logistics fixes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(prod): reconcile security headers
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2c76628413ef4686"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2ff129ad1dba4925"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Re24fa31e5e9345c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6bfa4817e4464a3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raaab071bc81d4903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5a5018a6a43947f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R21577fba22fa49b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9033d2a2a44841f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R904bbcbb051f4482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R197928887a6240ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rdebeacf8085b4b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R529827c5b9994cdc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,17 +2705,17 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-046 / SEC-002 CSP/security headers final reconciliation, then UX/logistics fixes.</x:v>
+        <x:v>Next queue item: UX/logistics fixes after SEC-002 header reconciliation.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Security backlog closed; production P1 web/Telegram user-story QA passed. 2026-07-02: QA-001 closed; prod-security-smoke accepts PGRST205 as anon-denied for service-role-only embed telemetry.</x:v>
+        <x:v>Owner note: security backlog closed; production P1 web/Telegram QA and CSP/security-header reconciliation passed on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="n"/>
       <x:c r="B3" s="8" t="n"/>
       <x:c r="C3" s="8" t="n"/>
-      <x:c r="D3" s="8" t="n"/>
+      <x:c r="D3" s="8"/>
       <x:c r="E3" s="8" t="n"/>
     </x:row>
     <x:row r="4">
@@ -2744,7 +2744,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2761,7 +2761,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="8" t="inlineStr">
         <x:is>
@@ -6139,40 +6139,26 @@
           <x:t xml:space="preserve">Main site avoids unnecessary unsafe-inline; embed CSP is documented and intentionally allows partner framing.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F50" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/server.ts; src/routes/embed.tsx</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G50" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roadmap Security Sprint; AUDIT feedback</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H50" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I50" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Build/manual QA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J50" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Remove/soften unsafe-inline where possible and document embed frame-ancestor policy.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K50" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L50" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do not break widget embedding while tightening main site CSP.</x:t>
-        </x:is>
+      <x:c r="F50" s="8" t="str">
+        <x:v>src/server.ts; src/lib/security/csp.ts; src/lib/security/csp.test.ts; src/server.security-headers.test.ts; scripts/prod-security-smoke.ts; ai_docs/DEPLOYMENT.md</x:v>
+      </x:c>
+      <x:c r="G50" s="8" t="str">
+        <x:v>Roadmap Security Sprint; AUDIT feedback; production header smoke 2026-07-02</x:v>
+      </x:c>
+      <x:c r="H50" s="14" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I50" s="8" t="str">
+        <x:v>Automated + production smoke</x:v>
+      </x:c>
+      <x:c r="J50" s="8" t="str">
+        <x:v>Closed 2026-07-02: server-level regression verifies baseline security headers, main-site frame-ancestors none, per-request script nonce, and embed allowlisted frame-ancestors without X-Frame-Options. prod:security-smoke now optionally verifies public /healthz and /embed/check headers by URL.</x:v>
+      </x:c>
+      <x:c r="K50" s="13" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L50" s="8" t="str">
+        <x:v>No remaining header gap found. Keep EMBED_ALLOWED_FRAME_ANCESTORS explicit for partners; partner query remains display-only and does not grant framing.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -10027,13 +10013,13 @@
         <x:v>SEC-002 either becomes Implemented with current production smoke evidence or gets a narrow remaining task for any real header gap.</x:v>
       </x:c>
       <x:c r="E47" s="596" t="str">
-        <x:v>Review current server CSP/header code, docs and production headers; update tracker/docs so the Partial row reflects reality.</x:v>
+        <x:v>Closed 2026-07-02: SEC-002 reconciled against code, docs and production headers; no remaining header gap found. Added server regression and optional public URL header checks to prod:security-smoke.</x:v>
       </x:c>
       <x:c r="F47" s="596" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G47" s="596" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Passed 2026-07-02: server header tests + CSP/env tests, scoped eslint, and production security smoke with public header checks plus Supabase/RLS.</x:v>
       </x:c>
       <x:c r="H47" s="596"/>
     </x:row>
@@ -12451,6 +12437,32 @@
         <x:v>Proceed to T-046 / SEC-002 CSP/security headers final reconciliation, then UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="52" ht="64" customHeight="1">
+      <x:c r="A52" t="str">
+        <x:v>QA-2026-07-02-008</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>SEC-002 headers reconciliation</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>Targeted tests, eslint, prod security smoke.</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>Passed: tests + prod smoke.</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>SEC-002, T-046</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>Verified main/embed headers; no broad https:. SEC-002 closed.</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>Proceed to UX/logistics fixes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
refactor(telegram): centralize emergency scenario profiles
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R21577fba22fa49b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9033d2a2a44841f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R904bbcbb051f4482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R197928887a6240ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rdebeacf8085b4b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R529827c5b9994cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rf03f152c412b46ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R889827088a844896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc217c6322dac49ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra0b4de23b4604b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc8f21657415d4c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R184093a3b9ed4b11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2699,16 +2699,16 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: UX/logistics fixes after SEC-002 header reconciliation.</x:v>
+        <x:v>Next queue item: UX/logistics fixes - choose next narrow user-facing polish slice.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog closed; production P1 web/Telegram QA and CSP/security-header reconciliation passed on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP reconciliation and emergency profile-map refactor passed on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2744,7 +2744,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -6835,6 +6835,44 @@
         <x:v>2026-07-02</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>UX-001</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>UX</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>Emergency profile-map refactor</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>As the team, we want SOS scenarios to be configured from one profile map before adding more emergency cases.</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>Panic scenario profile, menu page, contact-button role and family-first keyboard behavior are centralized without changing current SOS copy.</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>src/lib/telegram/emergency.ts; src/lib/telegram/emergency-wellformedness.property.test.ts; src/lib/telegram/i18n-completeness.test.ts</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/CHANGELOG_AI.md</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>Telegram regression suite + typecheck + scoped lint</x:v>
+      </x:c>
+      <x:c r="J65" t="str">
+        <x:v>Closed 2026-07-02: added PANIC_SCENARIO_PROFILES and PANIC_SCENARIO_IDS; panic menus, callback parsing, contact-button labels and family-first ordering now derive from the shared profile map. SOS text output is intentionally unchanged.</x:v>
+      </x:c>
+      <x:c r="K65" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L65" t="str">
+        <x:v>Next SOS additions should update the profile map once and rely on existing i18n/wellformedness tests.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10023,6 +10061,29 @@
       </x:c>
       <x:c r="H47" s="596"/>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>T-047</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>UX-001</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>SOS scenario profile map before adding more emergency cases.</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>Centralized profile/menu/button behavior; SOS copy unchanged.</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>Closed 2026-07-02: shared profile/id map drives menu, parsing and keyboards.</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>Passed: tests, tsc, eslint.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12463,6 +12524,32 @@
         <x:v>Proceed to UX/logistics fixes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>QA-2026-07-02-009</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>UX-001 emergency profile-map refactor</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>Targeted emergency/i18n/voice-out tests; full Telegram suite; tsc; scoped eslint.</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>Passed: 5 targeted files / 767 tests; full Telegram 49 files / 1333 tests; tsc and eslint clean.</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>UX-001, T-047</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>Verified panic menus, callback ids, button roles, i18n and SOS text coverage from shared profile data.</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>Proceed to next UX/logistics polish slice.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: close voice-out prerecorded QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rf03f152c412b46ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R889827088a844896"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc217c6322dac49ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra0b4de23b4604b8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc8f21657415d4c95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R184093a3b9ed4b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7f597599cdcf452e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R432877844133425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcfcaf2a885c644a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R4c8c7e112b054b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ref53ffaccf9a4b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R70a2dc78717c4d16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: UX/logistics fixes - choose next narrow user-facing polish slice.</x:v>
+        <x:v>Next queue item: Voice-in/STT real-audio regression corpus and confidence tuning.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP reconciliation and emergency profile-map refactor passed on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map and Voice-out prerecorded SOS assets verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4046,15 +4046,11 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I16" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit tests + static asset audit + deployed Telegram OGG playback smoke + provider-limit fallback regression</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J16" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-01: Deployed Railway build 962b98c9-b600-4c51-8e6d-98e14ebb15fd with 45 SOS OGG/Opus assets and smoke harness. Full production Voice-out smoke passed: direct Telegram sendAudio accepted panic-6 RU/UZ/EN OGG, and production webhook accepted voiceout:panic:6 callback against https://scam-guard-main-production.up.railway.app. General prod:smoke also passed. Provider-limit UX fixed: rate-limit fallback now removes Guardian/follow-up provider-only voice buttons while preserving static SOS voice and normal action buttons.</x:t>
-        </x:is>
+      <x:c r="I16" s="8" t="str">
+        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke + 2026-07-02 asset revalidation</x:v>
+      </x:c>
+      <x:c r="J16" s="8" t="str">
+        <x:v>Closed 2026-07-02: 45 committed SOS OGG/Opus assets for panic-1..15 in RU/UZ/EN revalidated locally; runtime still prefers OGG before WAV, TTS budget and provider calls. Human listen-through remains a release QA checklist item, not an architecture blocker.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="inlineStr">
         <x:is>
@@ -12550,6 +12546,32 @@
         <x:v>Proceed to next UX/logistics polish slice.</x:v>
       </x:c>
     </x:row>
+    <x:row r="54" ht="110" customHeight="1">
+      <x:c r="A54" s="596" t="str">
+        <x:v>QA-2026-07-02-010</x:v>
+      </x:c>
+      <x:c r="B54" s="596" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C54" s="596" t="str">
+        <x:v>TG-015 Voice-out prerecorded SOS asset revalidation</x:v>
+      </x:c>
+      <x:c r="D54" s="596" t="str">
+        <x:v>npm run tts:validate-assets; npm run test:run -- src/lib/telegram/voice-out.server.test.ts src/lib/telegram/emergency-followup.test.ts; git ls-files public/audio/voice-out</x:v>
+      </x:c>
+      <x:c r="E54" s="596" t="str">
+        <x:v>Passed: 45 OGG assets validated; 2 files / 42 tests; 91 tracked voice-out files including README/WAV fallbacks</x:v>
+      </x:c>
+      <x:c r="F54" s="596" t="str">
+        <x:v>TG-015, Voice-out pre-record architecture pass</x:v>
+      </x:c>
+      <x:c r="G54" s="596" t="str">
+        <x:v>Validator confirmed 45 RU/UZ/EN OGG assets, total 1,683,698 bytes, smallest panic-3-uz.ogg 27,662 bytes / 7.73s, largest panic-12-ru.ogg 48,611 bytes / 14.05s. Runtime tests confirm prerecorded SOS audio is selected before TTS budget/provider calls and OGG is preferred over WAV.</x:v>
+      </x:c>
+      <x:c r="H54" s="596" t="str">
+        <x:v>Proceed to Voice-in/STT real-audio regression corpus and confidence tuning; keep human listen-through of prerecorded audio in release QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): harden voice stt emergency corpus
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7f597599cdcf452e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R432877844133425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rcfcaf2a885c644a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R4c8c7e112b054b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ref53ffaccf9a4b0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R70a2dc78717c4d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6bcc259739534eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9717b4e9be664b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc4a431a902244260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6284068876674e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R172a72ff80784f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ref9cce0697124a17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: Voice-in/STT real-audio regression corpus and confidence tuning.</x:v>
+        <x:v>Next queue item: continue Voice-in/STT with real provider audio fixtures, then Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map and Voice-out prerecorded SOS assets verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets and first Voice-in STT corpus slice verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3984,25 +3984,19 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I15" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit tests + integration tests + live QA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J15" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closed 2026-06-30: friendly delivery/card voice stays below high-risk; sanitized hook phrase is shown for concrete risk triggers. Keep real-audio STT corpus/timing watch after provider/model changes.</x:t>
-        </x:is>
+      <x:c r="I15" s="8" t="str">
+        <x:v>Unit tests + integration tests + live QA + production-like STT corpus regression</x:v>
+      </x:c>
+      <x:c r="J15" s="8" t="str">
+        <x:v>Closed 2026-07-02 slice: production-like STT transcripts now cover card-security-code, remote-access, Telegram-login-QR and negated already-happened phrases across RU/UZ without raw audio fixtures. Keep collecting real provider audio/transcript examples for the next corpus expansion.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P1</x:t>
         </x:is>
       </x:c>
-      <x:c r="L15" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-30 verified: voice hook phrase is derived from sanitized transcript preview, so raw URLs, @handles and long digit runs remain hidden; long/unsupported/over-budget voice guard remains unchanged.</x:t>
-        </x:is>
+      <x:c r="L15" s="8" t="str">
+        <x:v>2026-07-02: first STT corpus/confidence slice shipped. Negated phrases like 'I did not send the code' no longer route to already-happened SOS; completed card/CVV, remote-access and Telegram QR phrases route to the matching SOS. Remaining: real provider audio fixture expansion.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -12572,6 +12566,32 @@
         <x:v>Proceed to Voice-in/STT real-audio regression corpus and confidence tuning; keep human listen-through of prerecorded audio in release QA.</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="120" customHeight="1">
+      <x:c r="A55" s="596" t="str">
+        <x:v>QA-2026-07-02-011</x:v>
+      </x:c>
+      <x:c r="B55" s="596" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C55" s="596" t="str">
+        <x:v>TG-014 Voice-in/STT production-like corpus tuning</x:v>
+      </x:c>
+      <x:c r="D55" s="596" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk/voice-transcription.test.ts src/lib/risk/rules.reason-codes.test.ts; npx eslint src/lib/telegram/handlers/check.ts src/lib/telegram/handlers/check.voice.test.ts --quiet; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E55" s="596" t="str">
+        <x:v>Passed: voice handler 1 file / 18 tests; full Telegram 49 files / 1335 tests; risk voice/rules 2 files / 153 tests; scoped eslint and tsc clean</x:v>
+      </x:c>
+      <x:c r="F55" s="596" t="str">
+        <x:v>TG-014, Voice-in/STT corpus and confidence tuning</x:v>
+      </x:c>
+      <x:c r="G55" s="596" t="str">
+        <x:v>Verified production-like STT transcript corpus for RU/UZ card-security-code/CVV, remote access, Telegram-login QR and negated already-happened phrases. Panic routing now avoids false SOS escalation for 'not sent/not scanned' wording while still routing completed high-impact actions to scenarios 2, 4 and 5.</x:v>
+      </x:c>
+      <x:c r="H55" s="596" t="str">
+        <x:v>Continue with real provider audio/transcript fixtures when available; then move to Phone Reputation v2 / Inline QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): cover english voice stt emergencies
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6bcc259739534eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9717b4e9be664b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc4a431a902244260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6284068876674e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R172a72ff80784f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ref9cce0697124a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R0099104574ee443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R607d39776dd34410"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5031e36142314c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2debcc09d580477d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R96d6710157d04263"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc14eef29aede48a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: continue Voice-in/STT with real provider audio fixtures, then Phone Reputation v2 / Inline QA.</x:v>
+        <x:v>Next queue item: real provider Voice-in/STT audio/transcript fixture expansion, then Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets and first Voice-in STT corpus slice verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ STT corpus and EN provider-like STT slice verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3969,20 +3969,14 @@
           <x:t xml:space="preserve">Short voice is transcribed, shown back to the user, and then checked; uncertain transcription should avoid hard verdicts.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F15" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/lib/telegram/voice.server.ts; src/lib/telegram/handlers/check.ts; src/lib/risk/check-core.ts</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G15" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">.kiro/specs/telegram-voice-stt-v1; .kiro/specs/telegram-voice-in-v2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H15" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented</x:t>
-        </x:is>
+      <x:c r="F15" s="8" t="str">
+        <x:v>Unit tests + integration tests + live QA + RU/UZ/EN provider-like STT corpus regression</x:v>
+      </x:c>
+      <x:c r="G15" s="8" t="str">
+        <x:v>Closed 2026-07-02 slice: EN provider-like transcripts now cover already-sent SMS code, card back digits, AnyDesk/screen access, money transfer, Telegram login QR and live-call routing; EN negated phrases stay on the normal check pipeline. Remaining: collect real provider audio/transcript fixtures from live QA.</x:v>
+      </x:c>
+      <x:c r="H15" s="14" t="str">
+        <x:v>2026-07-02: second STT corpus slice shipped. Direct voice-to-SOS routing now covers RU/UZ plus EN provider-like already-happened phrases; negated EN phrases like 'I did not send the code' do not open SOS. Remaining: real audio fixture expansion.</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
         <x:v>Unit tests + integration tests + live QA + production-like STT corpus regression</x:v>
@@ -12592,6 +12586,32 @@
         <x:v>Continue with real provider audio/transcript fixtures when available; then move to Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="96" customHeight="1">
+      <x:c r="A56" s="595" t="str">
+        <x:v>QA-2026-07-02-012</x:v>
+      </x:c>
+      <x:c r="B56" s="595" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C56" s="595" t="str">
+        <x:v>TG-014 Voice-in/STT EN provider-like corpus</x:v>
+      </x:c>
+      <x:c r="D56" s="595" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk/voice-transcription.test.ts src/lib/risk/rules.reason-codes.test.ts; npx eslint src/lib/telegram/handlers/check.ts src/lib/telegram/handlers/check.voice.test.ts --quiet; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E56" s="595" t="str">
+        <x:v>Passed: voice handler 1 file / 18 tests; full Telegram 49 files / 1335 tests; risk voice/rules 2 files / 153 tests; scoped eslint and tsc clean</x:v>
+      </x:c>
+      <x:c r="F56" s="595" t="str">
+        <x:v>TG-014, EN provider-like STT corpus and negation guard</x:v>
+      </x:c>
+      <x:c r="G56" s="595" t="str">
+        <x:v>EN provider-like transcripts for SMS code, card digits, AnyDesk/screen access, money transfer, Telegram login QR and live call route to matching SOS; EN negated already-happened phrases do not route to SOS.</x:v>
+      </x:c>
+      <x:c r="H56" s="595" t="str">
+        <x:v>Next: collect real provider audio/transcript examples from live QA before Phone Reputation v2 / Inline QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(telegram): add voice stt fixture workflow
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R0099104574ee443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R607d39776dd34410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5031e36142314c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2debcc09d580477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R96d6710157d04263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc14eef29aede48a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb352ae0593724149"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re6078ac2f3fb442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7184ce3263f448a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R622cfcd936c34741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rabbfb77ea1374294"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc726dd70af214368"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: real provider Voice-in/STT audio/transcript fixture expansion, then Phone Reputation v2 / Inline QA.</x:v>
+        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples with the new workflow, then Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ STT corpus and EN provider-like STT slice verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus and Voice-in fixture workflow verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3970,13 +3970,13 @@
         </x:is>
       </x:c>
       <x:c r="F15" s="8" t="str">
-        <x:v>Unit tests + integration tests + live QA + RU/UZ/EN provider-like STT corpus regression</x:v>
+        <x:v>Unit tests + integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + fixture workflow</x:v>
       </x:c>
       <x:c r="G15" s="8" t="str">
-        <x:v>Closed 2026-07-02 slice: EN provider-like transcripts now cover already-sent SMS code, card back digits, AnyDesk/screen access, money transfer, Telegram login QR and live-call routing; EN negated phrases stay on the normal check pipeline. Remaining: collect real provider audio/transcript fixtures from live QA.</x:v>
+        <x:v>Closed 2026-07-02 slice: replay corpus extracted to voice-stt-provider-fixtures.ts and local real-provider capture workflow added via npm run stt:transcribe-fixtures. Remaining: collect real provider audio/transcript fixtures from live QA and tune confidence heuristics from production examples.</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>2026-07-02: second STT corpus slice shipped. Direct voice-to-SOS routing now covers RU/UZ plus EN provider-like already-happened phrases; negated EN phrases like 'I did not send the code' do not open SOS. Remaining: real audio fixture expansion.</x:v>
+        <x:v>2026-07-02: Voice-in/STT fixture workflow shipped. Raw audio stays under ignored private/voice-stt-fixtures; collector emits sanitized transcripts only. Local live provider capture was not run because OPENAI_API_KEY is absent.</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
         <x:v>Unit tests + integration tests + live QA + production-like STT corpus regression</x:v>
@@ -12612,6 +12612,32 @@
         <x:v>Next: collect real provider audio/transcript examples from live QA before Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
     </x:row>
+    <x:row r="57" ht="110" customHeight="1">
+      <x:c r="A57" s="595" t="str">
+        <x:v>QA-2026-07-02-013</x:v>
+      </x:c>
+      <x:c r="B57" s="595" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C57" s="595" t="str">
+        <x:v>TG-014 Voice-in/STT fixture workflow</x:v>
+      </x:c>
+      <x:c r="D57" s="595" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk/voice-transcription.test.ts src/lib/risk/rules.reason-codes.test.ts; npx eslint src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/voice-stt-provider-fixtures.ts scripts/transcribe-voice-stt-fixtures.ts --quiet; npx tsc --noEmit --pretty false; npm run stt:transcribe-fixtures -- --help</x:v>
+      </x:c>
+      <x:c r="E57" s="595" t="str">
+        <x:v>Passed: voice handler 1 file / 18 tests; full Telegram 49 files / 1335 tests; risk voice/rules 2 files / 153 tests; scoped eslint and tsc clean; fixture script help works</x:v>
+      </x:c>
+      <x:c r="F57" s="595" t="str">
+        <x:v>TG-014, Voice-in/STT fixture replay and real-provider capture workflow</x:v>
+      </x:c>
+      <x:c r="G57" s="595" t="str">
+        <x:v>Verified replay corpus extraction, local ignored audio fixture capture path, sanitized transcript collector, docs and gitignore safety. Live provider capture was not run because OPENAI_API_KEY is absent in the local shell.</x:v>
+      </x:c>
+      <x:c r="H57" s="595" t="str">
+        <x:v>Next: collect real provider audio/transcript examples with the new manifest workflow, then proceed to Phone Reputation v2 / Inline QA.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): reuse risk passport in inline checks
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb352ae0593724149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re6078ac2f3fb442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R7184ce3263f448a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R622cfcd936c34741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rabbfb77ea1374294"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc726dd70af214368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R228a265ddbf94379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R519948da698044ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4ef031860b314326"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re39d540800c2443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1130fb160d934d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2bb052d3b4a341fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples with the new workflow, then Phone Reputation v2 / Inline QA.</x:v>
+        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then remaining Phone Reputation v2 / Inline QA polish.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus and Voice-in fixture workflow verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow and inline Risk Passport QA verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12638,6 +12638,32 @@
         <x:v>Next: collect real provider audio/transcript examples with the new manifest workflow, then proceed to Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
     </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="595" t="str">
+        <x:v>QA-2026-07-02-014</x:v>
+      </x:c>
+      <x:c r="B58" s="595" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C58" s="595" t="str">
+        <x:v>ROAD-013 Inline Risk Passport QA slice</x:v>
+      </x:c>
+      <x:c r="D58" s="595" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/inline.test.ts; npm run test:run -- src/lib/risk/risk-passport.test.ts src/lib/risk/phone-reputation.test.ts; npm run test:run -- src/lib/telegram; npx eslint src/lib/telegram/handlers/inline.ts src/lib/telegram/handlers/inline.test.ts; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E58" s="595" t="str">
+        <x:v>Passed: inline handler 1 file / 4 tests; risk passport + phone reputation 2 files / 6 tests; full Telegram 49 files / 1336 tests; scoped TS eslint 0 errors; tsc 0 errors.</x:v>
+      </x:c>
+      <x:c r="F58" s="595" t="str">
+        <x:v>ROAD-013, Telegram inline QA, Risk Passport, Phone Reputation v2</x:v>
+      </x:c>
+      <x:c r="G58" s="595" t="str">
+        <x:v>Low-signal phone/Telegram inline results now render shared Risk Passport sections with limitations, directory/reputation context and next-step prompts; high-risk inline results remain action-first.</x:v>
+      </x:c>
+      <x:c r="H58" s="595" t="str">
+        <x:v>Next: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then continue remaining Phone Reputation v2 / Inline QA polish.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(risk): clarify phone reputation source copy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R228a265ddbf94379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R519948da698044ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4ef031860b314326"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re39d540800c2443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1130fb160d934d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2bb052d3b4a341fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc201f51062bf429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf151559c82164f57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb79c18f414b74d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1532be76d3dd4f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e1c42b3ad1547ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc684d5098f434966"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then remaining Phone Reputation v2 / Inline QA polish.</x:v>
+        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then remaining inline/live QA examples for Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow and inline Risk Passport QA verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, inline Risk Passport QA and Phone Reputation v2 wording/source confidence verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12664,6 +12664,32 @@
         <x:v>Next: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then continue remaining Phone Reputation v2 / Inline QA polish.</x:v>
       </x:c>
     </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="595" t="str">
+        <x:v>QA-2026-07-02-015</x:v>
+      </x:c>
+      <x:c r="B59" s="595" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C59" s="595" t="str">
+        <x:v>ROAD-014 Phone Reputation v2 wording/source confidence</x:v>
+      </x:c>
+      <x:c r="D59" s="595" t="str">
+        <x:v>npm run test:run -- src/lib/risk/phone-reputation.test.ts src/lib/risk/risk-passport.test.ts src/lib/telegram/handlers/inline.test.ts src/lib/telegram/format.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk; npx eslint scoped touched TS files; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E59" s="595" t="str">
+        <x:v>Passed: focused 4 files / 46 tests; full Telegram 49 files / 1336 tests; full risk 30 files / 458 tests; scoped TS eslint 0 errors; tsc 0 errors.</x:v>
+      </x:c>
+      <x:c r="F59" s="595" t="str">
+        <x:v>ROAD-014, Phone Reputation v2, Risk Passport, Telegram inline QA</x:v>
+      </x:c>
+      <x:c r="G59" s="595" t="str">
+        <x:v>Phone reputation copy now names moderator-confirmed Ishonch Guard reports, conservative confidence and public-scope limits; it excludes unverified complaints, number owner data, carrier data and hidden external labels.</x:v>
+      </x:c>
+      <x:c r="H59" s="595" t="str">
+        <x:v>Next: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then remaining inline/live QA examples.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(telegram): cover inline passport regressions
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc201f51062bf429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf151559c82164f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb79c18f414b74d2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1532be76d3dd4f28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e1c42b3ad1547ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc684d5098f434966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc71148aae9b644c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rd396f98b8ae44230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R0b363da491204d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf765459afcdb46a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R59662681ba674793"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8aa08cfd34114913"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then remaining inline/live QA examples for Phone Reputation v2 / Inline QA.</x:v>
+        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then live Telegram inline QA examples for Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, inline Risk Passport QA and Phone Reputation v2 wording/source confidence verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, inline Risk Passport QA, Phone Reputation v2 wording/source confidence and inline QA regression matrix verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12690,6 +12690,32 @@
         <x:v>Next: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then remaining inline/live QA examples.</x:v>
       </x:c>
     </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>QA-2026-07-02-016</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>ROAD-015 Inline QA regression matrix</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/inline.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk; npx eslint src/lib/telegram/handlers/inline.test.ts; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>Passed: inline handler 1 file / 6 tests; full Telegram 49 files / 1338 tests; full risk 30 files / 458 tests; scoped TS eslint 0 errors; tsc 0 errors.</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>ROAD-015, Telegram inline QA, Risk Passport, Phone Reputation v2</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Expanded inline regression matrix for low-signal Telegram username passport and phone reputation source/scope rendering; high-risk inline cards remain action-first and inline checks stay non-persistent.</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>Next: collect live Telegram inline QA examples and real provider Voice-in/STT audio/transcript examples when key/audio access is available.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(stt): harden voice fixture collector
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc71148aae9b644c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rd396f98b8ae44230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R0b363da491204d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf765459afcdb46a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R59662681ba674793"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8aa08cfd34114913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R63e987f18c134bb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R461c53ed162e4d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9c500901631c49ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0078dd708d054bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R37b94788c6334a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ree8b49a0a6f641fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript examples when key/audio access is available, then live Telegram inline QA examples for Phone Reputation v2 / Inline QA.</x:v>
+        <x:v>Next queue item remains collecting real provider Voice-in/STT audio/transcript examples when OPENAI_API_KEY and local audio are available, then live Telegram inline QA examples for Phone Reputation v2 / Inline QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, inline Risk Passport QA, Phone Reputation v2 wording/source confidence and inline QA regression matrix verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, inline Risk Passport QA, Phone Reputation v2 wording/source confidence and inline QA regression matrix verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12716,6 +12716,32 @@
         <x:v>Next: collect live Telegram inline QA examples and real provider Voice-in/STT audio/transcript examples when key/audio access is available.</x:v>
       </x:c>
     </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>QA-2026-07-02-017</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>TG-014 Voice-in/STT collector validation hardening</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/voice-stt-fixture-collector.test.ts; npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk; npx eslint scripts/transcribe-voice-stt-fixtures.ts src/lib/telegram/voice-stt-fixture-collector.test.ts; npm run stt:transcribe-fixtures -- --help; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>Passed: fixture collector 1 file / 4 tests; voice handler 1 file / 18 tests; full Telegram 50 files / 1342 tests; full risk 30 files / 458 tests; scoped TS eslint 0 errors; STT collector --help prints usage; tsc 0 errors.</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>TG-014, Voice-in/STT, provider capture workflow, privacy guard</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>No local OPENAI_API_KEY or private audio fixtures were available for real provider capture. Hardened the local collector instead: manifest parsing, supported audio extensions, expected transcript fragments and relative audio paths are covered before provider calls; audioPath is scoped to the manifest directory to avoid accidental unrelated file reads.</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>Next: collect real provider audio/transcript fixtures from live QA when OPENAI_API_KEY and local audio are available, then continue live Telegram inline QA examples.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(telegram): add production inline smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R63e987f18c134bb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R461c53ed162e4d36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9c500901631c49ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R0078dd708d054bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R37b94788c6334a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ree8b49a0a6f641fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3a691299250142fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbe69fa95c3f54931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1816ac48c51749f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R20ea267576be47f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re884c97023844023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5c74f141d0dc4833"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item remains collecting real provider Voice-in/STT audio/transcript examples when OPENAI_API_KEY and local audio are available, then live Telegram inline QA examples for Phone Reputation v2 / Inline QA.</x:v>
+        <x:v>Next queue item: collect real Telegram-client inline QA examples/screenshots for Phone Reputation v2 / Inline QA, and real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, inline Risk Passport QA, Phone Reputation v2 wording/source confidence and inline QA regression matrix verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, inline Risk Passport QA, Phone Reputation v2 wording/source confidence, inline regression matrix and production inline smoke verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12742,6 +12742,32 @@
         <x:v>Next: collect real provider audio/transcript fixtures from live QA when OPENAI_API_KEY and local audio are available, then continue live Telegram inline QA examples.</x:v>
       </x:c>
     </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>QA-2026-07-02-018</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>ROAD-016 Production Telegram inline smoke</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>npm run prod:telegram-inline-smoke -- --help; npx eslint scripts/prod-telegram-inline-smoke.ts; npm run test:run -- src/lib/telegram/handlers/inline.test.ts src/lib/telegram/webhook.integration.test.ts; npm run test:run -- src/lib/telegram; npm run test:run -- src/lib/risk; npx tsc --noEmit --pretty false; railway run npm run prod:telegram-inline-smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>Passed: production Railway smoke high-risk text, low-signal phone and low-signal Telegram username inline previews all returned webhook 200 with no checks/session persisted; focused inline/webhook 2 files / 95 tests; full Telegram 50 files / 1342 tests; full risk 30 files / 458 tests; scoped TS eslint 0 errors; tsc 0 errors.</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>ROAD-016, Telegram inline QA, production webhook, non-persistence</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>Added production synthetic inline-query smoke and package script. It validates deployed webhook handling and privacy invariants for inline previews without TELEGRAM_QA_CHAT_ID; synthetic inline ids do not validate visual Telegram-client rendering.</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>Next: collect real Telegram-client inline screenshots/examples for visual article content; collect real provider Voice-in/STT audio/transcript fixtures when key/audio are available.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(telegram): add inline client qa checklist
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3a691299250142fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbe69fa95c3f54931"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1816ac48c51749f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R20ea267576be47f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re884c97023844023"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5c74f141d0dc4833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rf0fb522ad579439c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rdb88674ed4a94fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R34c082138f754b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rdffd90423f6749af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raef23f90af9c49f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rad59130d39e74b15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2705,10 +2705,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real Telegram-client inline QA examples/screenshots for Phone Reputation v2 / Inline QA, and real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
+        <x:v>Next queue item: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, inline Risk Passport QA, Phone Reputation v2 wording/source confidence, inline regression matrix and production inline smoke verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, inline Risk Passport QA, Phone Reputation v2 wording/source confidence, inline regression matrix, production inline smoke and inline client QA checklist verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12768,6 +12768,32 @@
         <x:v>Next: collect real Telegram-client inline screenshots/examples for visual article content; collect real provider Voice-in/STT audio/transcript fixtures when key/audio are available.</x:v>
       </x:c>
     </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>QA-2026-07-02-019</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>ROAD-017 Telegram inline client QA checklist</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>npm run prod:telegram-inline-smoke -- --help; npx eslint scripts/prod-telegram-inline-smoke.ts; npm run test:run -- src/lib/telegram/handlers/inline.test.ts src/lib/telegram/webhook.integration.test.ts; npm run test:run -- src/lib/telegram; npx tsc --noEmit --pretty false</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>Passed: production inline smoke --help; scoped TS eslint 0 errors; focused inline/webhook 2 files / 95 tests; full Telegram 50 files / 1342 tests; tsc 0 errors; workbook inspect/render 0 formula errors.</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>ROAD-017, Telegram inline QA, real client screenshot workflow</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>Added manual Telegram-client inline QA checklist with safe cases, capture/redaction rules, moderator-chat non-delivery expectation and evidence log template. It complements production synthetic inline smoke and does not commit raw screenshots.</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>Next: run the checklist in a real Telegram client and attach/summarize sanitized screenshots; collect real STT provider examples when key/audio are available.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(tracker): close tg006 risk passport status
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rf0fb522ad579439c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rdb88674ed4a94fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R34c082138f754b9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rdffd90423f6749af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raef23f90af9c49f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rad59130d39e74b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R45ffd4655b4d4655"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re34de34524fa408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Reb2323899aa044ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re89f93e3be994cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R016e47d332b742e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf1910a0eb11d4c30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2708,7 +2708,7 @@
         <x:v>Next queue item: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, inline Risk Passport QA, Phone Reputation v2 wording/source confidence, inline regression matrix, production inline smoke and inline client QA checklist verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, inline QA and production inline smoke verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2744,7 +2744,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2761,7 +2761,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="8" t="inlineStr">
         <x:is>
@@ -3483,30 +3483,20 @@
           <x:t xml:space="preserve">.kiro/specs/risk-passport-v1; ai_docs/EXECUTION_PLAN_2026-06-21.md</x:t>
         </x:is>
       </x:c>
-      <x:c r="H7" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I7" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit + live phone passport QA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J7" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phone passport production smoke passed for a synthetic UZ mobile number; P8.1/P8.2 username coach/heuristics remain.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K7" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L7" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Do not invent Telegram account age, hidden scam labels, or Telegram complaint history. 2026-06-30 production pass: synthetic +998 mobile persisted phone lastCheck with valid_uz_phone and no Guardian/high-risk.</x:t>
-        </x:is>
+      <x:c r="H7" s="14" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I7" s="8" t="str">
+        <x:v>Unit + live phone passport QA + Risk Passport / formatter / public metadata / inline regressions</x:v>
+      </x:c>
+      <x:c r="J7" s="8" t="str">
+        <x:v>Closed 2026-07-02: phone passport production smoke had passed earlier; current focused tests cover low-signal phone and Telegram username passport rendering, Bot API limitation copy, moderated phone reputation source/scope and no owner/hidden-label/account-age claims.</x:v>
+      </x:c>
+      <x:c r="K7" s="13" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L7" s="8" t="str">
+        <x:v>Reconciled after ROAD-011/013/014/015/016/017. Remaining work is manual real Telegram-client inline screenshots and future session-memory/pig-butchering UX, not TG-006 core passport behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -12794,6 +12784,32 @@
         <x:v>Next: run the checklist in a real Telegram client and attach/summarize sanitized screenshots; collect real STT provider examples when key/audio are available.</x:v>
       </x:c>
     </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>QA-2026-07-02-020</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>TG-006 Risk Passport tracker reconciliation</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>npm run test:run -- src/lib/risk/risk-passport.test.ts src/lib/telegram/format.test.ts src/lib/telegram/public-metadata.server.test.ts src/lib/telegram/handlers/inline.test.ts; npx eslint src/lib/risk/risk-passport.ts src/lib/risk/risk-passport.test.ts src/lib/telegram/format.test.ts src/lib/telegram/public-metadata.server.test.ts src/lib/telegram/handlers/inline.test.ts</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>Passed: focused Risk Passport / formatter / public metadata / inline suite 4 files / 64 tests; scoped TS eslint 0 errors; workbook inspect/render 0 formula errors.</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>TG-006, Risk Passport, Phone Reputation v2, Telegram inline QA</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>Reconciled stale TG-006 Partial tracker row. Existing code and tests cover phone/username Risk Passport, Bot API limitation copy, source-scoped moderated phone reputation, no owner/hidden-label/account-age claims, and inline low-signal passport rendering.</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>Next: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider STT examples when key/audio are available.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(tracker): reconcile conversation memory status
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R45ffd4655b4d4655"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re34de34524fa408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Reb2323899aa044ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re89f93e3be994cf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R016e47d332b742e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf1910a0eb11d4c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R0fae0d5971654aca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3d19141516b747af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9bd58c6b39174c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re91f108d10bc48e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R828e7080c4704b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc8658808b43c44bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2708,7 +2708,7 @@
         <x:v>Next queue item: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, inline QA and production inline smoke verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, conversation memory reconciliation, inline QA and production inline smoke verified on 2026-07-02.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -12810,6 +12810,32 @@
         <x:v>Next: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider STT examples when key/audio are available.</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>QA-2026-07-02-021</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>Conversation memory / pig-butchering reconciliation</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/conversation-check.test.ts src/lib/telegram/webhook.integration.test.ts; npx eslint src/lib/telegram/conversation-check.ts src/lib/telegram/conversation-check.test.ts src/lib/telegram/handlers/conversation.ts src/lib/telegram/webhook.integration.test.ts</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>Passed: focused conversation-check + webhook integration 2 files / 93 tests; scoped TS eslint 0 errors; workbook inspect/render 0 formula errors.</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>ROAD-004, /conversation, pig-butchering, romance grooming, privacy</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>Reconciled stale open-task wording. Explicit /conversation mode already stores only derived stage/action/reason metadata and catches romance/trust-building followed by investment/crypto/payment pressure without persisting raw chat text.</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>Next: real Telegram-client inline screenshots and real STT provider examples remain external live-evidence tasks; passive always-on conversation profiling remains a future privacy/product decision.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): route typed panic intents to sos
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R0fae0d5971654aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3d19141516b747af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9bd58c6b39174c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re91f108d10bc48e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R828e7080c4704b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc8658808b43c44bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R4a5dcbcddc254a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R72bd302705ee4fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc9accd1d4ab2468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1a9530a28b7343e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra8be2d5f42ca4468"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4704ebbcd2514411"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2688,10 +2688,8 @@
           <x:t xml:space="preserve">Next phase</x:t>
         </x:is>
       </x:c>
-      <x:c r="E1" s="594" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Owner note</x:t>
-        </x:is>
+      <x:c r="E1" s="594" t="str">
+        <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -2699,7 +2697,7 @@
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>64</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
@@ -2708,7 +2706,7 @@
         <x:v>Next queue item: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, conversation memory reconciliation, inline QA and production inline smoke verified on 2026-07-02.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, conversation memory reconciliation, inline QA and production inline smoke verified on 2026-07-02. P0 Text -&gt; Panic routing shipped/tested; fresh QA plan prioritizes image/profile fallback, live Telegram QA matrix, conversational follow-ups and proactive Family Shield.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2744,7 +2742,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2778,7 +2776,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C7" s="8" t="inlineStr">
         <x:is>
@@ -6847,6 +6845,158 @@
         <x:v>Next SOS additions should update the profile map once and rely on existing i18n/wellformedness tests.</x:v>
       </x:c>
     </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" t="str">
+        <x:v>P0-2026-07-02-001</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>Telegram UX / emergency routing</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>Text panic intent routing</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>As a stressed user who already sent a code, installed an APK or transferred money, I want typed first-person help messages to open the right SOS flow immediately.</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>Typed first-person already-happened emergencies open the matching SOS flow before the normal risk pipeline.</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>src/lib/telegram/handlers/check.ts; src/lib/telegram/handlers/check.followup-routing.test.ts</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>User feedback 2026-07-02; live Telegram QA notes</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I66" t="str">
+        <x:v>Focused unit tests</x:v>
+      </x:c>
+      <x:c r="J66" t="str">
+        <x:v>Text path now reuses panic intent detection before runCheck, while forwarded/quoted third-party messages stay on the normal risk pipeline.</x:v>
+      </x:c>
+      <x:c r="K66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L66" t="str">
+        <x:v>No raw evidence is stored; panic context stores only scenario metadata. Forwarded/quoted messages are guarded to avoid false SOS routing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" t="str">
+        <x:v>P1-2026-07-02-002</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>Telegram QA / image-profile fallback</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>Profile screenshot fallback</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>As a user sending a screenshot of a Telegram profile/chat, I want the bot to explain what it can and cannot infer, then ask for the actual request text/link/QR next.</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>The bot does not accuse from a profile screenshot, but recognizes the profile/chat context and asks for what the contact requested.</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>src/lib/telegram/image-fallback.ts; src/lib/risk/image-intelligence.ts</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>User feedback 2026-07-02 Lina profile screenshot</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>Needs live/harness QA</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>Feedback from Lina profile screenshot: fallback is safe but too generic. Needs profile-aware fallback and live QA cases.</x:v>
+      </x:c>
+      <x:c r="K67" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L67" t="str">
+        <x:v>Must avoid hidden Telegram claims, owner inference, account-age claims or unverified accusations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" t="str">
+        <x:v>P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>Telegram QA matrix</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>Live response quality QA</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>As the product owner, I want a repeatable live/harness QA matrix that checks bot replies for tone, routing, language and next-step usefulness.</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Each scenario records user input, actual bot answer, verdict on answer quality, and exact fix target.</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>ai_docs/TELEGRAM_BOT_QA_REPORT.md; npm run qa:telegram-report; npm run qa:telegram-visual</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>User feedback 2026-07-02 live bot QA request</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I68" t="str">
+        <x:v>Needs new matrix rows</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>Covers RU/UZ/EN free text, screenshots, profile images, QR, voice, follow-ups, panic, report and Family Shield.</x:v>
+      </x:c>
+      <x:c r="K68" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
+        <x:v>Live QA must use sanitized examples and avoid sending secrets or raw victim data to moderator channels.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" t="str">
+        <x:v>P2-2026-07-02-004</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>Family Shield / delivery</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>Proactive trusted-person alert</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>As a protected user, I want an opt-in proactive trusted-person alert after high-risk checks so help can arrive through someone not under pressure.</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>After explicit opt-in, high-confidence high-risk checks can send a redacted alert to the trusted contact with cooldown and acknowledgement.</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>src/lib/telegram/family-shield.server.ts; src/lib/telegram/guardian-angel.ts</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>User feedback 2026-07-02 delivery strategy</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>Needs design + tests</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>Requires explicit opt-in, redacted alert, cooldown, acknowledgement button and false-positive guardrails.</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L69" t="str">
+        <x:v>Alert must not include scammer number, codes, links, screenshots, card data or raw check evidence.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12836,6 +12986,32 @@
         <x:v>Next: real Telegram-client inline screenshots and real STT provider examples remain external live-evidence tasks; passive always-on conversation profiling remains a future privacy/product decision.</x:v>
       </x:c>
     </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" t="str">
+        <x:v>QA-2026-07-02-022</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>Telegram P0 Text -&gt; Panic routing</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.followup-routing.test.ts; npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>Passed: 15/15 follow-up routing tests and 18/18 voice tests. Typed first-person already-happened emergencies route to SOS; forwarded/quoted messages remain risk checks.</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>TG-005, TG-014, Telegram emergency routing</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>Added handleCheck regressions for typed already-transferred and already-sent-code phrases plus forwarded/quoted guardrails.</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>Proceed to P1 image/profile fallback QA and live Telegram QA matrix.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): add profile image triage fallback
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R4a5dcbcddc254a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R72bd302705ee4fc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc9accd1d4ab2468c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1a9530a28b7343e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra8be2d5f42ca4468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4704ebbcd2514411"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R8fc445d5d5fa4994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R75e787e2847e4324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb21b8fc7753c47fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6685a494a0044fe0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rac56af57d4a7498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3637f4d880024115"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, conversation memory reconciliation, inline QA and production inline smoke verified on 2026-07-02. P0 Text -&gt; Panic routing shipped/tested; fresh QA plan prioritizes image/profile fallback, live Telegram QA matrix, conversational follow-ups and proactive Family Shield.</x:v>
+        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, conversation memory reconciliation, inline QA and production inline smoke verified on 2026-07-02. P0 Text -&gt; Panic routing shipped/tested; fresh QA plan prioritizes image/profile fallback, live Telegram QA matrix, conversational follow-ups and proactive Family Shield. P1 image/profile fallback shipped/tested with profile/chat triage and safe Telegram-profile follow-up context.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2742,7 +2742,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -2776,7 +2776,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="8" t="inlineStr">
         <x:is>
@@ -6906,19 +6906,19 @@
         <x:v>User feedback 2026-07-02 Lina profile screenshot</x:v>
       </x:c>
       <x:c r="H67" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I67" t="str">
-        <x:v>Needs live/harness QA</x:v>
+        <x:v>Bot QA matrix + webhook integration + i18n completeness</x:v>
       </x:c>
       <x:c r="J67" t="str">
-        <x:v>Feedback from Lina profile screenshot: fallback is safe but too generic. Needs profile-aware fallback and live QA cases.</x:v>
+        <x:v>Closed 2026-07-02: unreadable image fallback now has Telegram profile/chat triage; callback answer avoids accusations and asks for the actual request; profile triage stores only safe telegram_profile follow-up context.</x:v>
       </x:c>
       <x:c r="K67" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L67" t="str">
-        <x:v>Must avoid hidden Telegram claims, owner inference, account-age claims or unverified accusations.</x:v>
+        <x:v>No raw screenshot, OCR text, phone, URL or Telegram identifier is persisted in the profile triage context.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
@@ -13012,6 +13012,32 @@
         <x:v>Proceed to P1 image/profile fallback QA and live Telegram QA matrix.</x:v>
       </x:c>
     </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" t="str">
+        <x:v>QA-2026-07-02-023</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>P1 Telegram profile/chat image fallback</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/bot-qa-matrix.test.ts src/lib/telegram/webhook.integration.test.ts src/lib/telegram/i18n-completeness.test.ts; npx eslint scoped files; git diff --check</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>Passed: 3 files / 766 tests; scoped eslint 0 errors; diff whitespace check clean. New profile/chat triage button and safe follow-up context verified.</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>P1-2026-07-02-002, Telegram unreadable image fallback, profile/chat triage</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>Regression verifies conservative profile answer: profile fields are clues, not proof; only request content matters. Webhook callback persists telegram_profile context without raw image data.</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>Proceed to P1 live Telegram QA matrix for RU/UZ/EN free text, screenshots, QR, voice, panic, report and Family Shield.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): align job source followup copy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R8fc445d5d5fa4994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R75e787e2847e4324"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb21b8fc7753c47fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6685a494a0044fe0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rac56af57d4a7498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3637f4d880024115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdcde998396384eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra3d2bf5a61a342fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rf828de73b3144d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2d87e43d92c74027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1e7c6f9dd856417e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R04248c8539ab4ee4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2694,7 +2694,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
         <x:v>68</x:v>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: capture real Telegram-client inline screenshots/examples using ai_docs/TELEGRAM_INLINE_QA.md; collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
+        <x:v>Next queue item: P1 web/Telegram residual QA; optional manual-only side effects only with action-time approval (trusted opt-out, live-call trusted alert, Guardian voice-out, staged report retry); collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog, P1 QA, CSP, emergency profile-map, Voice-out assets, RU/UZ/EN STT corpus, Voice-in fixture workflow, collector validation, Risk Passport TG-006 reconciliation, conversation memory reconciliation, inline QA and production inline smoke verified on 2026-07-02. P0 Text -&gt; Panic routing shipped/tested; fresh QA plan prioritizes image/profile fallback, live Telegram QA matrix, conversational follow-ups and proactive Family Shield. P1 image/profile fallback shipped/tested with profile/chat triage and safe Telegram-profile follow-up context.</x:v>
+        <x:v>Owner note: security backlog and P1 QA baseline are closed. Live Telegram button matrix covered start/menu/lang/conversation/trainer/image triage/SOS 1-15/follow-ups/Guardian/voice-out/Family invite/revoke/trusted alert/report submit through 2026-07-04. 2026-07-04 copy fix aligned job/easy-income Check source response with the button label and source-verification task. Remaining: optional side-effect retests, provider STT corpus, then UX/logistics/product backlog.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4266,15 +4266,11 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I20" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit + focused admin/report tests + build; live Telegram report smoke recommended</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J20" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-01: P7 polish closed. Web final copy is warmer; duplicate-as-signal language stays non-disclosing; admin uses active target_signal_count and target_last_report_at. Run live Telegram /report smoke after deploy.</x:t>
-        </x:is>
+      <x:c r="I20" s="8" t="str">
+        <x:v>Unit + focused admin/report tests + build + live Telegram report-submit smoke</x:v>
+      </x:c>
+      <x:c r="J20" s="8" t="str">
+        <x:v>Closed 2026-07-04: synthetic /report success path live-tested with https://example.invalid/live-qa-test and LIVE QA TEST description; bot confirmed moderation-only publication and moderator alert was observed.</x:v>
       </x:c>
       <x:c r="K20" s="13" t="inlineStr">
         <x:is>
@@ -4638,15 +4634,11 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I26" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit/property/i18n tests + Telegram QA report/visual + build</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J26" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closed 2026-07-01: first cards, detailed checklists and trusted-person follow-ups are distinct for sextortion, publication threats and minor safety; existing voice-clone and modern scenarios 12-15 remain covered. Live Telegram screenshot review remains release-check only.</x:t>
-        </x:is>
+      <x:c r="I26" s="8" t="str">
+        <x:v>Unit/property/i18n tests + Telegram QA report/visual + live Telegram button matrix</x:v>
+      </x:c>
+      <x:c r="J26" s="8" t="str">
+        <x:v>Closed 2026-07-04: live matrix covered modern SOS buttons; job/easy-income Check source copy polished so the answer starts with source verification instead of generic where-to-go wording. Optional live retest after deploy remains release-check only.</x:v>
       </x:c>
       <x:c r="K26" s="14" t="inlineStr">
         <x:is>
@@ -9015,20 +9007,14 @@
           <x:t xml:space="preserve">The flow validates target, description, type, city, loss; accepts 'none'; stores moderated report and masks public alerts.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E13" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closed 2026-07-01: warmer final copy, duplicate-as-signal language and admin active signal count/latest report time implemented; live report smoke after deploy remains release check.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F13" s="567" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G13" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Automated pass 2026-07-01: focused admin/report tests passed 3 files / 28 tests; scoped eslint and npm run build passed.</x:t>
-        </x:is>
+      <x:c r="E13" s="50" t="str">
+        <x:v>Closed 2026-07-04: live Telegram /report success path completed with synthetic example.invalid target and LIVE QA TEST description; bot confirmed signal accepted and moderation-only publication.</x:v>
+      </x:c>
+      <x:c r="F13" s="567" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="G13" s="50" t="str">
+        <x:v>Live pass 2026-07-04: action-time approval; moderator-chat alert observed; ai_docs/TELEGRAM_BUTTON_QA_MATRIX.md updated.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="76" customHeight="1">
@@ -9052,20 +9038,14 @@
           <x:t xml:space="preserve">Each modern scenario has a short first card, context-specific next step, ready phrase, where-to-go, trusted-contact option, and full checklist.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E14" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closed 2026-07-01: distinct copy for minors, sextortion and publication threats implemented; duplicate generic trusted-person branch removed for those cases.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F14" s="568" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G14" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Automated pass 2026-07-01: eslint; emergency/panic/voice-out suite 4 files / 135 tests; emergency property/i18n/follow-up suite 5 files / 632 tests; bot QA matrix 18 tests; qa:telegram-report, qa:telegram-visual and npm run build passed.</x:t>
-        </x:is>
+      <x:c r="E14" s="50" t="str">
+        <x:v>Closed 2026-07-04: job/easy-income Check source heading/copy polished to match the button label and emphasize company/vacancy verification before escalation contacts.</x:v>
+      </x:c>
+      <x:c r="F14" s="568" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="G14" s="50" t="str">
+        <x:v>Automated pass 2026-07-04: npm run test:run -- src/lib/telegram/emergency-followup.test.ts passed 28 tests; npm run qa:telegram-report regenerated the bot QA report.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">

</xml_diff>

<commit_message>
docs(tracker): record production job source retest
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdcde998396384eff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra3d2bf5a61a342fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rf828de73b3144d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2d87e43d92c74027"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1e7c6f9dd856417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R04248c8539ab4ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R530b34d7620743a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Raa6c61a7c0454385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6c3245189df24f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rda14ba5955464013"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re4d3bb9748b44ab3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R78bf9962b3104fd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: P1 web/Telegram residual QA; optional manual-only side effects only with action-time approval (trusted opt-out, live-call trusted alert, Guardian voice-out, staged report retry); collect real provider Voice-in/STT examples when OPENAI_API_KEY/local audio are available.</x:v>
+        <x:v>Next queue item: Voice-in/STT real-provider corpus or Voice-out human listen-through. Manual-only Telegram side effects remain approval-only.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog and P1 QA baseline are closed. Live Telegram button matrix covered start/menu/lang/conversation/trainer/image triage/SOS 1-15/follow-ups/Guardian/voice-out/Family invite/revoke/trusted alert/report submit through 2026-07-04. 2026-07-04 copy fix aligned job/easy-income Check source response with the button label and source-verification task. Remaining: optional side-effect retests, provider STT corpus, then UX/logistics/product backlog.</x:v>
+        <x:v>Owner note: production deploy dfc77c61 for commit 7d22868 succeeded on 2026-07-04; prod smoke and security smoke passed. Job/easy-income Check source was retested live in Telegram after deploy and now starts with "Проверить источник"; old "Куда обратиться" heading absent. Branch pushed to origin through 6b02789. Follow-up prod smoke confirmed AI provider healthy again: gemini-3.5-flash status=200.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4635,10 +4635,10 @@
         </x:is>
       </x:c>
       <x:c r="I26" s="8" t="str">
-        <x:v>Unit/property/i18n tests + Telegram QA report/visual + live Telegram button matrix</x:v>
+        <x:v>Unit/property/i18n tests + Telegram QA report/visual + live Telegram button matrix + post-deploy live retest.</x:v>
       </x:c>
       <x:c r="J26" s="8" t="str">
-        <x:v>Closed 2026-07-04: live matrix covered modern SOS buttons; job/easy-income Check source copy polished so the answer starts with source verification instead of generic where-to-go wording. Optional live retest after deploy remains release-check only.</x:v>
+        <x:v>Closed 2026-07-04: live matrix covered modern SOS buttons; job/easy-income Check source copy deployed via 7d22868 and live-retested after deploy. Next related work is real Voice-in/STT corpus or Voice-out human listen-through.</x:v>
       </x:c>
       <x:c r="K26" s="14" t="inlineStr">
         <x:is>
@@ -9039,13 +9039,13 @@
         </x:is>
       </x:c>
       <x:c r="E14" s="50" t="str">
-        <x:v>Closed 2026-07-04: job/easy-income Check source heading/copy polished to match the button label and emphasize company/vacancy verification before escalation contacts.</x:v>
+        <x:v>Closed 2026-07-04: modern SOS scenarios passed live button matrix; job/easy-income Check source heading/copy polished, deployed, and post-deploy live-retested in Telegram.</x:v>
       </x:c>
       <x:c r="F14" s="568" t="str">
         <x:v>P3</x:v>
       </x:c>
       <x:c r="G14" s="50" t="str">
-        <x:v>Automated pass 2026-07-04: npm run test:run -- src/lib/telegram/emergency-followup.test.ts passed 28 tests; npm run qa:telegram-report regenerated the bot QA report.</x:v>
+        <x:v>Passed 2026-07-04: emergency-followup tests 28/28, qa:telegram-report regenerated, Railway deploy dfc77c61 succeeded, prod:smoke and prod:security-smoke passed, live Telegram Check source retest confirmed "Проверить источник" and no old "Куда обратиться" heading.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">
@@ -13018,6 +13018,32 @@
         <x:v>Proceed to P1 live Telegram QA matrix for RU/UZ/EN free text, screenshots, QR, voice, panic, report and Family Shield.</x:v>
       </x:c>
     </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>QA-2026-07-04-001</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>TG-025 job/easy-income Check source deploy/live retest</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>railway up --ci; railway run npm run prod:smoke; railway run npm run prod:security-smoke; live Telegram /panic -&gt; Работа / лёгкий доход -&gt; Проверить источник; repeat prod:smoke</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Passed: deploy dfc77c61 succeeded, healthcheck passed, production smoke/security smoke passed, live Telegram reply starts with "Проверить источник" and old "Куда обратиться" heading is absent. Repeat prod:smoke confirmed AI provider status=200.</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>TG-025, T-013</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>Committed 7d22868 fix and 6b02789 QA docs; branch pushed to origin. Live retest used only safe non-side-effect Telegram actions.</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>Next: choose Voice-in/STT corpus or Voice-out human listen-through.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): cover uz cyrillic voice stt intents
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R530b34d7620743a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Raa6c61a7c0454385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6c3245189df24f62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rda14ba5955464013"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re4d3bb9748b44ab3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R78bf9962b3104fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R5ef8ac7773e94d14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R7a868335cb1549f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R62befeda834348da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5ac466951dc24c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2845bd7dc5ac4a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd4df5344a9b94370"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: Voice-in/STT real-provider corpus or Voice-out human listen-through. Manual-only Telegram side effects remain approval-only.</x:v>
+        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript fixtures or run Voice-out human listen-through. Manual-only Telegram side effects remain approval-only.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: production deploy dfc77c61 for commit 7d22868 succeeded on 2026-07-04; prod smoke and security smoke passed. Job/easy-income Check source was retested live in Telegram after deploy and now starts with "Проверить источник"; old "Куда обратиться" heading absent. Branch pushed to origin through 6b02789. Follow-up prod smoke confirmed AI provider healthy again: gemini-3.5-flash status=200.</x:v>
+        <x:v>Owner note: TG-014 Voice-in/STT Uzbek Cyrillic replay corpus shipped on 2026-07-04. UZ Cyrillic SMS-code sent, money transferred, active-call pressure and negated-code phrases now route through the existing SOS/normal-check boundaries. Full Telegram suite passed 50 files / 1369 tests. Remaining Voice-in work is real provider audio/transcript capture when local audio and provider key are available.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3958,19 +3958,19 @@
         </x:is>
       </x:c>
       <x:c r="F15" s="8" t="str">
-        <x:v>Unit tests + integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + fixture workflow</x:v>
+        <x:v>src/lib/telegram/handlers/check.ts; src/lib/telegram/voice-stt-provider-fixtures.ts; src/lib/risk/check-core.ts</x:v>
       </x:c>
       <x:c r="G15" s="8" t="str">
-        <x:v>Closed 2026-07-02 slice: replay corpus extracted to voice-stt-provider-fixtures.ts and local real-provider capture workflow added via npm run stt:transcribe-fixtures. Remaining: collect real provider audio/transcript fixtures from live QA and tune confidence heuristics from production examples.</x:v>
+        <x:v>.kiro/specs/telegram-voice-stt-v1; ai_docs/VOICE_STT_FIXTURES.md</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>2026-07-02: Voice-in/STT fixture workflow shipped. Raw audio stays under ignored private/voice-stt-fixtures; collector emits sanitized transcripts only. Local live provider capture was not run because OPENAI_API_KEY is absent.</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
-        <x:v>Unit tests + integration tests + live QA + production-like STT corpus regression</x:v>
+        <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-02 slice: production-like STT transcripts now cover card-security-code, remote-access, Telegram-login-QR and negated already-happened phrases across RU/UZ without raw audio fixtures. Keep collecting real provider audio/transcript examples for the next corpus expansion.</x:v>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic transcripts for sent SMS-code, transferred money and active-call pressure route to SOS; negated code wording stays on the normal check pipeline. Next: collect real provider audio/transcript fixtures from live QA.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -3978,7 +3978,7 @@
         </x:is>
       </x:c>
       <x:c r="L15" s="8" t="str">
-        <x:v>2026-07-02: first STT corpus/confidence slice shipped. Negated phrases like 'I did not send the code' no longer route to already-happened SOS; completed card/CVV, remote-access and Telegram QR phrases route to the matching SOS. Remaining: real provider audio fixture expansion.</x:v>
+        <x:v>No raw audio or Telegram file IDs committed; replay corpus stores sanitized transcripts only. Negated first-person phrases remain guarded against false SOS.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -8933,20 +8933,16 @@
           <x:t xml:space="preserve">Short voice is transcribed, shown back to the user, and then checked; uncertain transcription should avoid hard verdicts.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closed 2026-06-30: friendly delivery/card false positives covered; concrete voice hook phrase is extracted from sanitized transcript preview.</x:t>
-        </x:is>
+      <x:c r="E11" s="50" t="str">
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap covered for sent SMS-code, transferred money, active-call pressure and negated code wording; real provider audio/transcript capture remains next.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P1</x:t>
         </x:is>
       </x:c>
-      <x:c r="G11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Automated pass 2026-06-30; live voice/STT QA covered 2026-06-30; regression watch</x:t>
-        </x:is>
+      <x:c r="G11" s="50" t="str">
+        <x:v>Passed 2026-07-04: full Telegram suite 50 files / 1369 tests after adding UZ Cyrillic Voice-in/STT fixtures and routing normalization.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
@@ -13044,6 +13040,32 @@
         <x:v>Next: choose Voice-in/STT corpus or Voice-out human listen-through.</x:v>
       </x:c>
     </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>QA-2026-07-04-002</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>TG-014 Voice-in/STT Uzbek Cyrillic replay corpus</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts; npm run test:run -- src/lib/telegram</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>Passed: focused voice handler 18/18 after adding UZ Cyrillic fixtures; full Telegram suite 50 files / 1369 tests.</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>TG-014, T-010</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>Added Uzbek Cyrillic normalization and replay rows for SMS-code sent, money transferred, active call and negated code. No raw audio committed.</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>Next: collect real provider audio/transcript fixtures from live QA, or run Voice-out human listen-through.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(tracker): record voice-out release qa revalidation
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R5ef8ac7773e94d14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R7a868335cb1549f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R62befeda834348da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5ac466951dc24c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2845bd7dc5ac4a3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd4df5344a9b94370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R041c330a99444c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R907eef2ca45b4586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R551df41b502b4175"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6c63150ff90c4301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6043c56948cc41a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc38017b03c1a4365"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript fixtures or run Voice-out human listen-through. Manual-only Telegram side effects remain approval-only.</x:v>
+        <x:v>Next queue item: explicit approval for production Voice-out sendAudio/listen-through, or collect real provider Voice-in/STT audio/transcript fixtures. Manual-only Telegram side effects remain approval-only.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: TG-014 Voice-in/STT Uzbek Cyrillic replay corpus shipped on 2026-07-04. UZ Cyrillic SMS-code sent, money transferred, active-call pressure and negated-code phrases now route through the existing SOS/normal-check boundaries. Full Telegram suite passed 50 files / 1369 tests. Remaining Voice-in work is real provider audio/transcript capture when local audio and provider key are available.</x:v>
+        <x:v>Owner note: TG-014 UZ Cyrillic Voice-in replay corpus shipped on 2026-07-04. TG-015 prerecorded Voice-out release QA revalidated on 2026-07-04: 45 RU/UZ/EN OGG assets passed validation and the focused Telegram voice-out/emergency/webhook suite passed 3 files / 135 tests. Remaining real-provider Voice-in work needs local audio fixtures and a provider key; production Voice-out smoke needs action-time approval because it sends/deletes QA-chat audio.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4023,10 +4023,10 @@
         </x:is>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke + 2026-07-02 asset revalidation</x:v>
+        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke + 2026-07-02 asset revalidation + 2026-07-04 automated release QA</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>Closed 2026-07-02: 45 committed SOS OGG/Opus assets for panic-1..15 in RU/UZ/EN revalidated locally; runtime still prefers OGG before WAV, TTS budget and provider calls. Human listen-through remains a release QA checklist item, not an architecture blocker.</x:v>
+        <x:v>Closed 2026-07-04: 45 committed SOS OGG/Opus assets for panic-1..15 in RU/UZ/EN revalidated again; focused voice-out/emergency/webhook suite passed 3 files / 135 tests. Human/live listen-through and production sendAudio smoke remain action-time approval-only because they send/delete real QA-chat audio.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="inlineStr">
         <x:is>
@@ -8966,20 +8966,14 @@
           <x:t xml:space="preserve">The button voices only a short safe script, with text caption, cache/cooldown, and graceful daily-limit messaging.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closed 2026-07-01: SOS OGG static assets and deployed production webhook playback passed; provider-limit fallback now removes dynamic/provider-only voice buttons while preserving static SOS voice buttons.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F12" s="567" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Passed 2026-07-01: voice-out unit suite 14 tests, asset validator 45 files, build, deploy/full production smokes, and provider-limit keyboard regression passed.</x:t>
-        </x:is>
+      <x:c r="E12" s="50" t="str">
+        <x:v>Closed 2026-07-04: static SOS OGG assets and focused Telegram voice-out/emergency/webhook regressions passed. Production sendAudio/listen-through smoke is manual-only because it writes audio to the QA chat.</x:v>
+      </x:c>
+      <x:c r="F12" s="567" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="G12" s="50" t="str">
+        <x:v>Passed 2026-07-04: `npm run tts:validate-assets` validated 45 OGG assets, and focused Telegram suite passed 3 files / 135 tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
@@ -13066,6 +13060,32 @@
         <x:v>Next: collect real provider audio/transcript fixtures from live QA, or run Voice-out human listen-through.</x:v>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>QA-2026-07-04-003</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>TG-015 Voice-out automated release QA revalidation</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>npm run tts:validate-assets; npm run test:run -- src/lib/telegram/voice-out.server.test.ts src/lib/telegram/emergency-followup.test.ts src/lib/telegram/webhook.integration.test.ts</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Passed: 45 OGG assets / 1,683,698 bytes; focused Telegram suite 3 files / 135 tests. Local prod:telegram-voice-out-smoke was not run because local TELEGRAM_BOT_TOKEN is absent and the script sends/deletes real QA-chat audio.</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>TG-015, T-011</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Validator confirmed all RU/UZ/EN panic-1..15 OGG assets, smallest panic-3-uz.ogg 27,662 bytes / 7.73s, largest panic-12-ru.ogg 48,611 bytes / 14.05s. Tests cover static-first voice-out routing plus emergency/webhook callback paths.</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>Next: approve production Voice-out smoke/live listen-through at action time, or provide local Voice-in/STT audio fixtures and provider key for real-provider corpus capture.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(tracker): record voice-out production smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R041c330a99444c4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R907eef2ca45b4586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R551df41b502b4175"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6c63150ff90c4301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6043c56948cc41a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc38017b03c1a4365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc8a4f626f42c4b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R4aac98b817344d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc0bdbed96d3a4fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1d7e114501d24fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rafd5436dfb754d2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2dc32cb444be4d6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: explicit approval for production Voice-out sendAudio/listen-through, or collect real provider Voice-in/STT audio/transcript fixtures. Manual-only Telegram side effects remain approval-only.</x:v>
+        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript fixtures, or run optional full human listen-through of all prerecorded SOS assets. Manual-only Telegram side effects remain approval-only.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: TG-014 UZ Cyrillic Voice-in replay corpus shipped on 2026-07-04. TG-015 prerecorded Voice-out release QA revalidated on 2026-07-04: 45 RU/UZ/EN OGG assets passed validation and the focused Telegram voice-out/emergency/webhook suite passed 3 files / 135 tests. Remaining real-provider Voice-in work needs local audio fixtures and a provider key; production Voice-out smoke needs action-time approval because it sends/deletes QA-chat audio.</x:v>
+        <x:v>Owner note: TG-014 UZ Cyrillic Voice-in replay corpus shipped on 2026-07-04. TG-015 prerecorded Voice-out release QA and production Telegram smoke passed on 2026-07-04: 45 RU/UZ/EN OGG assets validated, focused Telegram suite passed 3 files / 135 tests, Telegram accepted RU/UZ/EN panic-6 OGG audio, and the production webhook accepted a voiceout:panic:6 callback. Remaining real-provider Voice-in work needs local audio fixtures and a provider key.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4023,10 +4023,10 @@
         </x:is>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke + 2026-07-02 asset revalidation + 2026-07-04 automated release QA</x:v>
+        <x:v>Unit tests + static asset audit + deployed Telegram OGG playback smoke + 2026-07-02 asset revalidation + 2026-07-04 automated release QA + 2026-07-04 production Telegram smoke</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>Closed 2026-07-04: 45 committed SOS OGG/Opus assets for panic-1..15 in RU/UZ/EN revalidated again; focused voice-out/emergency/webhook suite passed 3 files / 135 tests. Human/live listen-through and production sendAudio smoke remain action-time approval-only because they send/delete real QA-chat audio.</x:v>
+        <x:v>Closed 2026-07-04: 45 committed SOS OGG/Opus assets for panic-1..15 in RU/UZ/EN revalidated again; focused voice-out/emergency/webhook suite passed 3 files / 135 tests; production Telegram smoke accepted RU/UZ/EN panic-6 OGG sendAudio plus webhook callback. Full human listen-through remains optional release QA.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="inlineStr">
         <x:is>
@@ -8967,13 +8967,13 @@
         </x:is>
       </x:c>
       <x:c r="E12" s="50" t="str">
-        <x:v>Closed 2026-07-04: static SOS OGG assets and focused Telegram voice-out/emergency/webhook regressions passed. Production sendAudio/listen-through smoke is manual-only because it writes audio to the QA chat.</x:v>
+        <x:v>Closed 2026-07-04: static SOS OGG assets, focused Telegram voice-out/emergency/webhook regressions and production Telegram voice-out smoke passed. Full human listen-through remains optional for tone/pronunciation.</x:v>
       </x:c>
       <x:c r="F12" s="567" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="G12" s="50" t="str">
-        <x:v>Passed 2026-07-04: `npm run tts:validate-assets` validated 45 OGG assets, and focused Telegram suite passed 3 files / 135 tests.</x:v>
+        <x:v>Passed 2026-07-04: `npm run tts:validate-assets` validated 45 OGG assets; focused Telegram suite passed 3 files / 135 tests; production smoke accepted RU/UZ/EN panic-6 OGG audio and webhook callback.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
@@ -13086,6 +13086,32 @@
         <x:v>Next: approve production Voice-out smoke/live listen-through at action time, or provide local Voice-in/STT audio fixtures and provider key for real-provider corpus capture.</x:v>
       </x:c>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>QA-2026-07-04-004</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>TG-015 production Telegram Voice-out smoke</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>TELEGRAM_QA_CHAT_ID=&lt;private QA chat&gt; railway run npm run prod:telegram-voice-out-smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Passed: Telegram sendAudio accepted panic-6 RU/UZ/EN OGG assets; production webhook accepted voiceout:panic:6 callback; cleanup completed. App-generated audio may remain in QA chat as live playback evidence.</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>TG-015, T-011</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>Smoke marker QAVOICEOUTKANSJSLR. Initial run correctly failed closed because TELEGRAM_QA_CHAT_ID was unset and moderation chat fallback is forbidden. After setting the private QA chat id, the script accepted all three OGG files and the webhook callback.</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>Next: collect real provider Voice-in/STT audio/transcript fixtures, or run optional full human listen-through across all SOS assets/Guardian voice-out with action-time approval.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(telegram): add voice stt provider transcript fixtures
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc8a4f626f42c4b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R4aac98b817344d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rc0bdbed96d3a4fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R1d7e114501d24fd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rafd5436dfb754d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2dc32cb444be4d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Ra286ef666e6448dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb4f19fc85a604c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R71a5f182219a4e77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra7d79e7acfa544b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rffd9263976584f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb469335f3df544db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect real provider Voice-in/STT audio/transcript fixtures, or run optional full human listen-through of all prerecorded SOS assets. Manual-only Telegram side effects remain approval-only.</x:v>
+        <x:v>Next queue item: collect human/live RU and UZ Voice-in/STT provider examples, or run optional full human listen-through of prerecorded SOS assets. Manual-only Telegram side effects remain approval-only.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: TG-014 UZ Cyrillic Voice-in replay corpus shipped on 2026-07-04. TG-015 prerecorded Voice-out release QA and production Telegram smoke passed on 2026-07-04: 45 RU/UZ/EN OGG assets validated, focused Telegram suite passed 3 files / 135 tests, Telegram accepted RU/UZ/EN panic-6 OGG audio, and the production webhook accepted a voiceout:panic:6 callback. Remaining real-provider Voice-in work needs local audio fixtures and a provider key.</x:v>
+        <x:v>Owner note: TG-014 UZ Cyrillic replay corpus and first provider-sanitized Voice-in/STT capture shipped on 2026-07-04. English local audio through production STT provider now covers active-call SOS routing and negated SMS-code normal-check routing. Russian Windows TTS was noisy/empty and was not committed; next provider corpus needs human/live RU and UZ audio examples.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3967,10 +3967,10 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
-        <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures.</x:v>
+        <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized transcript capture.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic transcripts for sent SMS-code, transferred money and active-call pressure route to SOS; negated code wording stays on the normal check pipeline. Next: collect real provider audio/transcript fixtures from live QA.</x:v>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic transcripts route correctly; first production STT provider capture added English active-call -&gt; SOS and English negated SMS-code -&gt; normal-check. Next: collect human/live RU and UZ provider audio/transcript examples.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -8934,15 +8934,13 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap covered for sent SMS-code, transferred money, active-call pressure and negated code wording; real provider audio/transcript capture remains next.</x:v>
-      </x:c>
-      <x:c r="F11" s="566" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1</x:t>
-        </x:is>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap covered; first provider-sanitized transcript capture added English active-call and negated-code examples. RU/UZ human/live provider examples remain next.</x:v>
+      </x:c>
+      <x:c r="F11" s="566" t="str">
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Passed 2026-07-04: full Telegram suite 50 files / 1369 tests after adding UZ Cyrillic Voice-in/STT fixtures and routing normalization.</x:v>
+        <x:v>Passed 2026-07-04: focused voice handler + collector tests 2 files / 24 tests; scoped eslint passed. Provider capture produced sanitized English transcripts through production STT provider.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
@@ -13112,6 +13110,32 @@
         <x:v>Next: collect real provider Voice-in/STT audio/transcript fixtures, or run optional full human listen-through across all SOS assets/Guardian voice-out with action-time approval.</x:v>
       </x:c>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>QA-2026-07-04-005</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>TG-014 Voice-in/STT provider transcript capture</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>Generated ignored local Windows TTS WAV fixtures; railway run npx vite-node .codex-tmp/stt-provider-corpus/run-stt-fixtures.ts; npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/voice-stt-fixture-collector.test.ts; npx eslint scripts/transcribe-voice-stt-fixtures.ts src/lib/telegram/voice-stt-fixture-collector.test.ts src/lib/telegram/voice-stt-provider-fixtures.ts --quiet</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>Passed: production STT provider returned sanitized English transcripts for active-call and negated-code fixtures; focused tests 2 files / 24 tests; scoped eslint passed. Russian Windows TTS attempt was noisy/empty and was not committed.</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>TG-014, T-010</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>Committed replay corpus now has provider_sanitized_transcript rows for en-live-call-tts-001 (panic:6) and en-not-sent-code-tts-001 (normal_check). Local raw WAV, manifest and transcripts remain ignored under private/voice-stt-fixtures.</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>Next: collect human/live RU and UZ provider examples from Telegram voice notes or local audio fixtures, then tune confidence heuristics from real provider transcripts.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): cover live uz voice sent-code transcript
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Ra286ef666e6448dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb4f19fc85a604c33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R71a5f182219a4e77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra7d79e7acfa544b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rffd9263976584f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb469335f3df544db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3ace07679ea84ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1f7c4e3c29f84446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R484c529fb5124a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb10c794c45e04696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2c7670b28ca74b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3065dc70ab0c4d18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: collect human/live RU and UZ Voice-in/STT provider examples, or run optional full human listen-through of prerecorded SOS assets. Manual-only Telegram side effects remain approval-only.</x:v>
+        <x:v>Next queue item: deploy the live UZ Voice-in/STT routing fix, re-run the live Telegram UZ sent-code voice smoke, then continue full live Telegram QA matrix / UX polish.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: TG-014 UZ Cyrillic replay corpus and first provider-sanitized Voice-in/STT capture shipped on 2026-07-04. English local audio through production STT provider now covers active-call SOS routing and negated SMS-code normal-check routing. Russian Windows TTS was noisy/empty and was not committed; next provider corpus needs human/live RU and UZ audio examples.</x:v>
+        <x:v>Owner note: TG-014 live RU/UZ Voice-in/STT QA on 2026-07-04 found UZ `Men SMS kodni yubardim` fell through to not-enough-data. Code now tolerates provider `yubardim/yubordim` variants and committed sanitized live replay rows for UZ sent-code and RU negated-code transcripts. RU negated-code avoids SOS but still deserves warmer conversational UX polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3967,10 +3967,10 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I15" s="8" t="str">
-        <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized transcript capture.</x:v>
+        <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized and live Telegram transcript capture.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic transcripts route correctly; first production STT provider capture added English active-call -&gt; SOS and English negated SMS-code -&gt; normal-check. Next: collect human/live RU and UZ provider audio/transcript examples.</x:v>
+        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; provider-sanitized EN active-call/negated-code and live RU negated-code rows are in replay corpus. Next: deploy and re-run live UZ voice smoke; polish short negated-code voice UX.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -8934,13 +8934,13 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap covered; first provider-sanitized transcript capture added English active-call and negated-code examples. RU/UZ human/live provider examples remain next.</x:v>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered; provider-sanitized EN and live RU negated-code rows are committed. Short negated-code voice UX remains polish.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Passed 2026-07-04: focused voice handler + collector tests 2 files / 24 tests; scoped eslint passed. Provider capture produced sanitized English transcripts through production STT provider.</x:v>
+        <x:v>Passed 2026-07-04: focused voice handler + collector tests 2 files / 24 tests; full Telegram suite 50 files / 1371 tests; scoped eslint passed. Live Telegram observation showed UZ sent-code now has a regression fixture.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
@@ -13136,6 +13136,32 @@
         <x:v>Next: collect human/live RU and UZ provider examples from Telegram voice notes or local audio fixtures, then tune confidence heuristics from real provider transcripts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>QA-2026-07-04-006</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>TG-014 live RU/UZ Voice-in/STT Telegram replay fix</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>Live Telegram Web observation of four user-sent voice notes; npm run test:run -- src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/voice-stt-fixture-collector.test.ts; npm run test:run -- src/lib/telegram; npx eslint src/lib/telegram/handlers/check.ts src/lib/telegram/voice-stt-provider-fixtures.ts --quiet</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>Passed: RU already-sent-code routed to SOS in live production; UZ sent-code transcript fell through before the fix and is now covered by replay fixture. Focused tests 2 files / 24 tests, full Telegram suite 50 files / 1371 tests, scoped eslint passed.</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>TG-014, Voice-in/STT, live Telegram voice QA</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>Added sanitized live replay rows only: UZ provider transcript `Men SMS kodni yubardim.` -&gt; panic:1 and RU negated `Я не отправляла SMS-код` -&gt; normal-check/no SOS. No raw audio, Telegram file ids or provider payloads committed.</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>Next: deploy this fix and re-run live UZ sent-code voice smoke; then address short negated-code voice UX copy and continue live Telegram QA matrix.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs(tracker): record live voice fix deployment
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3ace07679ea84ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1f7c4e3c29f84446"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R484c529fb5124a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb10c794c45e04696"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2c7670b28ca74b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3065dc70ab0c4d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2e5d020070d74f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rfb9556ce6b4e4205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R2f70b6c082344755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra5758b2253e94b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R799836a4b9c943b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd0a99a8874ca462e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: deploy the live UZ Voice-in/STT routing fix, re-run the live Telegram UZ sent-code voice smoke, then continue full live Telegram QA matrix / UX polish.</x:v>
+        <x:v>Next queue item: re-run live Telegram UZ sent-code voice note against production, then polish short negated-code Voice-in UX and continue the full live Telegram QA matrix.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: TG-014 live RU/UZ Voice-in/STT QA on 2026-07-04 found UZ `Men SMS kodni yubardim` fell through to not-enough-data. Code now tolerates provider `yubardim/yubordim` variants and committed sanitized live replay rows for UZ sent-code and RU negated-code transcripts. RU negated-code avoids SOS but still deserves warmer conversational UX polish.</x:v>
+        <x:v>Owner note: TG-014 live UZ sent-code Voice-in/STT routing fix d9fe6f2 was deployed on 2026-07-04. Production smoke and security smoke passed with public URL/header checks. Remaining live proof is one post-deploy UZ voice note through the real Telegram bot; RU negated-code avoids SOS but still deserves warmer conversational UX polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3970,7 +3970,7 @@
         <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized and live Telegram transcript capture.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; provider-sanitized EN active-call/negated-code and live RU negated-code rows are in replay corpus. Next: deploy and re-run live UZ voice smoke; polish short negated-code voice UX.</x:v>
+        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; d9fe6f2 deployed and production smoke/security smoke passed. Provider-sanitized EN active-call/negated-code and live RU negated-code rows are in replay corpus. Next: post-deploy live UZ voice retest; polish short negated-code voice UX.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -8934,13 +8934,13 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered; provider-sanitized EN and live RU negated-code rows are committed. Short negated-code voice UX remains polish.</x:v>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered and deployed; provider-sanitized EN and live RU negated-code rows are committed. Short negated-code voice UX remains polish.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Passed 2026-07-04: focused voice handler + collector tests 2 files / 24 tests; full Telegram suite 50 files / 1371 tests; scoped eslint passed. Live Telegram observation showed UZ sent-code now has a regression fixture.</x:v>
+        <x:v>Passed 2026-07-04: focused voice handler + collector tests 2 files / 24 tests; full Telegram suite 50 files / 1371 tests; scoped eslint passed; railway deploy, prod:smoke and prod:security-smoke with public URL passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
@@ -13162,6 +13162,32 @@
         <x:v>Next: deploy this fix and re-run live UZ sent-code voice smoke; then address short negated-code voice UX copy and continue live Telegram QA matrix.</x:v>
       </x:c>
     </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>QA-2026-07-04-007</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>2026-07-04</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>TG-014 live UZ Voice-in/STT fix deployment proof</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>railway up --ci; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:security-smoke -- https://scam-guard-main-production.up.railway.app</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Passed: deploy complete; production smoke passed (home, healthz, webhook secret, Telegram webhook pending=0, AI provider 200); production security smoke passed with public header checks and Supabase/RLS checks.</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>TG-014, production deploy, security smoke</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>Commit d9fe6f2 deployed. Initial prod:smoke without URL failed closed as expected, then passed with the production URL. Security smoke first passed Supabase checks and then passed again with public header checks.</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>Next: re-run the live Telegram UZ sent-code voice note against production; then polish the short negated-code voice UX and continue full live Telegram QA matrix.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): guard negated Uzbek voice code transcript
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2e5d020070d74f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rfb9556ce6b4e4205"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R2f70b6c082344755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra5758b2253e94b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R799836a4b9c943b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rd0a99a8874ca462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1ea5c7c674ef41e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R573e9e8739ee42ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Re7e54c4e58494921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rdd3b99e67505469b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R62f0ef1d19944b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3bcdc820622f4a04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2694,7 +2694,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
-        <x:v>2026-07-04</x:v>
+        <x:v>2026-07-05</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
         <x:v>68</x:v>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: re-run live Telegram UZ sent-code voice note against production, then polish short negated-code Voice-in UX and continue the full live Telegram QA matrix.</x:v>
+        <x:v>Next queue item: deploy the live UZ negated-code Voice-in fix, re-run both Telegram voice notes against production, then continue short negated-code Voice-in UX polish and the full live Telegram QA matrix.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: TG-014 live UZ sent-code Voice-in/STT routing fix d9fe6f2 was deployed on 2026-07-04. Production smoke and security smoke passed with public URL/header checks. Remaining live proof is one post-deploy UZ voice note through the real Telegram bot; RU negated-code avoids SOS but still deserves warmer conversational UX polish.</x:v>
+        <x:v>Owner note: 2026-07-05 live Telegram QA found a false SOS for provider transcript `Men SMS-kod yubormadim.` after the positive `Men SMS-kod yubordim` case. Local fix adds punctuation-aware UZ negation and guards SMS positive verbs against `-ma` negation; focused voice test, scoped eslint and full Telegram suite passed before deploy.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3970,7 +3970,7 @@
         <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized and live Telegram transcript capture.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; d9fe6f2 deployed and production smoke/security smoke passed. Provider-sanitized EN active-call/negated-code and live RU negated-code rows are in replay corpus. Next: post-deploy live UZ voice retest; polish short negated-code voice UX.</x:v>
+        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; d9fe6f2 deployed and production smoke/security smoke passed. 2026-07-05 live Telegram retest found negated UZ `Men SMS-kod yubormadim.` falsely routed to SOS; local fix added replay coverage and negation guards. Next: deploy and re-run both live voice notes, then polish short negated-code voice UX.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -3978,7 +3978,7 @@
         </x:is>
       </x:c>
       <x:c r="L15" s="8" t="str">
-        <x:v>No raw audio or Telegram file IDs committed; replay corpus stores sanitized transcripts only. Negated first-person phrases remain guarded against false SOS.</x:v>
+        <x:v>No raw audio or Telegram file IDs committed; replay corpus stores sanitized transcripts only. Negated first-person phrases, including live `Men SMS-kod yubormadim.`, remain guarded against false SOS.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -8934,13 +8934,13 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered and deployed; provider-sanitized EN and live RU negated-code rows are committed. Short negated-code voice UX remains polish.</x:v>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered and deployed. 2026-07-05 live negated UZ `Men SMS-kod yubormadim.` false SOS fixed locally; deploy and live retest are next. Short negated-code voice UX remains polish.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Passed 2026-07-04: focused voice handler + collector tests 2 files / 24 tests; full Telegram suite 50 files / 1371 tests; scoped eslint passed; railway deploy, prod:smoke and prod:security-smoke with public URL passed.</x:v>
+        <x:v>Passed 2026-07-05 locally: check.voice.test.ts 18/18, scoped eslint passed, full Telegram suite 50 files / 1371 tests. Pending: Railway deploy and live two-voice retest in Telegram production.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">

</xml_diff>

<commit_message>
docs(tracker): record negated voice fix deployment
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R1ea5c7c674ef41e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R573e9e8739ee42ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Re7e54c4e58494921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rdd3b99e67505469b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R62f0ef1d19944b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3bcdc820622f4a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd98a924fd6334b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R86d467409b234d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ra931167e870d44cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9d55aa10d4dd49a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R647375638b6644f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8724e6f219d24758"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: deploy the live UZ negated-code Voice-in fix, re-run both Telegram voice notes against production, then continue short negated-code Voice-in UX polish and the full live Telegram QA matrix.</x:v>
+        <x:v>Next queue item: re-run both live Telegram UZ voice notes against production, then continue short negated-code Voice-in UX polish and the full live Telegram QA matrix.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: 2026-07-05 live Telegram QA found a false SOS for provider transcript `Men SMS-kod yubormadim.` after the positive `Men SMS-kod yubordim` case. Local fix adds punctuation-aware UZ negation and guards SMS positive verbs against `-ma` negation; focused voice test, scoped eslint and full Telegram suite passed before deploy.</x:v>
+        <x:v>Owner note: 2026-07-05 live Telegram QA found a false SOS for provider transcript `Men SMS-kod yubormadim.` after the positive sent-code case. Fix a5120cb adds punctuation-aware UZ negation and guards SMS positive verbs against `-ma` negation; deployed to Railway, prod:smoke and prod:security-smoke passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3970,7 +3970,7 @@
         <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized and live Telegram transcript capture.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; d9fe6f2 deployed and production smoke/security smoke passed. 2026-07-05 live Telegram retest found negated UZ `Men SMS-kod yubormadim.` falsely routed to SOS; local fix added replay coverage and negation guards. Next: deploy and re-run both live voice notes, then polish short negated-code voice UX.</x:v>
+        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; d9fe6f2 deployed and production smoke/security smoke passed. 2026-07-05 live Telegram retest found negated UZ `Men SMS-kod yubormadim.` falsely routed to SOS; a5120cb fixed it, deployed to Railway, and prod smoke/security smoke passed. Next: re-run both live voice notes, then polish short negated-code voice UX.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -8934,13 +8934,13 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered and deployed. 2026-07-05 live negated UZ `Men SMS-kod yubormadim.` false SOS fixed locally; deploy and live retest are next. Short negated-code voice UX remains polish.</x:v>
+        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered and deployed. 2026-07-05 live negated UZ `Men SMS-kod yubormadim.` false SOS fixed by a5120cb and deployed. Short negated-code voice UX remains polish.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Passed 2026-07-05 locally: check.voice.test.ts 18/18, scoped eslint passed, full Telegram suite 50 files / 1371 tests. Pending: Railway deploy and live two-voice retest in Telegram production.</x:v>
+        <x:v>Passed 2026-07-05: check.voice.test.ts 18/18, scoped eslint, full Telegram suite 50 files / 1371 tests, railway deploy, prod:smoke and prod:security-smoke. Pending: live two-voice retest in Telegram production.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">

</xml_diff>

<commit_message>
fix(telegram): acknowledge negated voice code phrases
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rd98a924fd6334b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R86d467409b234d20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ra931167e870d44cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9d55aa10d4dd49a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R647375638b6644f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8724e6f219d24758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R40565a546f0d43cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R6939693ef1fc44a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R53c98ad115d74793"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R88d678ddf3b8463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rbb95de51dee04eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R565b6264c25c4dc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: re-run both live Telegram UZ voice notes against production, then continue short negated-code Voice-in UX polish and the full live Telegram QA matrix.</x:v>
+        <x:v>Next queue item: deploy the negated Voice-in acknowledgement UX fix, re-run `Men esa SMS-kod yubormadim.` in live Telegram, then continue the full live Telegram QA matrix.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: 2026-07-05 live Telegram QA found a false SOS for provider transcript `Men SMS-kod yubormadim.` after the positive sent-code case. Fix a5120cb adds punctuation-aware UZ negation and guards SMS positive verbs against `-ma` negation; deployed to Railway, prod:smoke and prod:security-smoke passed.</x:v>
+        <x:v>Owner note: 2026-07-05 live Telegram QA confirmed the false SOS was fixed, but `Men esa SMS-kod yubormadim.` still produced generic insufficient-data. Local fix adds a dedicated negated Voice-in acknowledgement before runCheck, with replay fixture `uz-live-not-sent-code-telegram-002`; focused voice, i18n, full Telegram suite and scoped eslint passed locally.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -3970,7 +3970,7 @@
         <x:v>Unit/integration tests + live QA + RU/UZ/EN provider-like STT corpus regression + UZ Cyrillic replay fixtures + 2026-07-04 provider-sanitized and live Telegram transcript capture.</x:v>
       </x:c>
       <x:c r="J15" s="8" t="str">
-        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` now route to SMS-code SOS; d9fe6f2 deployed and production smoke/security smoke passed. 2026-07-05 live Telegram retest found negated UZ `Men SMS-kod yubormadim.` falsely routed to SOS; a5120cb fixed it, deployed to Railway, and prod smoke/security smoke passed. Next: re-run both live voice notes, then polish short negated-code voice UX.</x:v>
+        <x:v>Closed 2026-07-04: UZ Cyrillic and live UZ `Men SMS kodni yubardim` route to SMS-code SOS; d9fe6f2 deployed. 2026-07-05: false SOS for negated UZ `Men SMS-kod yubormadim.` fixed/deployed via a5120cb. Follow-up live phrase `Men esa SMS-kod yubormadim.` no longer SOS but returned insufficient-data; local UX fix now routes negated already-done voice transcripts to a calm acknowledgement before runCheck. Next: deploy and live retest.</x:v>
       </x:c>
       <x:c r="K15" s="12" t="inlineStr">
         <x:is>
@@ -3978,7 +3978,7 @@
         </x:is>
       </x:c>
       <x:c r="L15" s="8" t="str">
-        <x:v>No raw audio or Telegram file IDs committed; replay corpus stores sanitized transcripts only. Negated first-person phrases, including live `Men SMS-kod yubormadim.`, remain guarded against false SOS.</x:v>
+        <x:v>No raw audio or Telegram file IDs committed; replay corpus stores sanitized transcripts only. Negated first-person phrases, including live `Men esa SMS-kod yubormadim.`, use `negated_ack` and stay out of false SOS/generic insufficient-data.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -8934,13 +8934,13 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="50" t="str">
-        <x:v>Closed 2026-07-04 slice: UZ Cyrillic STT replay gap and live UZ `SMS kodni yubardim` provider variant are covered and deployed. 2026-07-05 live negated UZ `Men SMS-kod yubormadim.` false SOS fixed by a5120cb and deployed. Short negated-code voice UX remains polish.</x:v>
+        <x:v>2026-07-05 local slice: negated Voice-in acknowledgement UX added for short transcripts such as `Men esa SMS-kod yubormadim.`; this closes the generic insufficient-data response after false SOS was already fixed. Deploy/live retest pending.</x:v>
       </x:c>
       <x:c r="F11" s="566" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G11" s="50" t="str">
-        <x:v>Passed 2026-07-05: check.voice.test.ts 18/18, scoped eslint, full Telegram suite 50 files / 1371 tests, railway deploy, prod:smoke and prod:security-smoke. Pending: live two-voice retest in Telegram production.</x:v>
+        <x:v>Passed 2026-07-05 locally: check.voice.test.ts 18/18, i18n completeness 660/660, full Telegram suite 50 files / 1374 tests, scoped eslint. Pending: Railway deploy, prod smoke/security smoke, live Telegram retest.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">

</xml_diff>

<commit_message>
docs: update QA tracker after telegram hardening
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R40565a546f0d43cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R6939693ef1fc44a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R53c98ad115d74793"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R88d678ddf3b8463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rbb95de51dee04eff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R565b6264c25c4dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R285698870cc14979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb88ddbf4861b4cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R10fedc5267604a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2323f4b4951c4872"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb449772079af4906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rce7b0ed5b3494fdb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2694,7 +2694,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
-        <x:v>2026-07-05</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
         <x:v>68</x:v>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: deploy the negated Voice-in acknowledgement UX fix, re-run `Men esa SMS-kod yubormadim.` in live Telegram, then continue the full live Telegram QA matrix.</x:v>
+        <x:v>Next queue item: finish live Telegram QA residue: manual inline UI card verification in Telegram Web/mobile, broader RU/UZ direct/inline phrase sweep, then photo/screenshot and P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: 2026-07-05 live Telegram QA confirmed the false SOS was fixed, but `Men esa SMS-kod yubormadim.` still produced generic insufficient-data. Local fix adds a dedicated negated Voice-in acknowledgement before runCheck, with replay fixture `uz-live-not-sent-code-telegram-002`; focused voice, i18n, full Telegram suite and scoped eslint passed locally.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployment 7a93ecb2 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps; prod Telegram inline smoke passed. Open: live Telegram client inline preview did not surface in the current Web session although backend inline smoke passes; general prod AI smoke still needs separate provider-config review after Gemini 403.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2759,7 +2759,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="8" t="inlineStr">
         <x:is>
@@ -2776,7 +2776,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="8" t="inlineStr">
         <x:is>
@@ -6936,19 +6936,19 @@
         <x:v>User feedback 2026-07-02 live bot QA request</x:v>
       </x:c>
       <x:c r="H68" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="I68" t="str">
-        <x:v>Needs new matrix rows</x:v>
+        <x:v>Harness/live Telegram phrase matrix + production inline smoke + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J68" t="str">
-        <x:v>Covers RU/UZ/EN free text, screenshots, profile images, QR, voice, follow-ups, panic, report and Family Shield.</x:v>
+        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="K68" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L68" t="str">
-        <x:v>Live QA must use sanitized examples and avoid sending secrets or raw victim data to moderator channels.</x:v>
+        <x:v>Keep sanitized examples only; do not send secrets, raw victim data, cards, codes, screenshots with private details, or full scammer identifiers into shared chats.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
@@ -10573,6 +10573,32 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>ERR-2026-07-08-001</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Live Telegram Web inline QA</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>TG-002, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Inline preview card did not surface in the current Telegram Web UI session, while backend synthetic inline webhook smoke passed.</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>The backend can be correct while the real client UX still blocks discovery; users may think inline mode is broken or silent.</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>2026-07-08: prod:telegram-inline-smoke passed after Railway deployment 7a93ecb2; manual Telegram Web tab did not show inline result cards reliably. Needs mobile/Web client retest before closing.</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Open - manual client verification needed</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13188,6 +13214,32 @@
         <x:v>Next: re-run the live Telegram UZ sent-code voice note against production; then polish the short negated-code voice UX and continue full live Telegram QA matrix.</x:v>
       </x:c>
     </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>QA-2026-07-08-001</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>2026-07-08</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Telegram live-phrase/inline/cache hardening continuation</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>npm run test:run -- src/lib/telegram; npm run test:run -- inline/check.cache focused suite; npx eslint touched files; railway up --detach; railway run npm run prod:telegram-inline-smoke</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>Passed: focused suite 114 tests; full Telegram suite 53 files / 1828 tests; Railway deployment 7a93ecb2 SUCCESS; production inline smoke passed</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>TG-002, TG-010, TG-014, P1-2026-07-02-003, ROAD-003</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>Commits: 5d399f0 live phrase corpus, 37d67f2 inline preflight priorities, de43976 bounded check/voice/OCR caches. Open live UI note tracked as ERR-2026-07-08-001.</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>Continue manual live Telegram direct/inline QA, especially client inline preview, UZ voice spot-checks and photo/screenshot triage; then resume P1 web/Telegram flows.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record live inline retest
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R285698870cc14979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb88ddbf4861b4cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R10fedc5267604a15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2323f4b4951c4872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb449772079af4906"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rce7b0ed5b3494fdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc6008acfb4c04989"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R5d3e80c3d8254033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1debfbfcaa804d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbe4d29d35d1443d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R439fff0aa0494b8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0227bc093fdf4774"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: finish live Telegram QA residue: manual inline UI card verification in Telegram Web/mobile, broader RU/UZ direct/inline phrase sweep, then photo/screenshot and P1 web/Telegram flows.</x:v>
+        <x:v>Next queue item: finish live Telegram QA residue: broader RU/UZ direct phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployment 7a93ecb2 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps; prod Telegram inline smoke passed. Open: live Telegram client inline preview did not surface in the current Web session although backend inline smoke passes; general prod AI smoke still needs separate provider-config review after Gemini 403.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2 plus 3f3a0730 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; prod Telegram inline smoke passed and Telegram Web live inline retest passed. General prod AI smoke still needs separate provider-config review after Gemini 403.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10590,13 +10590,13 @@
         <x:v>The backend can be correct while the real client UX still blocks discovery; users may think inline mode is broken or silent.</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>2026-07-08: prod:telegram-inline-smoke passed after Railway deployment 7a93ecb2; manual Telegram Web tab did not show inline result cards reliably. Needs mobile/Web client retest before closing.</x:v>
+        <x:v>2026-07-08 update: prod:telegram-inline-smoke passed after Railway deployments 7a93ecb2 and 3f3a0730; manual Telegram Web live inline retest passed for 20+ news/user phrases. Specific retest after ed9d651: Uztelecom code call -&gt; operator card; known-contact urgent money -&gt; loved-one distress card.</x:v>
       </x:c>
       <x:c r="G10" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>Open - manual client verification needed</x:v>
+        <x:v>Closed - verified in Telegram Web; keep mobile spot-check in routine QA</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13240,6 +13240,32 @@
         <x:v>Continue manual live Telegram direct/inline QA, especially client inline preview, UZ voice spot-checks and photo/screenshot triage; then resume P1 web/Telegram flows.</x:v>
       </x:c>
     </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>QA-2026-07-08-002</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>2026-07-08</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Telegram live inline client retest after priority tuning</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/handlers/inline.test.ts src/lib/telegram/inline.mass.test.ts; npx eslint touched inline files; npm run test:run -- src/lib/telegram; railway up --detach; railway run npm run prod:telegram-inline-smoke; manual Telegram Web inline retest</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>Passed: focused inline 110 tests; full Telegram 53 files / 1830 tests; Railway deployment 3f3a0730 SUCCESS; prod inline smoke passed; Telegram Web inline cards passed for Uztelecom code call and known-contact urgent money retest</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>TG-002, TG-010, TG-014, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>Commit ed9d651 sharpened inline priority so operator-with-code is not collapsed into generic code copy and known-contact urgent loan requests use loved-one distress copy instead of romance copy. Manual live inline sweep covered 20+ current UZ/news phrases with no cold-card regression.</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>Next: direct bot live sweep for short RU/UZ phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram report/appeal/admin flows.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record direct received-code QA fix
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc6008acfb4c04989"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R5d3e80c3d8254033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1debfbfcaa804d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbe4d29d35d1443d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R439fff0aa0494b8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0227bc093fdf4774"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R953f0e27455c42bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra3862f928280485a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6e8442abde7445b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf26edb9a2ed24b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R90717d5bc49847ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R07d556ab03cd4594"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: finish live Telegram QA residue: broader RU/UZ direct phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
+        <x:v>Next queue item: finish live Telegram QA residue: UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2 plus 3f3a0730 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; prod Telegram inline smoke passed and Telegram Web live inline retest passed. General prod AI smoke still needs separate provider-config review after Gemini 403.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10599,6 +10599,32 @@
         <x:v>Closed - verified in Telegram Web; keep mobile spot-check in routine QA</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>ERR-2026-07-08-002</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Direct Telegram phrase QA harness</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>TG-002, TG-014, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Short victim phrase 'mne prishel kakoy-to kod / why did I get a code' fell through to the generic risk pipeline instead of giving code safety guidance.</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Users who receive an unexpected SMS/OTP may not know whether they initiated it; a cold or generic response loses the key safety moment.</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Fixed 2026-07-08: classifyVictimIntent now treats received-code confusion in RU/UZ/EN as code_request. Regression rows added to LIVE_PHRASE_CASES. Tests: focused 353 passed, full Telegram 53 files / 1833 tests passed, prod inline smoke passed, prod live QA smoke passed. Railway deployment c6f377e4 SUCCESS.</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Closed - fixed and deployed 2026-07-08</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13266,6 +13292,32 @@
         <x:v>Next: direct bot live sweep for short RU/UZ phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram report/appeal/admin flows.</x:v>
       </x:c>
     </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>QA-2026-07-08-003</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>2026-07-08</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Telegram direct short received-code phrase fix</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Temporary direct QA harness over 20 human phrases; npm run test:run -- src/lib/telegram/victim-intent.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts; npx eslint touched files; npm run test:run -- src/lib/telegram; railway up --detach; railway run npm run prod:telegram-inline-smoke; railway run npm run prod:telegram-live-qa-smoke</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>Passed: direct QA table found one gap and retest passed; focused 353 tests; full Telegram 53 files / 1833 tests; Railway deployment c6f377e4 SUCCESS; prod inline smoke passed; prod live QA smoke passed</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>TG-002, TG-014, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>Commit c22ae64 added RU/UZ/EN received-code confusion handling so 'mne prishel kod / why did I get a code?' routes to code safety guidance instead of generic risk pipeline.</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>Next: resume live Telegram QA with UZ voice spot-checks and photo/screenshot triage; then P1 web/Telegram report, appeal/admin, private/group scoping flows.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): smooth inline follow-up QA residue
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R953f0e27455c42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra3862f928280485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R6e8442abde7445b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf26edb9a2ed24b99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R90717d5bc49847ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R07d556ab03cd4594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7ba4332114bf4376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf50d6695d5764ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae8f963507ed4aec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R98f37f65968d4f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ref1c19110af54768"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R32e9d78ec3524e52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: finish live Telegram QA residue: UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6942,7 +6942,7 @@
         <x:v>Harness/live Telegram phrase matrix + production inline smoke + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J68" t="str">
-        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
+        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows. Inline/direct residue fixed 2026-07-08: already-supplied link/text cards no longer ask again, newline inline phrases route correctly, sibling/grandchild urgent-money phrases map to relative distress, and specific why-followups answer from lastCheck.</x:v>
       </x:c>
       <x:c r="K68" t="str">
         <x:v>P1</x:v>
@@ -10625,6 +10625,32 @@
         <x:v>Closed - fixed and deployed 2026-07-08</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>ERR-2026-07-08-003</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Live Telegram inline/direct QA</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>TG-002, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Inline cards kept asking for a link/full text after the user had already supplied it; newline-separated inline phrases could miss relative/code intent; specific why-followups about a suspicious domain fell back to a new insufficient-data check.</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Users experience the bot as stuck or cold exactly while trying to clarify a suspicious URL, admin-channel SMS request, or urgent relative money request.</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Fixed 2026-07-08: inline preview copy no longer repeats 'send the link/text' as a hard requirement, classifyHumanInlineIntent normalizes whitespace, sister/brother/grandchild terms were added to relative-distress news matching, and EXPLAIN_RE accepts specific why-questions. Tests: inline + followup focused suite 351/351; full src/lib/telegram 1839/1839; scoped eslint clean.</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Closed - fixed in current worktree; deploy pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record inline follow-up QA deploy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7ba4332114bf4376"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf50d6695d5764ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae8f963507ed4aec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R98f37f65968d4f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ref1c19110af54768"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R32e9d78ec3524e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rbc61f97cc25e44e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R014a155c6d2e409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3609e79f66894141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R8d5caa642c2940cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb74cb982ce2e46fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R20e477750c284e65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: finish live Telegram QA residue: UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6942,7 +6942,7 @@
         <x:v>Harness/live Telegram phrase matrix + production inline smoke + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J68" t="str">
-        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows. Inline/direct residue fixed 2026-07-08: already-supplied link/text cards no longer ask again, newline inline phrases route correctly, sibling/grandchild urgent-money phrases map to relative distress, and specific why-followups answer from lastCheck.</x:v>
+        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows. Inline/direct residue fixed 2026-07-08: already-supplied link/text cards no longer ask again, newline inline phrases route correctly, sibling/grandchild urgent-money phrases map to relative distress, and specific why-followups answer from lastCheck. Fixed in 9d80906 and deployed to Railway (1fe2a51e) on 2026-07-08. Prod inline and live QA smokes passed.</x:v>
       </x:c>
       <x:c r="K68" t="str">
         <x:v>P1</x:v>
@@ -10642,13 +10642,13 @@
         <x:v>Users experience the bot as stuck or cold exactly while trying to clarify a suspicious URL, admin-channel SMS request, or urgent relative money request.</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>Fixed 2026-07-08: inline preview copy no longer repeats 'send the link/text' as a hard requirement, classifyHumanInlineIntent normalizes whitespace, sister/brother/grandchild terms were added to relative-distress news matching, and EXPLAIN_RE accepts specific why-questions. Tests: inline + followup focused suite 351/351; full src/lib/telegram 1839/1839; scoped eslint clean.</x:v>
+        <x:v>Fixed 2026-07-08: inline preview copy no longer repeats 'send the link/text' as a hard requirement, classifyHumanInlineIntent normalizes whitespace, sister/brother/grandchild terms were added to relative-distress news matching, and EXPLAIN_RE accepts specific why-questions. Tests: inline + followup focused suite 351/351; full src/lib/telegram 1839/1839; scoped eslint clean. Fixed in 9d80906 and deployed to Railway (1fe2a51e) on 2026-07-08. Prod inline and live QA smokes passed.</x:v>
       </x:c>
       <x:c r="G12" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>Closed - fixed in current worktree; deploy pending</x:v>
+        <x:v>Closed - fixed and deployed 2026-07-08</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record relative distress live-call QA fix
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rbc61f97cc25e44e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R014a155c6d2e409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3609e79f66894141"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R8d5caa642c2940cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb74cb982ce2e46fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R20e477750c284e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R88fb47650f7a498c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R75e046eb1a434603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd26d4ac6d7254d48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Reb4881110b2842c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rfd45f0e7529c40ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf0edf25bb0a64e01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: finish live Telegram QA residue: UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed. Relative live-call family-copy fix deployed 2026-07-08 (dcf09ce / Railway a260c099): urgent sister/relative money calls now route to saved-number + codeword identity verification instead of generic organization/bank wording.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10651,6 +10651,32 @@
         <x:v>Closed - fixed and deployed 2026-07-08</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="69" customHeight="1">
+      <x:c r="A13" s="595" t="str">
+        <x:v>ERR-2026-07-08-004</x:v>
+      </x:c>
+      <x:c r="B13" s="595" t="str">
+        <x:v>Live Telegram direct QA</x:v>
+      </x:c>
+      <x:c r="C13" s="595" t="str">
+        <x:v>TG-002, TG-014, ROAD-006, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="D13" s="595" t="str">
+        <x:v>Relative distress calls such as 'sister urgently asks to transfer money because of car trouble' routed to live-call SOS, but used generic bank/organization callback wording.</x:v>
+      </x:c>
+      <x:c r="E13" s="595" t="str">
+        <x:v>For voice-clone and hacked-relative scams, the safe action is identity verification through a saved contact and family codeword, not an official organization callback.</x:v>
+      </x:c>
+      <x:c r="F13" s="595" t="str">
+        <x:v>Fixed 2026-07-08: classifyLiveCallContext now detects relative/loved-one money/code distress; Emergency Copilot uses family-specific RU/UZ/EN copy, saved-number callback, codeword/private-question guidance, and relative follow-up text. Tests: full src/lib/telegram 53 files / 1842 passed; prod Telegram live QA smoke passed after Railway deployment a260c099.</x:v>
+      </x:c>
+      <x:c r="G13" s="595" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H13" s="595" t="str">
+        <x:v>Closed - fixed and deployed 2026-07-08</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record relative full-plan button QA fix
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R88fb47650f7a498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R75e046eb1a434603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd26d4ac6d7254d48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Reb4881110b2842c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rfd45f0e7529c40ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf0edf25bb0a64e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rda817e77f398404f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc59326e927134558"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R62d388fffe3f499f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc8a56d1b3b384e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R35dbdf11d05343b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R9213e08ea63447ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: finish live Telegram QA residue: UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed. Relative live-call family-copy fix deployed 2026-07-08 (dcf09ce / Railway a260c099): urgent sister/relative money calls now route to saved-number + codeword identity verification instead of generic organization/bank wording.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed. Relative live-call family-copy fix deployed 2026-07-08 (dcf09ce / Railway a260c099): urgent sister/relative money calls now route to saved-number + codeword identity verification instead of generic organization/bank wording. Relative full-plan button residue fixed and live-verified 2026-07-08 (49f11d9 / Railway 5471ebd0): 'All urgent steps' now keeps the family verification plan.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10651,7 +10651,7 @@
         <x:v>Closed - fixed and deployed 2026-07-08</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="69" customHeight="1">
+    <x:row r="13" ht="88.5" customHeight="1">
       <x:c r="A13" s="595" t="str">
         <x:v>ERR-2026-07-08-004</x:v>
       </x:c>
@@ -10668,7 +10668,7 @@
         <x:v>For voice-clone and hacked-relative scams, the safe action is identity verification through a saved contact and family codeword, not an official organization callback.</x:v>
       </x:c>
       <x:c r="F13" s="595" t="str">
-        <x:v>Fixed 2026-07-08: classifyLiveCallContext now detects relative/loved-one money/code distress; Emergency Copilot uses family-specific RU/UZ/EN copy, saved-number callback, codeword/private-question guidance, and relative follow-up text. Tests: full src/lib/telegram 53 files / 1842 passed; prod Telegram live QA smoke passed after Railway deployment a260c099.</x:v>
+        <x:v>Fixed 2026-07-08: classifyLiveCallContext now detects relative/loved-one money/code distress; Emergency Copilot uses family-specific RU/UZ/EN copy, saved-number callback, codeword/private-question guidance, and relative follow-up text. Tests: full src/lib/telegram 53 files / 1842 passed; prod Telegram live QA smoke passed after Railway deployment a260c099. Follow-up live QA found the 'All urgent steps' button still used the generic bank/organization full checklist; fixed in 49f11d9 by adding a relative-specific full plan. Live Telegram retest after Railway deployment 5471ebd0 confirmed the button now says to end the call, callback via saved contact, ask the family codeword/private question, and only call the bank if money/code/card data was already sent.</x:v>
       </x:c>
       <x:c r="G13" s="595" t="str">
         <x:v>P1</x:v>

</xml_diff>

<commit_message>
docs: record Uzbek voice routing QA fix
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rda817e77f398404f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc59326e927134558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R62d388fffe3f499f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc8a56d1b3b384e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R35dbdf11d05343b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R9213e08ea63447ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdfe6d4da84354883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1cf1af2ae6484d06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R495c4bbf6061481b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc18a3a2830f842ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R16f5b95e71694f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R05ad1ccf02184957"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2697,16 +2697,16 @@
         <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: finish live Telegram QA residue: UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
+        <x:v>Next queue item: finish live Telegram QA residue: optional real-audio UZ voice spot-check if STT budget allows, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed. Relative live-call family-copy fix deployed 2026-07-08 (dcf09ce / Railway a260c099): urgent sister/relative money calls now route to saved-number + codeword identity verification instead of generic organization/bank wording. Relative full-plan button residue fixed and live-verified 2026-07-08 (49f11d9 / Railway 5471ebd0): 'All urgent steps' now keeps the family verification plan.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed. Relative live-call family-copy fix deployed 2026-07-08 (dcf09ce / Railway a260c099): urgent sister/relative money calls now route to saved-number + codeword identity verification instead of generic organization/bank wording. Relative full-plan button residue fixed and live-verified 2026-07-08 (49f11d9 / Railway 5471ebd0): 'All urgent steps' now keeps the family verification plan. UZ voice short live-call wording fixed 2026-07-08 (237adab): qo'ng'iroq/telefon qildi for akam urgent money, Beeline operator, and Soliq SMS-code calls now route to live-call SOS with correct context; full Telegram suite passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2742,7 +2742,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -6942,7 +6942,7 @@
         <x:v>Harness/live Telegram phrase matrix + production inline smoke + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J68" t="str">
-        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows. Inline/direct residue fixed 2026-07-08: already-supplied link/text cards no longer ask again, newline inline phrases route correctly, sibling/grandchild urgent-money phrases map to relative distress, and specific why-followups answer from lastCheck. Fixed in 9d80906 and deployed to Railway (1fe2a51e) on 2026-07-08. Prod inline and live QA smokes passed.</x:v>
+        <x:v>2026-07-08 update: broad live-phrase corpus now covers user feedback and 49+ news-derived UZ schemes across direct and inline paths; focused inline matrix passed, full Telegram suite passed, and cache hardening was deployed. Remaining work: manual Telegram client inline UI verification, 15-20 more live direct/inline phrases, UZ voice spot-checks, photo/screenshot triage, then P1 web/Telegram flows. Inline/direct residue fixed 2026-07-08: already-supplied link/text cards no longer ask again, newline inline phrases route correctly, sibling/grandchild urgent-money phrases map to relative distress, and specific why-followups answer from lastCheck. Fixed in 9d80906 and deployed to Railway (1fe2a51e) on 2026-07-08. Prod inline and live QA smokes passed. UZ voice code-regression slice fixed 2026-07-08 in 237adab: short qo'ng'iroq/telefon qildi phrases for relative distress, operator/SIM blocking, and Soliq SMS-code calls now route to live-call SOS with the correct context. Remaining work: optional real-audio Telegram spot-check if STT budget allows, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="K68" t="str">
         <x:v>P1</x:v>
@@ -6987,6 +6987,44 @@
       </x:c>
       <x:c r="L69" t="str">
         <x:v>Alert must not include scammer number, codes, links, screenshots, card data or raw check evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>P1-2026-07-08-004</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>Telegram QA / Uzbek voice</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>Short UZ live-call voice routing</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>As a Uzbek-speaking user who sends a short voice note about a caller from family, operator, or Soliq, I want the bot to open the right SOS plan instead of a generic risk check.</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Short UZ STT transcripts with qo'ng'iroq/telefon qildi plus relative, operator, or government cues route to panic scenario 6 and preserve live-call context.</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>src/lib/telegram/handlers/check.ts; src/lib/telegram/handlers/check.voice.test.ts; src/lib/telegram/voice-stt-provider-fixtures.ts</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>User feedback 2026-07-08 UZ voice QA; live Telegram screenshots</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>Full Telegram regression suite + focused UZ voice STT replay tests</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>Closed 2026-07-08 in 237adab: added qildi/qilgan/qilmoqda/telefon wording and replay fixtures for akam urgent money, Beeline operator, and Soliq SMS-code calls; src/lib/telegram suite passed (1840 tests).</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L70" t="str">
+        <x:v>Optional real-audio Telegram spot-check remains if STT daily budget is available; do not store raw audio or private transcripts.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record long Uzbek voice QA fix
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdfe6d4da84354883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1cf1af2ae6484d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R495c4bbf6061481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc18a3a2830f842ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R16f5b95e71694f32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R05ad1ccf02184957"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdf5c71f6845b48d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rac057ac51b0248de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3397ecf7a20047b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2df3f36ffa64437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc92715617750432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf73b161a65404c7e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2694,19 +2694,19 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="str">
-        <x:v>2026-07-08</x:v>
+        <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: finish live Telegram QA residue: optional real-audio UZ voice spot-check if STT budget allows, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
+        <x:v>Next queue item: finish live Telegram QA residue after the STT limit resets: real-audio UZ spot-check for long family/channel-admin phrases, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage, inline preflight priorities were tightened, Uzbek voice regression suites passed, image/QR/webhook suites passed, and Railway deployments 7a93ecb2, 3f3a0730, and c6f377e4 succeeded. Cache hardening commit de43976 bounds Telegram check/voice/OCR in-memory maps. Inline priority commit ed9d651 fixed live client copy for Uztelecom code calls and known-contact urgent money requests; direct received-code commit c22ae64 fixed short 'code arrived, why?' victim phrases. Prod inline and live QA smokes passed. General prod AI smoke still needs separate provider-config review after Gemini 403. Inline/direct residue ERR-2026-07-08-003 fixed in current worktree: no repeated send-link/text prompt after supplied details, newline inline normalization, expanded relative distress family terms, and last-check why-followups. Inline/direct QA residue closed and deployed (1fe2a51e); prod Telegram inline/live smokes passed. Relative live-call family-copy fix deployed 2026-07-08 (dcf09ce / Railway a260c099): urgent sister/relative money calls now route to saved-number + codeword identity verification instead of generic organization/bank wording. Relative full-plan button residue fixed and live-verified 2026-07-08 (49f11d9 / Railway 5471ebd0): 'All urgent steps' now keeps the family verification plan. UZ voice short live-call wording fixed 2026-07-08 (237adab): qo'ng'iroq/telefon qildi for akam urgent money, Beeline operator, and Soliq SMS-code calls now route to live-call SOS with correct context; full Telegram suite passed.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. Inline/direct residue was closed and deployed; relative live-call family copy and full-plan residue were fixed; short UZ voice routing was fixed 2026-07-08. Long UZ voice requested-action routing fixed 2026-07-09 in 4bba35c and deployed via Railway b156f8a8: STT timeout is 12s, prompt vocabulary covers singlim/kanal administratori/SMS kodini/pul o'tkazishimni so'rayapti, requested-action forms no longer route as already-completed emergencies, and Telegram/risk regression suites plus prod Telegram smokes passed. Optional real-audio Telegram spot-check remains after the user's STT daily limit resets.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7027,6 +7027,44 @@
         <x:v>Optional real-audio Telegram spot-check remains if STT daily budget is available; do not store raw audio or private transcripts.</x:v>
       </x:c>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>P1-2026-07-09-001</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>Telegram QA / Uzbek voice</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>Long UZ voice STT and requested-action routing</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>As a Uzbek-speaking user who sends a longer voice note about a relative requesting urgent money or a channel admin asking for an SMS code, I want the bot to understand the request and route to the right help path.</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Longer UZ audio gets a larger STT budget and prompt vocabulary; requested-action forms such as yuborishimni/o'tkazishimni so'rayapti do not get misread as already completed actions; family urgent money routes to live-call SOS and channel-admin SMS-code requests route through runCheck.</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>src/lib/telegram/handlers/check.ts; src/lib/telegram/handlers/check.voice.test.ts; src/lib/telegram/voice-stt-provider-fixtures.ts; src/lib/risk/check-core.ts; src/lib/risk/rules.ts; src/lib/risk/voice-transcription.test.ts; src/lib/risk/rules.reason-codes.test.ts</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>User feedback 2026-07-09 UZ long voice QA; live Telegram screenshots</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>Focused voice/risk tests + full Telegram/risk regression suites + production Telegram smokes</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>Closed 2026-07-09 in 4bba35c: default voice STT timeout raised to 12s; STT prompt expanded for UZ family/channel-admin phrases; live-call context handles singlim/zudlik/muammo; requested-action guard prevents UZ requests from being treated as completed emergencies; SMS-code and relative-distress rules expanded.</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>No raw audio or private transcript is persisted by this tracker entry. Live Telegram real-audio re-check remains recommended after the user's daily STT limit resets.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record screenshot triage QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rdf5c71f6845b48d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rac057ac51b0248de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R3397ecf7a20047b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2df3f36ffa64437c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc92715617750432f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf73b161a65404c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2ab6ff17bb6e4035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re083fd8a08cd478c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Re3ca809ee8524910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re10086062c0c45af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1e1a771f18f549ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8c18d47e21ea45a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2697,16 +2697,16 @@
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: finish live Telegram QA residue after the STT limit resets: real-audio UZ spot-check for long family/channel-admin phrases, photo/screenshot triage, then P1 web/Telegram flows.</x:v>
+        <x:v>Next queue item: manual live Telegram image/screenshot QA on real uploads (scam profile, QR, Apple popup, APK summons, Telegram fake profile), then P1 web/Telegram flows.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. Inline/direct residue was closed and deployed; relative live-call family copy and full-plan residue were fixed; short UZ voice routing was fixed 2026-07-08. Long UZ voice requested-action routing fixed 2026-07-09 in 4bba35c and deployed via Railway b156f8a8: STT timeout is 12s, prompt vocabulary covers singlim/kanal administratori/SMS kodini/pul o'tkazishimni so'rayapti, requested-action forms no longer route as already-completed emergencies, and Telegram/risk regression suites plus prod Telegram smokes passed. Optional real-audio Telegram spot-check remains after the user's STT daily limit resets.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca: fake Apple/iOS security popups, APK/.pdf.apk summons and fake Telegram deletion/verification screenshots are high-risk; QR login/payment and Telegram profile boundaries remain covered. Manual live image upload spot-check remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2742,7 +2742,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="8" t="inlineStr">
         <x:is>
@@ -7065,6 +7065,44 @@
         <x:v>No raw audio or private transcript is persisted by this tracker entry. Live Telegram real-audio re-check remains recommended after the user's daily STT limit resets.</x:v>
       </x:c>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>P1-2026-07-09-002</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>Telegram QA / image screenshots</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Screenshot scam triage</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>As a user who sends a scam screenshot, profile, QR, Apple popup, APK summons, or fake Telegram profile, I want the bot to recognize the visual scam pattern and give safe next steps without storing the raw image.</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>Image evidence recognizes fake device security popups, APK/.pdf.apk summons, fake Telegram deletion/verification, QR login/payment, and Telegram profile cards. High-risk image paths stay action-first; profile-only screenshots remain non-accusatory.</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>src/lib/risk/image-intelligence.ts; src/lib/risk/image-intelligence.test.ts; src/lib/telegram/webhook.integration.test.ts</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>User feedback 2026-07-09 photo/screenshot QA; live Telegram screenshots/news examples</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>Focused image intelligence + webhook integration + full risk/Telegram suites + production Telegram smokes</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>Closed 2026-07-09 in 33ec7e3: added image hints for fake device security popups and Telegram account-takeover screenshots, tightened APK detection to avoid QR-login false positives, and added webhook coverage for Apple popup, APK summons, and fake Telegram deletion. Railway f8c344ca deployed; prod live/inline/user-story/false-positive/scope smokes passed. Manual live upload spot-check remains pending.</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L72" t="str">
+        <x:v>No raw image, OCR text, QR payload, private Telegram id, or screenshot data is stored in this tracker entry. Webhook tests assert no data:image persistence.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10252,6 +10290,29 @@
         <x:v>Passed: tests, tsc, eslint.</x:v>
       </x:c>
     </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>T-048</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>P1-2026-07-09-002</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>As the product owner, I want real Telegram photo/screenshot uploads checked for scam profile, QR, Apple popup, APK summons, and fake Telegram account screens.</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Bot either reads/decodes and gives correct risk/action, or gives a useful image-specific fallback and asks for cropped text/link/QR. Profile-only screenshots must not accuse the account by screenshot alone.</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>Open manual live spot-check after deployment; automated evidence paths passed locally and production smokes passed.</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>Pending live manual Telegram image QA after image/OCR budget or real screenshots are available; local/prod automated checks passed 2026-07-09.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13446,6 +13507,32 @@
         <x:v>Next: resume live Telegram QA with UZ voice spot-checks and photo/screenshot triage; then P1 web/Telegram report, appeal/admin, private/group scoping flows.</x:v>
       </x:c>
     </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>QA-2026-07-09-002</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Telegram screenshot/image scam triage</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>npx eslint touched image/webhook files; npm run test:run -- src/lib/risk/image-intelligence.test.ts src/lib/telegram/webhook.integration.test.ts; npm run test:run -- src/lib/risk; npm run test:run -- src/lib/telegram; railway up --detach; railway run prod Telegram live/inline/user-story/false-positive/scope smokes</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>Passed: focused image/webhook 135 tests; full risk 30 files / 471 tests; full Telegram 53 files / 1852 tests; Railway deployment f8c344ca SUCCESS; production live/inline/user-story/false-positive/scope smokes passed.</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>P1-2026-07-09-002, TG-002, Telegram image OCR/QR path</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>Commit 33ec7e3 adds fake Apple/iOS popup, APK court summons, fake Telegram deletion/account-takeover evidence coverage; existing QR/profile behavior remains covered.</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>Next: manual live upload of real screenshots (scam profile, QR login/payment, Apple popup, APK-povestka, Telegram fake profile), then resume P1 web/Telegram report, appeal/admin, and private/group scoping flows.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record live image qa blocker
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R2ab6ff17bb6e4035"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re083fd8a08cd478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Re3ca809ee8524910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re10086062c0c45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1e1a771f18f549ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R8c18d47e21ea45a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R362afbfb3ca24b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb2321e821d224830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5c9f1aa18a8447d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R95d70d6312644eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra5812275ae514142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re6720d165d4e4e2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10814,6 +10814,23 @@
         <x:v>Closed - fixed and deployed 2026-07-08</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>ERR-2026-07-09-004</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Live Telegram image QA: text screenshots fall back when AI vision quota/provider is unavailable</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Evidence: manual live Telegram QA. QR-login screenshot worked through local QR decoder; scam profile, Apple popup, APK summons and fake Telegram deletion screenshots all returned OCR fallback. Railway logs show AI image-intelligence 403/429 / RESOURCE_EXHAUSTED. Next: provision working vision provider/fallback and rerun T-048.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13533,6 +13550,23 @@
         <x:v>Next: manual live upload of real screenshots (scam profile, QR login/payment, Apple popup, APK-povestka, Telegram fake profile), then resume P1 web/Telegram report, appeal/admin, and private/group scoping flows.</x:v>
       </x:c>
     </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>QA-2026-07-09-003</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>Live Telegram image QA partial</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Manual Telegram Web</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Partial / blocked</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>QR-login passed; non-QR text screenshots blocked by image-intelligence provider quota. No code regression confirmed yet.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): block dangerous MIME-spoofed filenames
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R362afbfb3ca24b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb2321e821d224830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5c9f1aa18a8447d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R95d70d6312644eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra5812275ae514142"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re6720d165d4e4e2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R89575f04e56f4275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R6483cad5c1db4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R628d7a8e4c9842c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R7cbaa5d63c5d48f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R62b20ea6b8b24a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R21adaaac97434cbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: manual live Telegram image/screenshot QA on real uploads (scam profile, QR, Apple popup, APK summons, Telegram fake profile), then P1 web/Telegram flows.</x:v>
+        <x:v>Next queue item: P1 web/Telegram flows (report success path, appeal/admin moderation, homepage high-risk, private/group Telegram report scoping), while continuing live direct/inline phrase QA as regressions appear.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca: fake Apple/iOS security popups, APK/.pdf.apk summons and fake Telegram deletion/verification screenshots are high-risk; QR login/payment and Telegram profile boundaries remain covered. Manual live image upload spot-check remains pending.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10822,13 +10822,30 @@
         <x:v>Live Telegram image QA: text screenshots fall back when AI vision quota/provider is unavailable</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="E14" t="str">
-        <x:v>Evidence: manual live Telegram QA. QR-login screenshot worked through local QR decoder; scam profile, Apple popup, APK summons and fake Telegram deletion screenshots all returned OCR fallback. Railway logs show AI image-intelligence 403/429 / RESOURCE_EXHAUSTED. Next: provision working vision provider/fallback and rerun T-048.</x:v>
+        <x:v>Resolved 2026-07-09 after Gemini quota/subscription was restored. Provider health returned 200; live Telegram uploads now process through image triage. Verified manually: QR-login =&gt; high-risk Telegram QR; Apple/iOS popup =&gt; high-risk APK/security-popup; APK summons =&gt; high-risk APK/legal-pressure; fake Telegram deletion/verification =&gt; high-risk account-takeover; scam profile alone =&gt; cautious boundary/follow-up prompt, no unsupported accusation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>ERR-2026-07-09-005</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Telegram MIME-spoofing: dangerous file_name routed into image/OCR or voice/STT when MIME was forged</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>Validated from attacking-scenarios v2 feedback. Fixed in src/lib/telegram/router.ts by checking dangerous file_name before trusting image/* or audio/* MIME. Covers app.apk\0.jpg, photo.jpg.apk, app.apk.jpg, update.apk trailing space, setup.exe image spoof, invoice.lnk.jpg, voice.apk audio/ogg and app.арк homoglyph. Verification: eslint router/router.test passed; router.test 84/84; full src/lib/telegram 1854/1854.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13561,10 +13578,27 @@
         <x:v>Manual Telegram Web</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Partial / blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>QR-login passed; non-QR text screenshots blocked by image-intelligence provider quota. No code regression confirmed yet.</x:v>
+        <x:v>Retested after Gemini quota/subscription restored. Manual live Telegram image QA passed: QR-login, Apple/iOS popup, APK summons, fake Telegram deletion/verification, and scam-profile boundary. Prior partial result was caused by AI image-intelligence provider quota/config exhaustion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>QA-2026-07-09-004</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>MIME-spoofing router guard regression</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Unit + full Telegram tests</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Added router tests for all v2 bypasses plus hidden dangerous-segment and .lnk variants. Dangerous filenames now return outOfScope/document before media download routes; legitimate image documents and audio documents still route normally.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record MIME spoofing deploy verification
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R89575f04e56f4275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R6483cad5c1db4002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R628d7a8e4c9842c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R7cbaa5d63c5d48f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R62b20ea6b8b24a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R21adaaac97434cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc98b10e1c8f642f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1011071bfeaa456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R2092b6f2270e49e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbd3dccda1e9247fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R767fa92da8044c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7ead49f10cf94b01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: P1 web/Telegram flows (report success path, appeal/admin moderation, homepage high-risk, private/group Telegram report scoping), while continuing live direct/inline phrase QA as regressions appear.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants. MIME-spoofing fix was deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b and post-deploy prod smokes passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10845,7 +10845,7 @@
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>Validated from attacking-scenarios v2 feedback. Fixed in src/lib/telegram/router.ts by checking dangerous file_name before trusting image/* or audio/* MIME. Covers app.apk\0.jpg, photo.jpg.apk, app.apk.jpg, update.apk trailing space, setup.exe image spoof, invoice.lnk.jpg, voice.apk audio/ogg and app.арк homoglyph. Verification: eslint router/router.test passed; router.test 84/84; full src/lib/telegram 1854/1854.</x:v>
+        <x:v>Validated from attacking-scenarios v2 feedback. Fixed in src/lib/telegram/router.ts by checking dangerous file_name before trusting image/* or audio/* MIME. Covers app.apk\0.jpg, photo.jpg.apk, app.apk.jpg, update.apk trailing space, setup.exe image spoof, invoice.lnk.jpg, voice.apk audio/ogg and app.арк homoglyph. Verification: eslint router/router.test passed; router.test 84/84; full src/lib/telegram 1854/1854. Deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b; prod smoke/security/Telegram inline/live/user-story/false-positive/scope/voice-out all passed against https://scam-guard-main-production.up.railway.app.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13598,7 +13598,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>Added router tests for all v2 bypasses plus hidden dangerous-segment and .lnk variants. Dangerous filenames now return outOfScope/document before media download routes; legitimate image documents and audio documents still route normally.</x:v>
+        <x:v>Added router tests for all v2 bypasses plus hidden dangerous-segment and .lnk variants. Dangerous filenames now return outOfScope/document before media download routes; legitimate image documents and audio documents still route normally. Post-deploy verification passed: prod:smoke, prod:security-smoke, prod:telegram-inline-smoke, prod:telegram-live-qa-smoke, prod:telegram-user-story-smoke, prod:telegram-false-positive-smoke, prod:telegram-scope-smoke, prod:telegram-voice-out-smoke.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(telegram): cover Soliq and short scam questions
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc98b10e1c8f642f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R1011071bfeaa456e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R2092b6f2270e49e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbd3dccda1e9247fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R767fa92da8044c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7ead49f10cf94b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re272c407c6644fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb582d11b5ae346bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8afd184c881745f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R11b1502c90da4f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra3c781a891144604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R404bd9beddd64ca8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2697,7 +2697,7 @@
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: P1 web/Telegram flows (report success path, appeal/admin moderation, homepage high-risk, private/group Telegram report scoping), while continuing live direct/inline phrase QA as regressions appear.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants. MIME-spoofing fix was deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b and post-deploy prod smokes passed.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants. MIME-spoofing fix was deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b and post-deploy prod smokes passed. Quality Gate residual direct phrases were fixed: Soliqdan qo'ng'iroq qilishdi and short mixed RU/UZ scam questions now route to human victim-intent guidance instead of cold fallback.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10848,6 +10848,23 @@
         <x:v>Validated from attacking-scenarios v2 feedback. Fixed in src/lib/telegram/router.ts by checking dangerous file_name before trusting image/* or audio/* MIME. Covers app.apk\0.jpg, photo.jpg.apk, app.apk.jpg, update.apk trailing space, setup.exe image spoof, invoice.lnk.jpg, voice.apk audio/ogg and app.арк homoglyph. Verification: eslint router/router.test passed; router.test 84/84; full src/lib/telegram 1854/1854. Deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b; prod smoke/security/Telegram inline/live/user-story/false-positive/scope/voice-out all passed against https://scam-guard-main-production.up.railway.app.</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>ERR-2026-07-09-006</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Quality gate leftovers: direct UZ Soliq call and short mixed RU/UZ scam question fell into cold fallback</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>Validated from Quality Gate feedback. Added direct victim-intent coverage for Soliqdan qo'ng'iroq qilishdi / soliqdan yozishdi and short questions like Salom это скам?, bu scammi?, bu firibgarlikmi?. Preserved scammer payload routing (Salom, men bank xodimi...) and report-question routing. Verification: victim-intent 123/123; focused Telegram victim/inline/check tests 476/476; full src/lib/telegram 1860/1860.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13601,6 +13618,23 @@
         <x:v>Added router tests for all v2 bypasses plus hidden dangerous-segment and .lnk variants. Dangerous filenames now return outOfScope/document before media download routes; legitimate image documents and audio documents still route normally. Post-deploy verification passed: prod:smoke, prod:security-smoke, prod:telegram-inline-smoke, prod:telegram-live-qa-smoke, prod:telegram-user-story-smoke, prod:telegram-false-positive-smoke, prod:telegram-scope-smoke, prod:telegram-voice-out-smoke.</x:v>
       </x:c>
     </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>QA-2026-07-09-005</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>Quality Gate residual direct phrase regression</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Unit + full Telegram tests</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>Covered the two remaining cold direct phrases from the Quality Gate report: UZ Soliq call/write variants and short mixed-language 'is this scam?' questions. No regression in inline, direct scammer payload, report-question or Telegram handler routing.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record quality gate phrase deploy
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re272c407c6644fa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb582d11b5ae346bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8afd184c881745f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R11b1502c90da4f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra3c781a891144604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R404bd9beddd64ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R16672fc31c3e4115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R719a3d33fd5c4853"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R472faa16f75044fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra2510070735645fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1f76c574f4b14e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R91a3c64a3fea4287"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: P1 web/Telegram flows (report success path, appeal/admin moderation, homepage high-risk, private/group Telegram report scoping), while continuing live direct/inline phrase QA as regressions appear.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants. MIME-spoofing fix was deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b and post-deploy prod smokes passed. Quality Gate residual direct phrases were fixed: Soliqdan qo'ng'iroq qilishdi and short mixed RU/UZ scam questions now route to human victim-intent guidance instead of cold fallback.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants. MIME-spoofing fix was deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b and post-deploy prod smokes passed. Quality Gate residual direct phrases were fixed: Soliqdan qo'ng'iroq qilishdi and short mixed RU/UZ scam questions now route to human victim-intent guidance instead of cold fallback. Quality Gate residual phrase fix was deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8; prod smoke, Telegram user-story and inline smokes passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10862,7 +10862,7 @@
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>Validated from Quality Gate feedback. Added direct victim-intent coverage for Soliqdan qo'ng'iroq qilishdi / soliqdan yozishdi and short questions like Salom это скам?, bu scammi?, bu firibgarlikmi?. Preserved scammer payload routing (Salom, men bank xodimi...) and report-question routing. Verification: victim-intent 123/123; focused Telegram victim/inline/check tests 476/476; full src/lib/telegram 1860/1860.</x:v>
+        <x:v>Validated from Quality Gate feedback. Added direct victim-intent coverage for Soliqdan qo'ng'iroq qilishdi / soliqdan yozishdi and short questions like Salom это скам?, bu scammi?, bu firibgarlikmi?. Preserved scammer payload routing (Salom, men bank xodimi...) and report-question routing. Verification: victim-intent 123/123; focused Telegram victim/inline/check tests 476/476; full src/lib/telegram 1860/1860. Deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8; prod:smoke, prod:telegram-user-story-smoke and prod:telegram-inline-smoke passed against https://scam-guard-main-production.up.railway.app.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13632,7 +13632,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>Covered the two remaining cold direct phrases from the Quality Gate report: UZ Soliq call/write variants and short mixed-language 'is this scam?' questions. No regression in inline, direct scammer payload, report-question or Telegram handler routing.</x:v>
+        <x:v>Covered the two remaining cold direct phrases from the Quality Gate report: UZ Soliq call/write variants and short mixed-language 'is this scam?' questions. No regression in inline, direct scammer payload, report-question or Telegram handler routing. Deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8; production smoke/user-story/inline verification passed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test: add production P1 web smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R16672fc31c3e4115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R719a3d33fd5c4853"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R472faa16f75044fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra2510070735645fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1f76c574f4b14e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R91a3c64a3fea4287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rce65c7a7c4e441b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3084f84266394983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R95276bef83a34d3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re108b19d97b04de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R65eb0c3013f344dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc663cff617194af6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: P1 web/Telegram flows (report success path, appeal/admin moderation, homepage high-risk, private/group Telegram report scoping), while continuing live direct/inline phrase QA as regressions appear.</x:v>
+        <x:v>Next queue item: UX/logistics fixes and residual live QA (direct/inline context stitching, short UZ voice spot-checks after STT reset, image provider spot-checks), then Family Shield proactive delivery.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. Previous image QA blocker is resolved as provider quota/config, not a code regression. MIME-spoofing report v2 was validated and fixed: dangerous document/audio filenames are blocked before image/OCR or voice/STT routing, including null-byte, double-extension, hidden dangerous-extension, trailing-space, EXE, LNK, audio-MIME and Cyrillic-homoglyph APK variants. MIME-spoofing fix was deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b and post-deploy prod smokes passed. Quality Gate residual direct phrases were fixed: Soliqdan qo'ng'iroq qilishdi and short mixed RU/UZ scam questions now route to human victim-intent guidance instead of cold fallback. Quality Gate residual phrase fix was deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8; prod smoke, Telegram user-story and inline smokes passed.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09: prod:web-p1-smoke now covers homepage/report/appeal/admin moderation; prod:telegram-user-story-smoke, prod:telegram-scope-smoke, prod:telegram-live-qa-smoke, prod:telegram-inline-smoke and prod:smoke passed against production.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6778,7 +6778,7 @@
         <x:v>Homepage high-risk, report success, appeal/admin moderation, live Telegram image/QR, Guardian Angel high-risk and private/group Telegram session scoping are verified against the configured production environment.</x:v>
       </x:c>
       <x:c r="F64" s="596" t="str">
-        <x:v>src/routes/index.tsx; src/routes/report.tsx; src/routes/appeal.tsx; scripts/prod-admin-moderation-smoke.ts; scripts/prod-telegram-user-story-smoke.ts; scripts/prod-telegram-live-qa-smoke.ts; scripts/prod-telegram-scope-smoke.ts; scripts/prod-security-smoke.ts</x:v>
+        <x:v>src/routes/index.tsx; src/routes/report.tsx; src/routes/appeal.tsx; scripts/prod-web-p1-smoke.ts; scripts/prod-admin-moderation-smoke.ts; scripts/prod-telegram-user-story-smoke.ts; scripts/prod-telegram-live-qa-smoke.ts; scripts/prod-telegram-scope-smoke.ts; scripts/prod-telegram-inline-smoke.ts; scripts/prod-smoke.ts</x:v>
       </x:c>
       <x:c r="G64" s="596" t="str">
         <x:v>ai_docs/OPEN_TASKS.md; ai_docs/ROADMAP.md; ai_docs/CHANGELOG_AI.md; production smoke notes</x:v>
@@ -6787,16 +6787,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I64" s="596" t="str">
-        <x:v>Production web/Telegram/admin/security smoke</x:v>
+        <x:v>Production web/Telegram/admin/security smoke + dedicated prod:web-p1-smoke</x:v>
       </x:c>
       <x:c r="J64" s="596" t="str">
-        <x:v>Closed 2026-07-02: Playwright production web smoke verified homepage high-risk result, report success and appeal success; admin moderation smoke verified report reject + appeal keep-reputation audit and cleanup. Telegram production user-story, live QR/Guardian, private/group scope smokes passed. prod-security-smoke passed after accepting PGRST205 as anon-denied for service-role-only embed_origin_events.</x:v>
+        <x:v>Re-verified 2026-07-09: prod:web-p1-smoke checked homepage/report/appeal pages, rules-only high-risk web check, synthetic report, synthetic appeal, admin reject/keep-reputation moderation, audit log and cleanup. Telegram user-story, private/group scope, live QR/Guardian and inline smokes also passed. Base prod smoke passed with Telegram webhook pending=0 and AI provider healthy.</x:v>
       </x:c>
       <x:c r="K64" s="596" t="str">
-        <x:v>Proceed to T-046 / SEC-002 CSP/security headers final reconciliation and UX/logistics cleanup.</x:v>
+        <x:v>Proceed to UX/logistics residuals: live direct/inline context stitching, UZ voice spot-checks after STT reset, image provider spot-checks, then Family Shield proactive delivery.</x:v>
       </x:c>
       <x:c r="L64" s="596" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-09</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -13635,6 +13635,32 @@
         <x:v>Covered the two remaining cold direct phrases from the Quality Gate report: UZ Soliq call/write variants and short mixed-language 'is this scam?' questions. No regression in inline, direct scammer payload, report-question or Telegram handler routing. Deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8; production smoke/user-story/inline verification passed.</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>QA-2026-07-09-006</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>P1 web/Telegram production user-story flow rerun</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>railway run npm run prod:web-p1-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-user-story-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-scope-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-live-qa-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:telegram-inline-smoke -- https://scam-guard-main-production.up.railway.app; railway run npm run prod:smoke -- https://scam-guard-main-production.up.railway.app; npm run test:run -- src/lib/admin.functions.test.ts src/lib/report.functions.test.ts src/lib/reputation-appeal.functions.test.ts</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>Passed: new prod:web-p1-smoke validated homepage/report/appeal 200s, rules-only web high-risk result, synthetic report/appeal submission, admin moderation/audit and cleanup. Telegram user-story, private/group scope, live QR/Guardian, inline and base prod smokes passed. Focused admin/report/appeal tests passed 24/24.</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>QA-001, TG-002, WEB-001, REP-001, APPEAL-001, ADMIN-001</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>Added scripts/prod-web-p1-smoke.ts and package script prod:web-p1-smoke so the P1 web/admin path can be rerun without manual DB setup.</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>Next: UX/logistics residual QA and fixes; no production deploy needed for this QA-script/tracker-only update.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record Telegram context QA closure
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rce65c7a7c4e441b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3084f84266394983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R95276bef83a34d3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re108b19d97b04de0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R65eb0c3013f344dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc663cff617194af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R20e9a6f6de3a4322"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rd1fba9ac8b5b4d71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9f25c16126034cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R613a4d343a7248fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf992aa567e454297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R17613aed9d2a49ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2697,16 +2697,16 @@
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: UX/logistics fixes and residual live QA (direct/inline context stitching, short UZ voice spot-checks after STT reset, image provider spot-checks), then Family Shield proactive delivery.</x:v>
+        <x:v>Next queue item: continue UX/logistics residual QA (manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, image provider routine spot-checks), then Family Shield proactive delivery.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09: prod:web-p1-smoke now covers homepage/report/appeal/admin moderation; prod:telegram-user-story-smoke, prod:telegram-scope-smoke, prod:telegram-live-qa-smoke, prod:telegram-inline-smoke and prod:smoke passed against production.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2736,52 +2736,40 @@
       <x:c r="E4" s="8" t="n"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented</x:t>
-        </x:is>
+      <x:c r="A5" s="8" t="str">
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="C5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Works in code; still needs regression/live QA per row.</x:t>
-        </x:is>
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>Works in code; still needs regression/live QA per row.</x:v>
       </x:c>
       <x:c r="D5" s="8" t="n"/>
       <x:c r="E5" s="8" t="n"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
-        </x:is>
+      <x:c r="A6" s="8" t="str">
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Code exists but known gaps remain.</x:t>
-        </x:is>
+      <x:c r="C6" s="8" t="str">
+        <x:v>Code exists but known gaps remain.</x:v>
       </x:c>
       <x:c r="D6" s="8" t="n"/>
       <x:c r="E6" s="8" t="n"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
-        </x:is>
+      <x:c r="A7" s="8" t="str">
+        <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roadmap item not yet implemented.</x:t>
-        </x:is>
+      <x:c r="C7" s="8" t="str">
+        <x:v>Roadmap item not yet implemented.</x:v>
       </x:c>
       <x:c r="D7" s="8" t="n"/>
       <x:c r="E7" s="8" t="n"/>
@@ -7103,6 +7091,44 @@
         <x:v>No raw image, OCR text, QR payload, private Telegram id, or screenshot data is stored in this tracker entry. Webhook tests assert no data:image persistence.</x:v>
       </x:c>
     </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>P1-2026-07-09-003</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>Telegram QA / context stitching</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Direct context prefaces and follow-up explanations</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>As a user who first sends a human preface like 'Мне прислали ссылку' or 'Мне пишет администратор канала', I want the bot to ask for the next piece and then understand the follow-up without a cold risk card.</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>Low-signal prefaces do not create checks; a follow-up URL creates a real URL check and why-question uses lastCheck; channel-admin preface stays conversational; SMS-code follow-up gives immediate code safety guidance.</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>src/lib/telegram/victim-intent.ts; src/lib/telegram/handlers/check.followup-routing.test.ts; src/lib/telegram/live-phrase-cases.ts; scripts/prod-telegram-context-smoke.ts</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>User feedback 2026-07-09 direct/inline context stitching; FEATURE_USER_STORY_TRACKER.xlsx</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>Focused victim/follow-up tests + full Telegram suite + production context/live/inline/user-story smokes</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>Closed 2026-07-09 in 0cf0ee2: channel-admin prefaces now route as Telegram-message context; direct SMS-code follow-up stays immediate code guidance. Railway deployment 9c12ac76-1bca-4a8c-b13e-78a966411feb reached SUCCESS. prod:telegram-context-smoke passed with marker QACTXDNAUNHBLUW, then prod live QA, inline and user-story smokes passed.</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>Continue residual UX/logistics: manual direct/inline 15-20 phrase sweep, UZ voice spot-checks after STT reset, image provider routine spot-checks, then Family Shield proactive alert.</x:v>
+      </x:c>
+      <x:c r="L73" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10865,6 +10891,32 @@
         <x:v>Validated from Quality Gate feedback. Added direct victim-intent coverage for Soliqdan qo'ng'iroq qilishdi / soliqdan yozishdi and short questions like Salom это скам?, bu scammi?, bu firibgarlikmi?. Preserved scammer payload routing (Salom, men bank xodimi...) and report-question routing. Verification: victim-intent 123/123; focused Telegram victim/inline/check tests 476/476; full src/lib/telegram 1860/1860. Deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8; prod:smoke, prod:telegram-user-story-smoke and prod:telegram-inline-smoke passed against https://scam-guard-main-production.up.railway.app.</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>ERR-2026-07-09-007</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Live Telegram direct QA / production context smoke</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>TG-002, TG-005, P1-2026-07-02-003</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Short preface 'Мне пишет администратор канала' created a check row/generic risk path instead of asking for the actual Telegram message or request.</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Users naturally send the situation in two steps. If the first preface creates a cold check, the bot feels stuck exactly before the user explains 'он просит СМС код'.</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Fixed 2026-07-09 in 0cf0ee2: channel-admin prefaces route to telegram_message; channel-admin SMS-code text keeps immediate code guidance. Verification: focused 370 tests, full Telegram 1869 tests, Railway deployment 9c12ac76 SUCCESS, prod:telegram-context-smoke passed.</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Closed - fixed and deployed 2026-07-09</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13661,6 +13713,32 @@
         <x:v>Next: UX/logistics residual QA and fixes; no production deploy needed for this QA-script/tracker-only update.</x:v>
       </x:c>
     </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>QA-2026-07-09-007</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>Telegram direct context-stitching production smoke</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>npm run test:run -- src/lib/telegram/victim-intent.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts; npm run test:run -- src/lib/telegram/handlers/inline.test.ts src/lib/telegram/inline.mass.test.ts; npm run test:run -- src/lib/risk/rules.reason-codes.test.ts src/lib/telegram/conversation-check.test.ts; npm run test:run -- src/lib/telegram; railway up --detach; railway run npm run prod:telegram-context-smoke -- https://scam-guard-main-production.up.railway.app; railway run prod Telegram live/inline/user-story smokes</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>Passed: focused victim/follow-up 370 tests; inline 115 tests; risk/conversation 164 tests; full Telegram 52 files / 1869 tests. Railway deployment 9c12ac76 SUCCESS. prod:telegram-context-smoke passed, then prod live QA, inline and user-story smokes passed.</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>TG-002, TG-005, P1-2026-07-02-003, P1-2026-07-09-003</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>Added scripts/prod-telegram-context-smoke.ts. It verifies low-signal link preface does not create a check, follow-up URL creates a URL check, why-question reuses lastCheck, channel-admin preface does not create a check, and SMS-code follow-up stays in direct guidance.</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>Next: continue residual live UX QA: 15-20 manual direct/inline phrases, UZ voice spot-checks when STT budget resets, image provider routine spot-checks, then Family Shield proactive delivery.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix(telegram): add proactive family shield alerts
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R20e9a6f6de3a4322"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rd1fba9ac8b5b4d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R9f25c16126034cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R613a4d343a7248fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rf992aa567e454297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R17613aed9d2a49ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R88a8b9d97ad74628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2f171ae9af2d4217"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R74a556bde9634ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf2619908cb724f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rcb4fbeb30e93431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R1caa57b8e2c84da4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: continue UX/logistics residual QA (manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, image provider routine spot-checks), then Family Shield proactive delivery.</x:v>
+        <x:v>Next queue item: post-deploy Family Shield live opt-in smoke, then residual UX/logistics QA: manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. Manual live Telegram image upload spot-check was repeated after Gemini quota/subscription was restored: QR-login, Apple/iOS popup, APK/.pdf.apk summons, fake Telegram deletion/verification and scam-profile boundary behaved as expected. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert is now implemented in code and ready for post-deploy live opt-in smoke.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2740,7 +2740,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -2766,7 +2766,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Roadmap item not yet implemented.</x:v>
@@ -6962,19 +6962,19 @@
         <x:v>User feedback 2026-07-02 delivery strategy</x:v>
       </x:c>
       <x:c r="H69" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I69" t="str">
-        <x:v>Needs design + tests</x:v>
+        <x:v>Focused Family Shield/follow-up/webhook/i18n tests + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J69" t="str">
-        <x:v>Requires explicit opt-in, redacted alert, cooldown, acknowledgement button and false-positive guardrails.</x:v>
+        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed.</x:v>
       </x:c>
       <x:c r="K69" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>Alert must not include scammer number, codes, links, screenshots, card data or raw check evidence.</x:v>
+        <x:v>Uses existing explicit active Family Shield link as opt-in. Alert must not include scammer number, codes, links, screenshots, card data, raw check evidence, or checked text; tests assert redaction and group no-alert behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">

</xml_diff>

<commit_message>
docs: record family shield prod smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R88a8b9d97ad74628"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2f171ae9af2d4217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R74a556bde9634ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf2619908cb724f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rcb4fbeb30e93431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R1caa57b8e2c84da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rec549a0d250444d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2dedee05a61143d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R964faff0ee004595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ref1adf55554743a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R420a9627056e4a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R442a5444220d4526"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: post-deploy Family Shield live opt-in smoke, then residual UX/logistics QA: manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
+        <x:v>Next queue item: manual real two-account Family Shield live opt-in smoke, then residual UX/logistics QA: manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert is now implemented in code and ready for post-deploy live opt-in smoke.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Remaining Family Shield item is manual live opt-in smoke with a real trusted contact.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6968,7 +6968,7 @@
         <x:v>Focused Family Shield/follow-up/webhook/i18n tests + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J69" t="str">
-        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed.</x:v>
+        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed. Railway deployment 3d187870-ce65-461b-b8b3-60c9a2ceafca is SUCCESS; prod Telegram context/live/inline/user-story smokes passed; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account opt-in smoke remains.</x:v>
       </x:c>
       <x:c r="K69" t="str">
         <x:v>P2</x:v>
@@ -7123,7 +7123,7 @@
         <x:v>Closed 2026-07-09 in 0cf0ee2: channel-admin prefaces now route as Telegram-message context; direct SMS-code follow-up stays immediate code guidance. Railway deployment 9c12ac76-1bca-4a8c-b13e-78a966411feb reached SUCCESS. prod:telegram-context-smoke passed with marker QACTXDNAUNHBLUW, then prod live QA, inline and user-story smokes passed.</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>Continue residual UX/logistics: manual direct/inline 15-20 phrase sweep, UZ voice spot-checks after STT reset, image provider routine spot-checks, then Family Shield proactive alert.</x:v>
+        <x:v>Continue residual UX/logistics: manual real two-account Family Shield live opt-in smoke, manual direct/inline 15-20 phrase sweep, UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
       </x:c>
       <x:c r="L73" t="str">
         <x:v>2026-07-09</x:v>
@@ -13736,7 +13736,7 @@
         <x:v>Added scripts/prod-telegram-context-smoke.ts. It verifies low-signal link preface does not create a check, follow-up URL creates a URL check, why-question reuses lastCheck, channel-admin preface does not create a check, and SMS-code follow-up stays in direct guidance.</x:v>
       </x:c>
       <x:c r="H83" t="str">
-        <x:v>Next: continue residual live UX QA: 15-20 manual direct/inline phrases, UZ voice spot-checks when STT budget resets, image provider routine spot-checks, then Family Shield proactive delivery.</x:v>
+        <x:v>Next: manual real two-account Family Shield live opt-in smoke; then continue residual live UX QA: 15-20 manual direct/inline phrases, UZ voice spot-checks when STT budget resets, and image provider routine spot-checks.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: close family shield live smoke
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rec549a0d250444d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2dedee05a61143d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R964faff0ee004595"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ref1adf55554743a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R420a9627056e4a54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R442a5444220d4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R38d22c2e90a84e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rdb823b309f744ce9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd373fafbbcda48d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9fda4da4c7044145"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R68e19e280c244d71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R45be7b8005a940b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: manual real two-account Family Shield live opt-in smoke, then residual UX/logistics QA: manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
+        <x:v>Next queue item: residual UX/logistics QA: manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, image provider routine spot-checks, then P1/P2 web/Telegram flow polish as needed.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Remaining Family Shield item is manual live opt-in smoke with a real trusted contact.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account Family Shield smoke passed 2026-07-09: trusted contact received proactive and manual alerts at 17:42 and 17:46, both redacted with acknowledgement and opt-out controls.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6968,7 +6968,7 @@
         <x:v>Focused Family Shield/follow-up/webhook/i18n tests + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J69" t="str">
-        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed. Railway deployment 3d187870-ce65-461b-b8b3-60c9a2ceafca is SUCCESS; prod Telegram context/live/inline/user-story smokes passed; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account opt-in smoke remains.</x:v>
+        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed. Railway deployment 3d187870-ce65-461b-b8b3-60c9a2ceafca is SUCCESS; prod Telegram context/live/inline/user-story smokes passed; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account live smoke passed: proactive trusted alert arrived at 17:42, and manual 'Позвать близкого' alert arrived at 17:46; both were redacted and showed acknowledgement/opt-out controls.</x:v>
       </x:c>
       <x:c r="K69" t="str">
         <x:v>P2</x:v>
@@ -7123,7 +7123,7 @@
         <x:v>Closed 2026-07-09 in 0cf0ee2: channel-admin prefaces now route as Telegram-message context; direct SMS-code follow-up stays immediate code guidance. Railway deployment 9c12ac76-1bca-4a8c-b13e-78a966411feb reached SUCCESS. prod:telegram-context-smoke passed with marker QACTXDNAUNHBLUW, then prod live QA, inline and user-story smokes passed.</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>Continue residual UX/logistics: manual real two-account Family Shield live opt-in smoke, manual direct/inline 15-20 phrase sweep, UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
+        <x:v>Continue residual UX/logistics: manual direct/inline 15-20 phrase sweep, UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
       </x:c>
       <x:c r="L73" t="str">
         <x:v>2026-07-09</x:v>
@@ -13736,7 +13736,33 @@
         <x:v>Added scripts/prod-telegram-context-smoke.ts. It verifies low-signal link preface does not create a check, follow-up URL creates a URL check, why-question reuses lastCheck, channel-admin preface does not create a check, and SMS-code follow-up stays in direct guidance.</x:v>
       </x:c>
       <x:c r="H83" t="str">
-        <x:v>Next: manual real two-account Family Shield live opt-in smoke; then continue residual live UX QA: 15-20 manual direct/inline phrases, UZ voice spot-checks when STT budget resets, and image provider routine spot-checks.</x:v>
+        <x:v>Next: continue residual live UX QA: 15-20 manual direct/inline phrases, UZ voice spot-checks when STT budget resets, and image provider routine spot-checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>QA-2026-07-09-010</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>2026-07-09</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>Family Shield real two-account live smoke</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Telegram Web: high-risk SMS-code call phrase in guardian chat, then manual 'Позвать близкого'; trusted account screenshot confirmation</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>P2-2026-07-02-004, Family Shield proactive delivery</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Guardian chat received SOS result. Trusted contact received two redacted Ishonch Guard alerts: proactive at 17:42 and manual at 17:46, with 'Я помогу сейчас' acknowledgement and 'Отключить эти сигналы' controls.</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>Proceed to residual UX/logistics QA: direct/inline phrase sweep, short UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record residual Telegram QA rerun
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R38d22c2e90a84e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rdb823b309f744ce9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd373fafbbcda48d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9fda4da4c7044145"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R68e19e280c244d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R45be7b8005a940b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R18b771d626f74509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R67be0736837e4f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R37f465fbdc344db9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6bf41e89e1bc4521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra9f71f72c7b04dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R07ebd8f27a794935"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: residual UX/logistics QA: manual direct/inline 15-20 phrase sweep, short UZ voice spot-checks after STT reset, image provider routine spot-checks, then P1/P2 web/Telegram flow polish as needed.</x:v>
+        <x:v>Next queue item: T-048 manual photo/screenshot spot-checks (scam profile, QR, Apple popup, APK summons, fake Telegram profile) once vision quota/provider is available; then short UZ voice spot-checks after STT reset and P1/P2 web/Telegram flow polish as needed.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account Family Shield smoke passed 2026-07-09: trusted contact received proactive and manual alerts at 17:42 and 17:46, both redacted with acknowledgement and opt-out controls.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account Family Shield smoke passed 2026-07-09: trusted contact received proactive and manual alerts at 17:42 and 17:46, both redacted with acknowledgement and opt-out controls. Residual Telegram text/context QA was rerun 2026-07-09: prod context, user-story, live-QR, false-positive, inline and voice-out smokes passed against Railway production; focused victim-intent/inline/webhook tests passed. T-048 remains open for manual real image/screenshot spot-checks when vision quota/provider is available.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10339,6 +10339,29 @@
         <x:v>Pending live manual Telegram image QA after image/OCR budget or real screenshots are available; local/prod automated checks passed 2026-07-09.</x:v>
       </x:c>
     </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>T-049</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>QA-2026-07-09-011</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>As the product owner, I want residual Telegram text/context UX rechecked after Family Shield and context fixes.</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Production context/user-story/live-QR/inline/voice-out/false-positive smokes pass, and focused victim-intent/inline/webhook tests keep recent RU/UZ/direct/inline phrases from regressing.</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>Closed 2026-07-09: production residual Telegram QA smokes passed against Railway production. The context-stitching cases from user screenshots are confirmed fixed.</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>Passed 2026-07-09: prod:telegram-context-smoke, prod:telegram-user-story-smoke, prod:telegram-live-qa-smoke, prod:telegram-false-positive-smoke, prod:telegram-inline-smoke, prod:telegram-voice-out-smoke; focused tests victim-intent 128/128, inline 114/114, webhook.integration 97/97.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record image screenshot QA closure
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R18b771d626f74509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R67be0736837e4f07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R37f465fbdc344db9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R6bf41e89e1bc4521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra9f71f72c7b04dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R07ebd8f27a794935"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb1b57cab6c3046a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R80a1f0ae9b334f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb7f042111bb94d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re12e3b0a807d4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ree97bbc6f4694d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0da6bdb9435b4a03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,10 +2703,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: T-048 manual photo/screenshot spot-checks (scam profile, QR, Apple popup, APK summons, fake Telegram profile) once vision quota/provider is available; then short UZ voice spot-checks after STT reset and P1/P2 web/Telegram flow polish as needed.</x:v>
+        <x:v>Next queue item: short UZ voice spot-checks after STT reset, then P1/P2 web/Telegram UX/logistics flow polish; keep routine image-provider spot-checks in QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account Family Shield smoke passed 2026-07-09: trusted contact received proactive and manual alerts at 17:42 and 17:46, both redacted with acknowledgement and opt-out controls. Residual Telegram text/context QA was rerun 2026-07-09: prod context, user-story, live-QR, false-positive, inline and voice-out smokes passed against Railway production; focused victim-intent/inline/webhook tests passed. T-048 remains open for manual real image/screenshot spot-checks when vision quota/provider is available.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed and manual real two-account smoke passed. Residual Telegram text/context QA was rerun 2026-07-09. T-048 image/screenshot core QA is now closed: profile-only remains non-accusatory, QR login live smoke passes, Apple/iOS popup and APK summons remain high-risk, and UZ fake Teiegram/Telegram freeze profile screenshots now route to Telegram account-takeover after f4655c7; Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS and prod live/inline/user-story/context/false-positive/voice-out smokes passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7079,16 +7079,16 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I72" t="str">
-        <x:v>Focused image intelligence + webhook integration + full risk/Telegram suites + production Telegram smokes</x:v>
+        <x:v>Focused image/risk tests + full risk/Telegram suites + core real screenshot QA + production Telegram smokes</x:v>
       </x:c>
       <x:c r="J72" t="str">
-        <x:v>Closed 2026-07-09 in 33ec7e3: added image hints for fake device security popups and Telegram account-takeover screenshots, tightened APK detection to avoid QR-login false positives, and added webhook coverage for Apple popup, APK summons, and fake Telegram deletion. Railway f8c344ca deployed; prod live/inline/user-story/false-positive/scope smokes passed. Manual live upload spot-check remains pending.</x:v>
+        <x:v>Closed 2026-07-09 in f4655c7: multiline UZ fake Telegram freeze/profile OCR now triggers telegram_account_takeover_phishing. Real screenshot core QA passed scam profile-only =&gt; non-accusatory unknown, fake Telegram deletion/freeze =&gt; high-risk Telegram takeover, Apple/iOS popup =&gt; high-risk device-security/APK, APK summons =&gt; high-risk APK/legal pressure, foreign +98 call =&gt; suspicious operator context. Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS; prod live/inline/user-story/context/false-positive/voice-out smokes passed.</x:v>
       </x:c>
       <x:c r="K72" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L72" t="str">
-        <x:v>No raw image, OCR text, QR payload, private Telegram id, or screenshot data is stored in this tracker entry. Webhook tests assert no data:image persistence.</x:v>
+        <x:v>No raw image, OCR text, QR payload, private Telegram id, or screenshot data is stored in this tracker entry. Core QA used local attachments and redacted output only; production smokes use synthetic IDs and cleanup.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -10940,6 +10940,32 @@
         <x:v>Closed - fixed and deployed 2026-07-09</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>ERR-2026-07-09-008</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Live Telegram image QA / core vision rerun</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>TG-010, P1-2026-07-09-002</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>UZ fake Teiegram/Telegram profile-freeze screenshot with multiline OCR stayed near profile-card/unknown instead of Telegram account-takeover high risk.</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Users sending this realistic fake official Telegram profile screenshot would get a weak answer despite visible account-freeze, unknown-device, urgency and link pressure.</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Fixed 2026-07-09 in f4655c7: Telegram account-takeover patterns now match multiline OCR and UZ cues such as noma'lum qurilmadan kirish, muzlatib qo'yildi and havolani bosing. Core real-image QA passed profile-only unknown, fake Telegram deletion/freeze high-risk, Apple popup high-risk, APK summons high-risk, +98 call suspicious. Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS; prod live/inline/user-story/context/false-positive/voice-out smokes passed.</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Closed - fixed and deployed 2026-07-09</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record family alert cooldown fix
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb1b57cab6c3046a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R80a1f0ae9b334f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb7f042111bb94d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re12e3b0a807d4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ree97bbc6f4694d6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R0da6bdb9435b4a03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R678b5b65f7a047f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbbf95ca5ac014c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8abf2a73d10e4fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R65dfcaf1e1bb4c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R309350c7b3af4297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7e8939f08bd649dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2706,7 +2706,7 @@
         <x:v>Next queue item: short UZ voice spot-checks after STT reset, then P1/P2 web/Telegram UX/logistics flow polish; keep routine image-provider spot-checks in QA.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed and manual real two-account smoke passed. Residual Telegram text/context QA was rerun 2026-07-09. T-048 image/screenshot core QA is now closed: profile-only remains non-accusatory, QR login live smoke passes, Apple/iOS popup and APK summons remain high-risk, and UZ fake Teiegram/Telegram freeze profile screenshots now route to Telegram account-takeover after f4655c7; Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS and prod live/inline/user-story/context/false-positive/voice-out smokes passed.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed and manual real two-account smoke passed. Residual Telegram text/context QA was rerun 2026-07-09. T-048 image/screenshot core QA is now closed: profile-only remains non-accusatory, QR login live smoke passes, Apple/iOS popup and APK summons remain high-risk, and UZ fake Teiegram/Telegram freeze profile screenshots now route to Telegram account-takeover after f4655c7; Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS and prod live/inline/user-story/context/false-positive/voice-out smokes passed. Family Shield proactive duplicate-alert QA was fixed in 5c01b8c by using a 30-minute auto-alert cooldown while keeping manual alerts on the short default window; Railway deployment 5b7cf352-45be-4c01-bba1-fb388239ff47 reached SUCCESS.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6968,13 +6968,13 @@
         <x:v>Focused Family Shield/follow-up/webhook/i18n tests + full Telegram regression suite</x:v>
       </x:c>
       <x:c r="J69" t="str">
-        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed. Railway deployment 3d187870-ce65-461b-b8b3-60c9a2ceafca is SUCCESS; prod Telegram context/live/inline/user-story smokes passed; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account live smoke passed: proactive trusted alert arrived at 17:42, and manual 'Позвать близкого' alert arrived at 17:46; both were redacted and showed acknowledgement/opt-out controls.</x:v>
+        <x:v>Closed 2026-07-09: private high-risk checks now attempt notifyTrustedContact for active Family Shield links after the Guardian SOS path; group checks are excluded. The trusted alert includes acknowledgement and opt-out buttons, and the auto path passes only guardian id, language and safe display name. Focused 1020/1020 and full src/lib/telegram 1878/1878 passed. Railway deployment 3d187870-ce65-461b-b8b3-60c9a2ceafca is SUCCESS; prod Telegram context/live/inline/user-story smokes passed; synthetic prod:family-smoke passed create invite -&gt; accept -&gt; safe notify failure -&gt; revoke -&gt; open_rows=0. Manual real two-account live smoke passed: proactive trusted alert arrived at 17:42, and manual 'Позвать близкого' alert arrived at 17:46; both were redacted and showed acknowledgement/opt-out controls. 2026-07-09 follow-up: duplicate-alert QA showed proactive high-risk checks could notify the trusted contact again after the 2-minute default cooldown; fixed in 5c01b8c with a 30-minute proactive cooldown, manual notify still uses the short default window, and deployment 5b7cf352-45be-4c01-bba1-fb388239ff47 reached SUCCESS.</x:v>
       </x:c>
       <x:c r="K69" t="str">
-        <x:v>P2</x:v>
+        <x:v>P2 Manual live check: trusted contact should not receive repeated proactive alerts for repeated high-risk checks inside 30 minutes; manual button may still be used after the default cooldown.</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>Uses existing explicit active Family Shield link as opt-in. Alert must not include scammer number, codes, links, screenshots, card data, raw check evidence, or checked text; tests assert redaction and group no-alert behavior.</x:v>
+        <x:v>2026-07-09</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -10966,6 +10966,32 @@
         <x:v>Closed - fixed and deployed 2026-07-09</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>ERR-2026-07-09-009</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Live Telegram Family Shield / trusted contact smoke</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>P2-2026-07-02-004</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Proactive trusted-person alerts could repeat after the 2-minute shared notify cooldown when the protected user ran several high-risk checks.</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>The trusted contact can receive duplicate-looking alerts within minutes, which makes Family Shield feel spammy during QA or an active incident.</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Fixed 2026-07-09 in 5c01b8c: notifyTrustedContact accepts a custom cooldown, proactive high-risk checks use 30 minutes, manual alerts retain the short default window. Focused Family Shield/follow-up tests passed (255/255), full src/lib/telegram passed (1879/1879), Railway deployment 5b7cf352-45be-4c01-bba1-fb388239ff47 SUCCESS.</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Closed - fixed and deployed 2026-07-09</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record residual image fallback QA
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R678b5b65f7a047f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbbf95ca5ac014c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8abf2a73d10e4fa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R65dfcaf1e1bb4c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R309350c7b3af4297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7e8939f08bd649dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R5792112d8b4744e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R0b1b853fa9f84ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb9e7a6fe48314d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R84f4a299233e4421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R475bec1837a54a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R28d9c582b0774df3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2697,16 +2697,16 @@
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C2" s="20" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="20" t="str">
-        <x:v>Next queue item: short UZ voice spot-checks after STT reset, then P1/P2 web/Telegram UX/logistics flow polish; keep routine image-provider spot-checks in QA.</x:v>
+        <x:v>Next queue item: deploy and live-check Telegram account screenshot fallback, then continue photo/QR/APK/profile spot-checks and P1/P2 web/Telegram UX/logistics flow polish.</x:v>
       </x:c>
       <x:c r="E2" s="20" t="str">
-        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed and manual real two-account smoke passed. Residual Telegram text/context QA was rerun 2026-07-09. T-048 image/screenshot core QA is now closed: profile-only remains non-accusatory, QR login live smoke passes, Apple/iOS popup and APK summons remain high-risk, and UZ fake Teiegram/Telegram freeze profile screenshots now route to Telegram account-takeover after f4655c7; Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS and prod live/inline/user-story/context/false-positive/voice-out smokes passed. Family Shield proactive duplicate-alert QA was fixed in 5c01b8c by using a 30-minute auto-alert cooldown while keeping manual alerts on the short default window; Railway deployment 5b7cf352-45be-4c01-bba1-fb388239ff47 reached SUCCESS.</x:v>
+        <x:v>Owner note: security backlog remains closed. Since 2026-07-05, live-phrase QA added broad RU/UZ/news-derived direct+inline coverage. UZ voice routing fixes were deployed 2026-07-09. Screenshot triage was strengthened in 33ec7e3 and deployed via Railway f8c344ca. MIME-spoofing report v2 was validated, fixed and deployed via Railway 0c851a61-54d9-4a21-b781-0419e6b51b1b with post-deploy smokes passing. Quality Gate residual direct phrases were fixed and deployed via Railway 193afe36-8392-44c9-9764-b4430aacacc8. P1 web/Telegram user-story flow rerun completed 2026-07-09. Context-stitching QA was fixed in 0cf0ee2 and deployed via Railway 9c12ac76-1bca-4a8c-b13e-78a966411feb; prod:telegram-context-smoke plus live/inline/user-story smokes passed against production. Family Shield proactive trusted-person alert was implemented in f0d5ab2 and deployed via Railway 3d187870-ce65-461b-b8b3-60c9a2ceafca; synthetic prod:family-smoke passed and manual real two-account smoke passed. Residual Telegram text/context QA was rerun 2026-07-09. T-048 image/screenshot core QA is now closed: profile-only remains non-accusatory, QR login live smoke passes, Apple/iOS popup and APK summons remain high-risk, and UZ fake Teiegram/Telegram freeze profile screenshots now route to Telegram account-takeover after f4655c7; Railway deployment 783183b4-195f-4034-8d3e-ef15fde76ad5 reached SUCCESS and prod live/inline/user-story/context/false-positive/voice-out smokes passed. Family Shield proactive duplicate-alert QA was fixed in 5c01b8c by using a 30-minute auto-alert cooldown while keeping manual alerts on the short default window; Railway deployment 5b7cf352-45be-4c01-bba1-fb388239ff47 reached SUCCESS. Telegram account screenshot unreadable fallback was strengthened 2026-07-09: image-intelligence prompt now exposes account-takeover/device-popup hints, and the fallback menu has a dedicated Telegram account rescue path.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2740,7 +2740,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
         <x:v>Works in code; still needs regression/live QA per row.</x:v>
@@ -7129,6 +7129,44 @@
         <x:v>2026-07-09</x:v>
       </x:c>
     </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>P1-2026-07-09-004</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>Telegram QA / image screenshots</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Unreadable Telegram account screenshot fallback</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>As a user who sends a fake Telegram deletion, freeze, verification, or account-warning screenshot that vision cannot read fully, I want the bot to still offer the right Telegram-account rescue path instead of a generic dead end.</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Vision prompt lists Telegram account-takeover and fake device-popup hints explicitly; unreadable image triage includes a dedicated Telegram account option with safe Settings &gt; Devices / 2FA guidance while keeping normal profile screenshots non-accusatory.</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>src/lib/risk/check-core.ts; src/lib/telegram/image-fallback.ts; src/lib/telegram/bot-i18n.ts; src/lib/telegram/bot-qa-matrix.test.ts</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>User feedback 2026-07-09 live Telegram fake Telegram screenshots; live Telegram image QA</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>Focused image triage tests + full Telegram/risk regression suites before deploy</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>Closed 2026-07-09: live fake Telegram screenshot still hit unreadable-image fallback after provider quota recovered. Added missing image-intelligence schema hints and a dedicated Telegram account fallback button/text for deletion/verification/freeze/link-bot screenshots.</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>No raw screenshot, OCR text, URL, QR payload, or Telegram identifier is stored. Fallback advice is conditional and non-accusatory unless the user confirms the Telegram-account scenario.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record production release verification
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R3da4c5b27f1949f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf31eecae665c4f66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R69f39ce98d064d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R2b2637fe2dea47ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rd835f211737f471c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R041fd6030f504b3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R0be079f04aa44136"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R9b0ebb2548584215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfeaee7bc0b834e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re16c2e8b86334408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae58f0db205947e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R39b958761c7c45c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e0747c5cee848a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4991b91a2c7e4b1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R850055f2750f4ce8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rcee7bd7e590f466e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="181">
+  <x:fills count="187">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -995,6 +995,36 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1082,7 +1112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1052">
+  <x:cellXfs count="1094">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -3795,11 +3825,105 @@
     <x:xf numFmtId="0" fontId="1" fillId="179" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="181" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="181" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="182" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="182" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="182" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="183" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="183" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="183" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="183" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="183" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="183" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="182" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="184" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="184" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="185" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="185" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="185" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="186" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="186" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="186" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="186" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="186" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="186" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="185" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="315">
+  <x:dxfs count="357">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7064,6 +7188,402 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -7125,6 +7645,28 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
@@ -7180,6 +7722,28 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
@@ -7229,6 +7793,28 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -7532,7 +8118,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="62" hidden="0" customWidth="1"/>
@@ -7540,39 +8126,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1031" t="str">
+      <x:c r="A1" s="1073" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1032" t="str">
+      <x:c r="B1" s="1074" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1032" t="str">
+      <x:c r="C1" s="1074" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1032" t="str">
+      <x:c r="D1" s="1074" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1033" t="str">
+      <x:c r="E1" s="1075" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1049" t="n">
+      <x:c r="A2" s="1091" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="B2" s="1050" t="n">
+      <x:c r="B2" s="1092" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1050" t="n">
+      <x:c r="C2" s="1092" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1050" t="str">
-        <x:v>Gate 1/2: deploy the durable Telegram polling lifecycle with no-drop cutover and live restart proof; then deploy/live-verify remaining local fixes and finish the 1100-row phrase/dialogue DSL plus real-client Inline matrix.</x:v>
-      </x:c>
-      <x:c r="E2" s="1050" t="str">
-        <x:v>All current P0/P1 security findings are fixed locally; SG-P1-009 awaits deploy/cutover proof. BOT-001/BOT-004 and live Inline evidence remain incomplete. Latest local proof: clean DB reset/lint, pgTAP 20/20, 2877 tests, TypeScript/build/audit, lint 0 errors.</x:v>
+      <x:c r="D2" s="1092" t="str">
+        <x:v>Gate 2/3: build a polling-compatible synthetic update QA harness; run real-client Inline RU/UZ/EN, multi-turn dialogue, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1092" t="str">
+        <x:v>Production release 6fb71ec8 is live: three migrations applied, no-drop polling cutover complete, restart/re-election proof passed, monitor/web/security/Family Shield smoke passed. BOT-001/BOT-004 and real-client Inline/provider/soak evidence remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -7583,13 +8169,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1051" t="str">
+      <x:c r="A4" s="1093" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1051" t="str">
+      <x:c r="B4" s="1093" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1051" t="str">
+      <x:c r="C4" s="1093" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -7645,16 +8231,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1051" t="str">
+      <x:c r="A9" s="1093" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1051" t="str">
+      <x:c r="B9" s="1093" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1051" t="str">
+      <x:c r="C9" s="1093" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1051" t="str">
+      <x:c r="D9" s="1093" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -7731,13 +8317,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1051" t="str">
+      <x:c r="A15" s="1093" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1051" t="str">
+      <x:c r="B15" s="1093" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1051" t="str">
+      <x:c r="C15" s="1093" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -7773,14 +8359,14 @@
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="629" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="B18" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A18)</x:f>
-        <x:v>20</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C18" s="629" t="str">
-        <x:v>Code/tests pass locally; deployment/live proof missing.</x:v>
+        <x:v>Code is in production; targeted real-client or failure-path proof remains.</x:v>
       </x:c>
       <x:c r="D18" s="629"/>
       <x:c r="E18" s="629"/>
@@ -7791,7 +8377,7 @@
       </x:c>
       <x:c r="B19" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A19)</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="629" t="str">
         <x:v>Original path revalidated after deployment.</x:v>
@@ -7821,13 +8407,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1051" t="str">
+      <x:c r="A22" s="1093" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1051" t="str">
+      <x:c r="B22" s="1093" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1051" t="str">
+      <x:c r="C22" s="1093" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -7839,7 +8425,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>30</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -7853,7 +8439,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>0</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -7867,7 +8453,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -7891,11 +8477,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="310" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="311" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="312" priority="3" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="313" priority="4" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="314" priority="5" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="350" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="351" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="352" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="353" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="354" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="355" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="356" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -18750,46 +19338,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1031" t="str">
+      <x:c r="A1" s="1073" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1032" t="str">
+      <x:c r="B1" s="1074" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1032" t="str">
+      <x:c r="C1" s="1074" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1032" t="str">
+      <x:c r="D1" s="1074" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1032" t="str">
+      <x:c r="E1" s="1074" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1032" t="str">
+      <x:c r="F1" s="1074" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1032" t="str">
+      <x:c r="G1" s="1074" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1032" t="str">
+      <x:c r="H1" s="1074" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1032" t="str">
+      <x:c r="I1" s="1074" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1032" t="str">
+      <x:c r="J1" s="1074" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1032" t="str">
+      <x:c r="K1" s="1074" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1032" t="str">
+      <x:c r="L1" s="1074" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1032" t="str">
+      <x:c r="M1" s="1074" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1033" t="str">
+      <x:c r="N1" s="1075" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -18968,7 +19556,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D6" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E6" s="615" t="str">
         <x:v>Passed</x:v>
@@ -18980,13 +19568,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H6" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I6" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J6" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K6" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -18998,7 +19586,7 @@
         <x:v>HOT-001</x:v>
       </x:c>
       <x:c r="N6" s="615" t="str">
-        <x:v>Regression reproducer removed raw OTP; malformed URL display fails closed.</x:v>
+        <x:v>Regression reproducer removed raw OTP; malformed URL display fails closed. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -19012,7 +19600,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D7" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E7" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19024,13 +19612,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H7" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I7" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J7" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K7" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -19040,7 +19628,7 @@
       </x:c>
       <x:c r="M7" s="615" t="str"/>
       <x:c r="N7" s="615" t="str">
-        <x:v>Saved session language remains authoritative.</x:v>
+        <x:v>Saved session language remains authoritative. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -19054,7 +19642,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D8" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E8" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19066,13 +19654,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H8" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I8" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J8" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K8" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -19082,7 +19670,7 @@
       </x:c>
       <x:c r="M8" s="615" t="str"/>
       <x:c r="N8" s="615" t="str">
-        <x:v>HTTP 200 with Bot API ok:false is no longer treated as silent success.</x:v>
+        <x:v>HTTP 200 with Bot API ok:false is no longer treated as silent success. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -19096,7 +19684,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D9" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E9" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19108,13 +19696,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H9" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I9" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J9" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K9" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -19126,7 +19714,7 @@
         <x:v>HOT-003</x:v>
       </x:c>
       <x:c r="N9" s="615" t="str">
-        <x:v>Rules-only/app-owned reputation remains available; external URL providers are skipped.</x:v>
+        <x:v>Rules-only/app-owned reputation remains available; external URL providers are skipped. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -19140,7 +19728,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D10" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E10" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19152,13 +19740,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H10" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I10" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J10" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K10" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -19170,7 +19758,7 @@
         <x:v>HOT-004</x:v>
       </x:c>
       <x:c r="N10" s="615" t="str">
-        <x:v>Verified contact can mark Safe only when every reason is informational/protective; 475 risk tests pass.</x:v>
+        <x:v>Verified contact can mark Safe only when every reason is informational/protective; 475 risk tests pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -19228,7 +19816,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D12" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E12" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19240,10 +19828,10 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H12" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I12" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J12" s="618" t="n">
         <x:v>46214</x:v>
@@ -19258,7 +19846,7 @@
         <x:v>HOT-004</x:v>
       </x:c>
       <x:c r="N12" s="615" t="str">
-        <x:v>All 55 codes have compile-time trust impact, protective-action and Inline evidence/limitation entries; every high-risk single/pair produces advice. Real-client proof remains.</x:v>
+        <x:v>All 55 codes have compile-time trust impact, protective-action and Inline evidence/limitation entries; every high-risk single/pair produces advice. Real-client proof remains. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -19272,7 +19860,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D13" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E13" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19284,13 +19872,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H13" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I13" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J13" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K13" s="615" t="str">
         <x:v>Risk / Privacy</x:v>
@@ -19302,7 +19890,7 @@
         <x:v>HOT-002</x:v>
       </x:c>
       <x:c r="N13" s="615" t="str">
-        <x:v>External reputation receives scheme/origin only; local deterministic rules retain full-path analysis. 479 risk tests pass.</x:v>
+        <x:v>External reputation receives scheme/origin only; local deterministic rules retain full-path analysis. 479 risk tests pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -19316,7 +19904,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D14" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E14" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19328,13 +19916,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H14" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I14" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J14" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K14" s="615" t="str">
         <x:v>Risk / Privacy</x:v>
@@ -19344,7 +19932,7 @@
       </x:c>
       <x:c r="M14" s="615" t="str"/>
       <x:c r="N14" s="615" t="str">
-        <x:v>Malformed URL display fails closed to [link]; tg/telegram custom schemes redact centrally. 528 owning-suite tests pass.</x:v>
+        <x:v>Malformed URL display fails closed to [link]; tg/telegram custom schemes redact centrally. 528 owning-suite tests pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -19358,7 +19946,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D15" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E15" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19370,13 +19958,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H15" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I15" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J15" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K15" s="615" t="str">
         <x:v>AI / Risk</x:v>
@@ -19386,7 +19974,7 @@
       </x:c>
       <x:c r="M15" s="615" t="str"/>
       <x:c r="N15" s="615" t="str">
-        <x:v>Typed Telegram evidence is physically separate from model explanation; action-clause safety regressions pass in RU/UZ/EN. 198 owning + 2667 full tests pass.</x:v>
+        <x:v>Typed Telegram evidence is physically separate from model explanation; action-clause safety regressions pass in RU/UZ/EN. 198 owning + 2667 full tests pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -19400,7 +19988,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D16" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E16" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19412,13 +20000,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H16" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I16" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J16" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K16" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -19428,7 +20016,7 @@
       </x:c>
       <x:c r="M16" s="615" t="str"/>
       <x:c r="N16" s="615" t="str">
-        <x:v>Two-sided NFKC/confusable/transliteration keys, Unicode text boundaries and one-root-dot removal cover every registered Cyrillic alias/official domain plus hybrid IDNs.</x:v>
+        <x:v>Two-sided NFKC/confusable/transliteration keys, Unicode text boundaries and one-root-dot removal cover every registered Cyrillic alias/official domain plus hybrid IDNs. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -19442,7 +20030,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D17" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E17" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19454,13 +20042,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H17" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I17" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J17" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K17" s="615" t="str">
         <x:v>Telegram / Data</x:v>
@@ -19470,7 +20058,7 @@
       </x:c>
       <x:c r="M17" s="615" t="str"/>
       <x:c r="N17" s="615" t="str">
-        <x:v>Both exact-count reads and aggregate upsert fail closed with typed stage-only error; admin cannot return ok. Reconciliation/atomicity remains operational work.</x:v>
+        <x:v>Both exact-count reads and aggregate upsert fail closed with typed stage-only error; admin cannot return ok. Reconciliation/atomicity remains operational work. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -19484,7 +20072,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D18" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E18" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19496,13 +20084,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H18" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I18" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J18" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K18" s="615" t="str">
         <x:v>Media / Security</x:v>
@@ -19512,7 +20100,7 @@
       </x:c>
       <x:c r="M18" s="615" t="str"/>
       <x:c r="N18" s="615" t="str">
-        <x:v>4 MiB/4 MP decode cap; 1.5 MP, 5-attempt and 350 ms QR scan budgets; PNG/JPEG QR regressions pass.</x:v>
+        <x:v>4 MiB/4 MP decode cap; 1.5 MP, 5-attempt and 350 ms QR scan budgets; PNG/JPEG QR regressions pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -19526,7 +20114,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D19" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E19" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19538,13 +20126,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H19" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I19" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J19" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K19" s="615" t="str">
         <x:v>Backend / Platform</x:v>
@@ -19554,7 +20142,7 @@
       </x:c>
       <x:c r="M19" s="615" t="str"/>
       <x:c r="N19" s="615" t="str">
-        <x:v>Single isolated worker, four-job total backlog, 900 ms deadline and 128 MiB old-generation cap keep untrusted decode off the Node event loop.</x:v>
+        <x:v>Single isolated worker, four-job total backlog, 900 ms deadline and 128 MiB old-generation cap keep untrusted decode off the Node event loop. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -19568,7 +20156,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D20" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E20" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19580,13 +20168,13 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H20" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I20" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J20" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
       <x:c r="K20" s="615" t="str">
         <x:v>Backend / Data</x:v>
@@ -19596,7 +20184,7 @@
       </x:c>
       <x:c r="M20" s="615" t="str"/>
       <x:c r="N20" s="615" t="str">
-        <x:v>Production/Railway fails closed on missing config, hash/RPC error or invalid shape; dev/test fallback caps 4096 TTL/LRU keys and denies overflow.</x:v>
+        <x:v>Production/Railway fails closed on missing config, hash/RPC error or invalid shape; dev/test fallback caps 4096 TTL/LRU keys and denies overflow. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -19694,7 +20282,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D23" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E23" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19706,10 +20294,10 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H23" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I23" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J23" s="618" t="n">
         <x:v>46214</x:v>
@@ -19722,7 +20310,7 @@
       </x:c>
       <x:c r="M23" s="615" t="str"/>
       <x:c r="N23" s="615" t="str">
-        <x:v>The scheduled workflow explicitly requires Telegram secrets; pure policy proves a required skip fails even with fail-on-warn disabled. Live Actions evidence remains.</x:v>
+        <x:v>The scheduled workflow explicitly requires Telegram secrets; pure policy proves a required skip fails even with fail-on-warn disabled. Live Actions evidence remains. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -19778,7 +20366,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D25" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E25" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19790,10 +20378,10 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H25" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I25" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J25" s="618" t="n">
         <x:v>46214</x:v>
@@ -19806,7 +20394,7 @@
       </x:c>
       <x:c r="M25" s="615" t="str"/>
       <x:c r="N25" s="615" t="str">
-        <x:v>LastCheckSnapshot stores at most three enum methods/source classes/limitations; no raw evidence. 306 focused tests pass.</x:v>
+        <x:v>LastCheckSnapshot stores at most three enum methods/source classes/limitations; no raw evidence. 306 focused tests pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -19820,7 +20408,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D26" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E26" s="615" t="str">
         <x:v>Passed</x:v>
@@ -19832,10 +20420,10 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H26" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I26" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J26" s="618" t="n">
         <x:v>46214</x:v>
@@ -19848,7 +20436,7 @@
       </x:c>
       <x:c r="M26" s="615" t="str"/>
       <x:c r="N26" s="615" t="str">
-        <x:v>Confidence/methodology/trusted-person/recheck/disagreement actions pass RU/UZ/EN; free-text trusted-person has no side effect.</x:v>
+        <x:v>Confidence/methodology/trusted-person/recheck/disagreement actions pass RU/UZ/EN; free-text trusted-person has no side effect. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -19904,22 +20492,22 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D28" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E28" s="615" t="str">
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F28" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G28" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H28" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I28" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J28" s="618" t="n">
         <x:v>46214</x:v>
@@ -19927,12 +20515,10 @@
       <x:c r="K28" s="615" t="str">
         <x:v>Telegram / Data</x:v>
       </x:c>
-      <x:c r="L28" s="615" t="str">
-        <x:v>Deploy migrations + polling leader cutover + live restart proof</x:v>
-      </x:c>
+      <x:c r="L28" s="615" t="str"/>
       <x:c r="M28" s="615" t="str"/>
       <x:c r="N28" s="615" t="str">
-        <x:v>D-072 single-leader getUpdates(limit=1), metadata-only processing/completion leases, fenced session I/O and outbound effects pass clean DB reset/lint, 20 pgTAP assertions, 119 files / 2877 tests, TypeScript, build and audit. Production cutover remains pending and delivery is at-least-once.</x:v>
+        <x:v>Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -20257,11 +20843,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="D2:I36">
-    <x:cfRule type="containsText" dxfId="300" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="301" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="302" priority="3" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="303" priority="4" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="304" priority="5" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="336" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="337" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="338" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="339" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="340" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="341" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -20309,40 +20897,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1031" t="str">
+      <x:c r="A1" s="1073" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1032" t="str">
+      <x:c r="B1" s="1074" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1032" t="str">
+      <x:c r="C1" s="1074" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1032" t="str">
+      <x:c r="D1" s="1074" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1032" t="str">
+      <x:c r="E1" s="1074" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1032" t="str">
+      <x:c r="F1" s="1074" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1032" t="str">
+      <x:c r="G1" s="1074" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1032" t="str">
+      <x:c r="H1" s="1074" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1032" t="str">
+      <x:c r="I1" s="1074" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1032" t="str">
+      <x:c r="J1" s="1074" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1032" t="str">
+      <x:c r="K1" s="1074" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1033" t="str">
+      <x:c r="L1" s="1075" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -20363,7 +20951,7 @@
         <x:v>src/lib/risk/check-core.ts; src/lib/risk/rules.ts</x:v>
       </x:c>
       <x:c r="F2" s="614" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G2" s="614" t="str">
         <x:v>Risk Engine</x:v>
@@ -20372,16 +20960,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I2" s="614" t="str">
-        <x:v>Reproducer + exhaustive 55-code trust map + 475 risk tests</x:v>
+        <x:v>Reproducer + exhaustive 55-code trust map + 475 risk tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J2" s="614" t="str">
-        <x:v>Deploy and run real-client conflict matrix</x:v>
+        <x:v>Run remaining targeted and run real-client conflict matrix</x:v>
       </x:c>
       <x:c r="K2" s="614" t="str">
         <x:v>No risk-classified reason + verified contact returns Safe</x:v>
       </x:c>
       <x:c r="L2" s="617" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -20401,7 +20989,7 @@
         <x:v>src/lib/risk/verified-contacts.ts; src/lib/trust/official-directory.ts</x:v>
       </x:c>
       <x:c r="F3" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G3" s="615" t="str">
         <x:v>Risk / Data</x:v>
@@ -20410,16 +20998,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I3" s="615" t="str">
-        <x:v>Expired-handle reproducer + 47 focused tests</x:v>
+        <x:v>Expired-handle reproducer + 47 focused tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J3" s="615" t="str">
-        <x:v>Deploy; re-verify primary sources before reactivation</x:v>
+        <x:v>Run remaining targeted re-verify primary sources before reactivation</x:v>
       </x:c>
       <x:c r="K3" s="615" t="str">
         <x:v>Expired Telegram contacts cannot show badge/link, enter counts or change verdict</x:v>
       </x:c>
       <x:c r="L3" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -20439,7 +21027,7 @@
         <x:v>src/lib/risk/qr-decoder.ts; src/lib/telegram/handlers/check.ts</x:v>
       </x:c>
       <x:c r="F4" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G4" s="615" t="str">
         <x:v>Backend / Platform</x:v>
@@ -20448,16 +21036,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I4" s="615" t="str">
-        <x:v>4.2 s reproducer; worker/cap/queue/deadline regressions; 104 focus + 2645 full tests</x:v>
+        <x:v>4.2 s reproducer; worker/cap/queue/deadline regressions; 104 focus + 2645 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J4" s="615" t="str">
-        <x:v>Deploy; run legitimate QR smoke and 60-minute worker soak/crash-restart</x:v>
+        <x:v>Run remaining targeted run legitimate QR smoke and 60-minute worker soak/crash-restart</x:v>
       </x:c>
       <x:c r="K4" s="615" t="str">
         <x:v>No untrusted PNG/JPEG/QR decode runs on the Node event loop; queue and per-job work stay bounded</x:v>
       </x:c>
       <x:c r="L4" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -20477,7 +21065,7 @@
         <x:v>src/lib/risk/check-core.ts; src/lib/risk/url-reputation.server.ts</x:v>
       </x:c>
       <x:c r="F5" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G5" s="615" t="str">
         <x:v>Risk / Privacy</x:v>
@@ -20486,16 +21074,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I5" s="615" t="str">
-        <x:v>Bearer-path reproducer + 52 focused + 479 risk tests</x:v>
+        <x:v>Bearer-path reproducer + 52 focused + 479 risk tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J5" s="615" t="str">
-        <x:v>Deploy and run provider compatibility smoke</x:v>
+        <x:v>Run remaining targeted and run provider compatibility smoke</x:v>
       </x:c>
       <x:c r="K5" s="615" t="str">
         <x:v>Outgoing provider capture contains origin only and no path/query/userinfo/fragment secrets</x:v>
       </x:c>
       <x:c r="L5" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -20515,7 +21103,7 @@
         <x:v>src/lib/risk/shared-rate-limit.server.ts; src/lib/risk/rate-limit.ts</x:v>
       </x:c>
       <x:c r="F6" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G6" s="615" t="str">
         <x:v>Backend / Data</x:v>
@@ -20524,16 +21112,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I6" s="615" t="str">
-        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests</x:v>
+        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J6" s="615" t="str">
-        <x:v>Deploy; force shared config/hash/RPC/shape failures and verify 429/no sink work</x:v>
+        <x:v>Run remaining targeted force shared config/hash/RPC/shape failures and verify 429/no sink work</x:v>
       </x:c>
       <x:c r="K6" s="615" t="str">
         <x:v>Production shared-control failure grants no local allowance; fallback state stays &lt;=4096 keys with bounded cleanup</x:v>
       </x:c>
       <x:c r="L6" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -20553,7 +21141,7 @@
         <x:v>src/lib/risk/detect.ts; report/appeal/Telegram draft paths</x:v>
       </x:c>
       <x:c r="F7" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G7" s="615" t="str">
         <x:v>Risk / Privacy</x:v>
@@ -20562,16 +21150,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I7" s="615" t="str">
-        <x:v>7-failure reproducer + 71 focused + 528 owning-suite tests</x:v>
+        <x:v>7-failure reproducer + 71 focused + 528 owning-suite tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J7" s="615" t="str">
-        <x:v>Deploy and run report/appeal/Telegram draft smoke</x:v>
+        <x:v>Run remaining targeted and run report/appeal/Telegram draft smoke</x:v>
       </x:c>
       <x:c r="K7" s="615" t="str">
         <x:v>No raw malformed URL or tg/telegram scheme reaches persistence/display/session/moderation</x:v>
       </x:c>
       <x:c r="L7" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -20591,7 +21179,7 @@
         <x:v>package.json; bun.lock; vite.config.ts; toolchain-config.test.ts</x:v>
       </x:c>
       <x:c r="F8" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="G8" s="615" t="str">
         <x:v>Platform</x:v>
@@ -20600,16 +21188,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I8" s="615" t="str">
-        <x:v>npm audit 7-&gt;0; bun audit 2-&gt;0; 127.0.0.1 listener proof; 3 security + 2655 full tests; Bun build</x:v>
+        <x:v>npm audit 7-&gt;0; bun audit 2-&gt;0; 127.0.0.1 listener proof; 3 security + 2655 full tests; Bun build. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J8" s="615" t="str">
-        <x:v>Commit/deploy; rerun Docker build when Docker Desktop engine is available</x:v>
+        <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
       </x:c>
       <x:c r="K8" s="615" t="str">
         <x:v>Canonical npm/Bun graphs have zero known advisories; default dev listener is loopback and external bind requires an explicit CLI flag</x:v>
       </x:c>
       <x:c r="L8" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -20629,7 +21217,7 @@
         <x:v>src/lib/telegram/handlers/inline.ts</x:v>
       </x:c>
       <x:c r="F9" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G9" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -20638,16 +21226,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I9" s="615" t="str">
-        <x:v>Regression test + 2026 Telegram suite</x:v>
+        <x:v>Regression test + 2026 Telegram suite. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J9" s="615" t="str">
-        <x:v>Deploy and verify real clients</x:v>
+        <x:v>Run remaining targeted and verify real clients</x:v>
       </x:c>
       <x:c r="K9" s="615" t="str">
         <x:v>No raw secret in any Inline article field</x:v>
       </x:c>
       <x:c r="L9" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -20667,7 +21255,7 @@
         <x:v>src/lib/telegram/router.ts</x:v>
       </x:c>
       <x:c r="F10" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G10" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -20676,16 +21264,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I10" s="615" t="str">
-        <x:v>Router regression + 2026 Telegram suite</x:v>
+        <x:v>Router regression + 2026 Telegram suite. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J10" s="615" t="str">
-        <x:v>Deploy and live-check RU/UZ/EN</x:v>
+        <x:v>Run remaining targeted and live-check RU/UZ/EN</x:v>
       </x:c>
       <x:c r="K10" s="615" t="str">
         <x:v>Telegram hint used only when no saved session exists</x:v>
       </x:c>
       <x:c r="L10" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -20705,7 +21293,7 @@
         <x:v>src/lib/telegram/api.server.ts; handlers/inline.ts</x:v>
       </x:c>
       <x:c r="F11" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G11" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -20714,16 +21302,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I11" s="615" t="str">
-        <x:v>Typed failure + parse retry tests</x:v>
+        <x:v>Typed failure + parse retry tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J11" s="615" t="str">
-        <x:v>Deploy and observe real answer result</x:v>
+        <x:v>Run remaining targeted and observe real answer result</x:v>
       </x:c>
       <x:c r="K11" s="615" t="str">
         <x:v>Bot API failure is observable without raw query/result</x:v>
       </x:c>
       <x:c r="L11" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -20743,7 +21331,7 @@
         <x:v>src/lib/telegram/handlers/inline.ts</x:v>
       </x:c>
       <x:c r="F12" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G12" s="615" t="str">
         <x:v>Telegram / Backend</x:v>
@@ -20752,16 +21340,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I12" s="615" t="str">
-        <x:v>256 boundary and skipUrlReputation tests</x:v>
+        <x:v>256 boundary and skipUrlReputation tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J12" s="615" t="str">
-        <x:v>Deploy and run 20-40 prefix sequence</x:v>
+        <x:v>Run remaining targeted and run 20-40 prefix sequence</x:v>
       </x:c>
       <x:c r="K12" s="615" t="str">
         <x:v>No external provider call or premature rate-limit while typing</x:v>
       </x:c>
       <x:c r="L12" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -20781,7 +21369,7 @@
         <x:v>src/lib/risk/risk-passport.ts; web/embed/Inline renderers</x:v>
       </x:c>
       <x:c r="F13" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G13" s="615" t="str">
         <x:v>AI / Risk</x:v>
@@ -20790,16 +21378,16 @@
         <x:v>Gate 1/2</x:v>
       </x:c>
       <x:c r="I13" s="615" t="str">
-        <x:v>Forged-marker reproducer + typed evidence isolation + 198 owning + 2667 full tests</x:v>
+        <x:v>Forged-marker reproducer + typed evidence isolation + 198 owning + 2667 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J13" s="615" t="str">
-        <x:v>Deploy and verify forged-marker corpus across web/embed/Inline</x:v>
+        <x:v>Run remaining targeted and verify forged-marker corpus across web/embed/Inline</x:v>
       </x:c>
       <x:c r="K13" s="615" t="str">
         <x:v>Model explanation cannot select a passport or become structured evidence; only separately typed deterministic text is parsed</x:v>
       </x:c>
       <x:c r="L13" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -20819,7 +21407,7 @@
         <x:v>src/lib/risk/ai-output-safety.ts</x:v>
       </x:c>
       <x:c r="F14" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G14" s="615" t="str">
         <x:v>AI / Risk</x:v>
@@ -20828,16 +21416,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I14" s="615" t="str">
-        <x:v>Six mixed-clause reproducers in RU/UZ/EN + five repeated focused runs + 2667 full tests</x:v>
+        <x:v>Six mixed-clause reproducers in RU/UZ/EN + five repeated focused runs + 2667 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J14" s="615" t="str">
-        <x:v>Deploy and run provider-output adversarial smoke</x:v>
+        <x:v>Run remaining targeted and run provider-output adversarial smoke</x:v>
       </x:c>
       <x:c r="K14" s="615" t="str">
         <x:v>Safe negation is clause-local; a sibling transfer/wallet/APK request is blocked and legitimate multi-clause warnings remain allowed</x:v>
       </x:c>
       <x:c r="L14" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -20857,7 +21445,7 @@
         <x:v>src/lib/telegram/advice-filter.ts; format.ts</x:v>
       </x:c>
       <x:c r="F15" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G15" s="615" t="str">
         <x:v>Telegram / Risk</x:v>
@@ -20866,16 +21454,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I15" s="615" t="str">
-        <x:v>8-failure reproducer + exhaustive 55-code action policy + 227 Telegram focus + 2675 full tests</x:v>
+        <x:v>8-failure reproducer + exhaustive 55-code action policy + 227 Telegram focus + 2675 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J15" s="615" t="str">
-        <x:v>Deploy and run RU/UZ/EN direct-bot smoke for confirmed report/phishing/malware</x:v>
+        <x:v>Run remaining targeted and run RU/UZ/EN direct-bot smoke for confirmed report/phishing/malware</x:v>
       </x:c>
       <x:c r="K15" s="615" t="str">
         <x:v>Every high-risk single/pair reason set produces immediate action; no high-risk context-request fallback</x:v>
       </x:c>
       <x:c r="L15" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -20895,7 +21483,7 @@
         <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
       </x:c>
       <x:c r="F16" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G16" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -20904,16 +21492,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I16" s="615" t="str">
-        <x:v>8-failure reproducer + full registry Cyrillic/official/hybrid corpus + 165 focus + 2733 full tests</x:v>
+        <x:v>8-failure reproducer + full registry Cyrillic/official/hybrid corpus + 165 focus + 2733 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J16" s="615" t="str">
-        <x:v>Deploy; run external reputation compatibility and RU/UZ/EN client smoke</x:v>
+        <x:v>Run remaining targeted run external reputation compatibility and RU/UZ/EN client smoke</x:v>
       </x:c>
       <x:c r="K16" s="615" t="str">
         <x:v>Cyrillic text and full/hybrid IDNs retain brand signal; one DNS root dot preserves official-domain suppression</x:v>
       </x:c>
       <x:c r="L16" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -20933,7 +21521,7 @@
         <x:v>src/lib/telegram/reputation.server.ts; admin.functions.ts</x:v>
       </x:c>
       <x:c r="F17" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G17" s="615" t="str">
         <x:v>Telegram / Data</x:v>
@@ -20942,16 +21530,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I17" s="615" t="str">
-        <x:v>5-failure reproducer + 158 ownership + 2738 full tests; stage-only privacy regression</x:v>
+        <x:v>5-failure reproducer + 158 ownership + 2738 full tests; stage-only privacy regression. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J17" s="615" t="str">
-        <x:v>Deploy; force both count failures and upsert failure; verify alert/retry UX</x:v>
+        <x:v>Run remaining targeted force both count failures and upsert failure; verify alert/retry UX</x:v>
       </x:c>
       <x:c r="K17" s="615" t="str">
         <x:v>Read/shape/upsert failure never becomes zero or admin success; telemetry omits target/DB message</x:v>
       </x:c>
       <x:c r="L17" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46214</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -20971,7 +21559,7 @@
         <x:v>.github/workflows/prod-monitor.yml; scripts/prod-monitor.ts; scripts/prod-monitor-policy.ts</x:v>
       </x:c>
       <x:c r="F18" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="G18" s="615" t="str">
         <x:v>DevOps</x:v>
@@ -20980,10 +21568,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I18" s="615" t="str">
-        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint</x:v>
+        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J18" s="615" t="str">
-        <x:v>Run Actions with secrets; controlled missing-secret failure; restore and pass</x:v>
+        <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
       </x:c>
       <x:c r="K18" s="615" t="str">
         <x:v>A required skipped check makes the run red independently of fail-on-warn and alert delivery</x:v>
@@ -21009,7 +21597,7 @@
         <x:v>src/lib/telegram/inline-reason-presentation.ts; handlers/inline.ts</x:v>
       </x:c>
       <x:c r="F19" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G19" s="615" t="str">
         <x:v>Telegram / Risk</x:v>
@@ -21018,10 +21606,10 @@
         <x:v>Gate 2/3</x:v>
       </x:c>
       <x:c r="I19" s="615" t="str">
-        <x:v>55x3 real-adapter matrix plus canonical collector/methodology regressions; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2</x:v>
+        <x:v>55x3 real-adapter matrix plus canonical collector/methodology regressions; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J19" s="615" t="str">
-        <x:v>Deploy; run Desktop/Android/iOS RU/UZ/EN visual/insertion matrix</x:v>
+        <x:v>Run remaining targeted run Desktop/Android/iOS RU/UZ/EN visual/insertion matrix</x:v>
       </x:c>
       <x:c r="K19" s="615" t="str">
         <x:v>All reason codes have typed priority, honest method/source and limitation; preview &lt;=120 chars and full insert &lt;=4096</x:v>
@@ -21047,7 +21635,7 @@
         <x:v>src/lib/telegram/check-followup.ts; session.server.ts; live-phrase-cases.ts</x:v>
       </x:c>
       <x:c r="F20" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G20" s="615" t="str">
         <x:v>Telegram / Product</x:v>
@@ -21056,10 +21644,10 @@
         <x:v>Gate 2</x:v>
       </x:c>
       <x:c r="I20" s="615" t="str">
-        <x:v>24 post-check rows inside the 239-phrase live matrix; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2</x:v>
+        <x:v>24 post-check rows inside the 239-phrase live matrix; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J20" s="615" t="str">
-        <x:v>Deploy; run real multi-turn transcripts and session-loss/restart cases</x:v>
+        <x:v>Run remaining targeted run real multi-turn transcripts and session-loss/restart cases</x:v>
       </x:c>
       <x:c r="K20" s="615" t="str">
         <x:v>Helper phrases never create checks or trusted-contact side effects; methodology is provenance-bound and RU/UZ/EN parallel</x:v>
@@ -21085,7 +21673,7 @@
         <x:v>src/lib/telegram/session.server.ts; update-{lifecycle,execution,dispatch}.server.ts; updates-poller.server.ts; outbound-effect-fence.server.ts; webhook.server.ts; api.server.ts; prod-monitor.ts; 20260711010000 + 20260711050337 migrations</x:v>
       </x:c>
       <x:c r="F21" s="615" t="str">
-        <x:v>Fixed Local / Awaiting Deploy</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="G21" s="615" t="str">
         <x:v>Telegram / Data</x:v>
@@ -21094,10 +21682,10 @@
         <x:v>Gate 2</x:v>
       </x:c>
       <x:c r="I21" s="615" t="str">
-        <x:v>Single leader, completion-gated offset, failure reacquisition, stale leader/update fence rejection, fenced session/effects; clean DB reset + no lint errors + pgTAP 20/20 + 2877 app tests + production build</x:v>
+        <x:v>Single leader, completion-gated offset, failure reacquisition, stale leader/update fence rejection, fenced session/effects; clean DB reset + no lint errors + pgTAP 20/20 + 2877 app tests + production build. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
       </x:c>
       <x:c r="J21" s="615" t="str">
-        <x:v>Deploy both 20260711 migrations and polling build; require authenticated leader health 200; run no-drop cutover; update scheduled monitor mode; capture restart and live multi-turn proof</x:v>
+        <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
       </x:c>
       <x:c r="K21" s="615" t="str">
         <x:v>No claimed-update loss; offset advances only after completion; stale worker cannot read/write session or send Bot API effect; no raw payload stored; cutover preserves pending updates; live restart proof passes</x:v>
@@ -21108,18 +21696,20 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="305" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="306" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="307" priority="3" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="308" priority="4" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="309" priority="5" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="343" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="344" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="345" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="346" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="347" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="348" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="349" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">
       <x:formula1>"P0,P1,P2"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F21">
-      <x:formula1>"Open,In Progress,Fixed Local / Awaiting Deploy,Closed,Accepted Risk"</x:formula1>
+      <x:formula1>"Open,In Progress,Fixed Local / Awaiting Deploy,Deployed / Awaiting Live Verification,Closed,Accepted Risk"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: record polling Telegram QA evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfeaee7bc0b834e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re16c2e8b86334408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae58f0db205947e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R39b958761c7c45c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R6e0747c5cee848a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4991b91a2c7e4b1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R850055f2750f4ce8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rcee7bd7e590f466e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcb59f627b8cd4a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9c8db7844cea48d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rfa61bc3e0ec14922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5c959531144f46bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R5076aa6d9d654b98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb24a201d182243ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re1ae6ddc44034564"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd96fa0f73dc044ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="187">
+  <x:fills count="190">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1025,6 +1025,21 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1112,7 +1127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1094">
+  <x:cellXfs count="1116">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -3919,11 +3934,59 @@
     <x:xf numFmtId="0" fontId="1" fillId="185" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="187" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="187" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="188" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="188" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="188" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="189" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="189" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="189" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="189" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="189" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="189" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="188" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="357">
+  <x:dxfs count="378">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7353,6 +7416,237 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -8126,39 +8420,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1073" t="str">
+      <x:c r="A1" s="1094" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1074" t="str">
+      <x:c r="B1" s="1095" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1074" t="str">
+      <x:c r="C1" s="1095" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1074" t="str">
+      <x:c r="D1" s="1095" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1075" t="str">
+      <x:c r="E1" s="1096" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1091" t="n">
+      <x:c r="A2" s="1113" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="B2" s="1092" t="n">
+      <x:c r="B2" s="1114" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1092" t="n">
+      <x:c r="C2" s="1114" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1092" t="str">
-        <x:v>Gate 2/3: build a polling-compatible synthetic update QA harness; run real-client Inline RU/UZ/EN, multi-turn dialogue, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
-      </x:c>
-      <x:c r="E2" s="1092" t="str">
-        <x:v>Production release 6fb71ec8 is live: three migrations applied, no-drop polling cutover complete, restart/re-election proof passed, monitor/web/security/Family Shield smoke passed. BOT-001/BOT-004 and real-client Inline/provider/soak evidence remain incomplete.</x:v>
+      <x:c r="D2" s="1114" t="str">
+        <x:v>Gate 2/3: finish live recheck/disagreement replies; run real-client Inline RU/UZ/EN, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1114" t="str">
+        <x:v>Production release 6fb71ec8 and QA PR #73 / ae182707 are live in main. Polling-compatible confidence/trusted-person/domain-methodology QA and cleanup read-back passed. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -8169,13 +8463,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1093" t="str">
+      <x:c r="A4" s="1115" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1093" t="str">
+      <x:c r="B4" s="1115" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1093" t="str">
+      <x:c r="C4" s="1115" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -8231,16 +8525,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1093" t="str">
+      <x:c r="A9" s="1115" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1093" t="str">
+      <x:c r="B9" s="1115" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1093" t="str">
+      <x:c r="C9" s="1115" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1093" t="str">
+      <x:c r="D9" s="1115" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -8270,7 +8564,7 @@
       </x:c>
       <x:c r="C11" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A11)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D11" s="629" t="n">
         <x:v>2</x:v>
@@ -8317,13 +8611,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1093" t="str">
+      <x:c r="A15" s="1115" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1093" t="str">
+      <x:c r="B15" s="1115" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1093" t="str">
+      <x:c r="C15" s="1115" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -8363,7 +8657,7 @@
       </x:c>
       <x:c r="B18" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A18)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C18" s="629" t="str">
         <x:v>Code is in production; targeted real-client or failure-path proof remains.</x:v>
@@ -8377,7 +8671,7 @@
       </x:c>
       <x:c r="B19" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A19)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C19" s="629" t="str">
         <x:v>Original path revalidated after deployment.</x:v>
@@ -8407,13 +8701,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1093" t="str">
+      <x:c r="A22" s="1115" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1093" t="str">
+      <x:c r="B22" s="1115" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1093" t="str">
+      <x:c r="C22" s="1115" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -8439,7 +8733,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -8453,7 +8747,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -8477,13 +8771,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="350" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="351" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="352" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="353" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="354" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="355" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="356" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="371" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="372" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="373" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="374" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="375" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="376" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="377" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19310,6 +19604,32 @@
       </x:c>
       <x:c r="H91" t="str">
         <x:v>Proceed to residual UX/logistics QA: direct/inline phrase sweep, short UZ voice spot-checks after STT reset, and image provider routine spot-checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>QA-POLLING-DISPATCH-2026-07-11</x:v>
+      </x:c>
+      <x:c r="B92" s="1097" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>Polling-compatible Telegram multi-turn production QA</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>railway run npm run prod:telegram-polling-dispatch-smoke -- https://scam-guard-main-production.up.railway.app; PR #73 CI app + Supabase/pgTAP</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Passed: active polling leader 200; confidence, trusted-person and suspicious-domain methodology replies delivered; no follow-up check rows; cleanup read-back passed; 2881/2881 tests; build/audit green.</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>SG-P1-008, BOT-002, BOT-003, BOT-006</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>Bot API guard allowed only sendMessage/sendChatAction to TELEGRAM_QA_CHAT_ID. Synthetic payload remained in-process and did not acquire the polling leader. PR #73 / ae182707 merged; production monitor passed with pending=0.</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>Complete live recheck/disagreement replies, then real Telegram Desktop/mobile Inline RU/UZ/EN visual matrix. Do not treat synthetic inline ids as client evidence.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19338,46 +19658,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1073" t="str">
+      <x:c r="A1" s="1094" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1074" t="str">
+      <x:c r="B1" s="1095" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1074" t="str">
+      <x:c r="C1" s="1095" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1074" t="str">
+      <x:c r="D1" s="1095" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1074" t="str">
+      <x:c r="E1" s="1095" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1074" t="str">
+      <x:c r="F1" s="1095" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1074" t="str">
+      <x:c r="G1" s="1095" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1074" t="str">
+      <x:c r="H1" s="1095" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1074" t="str">
+      <x:c r="I1" s="1095" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1074" t="str">
+      <x:c r="J1" s="1095" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1074" t="str">
+      <x:c r="K1" s="1095" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1074" t="str">
+      <x:c r="L1" s="1095" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1074" t="str">
+      <x:c r="M1" s="1095" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1075" t="str">
+      <x:c r="N1" s="1096" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -20372,16 +20692,16 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F25" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G25" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H25" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I25" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J25" s="618" t="n">
         <x:v>46214</x:v>
@@ -20389,12 +20709,10 @@
       <x:c r="K25" s="615" t="str">
         <x:v>Telegram / Risk</x:v>
       </x:c>
-      <x:c r="L25" s="615" t="str">
-        <x:v>TRUST-003</x:v>
-      </x:c>
+      <x:c r="L25" s="615" t="str"/>
       <x:c r="M25" s="615" t="str"/>
       <x:c r="N25" s="615" t="str">
-        <x:v>LastCheckSnapshot stores at most three enum methods/source classes/limitations; no raw evidence. 306 focused tests pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
+        <x:v>Production methodology follow-up named deterministic domain evidence and its limitation, did not claim a hidden owner/source, created no new check, and cleaned its synthetic session/check rows. PR #73 / ae182707; full suite 2881/2881.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -20432,11 +20750,11 @@
         <x:v>Telegram / Copy</x:v>
       </x:c>
       <x:c r="L26" s="615" t="str">
-        <x:v>BOT-001..002</x:v>
+        <x:v>BOT-001 + live recheck/disagreement</x:v>
       </x:c>
       <x:c r="M26" s="615" t="str"/>
       <x:c r="N26" s="615" t="str">
-        <x:v>Confidence/methodology/trusted-person/recheck/disagreement actions pass RU/UZ/EN; free-text trusted-person has no side effect. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
+        <x:v>RU production live QA passed confidence, methodology and trusted-person replies with no cold check or trusted-contact side effect. Automated RU/UZ/EN coverage passes all five actions; live recheck/disagreement remain before this row can pass. PR #73 / ae182707.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -20478,7 +20796,7 @@
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>24 RU/UZ/EN post-check rows are enforced inside the 239-row live matrix; the planned 1100-row canonical corpus and multi-turn dialogue DSL remain.</x:v>
+        <x:v>The polling-compatible production harness now covers three critical multi-turn replies, but the planned 1100-row canonical corpus/dialogue DSL and broader live transcript set remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -20518,36 +20836,36 @@
       <x:c r="L28" s="615" t="str"/>
       <x:c r="M28" s="615" t="str"/>
       <x:c r="N28" s="615" t="str">
-        <x:v>Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="615" t="str">
-        <x:v>INL-001</x:v>
+        <x:v>BOT-006</x:v>
       </x:c>
       <x:c r="B29" s="615" t="str">
-        <x:v>Inline full backend/protocol/failure/privacy matrix</x:v>
+        <x:v>Polling-compatible production Telegram response harness</x:v>
       </x:c>
       <x:c r="C29" s="615" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D29" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E29" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F29" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G29" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H29" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I29" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J29" s="618" t="n">
         <x:v>46214</x:v>
@@ -20555,28 +20873,24 @@
       <x:c r="K29" s="615" t="str">
         <x:v>Telegram / QA</x:v>
       </x:c>
-      <x:c r="L29" s="615" t="str">
-        <x:v>Gate 1 Inline deploy</x:v>
-      </x:c>
-      <x:c r="M29" s="615" t="str">
-        <x:v>INL-P0-01..04</x:v>
-      </x:c>
+      <x:c r="L29" s="615" t="str"/>
+      <x:c r="M29" s="615" t="str"/>
       <x:c r="N29" s="615" t="str">
-        <x:v>55x3 reason presentations now pass through the real adapter; remaining matrix includes webhook config, faults, prefix/load and stateless follow-ups.</x:v>
+        <x:v>PR #73 / ae182707. Authenticated leader health 200; synthetic payload stays in-process; Bot API is fail-closed to TELEGRAM_QA_CHAT_ID; exact confidence/trusted-person/domain-methodology replies passed; check/session cleanup read-back passed. Inline visual delivery remains a separate client gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="615" t="str">
-        <x:v>INL-002</x:v>
+        <x:v>INL-001</x:v>
       </x:c>
       <x:c r="B30" s="615" t="str">
-        <x:v>Telegram Desktop/Android/iOS real-client visual matrix</x:v>
+        <x:v>Inline full backend/protocol/failure/privacy matrix</x:v>
       </x:c>
       <x:c r="C30" s="615" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D30" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E30" s="615" t="str">
         <x:v>Pending</x:v>
@@ -20593,39 +20907,43 @@
       <x:c r="I30" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J30" s="618"/>
+      <x:c r="J30" s="618" t="n">
+        <x:v>46214</x:v>
+      </x:c>
       <x:c r="K30" s="615" t="str">
-        <x:v>QA / Product</x:v>
+        <x:v>Telegram / QA</x:v>
       </x:c>
       <x:c r="L30" s="615" t="str">
-        <x:v>Devices + staging deploy</x:v>
-      </x:c>
-      <x:c r="M30" s="615" t="str"/>
+        <x:v>Gate 1 Inline deploy</x:v>
+      </x:c>
+      <x:c r="M30" s="615" t="str">
+        <x:v>INL-P0-01..04</x:v>
+      </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients.</x:v>
+        <x:v>55x3 reason presentations now pass through the real adapter; remaining matrix includes webhook config, faults, prefix/load and stateless follow-ups.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="615" t="str">
-        <x:v>OPS-001</x:v>
+        <x:v>INL-002</x:v>
       </x:c>
       <x:c r="B31" s="615" t="str">
-        <x:v>Mandatory lint/format/type/coverage/SAST/secret/dependency/container gates</x:v>
+        <x:v>Telegram Desktop/Android/iOS real-client visual matrix</x:v>
       </x:c>
       <x:c r="C31" s="615" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="D31" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E31" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F31" s="615" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="G31" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="H31" s="615" t="str">
         <x:v>Not Deployed</x:v>
@@ -20633,30 +20951,30 @@
       <x:c r="I31" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J31" s="618" t="n">
-        <x:v>46214</x:v>
-      </x:c>
+      <x:c r="J31" s="618"/>
       <x:c r="K31" s="615" t="str">
-        <x:v>DevOps / Security</x:v>
-      </x:c>
-      <x:c r="L31" s="615" t="str"/>
+        <x:v>QA / Product</x:v>
+      </x:c>
+      <x:c r="L31" s="615" t="str">
+        <x:v>Devices + staging deploy</x:v>
+      </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>Full lint now passes with 0 errors/8 warnings; typecheck, 2863x2 tests, npm audits and build pass. Coverage/SAST/secret/container gates still require CI evidence; High/Critical blocks release or has an expiry-bound exception.</x:v>
+        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="615" t="str">
-        <x:v>OPS-002</x:v>
+        <x:v>OPS-001</x:v>
       </x:c>
       <x:c r="B32" s="615" t="str">
-        <x:v>SBOM, signing/provenance and immutable dependency pins</x:v>
+        <x:v>Mandatory lint/format/type/coverage/SAST/secret/dependency/container gates</x:v>
       </x:c>
       <x:c r="C32" s="615" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D32" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E32" s="615" t="str">
         <x:v>Pending</x:v>
@@ -20665,7 +20983,7 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="G32" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H32" s="615" t="str">
         <x:v>Not Deployed</x:v>
@@ -20673,22 +20991,24 @@
       <x:c r="I32" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J32" s="618"/>
+      <x:c r="J32" s="618" t="n">
+        <x:v>46214</x:v>
+      </x:c>
       <x:c r="K32" s="615" t="str">
         <x:v>DevOps / Security</x:v>
       </x:c>
       <x:c r="L32" s="615" t="str"/>
       <x:c r="M32" s="615" t="str"/>
       <x:c r="N32" s="615" t="str">
-        <x:v>Release artifact is bound to commit and immutable dependencies.</x:v>
+        <x:v>Full lint now passes with 0 errors/8 warnings; typecheck, 2863x2 tests, npm audits and build pass. Coverage/SAST/secret/container gates still require CI evidence; High/Critical blocks release or has an expiry-bound exception.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="615" t="str">
-        <x:v>OPS-003</x:v>
+        <x:v>OPS-002</x:v>
       </x:c>
       <x:c r="B33" s="615" t="str">
-        <x:v>Browser E2E, accessibility, visual and performance budgets</x:v>
+        <x:v>SBOM, signing/provenance and immutable dependency pins</x:v>
       </x:c>
       <x:c r="C33" s="615" t="str">
         <x:v>P2</x:v>
@@ -20700,7 +21020,7 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="F33" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="G33" s="615" t="str">
         <x:v>Pending</x:v>
@@ -20713,20 +21033,20 @@
       </x:c>
       <x:c r="J33" s="618"/>
       <x:c r="K33" s="615" t="str">
-        <x:v>Frontend / QA</x:v>
+        <x:v>DevOps / Security</x:v>
       </x:c>
       <x:c r="L33" s="615" t="str"/>
       <x:c r="M33" s="615" t="str"/>
       <x:c r="N33" s="615" t="str">
-        <x:v>Critical web journeys and agreed budgets block regressions.</x:v>
+        <x:v>Release artifact is bound to commit and immutable dependencies.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="615" t="str">
-        <x:v>OPS-004</x:v>
+        <x:v>OPS-003</x:v>
       </x:c>
       <x:c r="B34" s="615" t="str">
-        <x:v>Privacy/legal/appeal/retention/partner-governance review</x:v>
+        <x:v>Browser E2E, accessibility, visual and performance budgets</x:v>
       </x:c>
       <x:c r="C34" s="615" t="str">
         <x:v>P2</x:v>
@@ -20751,22 +21071,20 @@
       </x:c>
       <x:c r="J34" s="618"/>
       <x:c r="K34" s="615" t="str">
-        <x:v>Product / Legal</x:v>
-      </x:c>
-      <x:c r="L34" s="615" t="str">
-        <x:v>External legal review</x:v>
-      </x:c>
+        <x:v>Frontend / QA</x:v>
+      </x:c>
+      <x:c r="L34" s="615" t="str"/>
       <x:c r="M34" s="615" t="str"/>
       <x:c r="N34" s="615" t="str">
-        <x:v>One current approved privacy spec and truthful public copy.</x:v>
+        <x:v>Critical web journeys and agreed budgets block regressions.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="615" t="str">
-        <x:v>DR-001</x:v>
+        <x:v>OPS-004</x:v>
       </x:c>
       <x:c r="B35" s="615" t="str">
-        <x:v>Backup restore, RPO/RTO, rollback and key-rotation drill</x:v>
+        <x:v>Privacy/legal/appeal/retention/partner-governance review</x:v>
       </x:c>
       <x:c r="C35" s="615" t="str">
         <x:v>P2</x:v>
@@ -20791,25 +21109,25 @@
       </x:c>
       <x:c r="J35" s="618"/>
       <x:c r="K35" s="615" t="str">
-        <x:v>DevOps / Data</x:v>
+        <x:v>Product / Legal</x:v>
       </x:c>
       <x:c r="L35" s="615" t="str">
-        <x:v>Production access</x:v>
+        <x:v>External legal review</x:v>
       </x:c>
       <x:c r="M35" s="615" t="str"/>
       <x:c r="N35" s="615" t="str">
-        <x:v>Restore/rollback/key rotation evidence exists and is current.</x:v>
+        <x:v>One current approved privacy spec and truthful public copy.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="615" t="str">
-        <x:v>RC-001</x:v>
+        <x:v>DR-001</x:v>
       </x:c>
       <x:c r="B36" s="615" t="str">
-        <x:v>RC commit, fresh security scan and 72-hour closed canary</x:v>
+        <x:v>Backup restore, RPO/RTO, rollback and key-rotation drill</x:v>
       </x:c>
       <x:c r="C36" s="615" t="str">
-        <x:v>P1</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="D36" s="615" t="str">
         <x:v>Not Started</x:v>
@@ -20831,13 +21149,53 @@
       </x:c>
       <x:c r="J36" s="618"/>
       <x:c r="K36" s="615" t="str">
-        <x:v>Release Team</x:v>
+        <x:v>DevOps / Data</x:v>
       </x:c>
       <x:c r="L36" s="615" t="str">
-        <x:v>All P0/P1 gates</x:v>
+        <x:v>Production access</x:v>
       </x:c>
       <x:c r="M36" s="615" t="str"/>
       <x:c r="N36" s="615" t="str">
+        <x:v>Restore/rollback/key rotation evidence exists and is current.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="615" t="str">
+        <x:v>RC-001</x:v>
+      </x:c>
+      <x:c r="B37" s="615" t="str">
+        <x:v>RC commit, fresh security scan and 72-hour closed canary</x:v>
+      </x:c>
+      <x:c r="C37" s="615" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D37" s="615" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E37" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="F37" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G37" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="H37" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I37" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J37" s="618"/>
+      <x:c r="K37" s="615" t="str">
+        <x:v>Release Team</x:v>
+      </x:c>
+      <x:c r="L37" s="615" t="str">
+        <x:v>All P0/P1 gates</x:v>
+      </x:c>
+      <x:c r="M37" s="615" t="str"/>
+      <x:c r="N37" s="615" t="str">
         <x:v>Go requires 0 open P0/P1 and fresh production/security/restore evidence.</x:v>
       </x:c>
     </x:row>
@@ -20851,7 +21209,16 @@
     <x:cfRule type="containsText" dxfId="341" priority="6" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="7">
+  <x:conditionalFormatting sqref="D2:I37">
+    <x:cfRule type="containsText" dxfId="357" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="358" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="359" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="360" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="361" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="362" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="363" priority="14" operator="containsText" text="In Progress"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
       <x:formula1>"P0,P1,P2,P3"</x:formula1>
     </x:dataValidation>
@@ -20871,6 +21238,27 @@
       <x:formula1>"Not Deployed,Pending,Deployed,N/A"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:I36">
+      <x:formula1>"Blocked,In Progress,Passed,Deferred"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C2:C37">
+      <x:formula1>"P0,P1,P2,P3"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D2:D37">
+      <x:formula1>"Not Started,In Progress,Fixed Local,Implemented,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E2:E37">
+      <x:formula1>"Pending,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F2:F37">
+      <x:formula1>"Pending,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G2:G37">
+      <x:formula1>"Pending,Passed Local,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H2:H37">
+      <x:formula1>"Not Deployed,Pending,Deployed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I2:I37">
       <x:formula1>"Blocked,In Progress,Passed,Deferred"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -20897,40 +21285,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1073" t="str">
+      <x:c r="A1" s="1094" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1074" t="str">
+      <x:c r="B1" s="1095" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1074" t="str">
+      <x:c r="C1" s="1095" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1074" t="str">
+      <x:c r="D1" s="1095" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1074" t="str">
+      <x:c r="E1" s="1095" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1074" t="str">
+      <x:c r="F1" s="1095" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1074" t="str">
+      <x:c r="G1" s="1095" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1074" t="str">
+      <x:c r="H1" s="1095" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1074" t="str">
+      <x:c r="I1" s="1095" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1074" t="str">
+      <x:c r="J1" s="1095" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1074" t="str">
+      <x:c r="K1" s="1095" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1075" t="str">
+      <x:c r="L1" s="1096" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -20960,7 +21348,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I2" s="614" t="str">
-        <x:v>Reproducer + exhaustive 55-code trust map + 475 risk tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Reproducer + exhaustive 55-code trust map + 475 risk tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J2" s="614" t="str">
         <x:v>Run remaining targeted and run real-client conflict matrix</x:v>
@@ -20998,7 +21386,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I3" s="615" t="str">
-        <x:v>Expired-handle reproducer + 47 focused tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Expired-handle reproducer + 47 focused tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J3" s="615" t="str">
         <x:v>Run remaining targeted re-verify primary sources before reactivation</x:v>
@@ -21036,7 +21424,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I4" s="615" t="str">
-        <x:v>4.2 s reproducer; worker/cap/queue/deadline regressions; 104 focus + 2645 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>4.2 s reproducer; worker/cap/queue/deadline regressions; 104 focus + 2645 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J4" s="615" t="str">
         <x:v>Run remaining targeted run legitimate QR smoke and 60-minute worker soak/crash-restart</x:v>
@@ -21074,7 +21462,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I5" s="615" t="str">
-        <x:v>Bearer-path reproducer + 52 focused + 479 risk tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Bearer-path reproducer + 52 focused + 479 risk tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J5" s="615" t="str">
         <x:v>Run remaining targeted and run provider compatibility smoke</x:v>
@@ -21112,7 +21500,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I6" s="615" t="str">
-        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J6" s="615" t="str">
         <x:v>Run remaining targeted force shared config/hash/RPC/shape failures and verify 429/no sink work</x:v>
@@ -21150,7 +21538,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I7" s="615" t="str">
-        <x:v>7-failure reproducer + 71 focused + 528 owning-suite tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>7-failure reproducer + 71 focused + 528 owning-suite tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J7" s="615" t="str">
         <x:v>Run remaining targeted and run report/appeal/Telegram draft smoke</x:v>
@@ -21188,7 +21576,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I8" s="615" t="str">
-        <x:v>npm audit 7-&gt;0; bun audit 2-&gt;0; 127.0.0.1 listener proof; 3 security + 2655 full tests; Bun build. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>npm audit 7-&gt;0; bun audit 2-&gt;0; 127.0.0.1 listener proof; 3 security + 2655 full tests; Bun build. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J8" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -21226,7 +21614,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I9" s="615" t="str">
-        <x:v>Regression test + 2026 Telegram suite. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Regression test + 2026 Telegram suite. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J9" s="615" t="str">
         <x:v>Run remaining targeted and verify real clients</x:v>
@@ -21264,7 +21652,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I10" s="615" t="str">
-        <x:v>Router regression + 2026 Telegram suite. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Router regression + 2026 Telegram suite. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J10" s="615" t="str">
         <x:v>Run remaining targeted and live-check RU/UZ/EN</x:v>
@@ -21302,7 +21690,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I11" s="615" t="str">
-        <x:v>Typed failure + parse retry tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Typed failure + parse retry tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J11" s="615" t="str">
         <x:v>Run remaining targeted and observe real answer result</x:v>
@@ -21340,7 +21728,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I12" s="615" t="str">
-        <x:v>256 boundary and skipUrlReputation tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>256 boundary and skipUrlReputation tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J12" s="615" t="str">
         <x:v>Run remaining targeted and run 20-40 prefix sequence</x:v>
@@ -21378,7 +21766,7 @@
         <x:v>Gate 1/2</x:v>
       </x:c>
       <x:c r="I13" s="615" t="str">
-        <x:v>Forged-marker reproducer + typed evidence isolation + 198 owning + 2667 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Forged-marker reproducer + typed evidence isolation + 198 owning + 2667 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J13" s="615" t="str">
         <x:v>Run remaining targeted and verify forged-marker corpus across web/embed/Inline</x:v>
@@ -21416,7 +21804,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I14" s="615" t="str">
-        <x:v>Six mixed-clause reproducers in RU/UZ/EN + five repeated focused runs + 2667 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Six mixed-clause reproducers in RU/UZ/EN + five repeated focused runs + 2667 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J14" s="615" t="str">
         <x:v>Run remaining targeted and run provider-output adversarial smoke</x:v>
@@ -21454,7 +21842,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I15" s="615" t="str">
-        <x:v>8-failure reproducer + exhaustive 55-code action policy + 227 Telegram focus + 2675 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>8-failure reproducer + exhaustive 55-code action policy + 227 Telegram focus + 2675 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J15" s="615" t="str">
         <x:v>Run remaining targeted and run RU/UZ/EN direct-bot smoke for confirmed report/phishing/malware</x:v>
@@ -21492,7 +21880,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I16" s="615" t="str">
-        <x:v>8-failure reproducer + full registry Cyrillic/official/hybrid corpus + 165 focus + 2733 full tests. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>8-failure reproducer + full registry Cyrillic/official/hybrid corpus + 165 focus + 2733 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J16" s="615" t="str">
         <x:v>Run remaining targeted run external reputation compatibility and RU/UZ/EN client smoke</x:v>
@@ -21530,7 +21918,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I17" s="615" t="str">
-        <x:v>5-failure reproducer + 158 ownership + 2738 full tests; stage-only privacy regression. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>5-failure reproducer + 158 ownership + 2738 full tests; stage-only privacy regression. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J17" s="615" t="str">
         <x:v>Run remaining targeted force both count failures and upsert failure; verify alert/retry UX</x:v>
@@ -21568,7 +21956,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I18" s="615" t="str">
-        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J18" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -21606,7 +21994,7 @@
         <x:v>Gate 2/3</x:v>
       </x:c>
       <x:c r="I19" s="615" t="str">
-        <x:v>55x3 real-adapter matrix plus canonical collector/methodology regressions; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>55x3 real-adapter matrix plus canonical collector/methodology regressions; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J19" s="615" t="str">
         <x:v>Run remaining targeted run Desktop/Android/iOS RU/UZ/EN visual/insertion matrix</x:v>
@@ -21635,7 +22023,7 @@
         <x:v>src/lib/telegram/check-followup.ts; session.server.ts; live-phrase-cases.ts</x:v>
       </x:c>
       <x:c r="F20" s="615" t="str">
-        <x:v>Deployed / Awaiting Live Verification</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="G20" s="615" t="str">
         <x:v>Telegram / Product</x:v>
@@ -21644,10 +22032,10 @@
         <x:v>Gate 2</x:v>
       </x:c>
       <x:c r="I20" s="615" t="str">
-        <x:v>24 post-check rows inside the 239-phrase live matrix; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>24 post-check rows inside the 239-phrase live matrix; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J20" s="615" t="str">
-        <x:v>Run remaining targeted run real multi-turn transcripts and session-loss/restart cases</x:v>
+        <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
       </x:c>
       <x:c r="K20" s="615" t="str">
         <x:v>Helper phrases never create checks or trusted-contact side effects; methodology is provenance-bound and RU/UZ/EN parallel</x:v>
@@ -21682,7 +22070,7 @@
         <x:v>Gate 2</x:v>
       </x:c>
       <x:c r="I21" s="615" t="str">
-        <x:v>Single leader, completion-gated offset, failure reacquisition, stale leader/update fence rejection, fenced session/effects; clean DB reset + no lint errors + pgTAP 20/20 + 2877 app tests + production build. Prod 6fb71ec8: three migrations applied; polling cutover and restart passed; monitor, web P1, security and Family Shield smoke passed with cleanup.</x:v>
+        <x:v>Single leader, completion-gated offset, failure reacquisition, stale leader/update fence rejection, fenced session/effects; clean DB reset + no lint errors + pgTAP 20/20 + 2877 app tests + production build. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J21" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -21696,13 +22084,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="343" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="344" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="345" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="346" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="347" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="348" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="349" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="364" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="365" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="366" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="367" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="368" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="369" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="370" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
docs: close polling follow-up QA gate
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rcb59f627b8cd4a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9c8db7844cea48d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rfa61bc3e0ec14922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R5c959531144f46bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R5076aa6d9d654b98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb24a201d182243ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re1ae6ddc44034564"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd96fa0f73dc044ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rf7f31773bb9444c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R0f178f0a3c014512"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5b02a540a1104074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R4bc6a07a04264127"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R56ceb83610b04b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3f25b48ca73d4f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf1da4f2a0fb84dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R6f49add54bb3448b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="190">
+  <x:fills count="193">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1040,6 +1040,21 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1127,7 +1142,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1116">
+  <x:cellXfs count="1137">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -3982,11 +3997,58 @@
     <x:xf numFmtId="0" fontId="1" fillId="188" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="190" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="190" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="191" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="191" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="191" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="192" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="192" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="192" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="192" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="192" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="192" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="191" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="378">
+  <x:dxfs count="399">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7416,6 +7478,237 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -8420,39 +8713,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1094" t="str">
+      <x:c r="A1" s="1116" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1095" t="str">
+      <x:c r="B1" s="1117" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1095" t="str">
+      <x:c r="C1" s="1117" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1095" t="str">
+      <x:c r="D1" s="1117" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1096" t="str">
+      <x:c r="E1" s="1118" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1113" t="n">
+      <x:c r="A2" s="1134" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="B2" s="1114" t="n">
+      <x:c r="B2" s="1135" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1114" t="n">
+      <x:c r="C2" s="1135" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1114" t="str">
-        <x:v>Gate 2/3: finish live recheck/disagreement replies; run real-client Inline RU/UZ/EN, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
-      </x:c>
-      <x:c r="E2" s="1114" t="str">
-        <x:v>Production release 6fb71ec8 and QA PR #73 / ae182707 are live in main. Polling-compatible confidence/trusted-person/domain-methodology QA and cleanup read-back passed. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
+      <x:c r="D2" s="1135" t="str">
+        <x:v>Gate 2/3: finish BOT-001 intent/action contract and BOT-004 canonical corpus; run real-client Inline RU/UZ/EN, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1135" t="str">
+        <x:v>Production release 6fb71ec8 and QA PR #75 / 74066f1 are live in main. All five post-check actions and cleanup read-back passed. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -8463,13 +8756,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1115" t="str">
+      <x:c r="A4" s="1136" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1115" t="str">
+      <x:c r="B4" s="1136" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1115" t="str">
+      <x:c r="C4" s="1136" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -8525,16 +8818,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1115" t="str">
+      <x:c r="A9" s="1136" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1115" t="str">
+      <x:c r="B9" s="1136" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1115" t="str">
+      <x:c r="C9" s="1136" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1115" t="str">
+      <x:c r="D9" s="1136" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -8611,13 +8904,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1115" t="str">
+      <x:c r="A15" s="1136" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1115" t="str">
+      <x:c r="B15" s="1136" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1115" t="str">
+      <x:c r="C15" s="1136" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -8701,13 +8994,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1115" t="str">
+      <x:c r="A22" s="1136" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1115" t="str">
+      <x:c r="B22" s="1136" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1115" t="str">
+      <x:c r="C22" s="1136" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -8733,7 +9026,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -8747,7 +9040,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -8771,13 +9064,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="371" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="372" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="373" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="374" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="375" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="376" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="377" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="392" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="393" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="394" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="395" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="396" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="397" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="398" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19617,19 +19910,19 @@
         <x:v>Polling-compatible Telegram multi-turn production QA</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>railway run npm run prod:telegram-polling-dispatch-smoke -- https://scam-guard-main-production.up.railway.app; PR #73 CI app + Supabase/pgTAP</x:v>
+        <x:v>railway run npm run prod:telegram-polling-dispatch-smoke -- https://scam-guard-main-production.up.railway.app; PR #75 CI app + Supabase/pgTAP</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>Passed: active polling leader 200; confidence, trusted-person and suspicious-domain methodology replies delivered; no follow-up check rows; cleanup read-back passed; 2881/2881 tests; build/audit green.</x:v>
+        <x:v>Passed: active polling leader 200; confidence, trusted-person, recheck, disagreement and suspicious-domain methodology replies delivered; no follow-up check rows; cleanup read-back passed; 2881/2881 tests; build/audit green.</x:v>
       </x:c>
       <x:c r="F92" t="str">
         <x:v>SG-P1-008, BOT-002, BOT-003, BOT-006</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>Bot API guard allowed only sendMessage/sendChatAction to TELEGRAM_QA_CHAT_ID. Synthetic payload remained in-process and did not acquire the polling leader. PR #73 / ae182707 merged; production monitor passed with pending=0.</x:v>
+        <x:v>Bot API guard allowed only sendMessage/sendChatAction to TELEGRAM_QA_CHAT_ID. Synthetic payload remained in-process and did not acquire the polling leader. PR #75 / 74066f1 merged; app and Supabase/pgTAP CI passed.</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>Complete live recheck/disagreement replies, then real Telegram Desktop/mobile Inline RU/UZ/EN visual matrix. Do not treat synthetic inline ids as client evidence.</x:v>
+        <x:v>Proceed to BOT-001/BOT-004 contract/corpus work and real Telegram Desktop/mobile Inline RU/UZ/EN visual matrix. Do not treat synthetic inline ids as client evidence.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19658,46 +19951,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1094" t="str">
+      <x:c r="A1" s="1116" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1095" t="str">
+      <x:c r="B1" s="1117" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1095" t="str">
+      <x:c r="C1" s="1117" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1095" t="str">
+      <x:c r="D1" s="1117" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1095" t="str">
+      <x:c r="E1" s="1117" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1095" t="str">
+      <x:c r="F1" s="1117" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1095" t="str">
+      <x:c r="G1" s="1117" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1095" t="str">
+      <x:c r="H1" s="1117" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1095" t="str">
+      <x:c r="I1" s="1117" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1095" t="str">
+      <x:c r="J1" s="1117" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1095" t="str">
+      <x:c r="K1" s="1117" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1095" t="str">
+      <x:c r="L1" s="1117" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1095" t="str">
+      <x:c r="M1" s="1117" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1096" t="str">
+      <x:c r="N1" s="1118" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -20732,16 +21025,16 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F26" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G26" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H26" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I26" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J26" s="618" t="n">
         <x:v>46214</x:v>
@@ -20749,12 +21042,10 @@
       <x:c r="K26" s="615" t="str">
         <x:v>Telegram / Copy</x:v>
       </x:c>
-      <x:c r="L26" s="615" t="str">
-        <x:v>BOT-001 + live recheck/disagreement</x:v>
-      </x:c>
+      <x:c r="L26" s="615" t="str"/>
       <x:c r="M26" s="615" t="str"/>
       <x:c r="N26" s="615" t="str">
-        <x:v>RU production live QA passed confidence, methodology and trusted-person replies with no cold check or trusted-contact side effect. Automated RU/UZ/EN coverage passes all five actions; live recheck/disagreement remain before this row can pass. PR #73 / ae182707.</x:v>
+        <x:v>RU production live QA passed confidence, methodology, trusted-person, recheck and disagreement with no cold check or trusted-contact side effect. Recheck requires resubmission without pretending analysis ran; disagreement remains non-accusatory. Automated RU/UZ/EN coverage passes all five actions. PR #75 / 74066f1.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -20836,7 +21127,7 @@
       <x:c r="L28" s="615" t="str"/>
       <x:c r="M28" s="615" t="str"/>
       <x:c r="N28" s="615" t="str">
-        <x:v>Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -21210,13 +21501,13 @@
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I37">
-    <x:cfRule type="containsText" dxfId="357" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="358" priority="9" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="359" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="360" priority="11" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="361" priority="12" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="362" priority="13" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="363" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="378" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="379" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="380" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="381" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="382" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="383" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="384" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -21285,40 +21576,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1094" t="str">
+      <x:c r="A1" s="1116" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1095" t="str">
+      <x:c r="B1" s="1117" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1095" t="str">
+      <x:c r="C1" s="1117" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1095" t="str">
+      <x:c r="D1" s="1117" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1095" t="str">
+      <x:c r="E1" s="1117" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1095" t="str">
+      <x:c r="F1" s="1117" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1095" t="str">
+      <x:c r="G1" s="1117" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1095" t="str">
+      <x:c r="H1" s="1117" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1095" t="str">
+      <x:c r="I1" s="1117" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1095" t="str">
+      <x:c r="J1" s="1117" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1095" t="str">
+      <x:c r="K1" s="1117" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1096" t="str">
+      <x:c r="L1" s="1118" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -21348,7 +21639,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I2" s="614" t="str">
-        <x:v>Reproducer + exhaustive 55-code trust map + 475 risk tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Reproducer + exhaustive 55-code trust map + 475 risk tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J2" s="614" t="str">
         <x:v>Run remaining targeted and run real-client conflict matrix</x:v>
@@ -21386,7 +21677,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I3" s="615" t="str">
-        <x:v>Expired-handle reproducer + 47 focused tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Expired-handle reproducer + 47 focused tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J3" s="615" t="str">
         <x:v>Run remaining targeted re-verify primary sources before reactivation</x:v>
@@ -21424,7 +21715,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I4" s="615" t="str">
-        <x:v>4.2 s reproducer; worker/cap/queue/deadline regressions; 104 focus + 2645 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>4.2 s reproducer; worker/cap/queue/deadline regressions; 104 focus + 2645 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J4" s="615" t="str">
         <x:v>Run remaining targeted run legitimate QR smoke and 60-minute worker soak/crash-restart</x:v>
@@ -21462,7 +21753,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I5" s="615" t="str">
-        <x:v>Bearer-path reproducer + 52 focused + 479 risk tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Bearer-path reproducer + 52 focused + 479 risk tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J5" s="615" t="str">
         <x:v>Run remaining targeted and run provider compatibility smoke</x:v>
@@ -21500,7 +21791,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I6" s="615" t="str">
-        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J6" s="615" t="str">
         <x:v>Run remaining targeted force shared config/hash/RPC/shape failures and verify 429/no sink work</x:v>
@@ -21538,7 +21829,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I7" s="615" t="str">
-        <x:v>7-failure reproducer + 71 focused + 528 owning-suite tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>7-failure reproducer + 71 focused + 528 owning-suite tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J7" s="615" t="str">
         <x:v>Run remaining targeted and run report/appeal/Telegram draft smoke</x:v>
@@ -21576,7 +21867,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I8" s="615" t="str">
-        <x:v>npm audit 7-&gt;0; bun audit 2-&gt;0; 127.0.0.1 listener proof; 3 security + 2655 full tests; Bun build. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>npm audit 7-&gt;0; bun audit 2-&gt;0; 127.0.0.1 listener proof; 3 security + 2655 full tests; Bun build. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J8" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -21614,7 +21905,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I9" s="615" t="str">
-        <x:v>Regression test + 2026 Telegram suite. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Regression test + 2026 Telegram suite. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J9" s="615" t="str">
         <x:v>Run remaining targeted and verify real clients</x:v>
@@ -21652,7 +21943,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I10" s="615" t="str">
-        <x:v>Router regression + 2026 Telegram suite. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Router regression + 2026 Telegram suite. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J10" s="615" t="str">
         <x:v>Run remaining targeted and live-check RU/UZ/EN</x:v>
@@ -21690,7 +21981,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I11" s="615" t="str">
-        <x:v>Typed failure + parse retry tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Typed failure + parse retry tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J11" s="615" t="str">
         <x:v>Run remaining targeted and observe real answer result</x:v>
@@ -21728,7 +22019,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I12" s="615" t="str">
-        <x:v>256 boundary and skipUrlReputation tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>256 boundary and skipUrlReputation tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J12" s="615" t="str">
         <x:v>Run remaining targeted and run 20-40 prefix sequence</x:v>
@@ -21766,7 +22057,7 @@
         <x:v>Gate 1/2</x:v>
       </x:c>
       <x:c r="I13" s="615" t="str">
-        <x:v>Forged-marker reproducer + typed evidence isolation + 198 owning + 2667 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Forged-marker reproducer + typed evidence isolation + 198 owning + 2667 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J13" s="615" t="str">
         <x:v>Run remaining targeted and verify forged-marker corpus across web/embed/Inline</x:v>
@@ -21804,7 +22095,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I14" s="615" t="str">
-        <x:v>Six mixed-clause reproducers in RU/UZ/EN + five repeated focused runs + 2667 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Six mixed-clause reproducers in RU/UZ/EN + five repeated focused runs + 2667 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J14" s="615" t="str">
         <x:v>Run remaining targeted and run provider-output adversarial smoke</x:v>
@@ -21842,7 +22133,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I15" s="615" t="str">
-        <x:v>8-failure reproducer + exhaustive 55-code action policy + 227 Telegram focus + 2675 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>8-failure reproducer + exhaustive 55-code action policy + 227 Telegram focus + 2675 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J15" s="615" t="str">
         <x:v>Run remaining targeted and run RU/UZ/EN direct-bot smoke for confirmed report/phishing/malware</x:v>
@@ -21880,7 +22171,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I16" s="615" t="str">
-        <x:v>8-failure reproducer + full registry Cyrillic/official/hybrid corpus + 165 focus + 2733 full tests. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>8-failure reproducer + full registry Cyrillic/official/hybrid corpus + 165 focus + 2733 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J16" s="615" t="str">
         <x:v>Run remaining targeted run external reputation compatibility and RU/UZ/EN client smoke</x:v>
@@ -21918,7 +22209,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I17" s="615" t="str">
-        <x:v>5-failure reproducer + 158 ownership + 2738 full tests; stage-only privacy regression. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>5-failure reproducer + 158 ownership + 2738 full tests; stage-only privacy regression. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J17" s="615" t="str">
         <x:v>Run remaining targeted force both count failures and upsert failure; verify alert/retry UX</x:v>
@@ -21956,7 +22247,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I18" s="615" t="str">
-        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J18" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -21994,7 +22285,7 @@
         <x:v>Gate 2/3</x:v>
       </x:c>
       <x:c r="I19" s="615" t="str">
-        <x:v>55x3 real-adapter matrix plus canonical collector/methodology regressions; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>55x3 real-adapter matrix plus canonical collector/methodology regressions; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J19" s="615" t="str">
         <x:v>Run remaining targeted run Desktop/Android/iOS RU/UZ/EN visual/insertion matrix</x:v>
@@ -22032,7 +22323,7 @@
         <x:v>Gate 2</x:v>
       </x:c>
       <x:c r="I20" s="615" t="str">
-        <x:v>24 post-check rows inside the 239-phrase live matrix; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>24 post-check rows inside the 239-phrase live matrix; 634 critical tests x5, expanded focus 713, 2159 Telegram and 2863 full tests x2. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J20" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -22070,7 +22361,7 @@
         <x:v>Gate 2</x:v>
       </x:c>
       <x:c r="I21" s="615" t="str">
-        <x:v>Single leader, completion-gated offset, failure reacquisition, stale leader/update fence rejection, fenced session/effects; clean DB reset + no lint errors + pgTAP 20/20 + 2877 app tests + production build. Prod 6fb71ec8 + QA ae182707: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified confidence, trusted-person and domain-methodology replies with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Single leader, completion-gated offset, failure reacquisition, stale leader/update fence rejection, fenced session/effects; clean DB reset + no lint errors + pgTAP 20/20 + 2877 app tests + production build. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
       </x:c>
       <x:c r="J21" s="615" t="str">
         <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
@@ -22084,13 +22375,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="364" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="365" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="366" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="367" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="368" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="369" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="370" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="385" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="386" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="387" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="388" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="389" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="390" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="391" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
docs: close production monitor gate
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rf7f31773bb9444c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R0f178f0a3c014512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R5b02a540a1104074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R4bc6a07a04264127"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R56ceb83610b04b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R3f25b48ca73d4f2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rf1da4f2a0fb84dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R6f49add54bb3448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R77e617c7fc46416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re891b337460b491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1973335bfd3947d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9c15ea568d3347ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rfa8ccd57d888449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4d23201c7310469b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re30527dbc05547e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R22f7abb837ee47a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="193">
+  <x:fills count="199">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1055,6 +1055,36 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1142,7 +1172,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1137">
+  <x:cellXfs count="1179">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4044,11 +4074,105 @@
     <x:xf numFmtId="0" fontId="1" fillId="191" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="193" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="193" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="194" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="194" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="194" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="195" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="195" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="195" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="195" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="195" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="195" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="194" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="196" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="196" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="197" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="197" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="197" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="198" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="198" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="198" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="198" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="198" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="198" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="197" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="399">
+  <x:dxfs count="441">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7478,6 +7602,468 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -8713,39 +9299,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1116" t="str">
+      <x:c r="A1" s="1158" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1117" t="str">
+      <x:c r="B1" s="1159" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1117" t="str">
+      <x:c r="C1" s="1159" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1117" t="str">
+      <x:c r="D1" s="1159" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1118" t="str">
+      <x:c r="E1" s="1160" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1134" t="n">
+      <x:c r="A2" s="1176" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="B2" s="1135" t="n">
+      <x:c r="B2" s="1177" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1135" t="n">
+      <x:c r="C2" s="1177" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1135" t="str">
+      <x:c r="D2" s="1177" t="str">
         <x:v>Gate 2/3: finish BOT-001 intent/action contract and BOT-004 canonical corpus; run real-client Inline RU/UZ/EN, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
       </x:c>
-      <x:c r="E2" s="1135" t="str">
-        <x:v>Production release 6fb71ec8 and QA PR #75 / 74066f1 are live in main. All five post-check actions and cleanup read-back passed. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
+      <x:c r="E2" s="1177" t="str">
+        <x:v>Production release 6fb71ec8, QA PR #75 / 74066f1 and monitor PR #77 / 7466d00 are live in main. All five post-check actions passed; the scheduled polling monitor and controlled missing-secret/restore drill are green. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -8756,13 +9342,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1136" t="str">
+      <x:c r="A4" s="1178" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1136" t="str">
+      <x:c r="B4" s="1178" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1136" t="str">
+      <x:c r="C4" s="1178" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -8818,16 +9404,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1136" t="str">
+      <x:c r="A9" s="1178" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1136" t="str">
+      <x:c r="B9" s="1178" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1136" t="str">
+      <x:c r="C9" s="1178" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1136" t="str">
+      <x:c r="D9" s="1178" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -8904,13 +9490,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1136" t="str">
+      <x:c r="A15" s="1178" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1136" t="str">
+      <x:c r="B15" s="1178" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1136" t="str">
+      <x:c r="C15" s="1178" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -8994,13 +9580,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1136" t="str">
+      <x:c r="A22" s="1178" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1136" t="str">
+      <x:c r="B22" s="1178" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1136" t="str">
+      <x:c r="C22" s="1178" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -9026,7 +9612,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -9040,7 +9626,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -9064,13 +9650,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="392" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="393" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="394" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="395" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="396" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="397" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="398" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="434" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="435" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="436" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="437" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="438" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="439" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="440" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19923,6 +20509,32 @@
       </x:c>
       <x:c r="H92" t="str">
         <x:v>Proceed to BOT-001/BOT-004 contract/corpus work and real Telegram Desktop/mobile Inline RU/UZ/EN visual matrix. Do not treat synthetic inline ids as client evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>QA-PROD-MONITOR-2026-07-11</x:v>
+      </x:c>
+      <x:c r="B93" s="1097" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>Scheduled production monitor polling alignment and fail-hard drill</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>PR #77 CI; GitHub Production Monitor runs 29163086372 and 29163166938 from main; process-only missing TELEGRAM_BOT_TOKEN drill with MONITOR_REQUIRE_SECRET_CHECKS=true</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Passed: both GitHub runs succeeded; home/health 200, disabled webhook 503/503, mode=polling, url_ok=true, pending=0, polling leader 200, AI provider 200. Missing-token drill exited 1 as required, then restore run passed.</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>PLAT-002, SG-P1-006</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Production secrets were not removed or changed. The drill cleared the token and alert chat only inside one child process, preventing a test alert while proving the fail-hard policy. PR #77 / 7466d00 merged.</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>Continue scheduled monitoring; investigate only new failures after commit 7466d00 rather than the retired webhook-mode false alert.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19951,46 +20563,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1116" t="str">
+      <x:c r="A1" s="1158" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1117" t="str">
+      <x:c r="B1" s="1159" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1117" t="str">
+      <x:c r="C1" s="1159" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1117" t="str">
+      <x:c r="D1" s="1159" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1117" t="str">
+      <x:c r="E1" s="1159" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1117" t="str">
+      <x:c r="F1" s="1159" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1117" t="str">
+      <x:c r="G1" s="1159" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1117" t="str">
+      <x:c r="H1" s="1159" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1117" t="str">
+      <x:c r="I1" s="1159" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1117" t="str">
+      <x:c r="J1" s="1159" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1117" t="str">
+      <x:c r="K1" s="1159" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1117" t="str">
+      <x:c r="L1" s="1159" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1117" t="str">
+      <x:c r="M1" s="1159" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1118" t="str">
+      <x:c r="N1" s="1160" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -20901,16 +21513,16 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F23" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G23" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H23" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I23" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J23" s="618" t="n">
         <x:v>46214</x:v>
@@ -20918,12 +21530,10 @@
       <x:c r="K23" s="615" t="str">
         <x:v>DevOps</x:v>
       </x:c>
-      <x:c r="L23" s="615" t="str">
-        <x:v>GitHub Actions run + controlled missing-secret/restore drill</x:v>
-      </x:c>
+      <x:c r="L23" s="615" t="str"/>
       <x:c r="M23" s="615" t="str"/>
       <x:c r="N23" s="615" t="str">
-        <x:v>The scheduled workflow explicitly requires Telegram secrets; pure policy proves a required skip fails even with fail-on-warn disabled. Live Actions evidence remains. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
+        <x:v>PR #77 / 7466d00 aligned the scheduled GitHub monitor with production polling. GitHub Actions runs 29163086372 and 29163166938 passed from main: home/health 200, disabled webhook 503/503, Telegram polling URL valid, pending 0, leader 200 and AI provider 200. A controlled process-only missing TELEGRAM_BOT_TOKEN drill failed hard with exit 1; production secrets were not changed, and the subsequent restore run passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -21501,13 +22111,13 @@
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I37">
-    <x:cfRule type="containsText" dxfId="378" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="379" priority="9" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="380" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="381" priority="11" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="382" priority="12" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="383" priority="13" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="384" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="420" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="421" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="422" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="423" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="424" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="425" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="426" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -21576,40 +22186,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1116" t="str">
+      <x:c r="A1" s="1158" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1117" t="str">
+      <x:c r="B1" s="1159" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1117" t="str">
+      <x:c r="C1" s="1159" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1117" t="str">
+      <x:c r="D1" s="1159" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1117" t="str">
+      <x:c r="E1" s="1159" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1117" t="str">
+      <x:c r="F1" s="1159" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1117" t="str">
+      <x:c r="G1" s="1159" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1117" t="str">
+      <x:c r="H1" s="1159" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1117" t="str">
+      <x:c r="I1" s="1159" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1117" t="str">
+      <x:c r="J1" s="1159" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1117" t="str">
+      <x:c r="K1" s="1159" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1118" t="str">
+      <x:c r="L1" s="1160" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -22247,10 +22857,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I18" s="615" t="str">
-        <x:v>3 policy/workflow regressions + 2741 full tests; TypeScript/scoped lint. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>3 policy/workflow regressions plus full repository CI. PR #77 / 7466d00 explicitly configured the scheduled monitor for polling. GitHub Actions runs 29163086372 and 29163166938 passed from main; a controlled child-process missing TELEGRAM_BOT_TOKEN drill with required secret checks exited 1, and the subsequent normal restore run passed. Production secrets were not changed.</x:v>
       </x:c>
       <x:c r="J18" s="615" t="str">
-        <x:v>Closed after production deployment and targeted post-deploy verification.</x:v>
+        <x:v>Closed after the polling-aligned GitHub workflow, fail-hard missing-secret drill and successful restore run.</x:v>
       </x:c>
       <x:c r="K18" s="615" t="str">
         <x:v>A required skipped check makes the run red independently of fail-on-warn and alert delivery</x:v>
@@ -22375,13 +22985,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="385" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="386" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="387" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="388" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="389" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="390" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="391" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="427" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="428" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="429" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="430" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="431" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="432" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="433" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
docs: update Telegram contract release evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R77e617c7fc46416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re891b337460b491b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1973335bfd3947d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9c15ea568d3347ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rfa8ccd57d888449f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4d23201c7310469b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re30527dbc05547e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R22f7abb837ee47a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc72721937bf442f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R29020785b8f54fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd658b958aa6d465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rcdff9710188c4cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8b03fd02d5c7453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf125533db6714da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R73fdd7c7eef44a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R7c4989cf42ff41c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="199">
+  <x:fills count="202">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1085,6 +1085,21 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1172,7 +1187,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1179">
+  <x:cellXfs count="1200">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4168,11 +4183,58 @@
     <x:xf numFmtId="0" fontId="1" fillId="197" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="199" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="200" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="200" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="200" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="201" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="200" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="441">
+  <x:dxfs count="462">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7602,6 +7664,237 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9299,39 +9592,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1158" t="str">
+      <x:c r="A1" s="1179" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1159" t="str">
+      <x:c r="B1" s="1180" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1159" t="str">
+      <x:c r="C1" s="1180" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1159" t="str">
+      <x:c r="D1" s="1180" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1160" t="str">
+      <x:c r="E1" s="1181" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1176" t="n">
+      <x:c r="A2" s="1197" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="B2" s="1177" t="n">
+      <x:c r="B2" s="1198" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1177" t="n">
+      <x:c r="C2" s="1198" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1177" t="str">
-        <x:v>Gate 2/3: finish BOT-001 intent/action contract and BOT-004 canonical corpus; run real-client Inline RU/UZ/EN, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
-      </x:c>
-      <x:c r="E2" s="1177" t="str">
-        <x:v>Production release 6fb71ec8, QA PR #75 / 74066f1 and monitor PR #77 / 7466d00 are live in main. All five post-check actions passed; the scheduled polling monitor and controlled missing-secret/restore drill are green. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
+      <x:c r="D2" s="1198" t="str">
+        <x:v>Restore Railway deployment capability, deploy b4cabb9 or later, then verify BOT-001 with the bounded production smoke and expand BOT-004 into real-client RU/UZ/EN transcripts. Continue Inline client, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1198" t="str">
+        <x:v>PR #79 / b4cabb9 implemented the canonical Telegram contract and 1248-row dialogue DSL; all 238 legacy rows map and CI is green. Railway rejected deployment because the trial expired, so production remains on 6714227 and BOT-001/BOT-004 live gates stay blocked. Existing production health remains 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -9342,13 +9635,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1178" t="str">
+      <x:c r="A4" s="1199" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1178" t="str">
+      <x:c r="B4" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1178" t="str">
+      <x:c r="C4" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -9404,16 +9697,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1178" t="str">
+      <x:c r="A9" s="1199" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1178" t="str">
+      <x:c r="B9" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1178" t="str">
+      <x:c r="C9" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1178" t="str">
+      <x:c r="D9" s="1199" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -9490,13 +9783,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1178" t="str">
+      <x:c r="A15" s="1199" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1178" t="str">
+      <x:c r="B15" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1178" t="str">
+      <x:c r="C15" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -9580,13 +9873,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1178" t="str">
+      <x:c r="A22" s="1199" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1178" t="str">
+      <x:c r="B22" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1178" t="str">
+      <x:c r="C22" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -9650,13 +9943,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="434" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="435" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="436" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="437" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="438" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="439" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="440" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="455" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="456" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="457" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="458" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="459" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="460" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="461" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -20535,6 +20828,32 @@
       </x:c>
       <x:c r="H93" t="str">
         <x:v>Continue scheduled monitoring; investigate only new failures after commit 7466d00 rather than the retired webhook-mode false alert.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>QA-TELEGRAM-CONTRACT-2026-07-11</x:v>
+      </x:c>
+      <x:c r="B94" s="1097" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Canonical Telegram intent/action contract and 1248-row dialogue DSL</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>PR #79 / b4cabb9; GitHub CI run 29164500392; local full/Telegram suites; Railway deployment attempt from clean main</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Automated QA passed: 4135/4135 full tests, 3431/3431 Telegram tests, all 238 legacy phrase rows mapped, exactly 1248 unique RU/UZ/EN dialogue-state rows, TypeScript/lint/build/format/npm audit green. GitHub app and Supabase reset/schema lint/pgTAP jobs passed.</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>BOT-001, BOT-004</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Reply-only contracts forbid check persistence and trusted-contact effects; direct versus Inline risk persistence is explicit; response length is enforced before Bot API delivery. No schema, migration, dependency, secret or production-data changes. Railway rejected the new deployment because the trial expired; production remains on commit 6714227.</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>Renew/select a Railway plan, deploy b4cabb9 or later, verify /healthz and polling leader, rerun the bounded five-action production smoke, then capture broader real-client RU/UZ/EN transcripts before marking BOT-001/BOT-004 release gates Passed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20563,46 +20882,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1158" t="str">
+      <x:c r="A1" s="1179" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1159" t="str">
+      <x:c r="B1" s="1180" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1159" t="str">
+      <x:c r="C1" s="1180" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1159" t="str">
+      <x:c r="D1" s="1180" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1159" t="str">
+      <x:c r="E1" s="1180" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1159" t="str">
+      <x:c r="F1" s="1180" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1159" t="str">
+      <x:c r="G1" s="1180" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1159" t="str">
+      <x:c r="H1" s="1180" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1159" t="str">
+      <x:c r="I1" s="1180" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1159" t="str">
+      <x:c r="J1" s="1180" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1159" t="str">
+      <x:c r="K1" s="1180" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1159" t="str">
+      <x:c r="L1" s="1180" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1159" t="str">
+      <x:c r="M1" s="1180" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1160" t="str">
+      <x:c r="N1" s="1181" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -21547,16 +21866,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D24" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E24" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F24" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G24" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H24" s="615" t="str">
         <x:v>Not Deployed</x:v>
@@ -21571,11 +21890,11 @@
         <x:v>Telegram / Product</x:v>
       </x:c>
       <x:c r="L24" s="615" t="str">
-        <x:v>Gate 1 trust contract</x:v>
+        <x:v>Railway plan expired; deploy b4cabb9 + live smoke</x:v>
       </x:c>
       <x:c r="M24" s="615" t="str"/>
       <x:c r="N24" s="615" t="str">
-        <x:v>Post-check helper actions are now typed/shared; the broader direct/Inline intent and response contract remains incomplete.</x:v>
+        <x:v>Canonical meta.*, victim.*, followup.*, panic.* and input.risk_check registry now binds response actions to direct/Inline persistence, trusted-contact and reply-size boundaries. Runtime reply enforcement is active in direct handlers. PR #79 / b4cabb9; GitHub app CI and Supabase reset/schema lint/pgTAP passed; full suite 4135/4135, Telegram 3431/3431, TypeScript, lint, build and npm audit green. Railway rejected deployment because the trial expired, so production still runs 6714227.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -21669,16 +21988,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D27" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E27" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F27" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
         <x:v>Not Deployed</x:v>
@@ -21693,11 +22012,11 @@
         <x:v>QA Automation</x:v>
       </x:c>
       <x:c r="L27" s="615" t="str">
-        <x:v>BOT-001</x:v>
+        <x:v>Railway plan expired; deploy + broader real-client transcript matrix</x:v>
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>The polling-compatible production harness now covers three critical multi-turn replies, but the planned 1100-row canonical corpus/dialogue DSL and broader live transcript set remain incomplete.</x:v>
+        <x:v>Deterministic DSL now covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. Recent, orphan, stale and new-artifact routing plus &lt;=4096 response bounds pass. PR #79 / b4cabb9. Broader real Telegram-client transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -22111,13 +22430,13 @@
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I37">
-    <x:cfRule type="containsText" dxfId="420" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="421" priority="9" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="422" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="423" priority="11" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="424" priority="12" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="425" priority="13" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="426" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="441" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="442" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="443" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="444" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="445" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="446" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="447" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -22186,40 +22505,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1158" t="str">
+      <x:c r="A1" s="1179" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1159" t="str">
+      <x:c r="B1" s="1180" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1159" t="str">
+      <x:c r="C1" s="1180" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1159" t="str">
+      <x:c r="D1" s="1180" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1159" t="str">
+      <x:c r="E1" s="1180" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1159" t="str">
+      <x:c r="F1" s="1180" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1159" t="str">
+      <x:c r="G1" s="1180" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1159" t="str">
+      <x:c r="H1" s="1180" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1159" t="str">
+      <x:c r="I1" s="1180" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1159" t="str">
+      <x:c r="J1" s="1180" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1159" t="str">
+      <x:c r="K1" s="1180" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1160" t="str">
+      <x:c r="L1" s="1181" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -22985,13 +23304,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="427" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="428" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="429" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="430" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="431" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="432" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="433" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="448" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="449" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="450" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="451" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="452" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="453" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="454" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
docs: update Telegram contract release evidence (#80)
Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R77e617c7fc46416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Re891b337460b491b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R1973335bfd3947d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R9c15ea568d3347ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rfa8ccd57d888449f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R4d23201c7310469b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re30527dbc05547e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R22f7abb837ee47a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc72721937bf442f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R29020785b8f54fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd658b958aa6d465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rcdff9710188c4cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8b03fd02d5c7453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf125533db6714da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R73fdd7c7eef44a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R7c4989cf42ff41c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="199">
+  <x:fills count="202">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1085,6 +1085,21 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1172,7 +1187,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1179">
+  <x:cellXfs count="1200">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4168,11 +4183,58 @@
     <x:xf numFmtId="0" fontId="1" fillId="197" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="199" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="199" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="200" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="200" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="200" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="201" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="201" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="201" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="200" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="441">
+  <x:dxfs count="462">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7602,6 +7664,237 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9299,39 +9592,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1158" t="str">
+      <x:c r="A1" s="1179" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1159" t="str">
+      <x:c r="B1" s="1180" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1159" t="str">
+      <x:c r="C1" s="1180" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1159" t="str">
+      <x:c r="D1" s="1180" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1160" t="str">
+      <x:c r="E1" s="1181" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1176" t="n">
+      <x:c r="A2" s="1197" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="B2" s="1177" t="n">
+      <x:c r="B2" s="1198" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1177" t="n">
+      <x:c r="C2" s="1198" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1177" t="str">
-        <x:v>Gate 2/3: finish BOT-001 intent/action contract and BOT-004 canonical corpus; run real-client Inline RU/UZ/EN, provider compatibility and resource-soak matrices; close remaining deployed findings and enable leaked-password protection.</x:v>
-      </x:c>
-      <x:c r="E2" s="1177" t="str">
-        <x:v>Production release 6fb71ec8, QA PR #75 / 74066f1 and monitor PR #77 / 7466d00 are live in main. All five post-check actions passed; the scheduled polling monitor and controlled missing-secret/restore drill are green. BOT-001/BOT-004, real-client Inline, provider and soak evidence remain incomplete.</x:v>
+      <x:c r="D2" s="1198" t="str">
+        <x:v>Restore Railway deployment capability, deploy b4cabb9 or later, then verify BOT-001 with the bounded production smoke and expand BOT-004 into real-client RU/UZ/EN transcripts. Continue Inline client, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1198" t="str">
+        <x:v>PR #79 / b4cabb9 implemented the canonical Telegram contract and 1248-row dialogue DSL; all 238 legacy rows map and CI is green. Railway rejected deployment because the trial expired, so production remains on 6714227 and BOT-001/BOT-004 live gates stay blocked. Existing production health remains 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -9342,13 +9635,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1178" t="str">
+      <x:c r="A4" s="1199" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1178" t="str">
+      <x:c r="B4" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1178" t="str">
+      <x:c r="C4" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -9404,16 +9697,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1178" t="str">
+      <x:c r="A9" s="1199" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1178" t="str">
+      <x:c r="B9" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1178" t="str">
+      <x:c r="C9" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1178" t="str">
+      <x:c r="D9" s="1199" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -9490,13 +9783,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1178" t="str">
+      <x:c r="A15" s="1199" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1178" t="str">
+      <x:c r="B15" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1178" t="str">
+      <x:c r="C15" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -9580,13 +9873,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1178" t="str">
+      <x:c r="A22" s="1199" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1178" t="str">
+      <x:c r="B22" s="1199" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1178" t="str">
+      <x:c r="C22" s="1199" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -9650,13 +9943,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="434" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="435" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="436" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="437" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="438" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="439" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="440" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="455" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="456" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="457" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="458" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="459" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="460" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="461" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -20535,6 +20828,32 @@
       </x:c>
       <x:c r="H93" t="str">
         <x:v>Continue scheduled monitoring; investigate only new failures after commit 7466d00 rather than the retired webhook-mode false alert.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>QA-TELEGRAM-CONTRACT-2026-07-11</x:v>
+      </x:c>
+      <x:c r="B94" s="1097" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Canonical Telegram intent/action contract and 1248-row dialogue DSL</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>PR #79 / b4cabb9; GitHub CI run 29164500392; local full/Telegram suites; Railway deployment attempt from clean main</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Automated QA passed: 4135/4135 full tests, 3431/3431 Telegram tests, all 238 legacy phrase rows mapped, exactly 1248 unique RU/UZ/EN dialogue-state rows, TypeScript/lint/build/format/npm audit green. GitHub app and Supabase reset/schema lint/pgTAP jobs passed.</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>BOT-001, BOT-004</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Reply-only contracts forbid check persistence and trusted-contact effects; direct versus Inline risk persistence is explicit; response length is enforced before Bot API delivery. No schema, migration, dependency, secret or production-data changes. Railway rejected the new deployment because the trial expired; production remains on commit 6714227.</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>Renew/select a Railway plan, deploy b4cabb9 or later, verify /healthz and polling leader, rerun the bounded five-action production smoke, then capture broader real-client RU/UZ/EN transcripts before marking BOT-001/BOT-004 release gates Passed.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20563,46 +20882,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1158" t="str">
+      <x:c r="A1" s="1179" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1159" t="str">
+      <x:c r="B1" s="1180" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1159" t="str">
+      <x:c r="C1" s="1180" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1159" t="str">
+      <x:c r="D1" s="1180" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1159" t="str">
+      <x:c r="E1" s="1180" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1159" t="str">
+      <x:c r="F1" s="1180" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1159" t="str">
+      <x:c r="G1" s="1180" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1159" t="str">
+      <x:c r="H1" s="1180" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1159" t="str">
+      <x:c r="I1" s="1180" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1159" t="str">
+      <x:c r="J1" s="1180" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1159" t="str">
+      <x:c r="K1" s="1180" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1159" t="str">
+      <x:c r="L1" s="1180" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1159" t="str">
+      <x:c r="M1" s="1180" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1160" t="str">
+      <x:c r="N1" s="1181" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -21547,16 +21866,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D24" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E24" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F24" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G24" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H24" s="615" t="str">
         <x:v>Not Deployed</x:v>
@@ -21571,11 +21890,11 @@
         <x:v>Telegram / Product</x:v>
       </x:c>
       <x:c r="L24" s="615" t="str">
-        <x:v>Gate 1 trust contract</x:v>
+        <x:v>Railway plan expired; deploy b4cabb9 + live smoke</x:v>
       </x:c>
       <x:c r="M24" s="615" t="str"/>
       <x:c r="N24" s="615" t="str">
-        <x:v>Post-check helper actions are now typed/shared; the broader direct/Inline intent and response contract remains incomplete.</x:v>
+        <x:v>Canonical meta.*, victim.*, followup.*, panic.* and input.risk_check registry now binds response actions to direct/Inline persistence, trusted-contact and reply-size boundaries. Runtime reply enforcement is active in direct handlers. PR #79 / b4cabb9; GitHub app CI and Supabase reset/schema lint/pgTAP passed; full suite 4135/4135, Telegram 3431/3431, TypeScript, lint, build and npm audit green. Railway rejected deployment because the trial expired, so production still runs 6714227.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -21669,16 +21988,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D27" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E27" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F27" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
         <x:v>Not Deployed</x:v>
@@ -21693,11 +22012,11 @@
         <x:v>QA Automation</x:v>
       </x:c>
       <x:c r="L27" s="615" t="str">
-        <x:v>BOT-001</x:v>
+        <x:v>Railway plan expired; deploy + broader real-client transcript matrix</x:v>
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>The polling-compatible production harness now covers three critical multi-turn replies, but the planned 1100-row canonical corpus/dialogue DSL and broader live transcript set remain incomplete.</x:v>
+        <x:v>Deterministic DSL now covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. Recent, orphan, stale and new-artifact routing plus &lt;=4096 response bounds pass. PR #79 / b4cabb9. Broader real Telegram-client transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -22111,13 +22430,13 @@
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I37">
-    <x:cfRule type="containsText" dxfId="420" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="421" priority="9" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="422" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="423" priority="11" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="424" priority="12" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="425" priority="13" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="426" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="441" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="442" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="443" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="444" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="445" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="446" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="447" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -22186,40 +22505,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1158" t="str">
+      <x:c r="A1" s="1179" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1159" t="str">
+      <x:c r="B1" s="1180" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1159" t="str">
+      <x:c r="C1" s="1180" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1159" t="str">
+      <x:c r="D1" s="1180" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1159" t="str">
+      <x:c r="E1" s="1180" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1159" t="str">
+      <x:c r="F1" s="1180" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1159" t="str">
+      <x:c r="G1" s="1180" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1159" t="str">
+      <x:c r="H1" s="1180" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1159" t="str">
+      <x:c r="I1" s="1180" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1159" t="str">
+      <x:c r="J1" s="1180" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1159" t="str">
+      <x:c r="K1" s="1180" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1160" t="str">
+      <x:c r="L1" s="1181" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -22985,13 +23304,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="427" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="428" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="429" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="430" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="431" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="432" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="433" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="448" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="449" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="450" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="451" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="452" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="453" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="454" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
docs: record Telegram contract production verification
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc72721937bf442f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R29020785b8f54fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd658b958aa6d465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rcdff9710188c4cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8b03fd02d5c7453e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf125533db6714da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R73fdd7c7eef44a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R7c4989cf42ff41c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R44f303add1cb497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rce01bdcc5c7f4580"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4cd76356b43849eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd60d1bdc9576485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4964852fc6e4e3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5704deac18cf4975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R2052ccc65c9c442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R9fea1affd62241aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="202">
+  <x:fills count="205">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1100,6 +1100,21 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1187,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1200">
+  <x:cellXfs count="1221">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4230,11 +4245,58 @@
     <x:xf numFmtId="0" fontId="1" fillId="200" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="202" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="203" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="203" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="203" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="204" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="203" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="462">
+  <x:dxfs count="483">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7664,6 +7726,237 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9592,39 +9885,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1179" t="str">
+      <x:c r="A1" s="1200" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1180" t="str">
+      <x:c r="B1" s="1201" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1180" t="str">
+      <x:c r="C1" s="1201" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1180" t="str">
+      <x:c r="D1" s="1201" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1181" t="str">
+      <x:c r="E1" s="1202" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1197" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B2" s="1198" t="n">
+      <x:c r="A2" s="1218" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="B2" s="1219" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1198" t="n">
+      <x:c r="C2" s="1219" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1198" t="str">
-        <x:v>Restore Railway deployment capability, deploy b4cabb9 or later, then verify BOT-001 with the bounded production smoke and expand BOT-004 into real-client RU/UZ/EN transcripts. Continue Inline client, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
-      </x:c>
-      <x:c r="E2" s="1198" t="str">
-        <x:v>PR #79 / b4cabb9 implemented the canonical Telegram contract and 1248-row dialogue DSL; all 238 legacy rows map and CI is green. Railway rejected deployment because the trial expired, so production remains on 6714227 and BOT-001/BOT-004 live gates stay blocked. Existing production health remains 200.</x:v>
+      <x:c r="D2" s="1219" t="str">
+        <x:v>Expand BOT-004 into broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts. Continue the separate Inline visual/client matrix, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1219" t="str">
+        <x:v>Railway 37a91c7a deployed clean main 4050172 after plan renewal. Health 200, polling-aware monitor and five-action production dispatch smoke passed with cleanup. BOT-001 is Passed; BOT-004 is deployed and automated but remains In Progress until broader real-client transcripts exist.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -9635,13 +9928,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1199" t="str">
+      <x:c r="A4" s="1220" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1199" t="str">
+      <x:c r="B4" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1199" t="str">
+      <x:c r="C4" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -9697,16 +9990,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1199" t="str">
+      <x:c r="A9" s="1220" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1199" t="str">
+      <x:c r="B9" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1199" t="str">
+      <x:c r="C9" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1199" t="str">
+      <x:c r="D9" s="1220" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -9783,13 +10076,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1199" t="str">
+      <x:c r="A15" s="1220" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1199" t="str">
+      <x:c r="B15" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1199" t="str">
+      <x:c r="C15" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -9873,13 +10166,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1199" t="str">
+      <x:c r="A22" s="1220" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1199" t="str">
+      <x:c r="B22" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1199" t="str">
+      <x:c r="C22" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -9891,7 +10184,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -9905,7 +10198,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -9919,7 +10212,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -9943,13 +10236,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="455" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="456" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="457" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="458" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="459" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="460" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="461" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="476" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="477" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="478" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="479" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="480" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="481" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="482" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -20854,6 +21147,32 @@
       </x:c>
       <x:c r="H94" t="str">
         <x:v>Renew/select a Railway plan, deploy b4cabb9 or later, verify /healthz and polling leader, rerun the bounded five-action production smoke, then capture broader real-client RU/UZ/EN transcripts before marking BOT-001/BOT-004 release gates Passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>QA-TELEGRAM-CONTRACT-PROD-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B95" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>Canonical Telegram contract production deployment and bounded live dispatch QA</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Railway deployment 37a91c7a from clean main 4050172; healthz; polling-aware monitor:prod; prod:telegram-polling-dispatch-smoke</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Passed: deployment SUCCESS; home/health 200; polling webhook boundary 401/503; getMe, pending=0, singleton leader and AI provider passed; confidence, trusted-person, recheck, disagreement and domain-methodology replies passed; Bot API replies and synthetic DB rows were cleaned up.</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>BOT-001, BOT-004, BOT-006</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>The dispatch harness was restricted to TELEGRAM_QA_CHAT_ID, acquired no polling lease and did not expose identifiers. Follow-ups reused prior results, did not auto-alert a trusted person, did not pretend to re-run analysis and stayed non-accusatory. The legacy webhook-only prod:smoke reported its expected polling-mode 503/empty-URL mismatch; the polling-aware monitor passed.</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>BOT-001 is release-passed. Continue BOT-004 with broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts and keep Inline visual delivery separate because it requires a real client-generated inline_query_id.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20882,46 +21201,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1179" t="str">
+      <x:c r="A1" s="1200" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1180" t="str">
+      <x:c r="B1" s="1201" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1180" t="str">
+      <x:c r="C1" s="1201" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1180" t="str">
+      <x:c r="D1" s="1201" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1180" t="str">
+      <x:c r="E1" s="1201" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1180" t="str">
+      <x:c r="F1" s="1201" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1180" t="str">
+      <x:c r="G1" s="1201" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1180" t="str">
+      <x:c r="H1" s="1201" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1180" t="str">
+      <x:c r="I1" s="1201" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1180" t="str">
+      <x:c r="J1" s="1201" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1180" t="str">
+      <x:c r="K1" s="1201" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1180" t="str">
+      <x:c r="L1" s="1201" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1180" t="str">
+      <x:c r="M1" s="1201" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1181" t="str">
+      <x:c r="N1" s="1202" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -21872,29 +22191,27 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F24" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G24" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H24" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I24" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J24" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K24" s="615" t="str">
         <x:v>Telegram / Product</x:v>
       </x:c>
-      <x:c r="L24" s="615" t="str">
-        <x:v>Railway plan expired; deploy b4cabb9 + live smoke</x:v>
-      </x:c>
+      <x:c r="L24" s="615" t="str"/>
       <x:c r="M24" s="615" t="str"/>
       <x:c r="N24" s="615" t="str">
-        <x:v>Canonical meta.*, victim.*, followup.*, panic.* and input.risk_check registry now binds response actions to direct/Inline persistence, trusted-contact and reply-size boundaries. Runtime reply enforcement is active in direct handlers. PR #79 / b4cabb9; GitHub app CI and Supabase reset/schema lint/pgTAP passed; full suite 4135/4135, Telegram 3431/3431, TypeScript, lint, build and npm audit green. Railway rejected deployment because the trial expired, so production still runs 6714227.</x:v>
+        <x:v>Canonical meta.*, victim.*, followup.*, panic.* and input.risk_check registry binds response actions to direct/Inline persistence, trusted-contact and reply-size boundaries. PR #79 / b4cabb9 passed 4135/4135 full and 3431/3431 Telegram tests plus GitHub app and Supabase CI. Railway deployment 37a91c7a from clean main 4050172 succeeded after plan renewal; health 200, polling-aware production monitor passed, and the bounded five-action production dispatch smoke passed with Bot API/synthetic DB cleanup read-back.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -21997,26 +22314,24 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J27" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
       </x:c>
-      <x:c r="L27" s="615" t="str">
-        <x:v>Railway plan expired; deploy + broader real-client transcript matrix</x:v>
-      </x:c>
+      <x:c r="L27" s="615" t="str"/>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>Deterministic DSL now covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. Recent, orphan, stale and new-artifact routing plus &lt;=4096 response bounds pass. PR #79 / b4cabb9. Broader real Telegram-client transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
+        <x:v>Deterministic DSL covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. PR #79 / b4cabb9 is deployed via Railway 37a91c7a; polling monitor and the five-action production dispatch smoke passed. Broader real Telegram-client RU/UZ/EN transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -22430,13 +22745,13 @@
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I37">
-    <x:cfRule type="containsText" dxfId="441" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="442" priority="9" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="443" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="444" priority="11" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="445" priority="12" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="446" priority="13" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="447" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="462" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="463" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="464" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="465" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="466" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="467" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -22505,40 +22820,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1179" t="str">
+      <x:c r="A1" s="1200" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1180" t="str">
+      <x:c r="B1" s="1201" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1180" t="str">
+      <x:c r="C1" s="1201" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1180" t="str">
+      <x:c r="D1" s="1201" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1180" t="str">
+      <x:c r="E1" s="1201" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1180" t="str">
+      <x:c r="F1" s="1201" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1180" t="str">
+      <x:c r="G1" s="1201" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1180" t="str">
+      <x:c r="H1" s="1201" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1180" t="str">
+      <x:c r="I1" s="1201" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1180" t="str">
+      <x:c r="J1" s="1201" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1180" t="str">
+      <x:c r="K1" s="1201" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1181" t="str">
+      <x:c r="L1" s="1202" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -23304,13 +23619,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="448" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="449" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="450" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="451" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="452" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="453" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="454" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="469" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="470" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="471" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="472" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="473" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="474" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
docs: record Telegram contract production verification (#81)
Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rc72721937bf442f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R29020785b8f54fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd658b958aa6d465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rcdff9710188c4cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R8b03fd02d5c7453e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rf125533db6714da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R73fdd7c7eef44a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R7c4989cf42ff41c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R44f303add1cb497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rce01bdcc5c7f4580"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4cd76356b43849eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd60d1bdc9576485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4964852fc6e4e3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5704deac18cf4975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R2052ccc65c9c442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R9fea1affd62241aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -93,7 +93,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="202">
+  <x:fills count="205">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1100,6 +1100,21 @@
         <x:fgColor rgb="FFF8FAFC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="11">
     <x:border/>
@@ -1187,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1200">
+  <x:cellXfs count="1221">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4230,11 +4245,58 @@
     <x:xf numFmtId="0" fontId="1" fillId="200" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="202" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="202" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="203" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="203" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="203" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="204" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="204" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="204" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="203" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="462">
+  <x:dxfs count="483">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -7664,6 +7726,237 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9592,39 +9885,39 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1179" t="str">
+      <x:c r="A1" s="1200" t="str">
         <x:v>Generated</x:v>
       </x:c>
-      <x:c r="B1" s="1180" t="str">
+      <x:c r="B1" s="1201" t="str">
         <x:v>Feature rows</x:v>
       </x:c>
-      <x:c r="C1" s="1180" t="str">
+      <x:c r="C1" s="1201" t="str">
         <x:v>Current security items</x:v>
       </x:c>
-      <x:c r="D1" s="1180" t="str">
+      <x:c r="D1" s="1201" t="str">
         <x:v>Next phase</x:v>
       </x:c>
-      <x:c r="E1" s="1181" t="str">
+      <x:c r="E1" s="1202" t="str">
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="72" customHeight="1">
-      <x:c r="A2" s="1197" t="n">
-        <x:v>46214</x:v>
-      </x:c>
-      <x:c r="B2" s="1198" t="n">
+      <x:c r="A2" s="1218" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="B2" s="1219" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C2" s="1198" t="n">
+      <x:c r="C2" s="1219" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D2" s="1198" t="str">
-        <x:v>Restore Railway deployment capability, deploy b4cabb9 or later, then verify BOT-001 with the bounded production smoke and expand BOT-004 into real-client RU/UZ/EN transcripts. Continue Inline client, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
-      </x:c>
-      <x:c r="E2" s="1198" t="str">
-        <x:v>PR #79 / b4cabb9 implemented the canonical Telegram contract and 1248-row dialogue DSL; all 238 legacy rows map and CI is green. Railway rejected deployment because the trial expired, so production remains on 6714227 and BOT-001/BOT-004 live gates stay blocked. Existing production health remains 200.</x:v>
+      <x:c r="D2" s="1219" t="str">
+        <x:v>Expand BOT-004 into broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts. Continue the separate Inline visual/client matrix, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
+      </x:c>
+      <x:c r="E2" s="1219" t="str">
+        <x:v>Railway 37a91c7a deployed clean main 4050172 after plan renewal. Health 200, polling-aware monitor and five-action production dispatch smoke passed with cleanup. BOT-001 is Passed; BOT-004 is deployed and automated but remains In Progress until broader real-client transcripts exist.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -9635,13 +9928,13 @@
       <x:c r="E3" s="629"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="1199" t="str">
+      <x:c r="A4" s="1220" t="str">
         <x:v>Feature Status</x:v>
       </x:c>
-      <x:c r="B4" s="1199" t="str">
+      <x:c r="B4" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C4" s="1199" t="str">
+      <x:c r="C4" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D4" s="629"/>
@@ -9697,16 +9990,16 @@
       <x:c r="E8" s="629"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="1199" t="str">
+      <x:c r="A9" s="1220" t="str">
         <x:v>Release Priority</x:v>
       </x:c>
-      <x:c r="B9" s="1199" t="str">
+      <x:c r="B9" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
-      <x:c r="C9" s="1199" t="str">
+      <x:c r="C9" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="D9" s="1199" t="str">
+      <x:c r="D9" s="1220" t="str">
         <x:v>Order</x:v>
       </x:c>
       <x:c r="E9" s="629"/>
@@ -9783,13 +10076,13 @@
       <x:c r="E14" s="629"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="1199" t="str">
+      <x:c r="A15" s="1220" t="str">
         <x:v>Current Security Status</x:v>
       </x:c>
-      <x:c r="B15" s="1199" t="str">
+      <x:c r="B15" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C15" s="1199" t="str">
+      <x:c r="C15" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D15" s="629"/>
@@ -9873,13 +10166,13 @@
       <x:c r="E21" s="629"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="1199" t="str">
+      <x:c r="A22" s="1220" t="str">
         <x:v>Release Gate State</x:v>
       </x:c>
-      <x:c r="B22" s="1199" t="str">
+      <x:c r="B22" s="1220" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C22" s="1199" t="str">
+      <x:c r="C22" s="1220" t="str">
         <x:v>Meaning</x:v>
       </x:c>
       <x:c r="D22" s="629"/>
@@ -9891,7 +10184,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -9905,7 +10198,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -9919,7 +10212,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -9943,13 +10236,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="A16:B26">
-    <x:cfRule type="containsText" dxfId="455" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="456" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="457" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="458" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="459" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="460" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="461" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="476" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="477" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="478" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="479" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="480" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="481" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="482" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -20854,6 +21147,32 @@
       </x:c>
       <x:c r="H94" t="str">
         <x:v>Renew/select a Railway plan, deploy b4cabb9 or later, verify /healthz and polling leader, rerun the bounded five-action production smoke, then capture broader real-client RU/UZ/EN transcripts before marking BOT-001/BOT-004 release gates Passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>QA-TELEGRAM-CONTRACT-PROD-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B95" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>Canonical Telegram contract production deployment and bounded live dispatch QA</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Railway deployment 37a91c7a from clean main 4050172; healthz; polling-aware monitor:prod; prod:telegram-polling-dispatch-smoke</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Passed: deployment SUCCESS; home/health 200; polling webhook boundary 401/503; getMe, pending=0, singleton leader and AI provider passed; confidence, trusted-person, recheck, disagreement and domain-methodology replies passed; Bot API replies and synthetic DB rows were cleaned up.</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>BOT-001, BOT-004, BOT-006</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>The dispatch harness was restricted to TELEGRAM_QA_CHAT_ID, acquired no polling lease and did not expose identifiers. Follow-ups reused prior results, did not auto-alert a trusted person, did not pretend to re-run analysis and stayed non-accusatory. The legacy webhook-only prod:smoke reported its expected polling-mode 503/empty-URL mismatch; the polling-aware monitor passed.</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>BOT-001 is release-passed. Continue BOT-004 with broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts and keep Inline visual delivery separate because it requires a real client-generated inline_query_id.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20882,46 +21201,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1179" t="str">
+      <x:c r="A1" s="1200" t="str">
         <x:v>Gate ID</x:v>
       </x:c>
-      <x:c r="B1" s="1180" t="str">
+      <x:c r="B1" s="1201" t="str">
         <x:v>Work Item</x:v>
       </x:c>
-      <x:c r="C1" s="1180" t="str">
+      <x:c r="C1" s="1201" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="D1" s="1180" t="str">
+      <x:c r="D1" s="1201" t="str">
         <x:v>Implementation</x:v>
       </x:c>
-      <x:c r="E1" s="1180" t="str">
+      <x:c r="E1" s="1201" t="str">
         <x:v>Automated QA</x:v>
       </x:c>
-      <x:c r="F1" s="1180" t="str">
+      <x:c r="F1" s="1201" t="str">
         <x:v>Live QA</x:v>
       </x:c>
-      <x:c r="G1" s="1180" t="str">
+      <x:c r="G1" s="1201" t="str">
         <x:v>Security Validation</x:v>
       </x:c>
-      <x:c r="H1" s="1180" t="str">
+      <x:c r="H1" s="1201" t="str">
         <x:v>Deployment</x:v>
       </x:c>
-      <x:c r="I1" s="1180" t="str">
+      <x:c r="I1" s="1201" t="str">
         <x:v>Release Gate</x:v>
       </x:c>
-      <x:c r="J1" s="1180" t="str">
+      <x:c r="J1" s="1201" t="str">
         <x:v>Evidence Date</x:v>
       </x:c>
-      <x:c r="K1" s="1180" t="str">
+      <x:c r="K1" s="1201" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="L1" s="1180" t="str">
+      <x:c r="L1" s="1201" t="str">
         <x:v>Blocked By</x:v>
       </x:c>
-      <x:c r="M1" s="1180" t="str">
+      <x:c r="M1" s="1201" t="str">
         <x:v>Supersedes</x:v>
       </x:c>
-      <x:c r="N1" s="1181" t="str">
+      <x:c r="N1" s="1202" t="str">
         <x:v>Evidence / Notes</x:v>
       </x:c>
     </x:row>
@@ -21872,29 +22191,27 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F24" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G24" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H24" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I24" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J24" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K24" s="615" t="str">
         <x:v>Telegram / Product</x:v>
       </x:c>
-      <x:c r="L24" s="615" t="str">
-        <x:v>Railway plan expired; deploy b4cabb9 + live smoke</x:v>
-      </x:c>
+      <x:c r="L24" s="615" t="str"/>
       <x:c r="M24" s="615" t="str"/>
       <x:c r="N24" s="615" t="str">
-        <x:v>Canonical meta.*, victim.*, followup.*, panic.* and input.risk_check registry now binds response actions to direct/Inline persistence, trusted-contact and reply-size boundaries. Runtime reply enforcement is active in direct handlers. PR #79 / b4cabb9; GitHub app CI and Supabase reset/schema lint/pgTAP passed; full suite 4135/4135, Telegram 3431/3431, TypeScript, lint, build and npm audit green. Railway rejected deployment because the trial expired, so production still runs 6714227.</x:v>
+        <x:v>Canonical meta.*, victim.*, followup.*, panic.* and input.risk_check registry binds response actions to direct/Inline persistence, trusted-contact and reply-size boundaries. PR #79 / b4cabb9 passed 4135/4135 full and 3431/3431 Telegram tests plus GitHub app and Supabase CI. Railway deployment 37a91c7a from clean main 4050172 succeeded after plan renewal; health 200, polling-aware production monitor passed, and the bounded five-action production dispatch smoke passed with Bot API/synthetic DB cleanup read-back.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -21997,26 +22314,24 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J27" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
       </x:c>
-      <x:c r="L27" s="615" t="str">
-        <x:v>Railway plan expired; deploy + broader real-client transcript matrix</x:v>
-      </x:c>
+      <x:c r="L27" s="615" t="str"/>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>Deterministic DSL now covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. Recent, orphan, stale and new-artifact routing plus &lt;=4096 response bounds pass. PR #79 / b4cabb9. Broader real Telegram-client transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
+        <x:v>Deterministic DSL covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. PR #79 / b4cabb9 is deployed via Railway 37a91c7a; polling monitor and the five-action production dispatch smoke passed. Broader real Telegram-client RU/UZ/EN transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -22430,13 +22745,13 @@
     <x:cfRule type="containsText" dxfId="342" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I37">
-    <x:cfRule type="containsText" dxfId="441" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="442" priority="9" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="443" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="444" priority="11" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="445" priority="12" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="446" priority="13" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="447" priority="14" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="462" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="463" priority="9" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="464" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="465" priority="11" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="466" priority="12" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="467" priority="13" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -22505,40 +22820,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="1179" t="str">
+      <x:c r="A1" s="1200" t="str">
         <x:v>Finding ID</x:v>
       </x:c>
-      <x:c r="B1" s="1180" t="str">
+      <x:c r="B1" s="1201" t="str">
         <x:v>Priority</x:v>
       </x:c>
-      <x:c r="C1" s="1180" t="str">
+      <x:c r="C1" s="1201" t="str">
         <x:v>Area</x:v>
       </x:c>
-      <x:c r="D1" s="1180" t="str">
+      <x:c r="D1" s="1201" t="str">
         <x:v>Finding</x:v>
       </x:c>
-      <x:c r="E1" s="1180" t="str">
+      <x:c r="E1" s="1201" t="str">
         <x:v>Affected Path</x:v>
       </x:c>
-      <x:c r="F1" s="1180" t="str">
+      <x:c r="F1" s="1201" t="str">
         <x:v>Current Status</x:v>
       </x:c>
-      <x:c r="G1" s="1180" t="str">
+      <x:c r="G1" s="1201" t="str">
         <x:v>Owner</x:v>
       </x:c>
-      <x:c r="H1" s="1180" t="str">
+      <x:c r="H1" s="1201" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="I1" s="1180" t="str">
+      <x:c r="I1" s="1201" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="J1" s="1180" t="str">
+      <x:c r="J1" s="1201" t="str">
         <x:v>Next Step</x:v>
       </x:c>
-      <x:c r="K1" s="1180" t="str">
+      <x:c r="K1" s="1201" t="str">
         <x:v>Acceptance Criteria</x:v>
       </x:c>
-      <x:c r="L1" s="1181" t="str">
+      <x:c r="L1" s="1202" t="str">
         <x:v>Last Verified</x:v>
       </x:c>
     </x:row>
@@ -23304,13 +23619,13 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
-    <x:cfRule type="containsText" dxfId="448" priority="1" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="449" priority="2" operator="containsText" text="Fixed Local"/>
-    <x:cfRule type="containsText" dxfId="450" priority="3" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="451" priority="4" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="452" priority="5" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="453" priority="6" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="454" priority="7" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="469" priority="1" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="470" priority="2" operator="containsText" text="Fixed Local"/>
+    <x:cfRule type="containsText" dxfId="471" priority="3" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="472" priority="4" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="473" priority="5" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="474" priority="6" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
Fix security revalidation findings
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R44f303add1cb497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rce01bdcc5c7f4580"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4cd76356b43849eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd60d1bdc9576485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4964852fc6e4e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5704deac18cf4975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R2052ccc65c9c442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R9fea1affd62241aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R752edd750c7d439d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf51954a7b3cf43ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R56295e6b3f494817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc509fa81914d474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4b27414a6734dab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra9bec3428dd14783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R9309644b54b4491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0f1c9dc1b572465b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1202,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1221">
+  <x:cellXfs count="1227">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4292,11 +4292,23 @@
     <x:xf numFmtId="0" fontId="1" fillId="203" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="483">
+  <x:dxfs count="567">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -9376,6 +9388,1007 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9393,11 +10406,11 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF92400E"/>
+        <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9415,6 +10428,50 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
@@ -9426,6 +10483,28 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
@@ -9459,154 +10538,11 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF166534"/>
+        <x:color rgb="FF4B5563"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF92400E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF115E59"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFCCFBF1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF1E40AF"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDBEAFE"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF92400E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF115E59"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFCCFBF1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF1E40AF"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDBEAFE"/>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9911,13 +10847,13 @@
       </x:c>
       <x:c r="C2" s="1219" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
-        <x:v>20</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Expand BOT-004 into broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts. Continue the separate Inline visual/client matrix, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
+        <x:v>All 15 validated findings are fixed locally and the count-only production admin preflight is green. Next: commit and CI, apply the production migration, deploy the exact commit, run targeted trust/privacy/Inline/media/provider/monitor smokes and read-back, complete historical count-only privacy review and close a 72-hour canary. Keep broad real-client RU/UZ/EN bot/Inline evidence separate.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Railway 37a91c7a deployed clean main 4050172 after plan renewal. Health 200, polling-aware monitor and five-action production dispatch smoke passed with cleanup. BOT-001 is Passed; BOT-004 is deployed and automated but remains In Progress until broader real-client transcripts exist.</x:v>
+        <x:v>Local remediation evidence: 4222/4222 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint and original-path PoCs. Production count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Current security rows are In Progress until deployment/read-back; no production state was changed by this verification. Canonical source and evidence copy are synchronized.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -10029,7 +10965,7 @@
       </x:c>
       <x:c r="C11" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A11)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D11" s="629" t="n">
         <x:v>2</x:v>
@@ -10045,7 +10981,7 @@
       </x:c>
       <x:c r="C12" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A12)</x:f>
-        <x:v>5</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D12" s="629" t="n">
         <x:v>3</x:v>
@@ -10061,7 +10997,7 @@
       </x:c>
       <x:c r="C13" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A13)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D13" s="629" t="n">
         <x:v>4</x:v>
@@ -10108,10 +11044,10 @@
       </x:c>
       <x:c r="B17" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A17)</x:f>
-        <x:v>0</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C17" s="629" t="str">
-        <x:v>Implementation is underway.</x:v>
+        <x:v>Local fixes and regressions pass; deployment/read-back is pending.</x:v>
       </x:c>
       <x:c r="D17" s="629"/>
       <x:c r="E17" s="629"/>
@@ -10184,7 +11120,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -10226,7 +11162,7 @@
       </x:c>
       <x:c r="B26" s="631" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A26)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C26" s="631" t="str">
         <x:v>Outside the current release scope.</x:v>
@@ -21175,6 +22111,58 @@
         <x:v>BOT-001 is release-passed. Continue BOT-004 with broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts and keep Inline visual delivery separate because it requires a real client-generated inline_query_id.</x:v>
       </x:c>
     </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>QA-SECURITY-REVALIDATION-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B96" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>Full repository security revalidation</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>388-file inventory; 109 review receipts; 62 raw candidates; 38 independently validated; 24 attack-path candidates; local canonical finalizer and report validator; 4135 tests; TypeScript/lint/build/npm audit; production health/monitor read-only checks</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Completed: 15 final instances (1 High, 9 Medium, 5 Low), 27 reviewed surfaces, 5 explicitly deferred live/product-intent questions.</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>RC-001, OPS-001, SEC-2026-0712-001..015</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>No production data, secrets or repository source changed. Reports, JSON, hardening portfolio and PoCs are in outputs/security_revalidation_2026-07-12.</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>Fix High/P1 first, then nine Medium/P2; keep five Low/P3 tracked. Re-run all original probes, deploy, run targeted smokes and 72-hour canary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>QA-SECURITY-FIX-VERIFICATION-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B97" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Local remediation verification for 15 revalidation findings</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; supabase db reset --local --yes; supabase test db --local; supabase db lint --local --level error --fail-on error; railway run npm run admin-role:preflight; fixed-state and old-assertion PoCs</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Passed locally: 4222/4222 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; fixed-state redaction/QR; old contact/provider/domain/Inline/public-post/moderation/passport/media-order assertions rejected. Production count-only admin preflight passed: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>SEC-2026-0712-001..015, OPS-001, RC-001</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>No production deployment, migration or production-data mutation. The production admin preflight was read-only and logged counts only. One external appeal PoC is excluded by the repository Vitest include pattern; the equivalent real mocked-insert regression is included in the green suite. GitHub action tag SHAs were verified with git ls-remote.</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Commit and run CI; apply the production migration; deploy exact commit; run target smokes/read-back; historical count-only privacy review; 72-hour canary; then reclassify findings.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -22437,7 +23425,7 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H30" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I30" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -22449,13 +23437,13 @@
         <x:v>Telegram / QA</x:v>
       </x:c>
       <x:c r="L30" s="615" t="str">
-        <x:v>Gate 1 Inline deploy</x:v>
+        <x:v>Telegram Desktop/Android/iOS real-client visual and insertion QA</x:v>
       </x:c>
       <x:c r="M30" s="615" t="str">
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>55x3 reason presentations now pass through the real adapter; remaining matrix includes webhook config, faults, prefix/load and stateless follow-ups.</x:v>
+        <x:v>Backend is deployed at 4bd9403. Automated Inline protocol/privacy coverage is green; real-client visual/insertion evidence remains the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -22732,6 +23720,636 @@
       <x:c r="M37" s="615" t="str"/>
       <x:c r="N37" s="615" t="str">
         <x:v>Go requires 0 open P0/P1 and fresh production/security/restore evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="614" t="str">
+        <x:v>SEC-2026-0712-001</x:v>
+      </x:c>
+      <x:c r="B38" s="614" t="str">
+        <x:v>Embedded official contact tokens can mark unrelated attacker content Safe</x:v>
+      </x:c>
+      <x:c r="C38" s="614" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D38" s="614" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E38" s="614" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F38" s="614" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G38" s="614" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H38" s="614" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I38" s="614" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J38" s="617" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K38" s="614" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="L38" s="614" t="str">
+        <x:v>SEC-2026-0712-001</x:v>
+      </x:c>
+      <x:c r="M38" s="614"/>
+      <x:c r="N38" s="614" t="str">
+        <x:v>High/P1 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="615" t="str">
+        <x:v>SEC-2026-0712-002</x:v>
+      </x:c>
+      <x:c r="B39" s="615" t="str">
+        <x:v>Public reports retain passwords, separated OTPs and recovery phrases</x:v>
+      </x:c>
+      <x:c r="C39" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D39" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E39" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F39" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G39" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H39" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I39" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J39" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K39" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="L39" s="615" t="str">
+        <x:v>SEC-2026-0712-002</x:v>
+      </x:c>
+      <x:c r="M39" s="615"/>
+      <x:c r="N39" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="615" t="str">
+        <x:v>SEC-2026-0712-003</x:v>
+      </x:c>
+      <x:c r="B40" s="615" t="str">
+        <x:v>Appeal reason/contact fields can retain secrets</x:v>
+      </x:c>
+      <x:c r="C40" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D40" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E40" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F40" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G40" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H40" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I40" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J40" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K40" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="L40" s="615" t="str">
+        <x:v>SEC-2026-0712-003</x:v>
+      </x:c>
+      <x:c r="M40" s="615"/>
+      <x:c r="N40" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="615" t="str">
+        <x:v>SEC-2026-0712-004</x:v>
+      </x:c>
+      <x:c r="B41" s="615" t="str">
+        <x:v>Decoded QR credentials can be retained in check records</x:v>
+      </x:c>
+      <x:c r="C41" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D41" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E41" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F41" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G41" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H41" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I41" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J41" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K41" s="615" t="str">
+        <x:v>Media / Privacy</x:v>
+      </x:c>
+      <x:c r="L41" s="615" t="str">
+        <x:v>SEC-2026-0712-004</x:v>
+      </x:c>
+      <x:c r="M41" s="615"/>
+      <x:c r="N41" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="615" t="str">
+        <x:v>SEC-2026-0712-005</x:v>
+      </x:c>
+      <x:c r="B42" s="615" t="str">
+        <x:v>Inline results can republish secrets into selected chats</x:v>
+      </x:c>
+      <x:c r="C42" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D42" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E42" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F42" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G42" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H42" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I42" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J42" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K42" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="L42" s="615" t="str">
+        <x:v>SEC-2026-0712-005</x:v>
+      </x:c>
+      <x:c r="M42" s="615"/>
+      <x:c r="N42" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="615" t="str">
+        <x:v>SEC-2026-0712-006</x:v>
+      </x:c>
+      <x:c r="B43" s="615" t="str">
+        <x:v>Public-post checks can retain passwords and recovery phrases</x:v>
+      </x:c>
+      <x:c r="C43" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D43" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E43" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F43" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G43" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H43" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I43" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J43" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K43" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="L43" s="615" t="str">
+        <x:v>SEC-2026-0712-006</x:v>
+      </x:c>
+      <x:c r="M43" s="615"/>
+      <x:c r="N43" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="615" t="str">
+        <x:v>SEC-2026-0712-007</x:v>
+      </x:c>
+      <x:c r="B44" s="615" t="str">
+        <x:v>Report metadata can forward secrets to moderator Telegram</x:v>
+      </x:c>
+      <x:c r="C44" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D44" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E44" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F44" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G44" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H44" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I44" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J44" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K44" s="615" t="str">
+        <x:v>Telegram / Moderation</x:v>
+      </x:c>
+      <x:c r="L44" s="615" t="str">
+        <x:v>SEC-2026-0712-007</x:v>
+      </x:c>
+      <x:c r="M44" s="615"/>
+      <x:c r="N44" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="615" t="str">
+        <x:v>SEC-2026-0712-008</x:v>
+      </x:c>
+      <x:c r="B45" s="615" t="str">
+        <x:v>Removed admin eligibility is not revoked from durable roles</x:v>
+      </x:c>
+      <x:c r="C45" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D45" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E45" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F45" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G45" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H45" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I45" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J45" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K45" s="615" t="str">
+        <x:v>Data / Security</x:v>
+      </x:c>
+      <x:c r="L45" s="615" t="str">
+        <x:v>SEC-2026-0712-008</x:v>
+      </x:c>
+      <x:c r="M45" s="615"/>
+      <x:c r="N45" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="615" t="str">
+        <x:v>SEC-2026-0712-009</x:v>
+      </x:c>
+      <x:c r="B46" s="615" t="str">
+        <x:v>Embed meta-intents bypass shared limit and append telemetry</x:v>
+      </x:c>
+      <x:c r="C46" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D46" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E46" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F46" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G46" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H46" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I46" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J46" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K46" s="615" t="str">
+        <x:v>Backend / Data</x:v>
+      </x:c>
+      <x:c r="L46" s="615" t="str">
+        <x:v>SEC-2026-0712-009</x:v>
+      </x:c>
+      <x:c r="M46" s="615"/>
+      <x:c r="N46" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="615" t="str">
+        <x:v>SEC-2026-0712-010</x:v>
+      </x:c>
+      <x:c r="B47" s="615" t="str">
+        <x:v>Production-monitor secrets are visible to mutable setup code</x:v>
+      </x:c>
+      <x:c r="C47" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D47" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E47" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F47" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G47" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H47" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I47" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J47" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K47" s="615" t="str">
+        <x:v>DevOps / Security</x:v>
+      </x:c>
+      <x:c r="L47" s="615" t="str">
+        <x:v>SEC-2026-0712-010</x:v>
+      </x:c>
+      <x:c r="M47" s="615"/>
+      <x:c r="N47" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="615" t="str">
+        <x:v>SEC-2026-0712-011</x:v>
+      </x:c>
+      <x:c r="B48" s="615" t="str">
+        <x:v>Report images download before shared media admission</x:v>
+      </x:c>
+      <x:c r="C48" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D48" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E48" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F48" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G48" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H48" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I48" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J48" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K48" s="615" t="str">
+        <x:v>Telegram / Platform</x:v>
+      </x:c>
+      <x:c r="L48" s="615" t="str">
+        <x:v>SEC-2026-0712-011</x:v>
+      </x:c>
+      <x:c r="M48" s="615"/>
+      <x:c r="N48" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="615" t="str">
+        <x:v>SEC-2026-0712-012</x:v>
+      </x:c>
+      <x:c r="B49" s="615" t="str">
+        <x:v>Benign provider evidence can omit phishing URL and return Safe</x:v>
+      </x:c>
+      <x:c r="C49" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D49" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E49" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F49" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G49" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H49" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I49" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J49" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K49" s="615" t="str">
+        <x:v>AI / Risk</x:v>
+      </x:c>
+      <x:c r="L49" s="615" t="str">
+        <x:v>SEC-2026-0712-012</x:v>
+      </x:c>
+      <x:c r="M49" s="615"/>
+      <x:c r="N49" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="615" t="str">
+        <x:v>SEC-2026-0712-013</x:v>
+      </x:c>
+      <x:c r="B50" s="615" t="str">
+        <x:v>Official-domain skeleton collisions suppress brand detection</x:v>
+      </x:c>
+      <x:c r="C50" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D50" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E50" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F50" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G50" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H50" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I50" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J50" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K50" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="L50" s="615" t="str">
+        <x:v>SEC-2026-0712-013</x:v>
+      </x:c>
+      <x:c r="M50" s="615"/>
+      <x:c r="N50" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="615" t="str">
+        <x:v>SEC-2026-0712-014</x:v>
+      </x:c>
+      <x:c r="B51" s="615" t="str">
+        <x:v>News-domain skeleton collisions suppress path-brand warning</x:v>
+      </x:c>
+      <x:c r="C51" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D51" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E51" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F51" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G51" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H51" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I51" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J51" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K51" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="L51" s="615" t="str">
+        <x:v>SEC-2026-0712-014</x:v>
+      </x:c>
+      <x:c r="M51" s="615"/>
+      <x:c r="N51" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="615" t="str">
+        <x:v>SEC-2026-0712-015</x:v>
+      </x:c>
+      <x:c r="B52" s="615" t="str">
+        <x:v>Passport request can be answered as stale Safe follow-up</x:v>
+      </x:c>
+      <x:c r="C52" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D52" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E52" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F52" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G52" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H52" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I52" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J52" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K52" s="615" t="str">
+        <x:v>Telegram / Product</x:v>
+      </x:c>
+      <x:c r="L52" s="615" t="str">
+        <x:v>SEC-2026-0712-015</x:v>
+      </x:c>
+      <x:c r="M52" s="615"/>
+      <x:c r="N52" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -22753,7 +24371,16 @@
     <x:cfRule type="containsText" dxfId="467" priority="13" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="14">
+  <x:conditionalFormatting sqref="D2:I52">
+    <x:cfRule type="containsText" dxfId="560" priority="15" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="561" priority="16" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="562" priority="17" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="563" priority="18" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="564" priority="19" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="565" priority="20" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="566" priority="21" operator="containsText" text="Deferred"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="C2:C36">
       <x:formula1>"P0,P1,P2,P3"</x:formula1>
     </x:dataValidation>
@@ -22796,6 +24423,24 @@
     <x:dataValidation type="list" sqref="I2:I37">
       <x:formula1>"Blocked,In Progress,Passed,Deferred"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="C38:C52">
+      <x:formula1>"P0,P1,P2,P3"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D38:D52">
+      <x:formula1>"Not Started,In Progress,Fixed Local,Implemented,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E38:F52">
+      <x:formula1>"Pending,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G38:G52">
+      <x:formula1>"Pending,Passed Local,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H38:H52">
+      <x:formula1>"Not Deployed,Pending,Deployed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I38:I52">
+      <x:formula1>"Blocked,In Progress,Passed,Deferred"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -23617,6 +25262,576 @@
         <x:v>46214</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="614" t="str">
+        <x:v>SEC-2026-0712-001</x:v>
+      </x:c>
+      <x:c r="B22" s="614" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C22" s="614" t="str">
+        <x:v>Trust decision</x:v>
+      </x:c>
+      <x:c r="D22" s="614" t="str">
+        <x:v>Embedded official contact tokens can mark unrelated attacker content Safe</x:v>
+      </x:c>
+      <x:c r="E22" s="614" t="str">
+        <x:v>src/lib/risk/check-core.ts:125-143,338-350; src/lib/risk/rules.ts:302-307</x:v>
+      </x:c>
+      <x:c r="F22" s="614" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G22" s="614" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="H22" s="614" t="str">
+        <x:v>Gate 0</x:v>
+      </x:c>
+      <x:c r="I22" s="614" t="str">
+        <x:v>High/P1 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
+      </x:c>
+      <x:c r="J22" s="614" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K22" s="614" t="str">
+        <x:v>Unrelated content cannot become Safe because it merely contains an official token.</x:v>
+      </x:c>
+      <x:c r="L22" s="617" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="615" t="str">
+        <x:v>SEC-2026-0712-002</x:v>
+      </x:c>
+      <x:c r="B23" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C23" s="615" t="str">
+        <x:v>Report privacy</x:v>
+      </x:c>
+      <x:c r="D23" s="615" t="str">
+        <x:v>Public reports retain passwords, separated OTPs and recovery phrases</x:v>
+      </x:c>
+      <x:c r="E23" s="615" t="str">
+        <x:v>src/lib/risk/detect.ts; src/lib/report.functions.ts</x:v>
+      </x:c>
+      <x:c r="F23" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G23" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="H23" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I23" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
+      </x:c>
+      <x:c r="J23" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K23" s="615" t="str">
+        <x:v>Complete reports/entities insert payload contains no supported secret marker.</x:v>
+      </x:c>
+      <x:c r="L23" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="615" t="str">
+        <x:v>SEC-2026-0712-003</x:v>
+      </x:c>
+      <x:c r="B24" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C24" s="615" t="str">
+        <x:v>Appeal privacy</x:v>
+      </x:c>
+      <x:c r="D24" s="615" t="str">
+        <x:v>Appeal reason/contact fields can retain secrets</x:v>
+      </x:c>
+      <x:c r="E24" s="615" t="str">
+        <x:v>src/lib/reputation-appeal.functions.ts; src/lib/risk/detect.ts</x:v>
+      </x:c>
+      <x:c r="F24" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G24" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="H24" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I24" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
+      </x:c>
+      <x:c r="J24" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K24" s="615" t="str">
+        <x:v>No secret marker reaches reason or contact_display; generic unsafe contact is rejected.</x:v>
+      </x:c>
+      <x:c r="L24" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="615" t="str">
+        <x:v>SEC-2026-0712-004</x:v>
+      </x:c>
+      <x:c r="B25" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C25" s="615" t="str">
+        <x:v>QR privacy</x:v>
+      </x:c>
+      <x:c r="D25" s="615" t="str">
+        <x:v>Decoded QR credentials can be retained in check records</x:v>
+      </x:c>
+      <x:c r="E25" s="615" t="str">
+        <x:v>src/lib/risk/qr-decoder.ts; image-intelligence.ts; check-core.ts</x:v>
+      </x:c>
+      <x:c r="F25" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G25" s="615" t="str">
+        <x:v>Media / Privacy</x:v>
+      </x:c>
+      <x:c r="H25" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I25" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
+      </x:c>
+      <x:c r="J25" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K25" s="615" t="str">
+        <x:v>Wi-Fi passwords, otpauth secrets and mnemonic candidates never enter redacted_input.</x:v>
+      </x:c>
+      <x:c r="L25" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="615" t="str">
+        <x:v>SEC-2026-0712-005</x:v>
+      </x:c>
+      <x:c r="B26" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C26" s="615" t="str">
+        <x:v>Telegram Inline privacy</x:v>
+      </x:c>
+      <x:c r="D26" s="615" t="str">
+        <x:v>Inline results can republish secrets into selected chats</x:v>
+      </x:c>
+      <x:c r="E26" s="615" t="str">
+        <x:v>src/lib/telegram/handlers/inline.ts; src/lib/risk/detect.ts</x:v>
+      </x:c>
+      <x:c r="F26" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G26" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="H26" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I26" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
+      </x:c>
+      <x:c r="J26" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K26" s="615" t="str">
+        <x:v>No supported secret marker appears in any Inline article field on real clients.</x:v>
+      </x:c>
+      <x:c r="L26" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="615" t="str">
+        <x:v>SEC-2026-0712-006</x:v>
+      </x:c>
+      <x:c r="B27" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C27" s="615" t="str">
+        <x:v>Public-post privacy</x:v>
+      </x:c>
+      <x:c r="D27" s="615" t="str">
+        <x:v>Public-post checks can retain passwords and recovery phrases</x:v>
+      </x:c>
+      <x:c r="E27" s="615" t="str">
+        <x:v>src/lib/telegram/public-post.server.ts; src/lib/risk/check-core.ts</x:v>
+      </x:c>
+      <x:c r="F27" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G27" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="H27" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I27" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
+      </x:c>
+      <x:c r="J27" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K27" s="615" t="str">
+        <x:v>Mocked check insert contains no secret marker from public-post fixtures.</x:v>
+      </x:c>
+      <x:c r="L27" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="615" t="str">
+        <x:v>SEC-2026-0712-007</x:v>
+      </x:c>
+      <x:c r="B28" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C28" s="615" t="str">
+        <x:v>Moderation privacy</x:v>
+      </x:c>
+      <x:c r="D28" s="615" t="str">
+        <x:v>Report metadata can forward secrets to moderator Telegram</x:v>
+      </x:c>
+      <x:c r="E28" s="615" t="str">
+        <x:v>src/lib/report.functions.ts; moderation-notifier.server.ts</x:v>
+      </x:c>
+      <x:c r="F28" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G28" s="615" t="str">
+        <x:v>Telegram / Moderation</x:v>
+      </x:c>
+      <x:c r="H28" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I28" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
+      </x:c>
+      <x:c r="J28" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K28" s="615" t="str">
+        <x:v>Markdown and plaintext notification payloads contain no secret marker.</x:v>
+      </x:c>
+      <x:c r="L28" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="615" t="str">
+        <x:v>SEC-2026-0712-008</x:v>
+      </x:c>
+      <x:c r="B29" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C29" s="615" t="str">
+        <x:v>Admin authorization</x:v>
+      </x:c>
+      <x:c r="D29" s="615" t="str">
+        <x:v>Removed admin eligibility is not revoked from durable roles</x:v>
+      </x:c>
+      <x:c r="E29" s="615" t="str">
+        <x:v>supabase/migrations/20260629085533_*; src/lib/admin.functions.ts</x:v>
+      </x:c>
+      <x:c r="F29" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G29" s="615" t="str">
+        <x:v>Data / Security</x:v>
+      </x:c>
+      <x:c r="H29" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I29" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+      </x:c>
+      <x:c r="J29" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K29" s="615" t="str">
+        <x:v>Allowlist delete, email drift and confirmation loss immediately deny existing sessions.</x:v>
+      </x:c>
+      <x:c r="L29" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="615" t="str">
+        <x:v>SEC-2026-0712-009</x:v>
+      </x:c>
+      <x:c r="B30" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C30" s="615" t="str">
+        <x:v>Embed availability</x:v>
+      </x:c>
+      <x:c r="D30" s="615" t="str">
+        <x:v>Embed meta-intents bypass shared limit and append telemetry</x:v>
+      </x:c>
+      <x:c r="E30" s="615" t="str">
+        <x:v>src/lib/check.functions.ts; embed-origin-analytics.server.ts</x:v>
+      </x:c>
+      <x:c r="F30" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G30" s="615" t="str">
+        <x:v>Backend / Data</x:v>
+      </x:c>
+      <x:c r="H30" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I30" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
+      </x:c>
+      <x:c r="J30" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K30" s="615" t="str">
+        <x:v>Denied request performs zero analytics inserts; production storage failure fails closed.</x:v>
+      </x:c>
+      <x:c r="L30" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="615" t="str">
+        <x:v>SEC-2026-0712-010</x:v>
+      </x:c>
+      <x:c r="B31" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C31" s="615" t="str">
+        <x:v>CI supply chain</x:v>
+      </x:c>
+      <x:c r="D31" s="615" t="str">
+        <x:v>Production-monitor secrets are visible to mutable setup code</x:v>
+      </x:c>
+      <x:c r="E31" s="615" t="str">
+        <x:v>.github/workflows/prod-monitor.yml</x:v>
+      </x:c>
+      <x:c r="F31" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G31" s="615" t="str">
+        <x:v>DevOps / Security</x:v>
+      </x:c>
+      <x:c r="H31" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I31" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
+      </x:c>
+      <x:c r="J31" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K31" s="615" t="str">
+        <x:v>Policy rejects job-scoped secrets, non-SHA actions and pre-secret install hooks.</x:v>
+      </x:c>
+      <x:c r="L31" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="615" t="str">
+        <x:v>SEC-2026-0712-011</x:v>
+      </x:c>
+      <x:c r="B32" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C32" s="615" t="str">
+        <x:v>Telegram availability</x:v>
+      </x:c>
+      <x:c r="D32" s="615" t="str">
+        <x:v>Report images download before shared media admission</x:v>
+      </x:c>
+      <x:c r="E32" s="615" t="str">
+        <x:v>src/lib/telegram/handlers/report.ts; handlers/check.ts</x:v>
+      </x:c>
+      <x:c r="F32" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G32" s="615" t="str">
+        <x:v>Telegram / Platform</x:v>
+      </x:c>
+      <x:c r="H32" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I32" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
+      </x:c>
+      <x:c r="J32" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K32" s="615" t="str">
+        <x:v>Rate-limited report image makes zero getFile/download calls under concurrency.</x:v>
+      </x:c>
+      <x:c r="L32" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="615" t="str">
+        <x:v>SEC-2026-0712-012</x:v>
+      </x:c>
+      <x:c r="B33" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C33" s="615" t="str">
+        <x:v>Image evidence trust</x:v>
+      </x:c>
+      <x:c r="D33" s="615" t="str">
+        <x:v>Benign provider evidence can omit phishing URL and return Safe</x:v>
+      </x:c>
+      <x:c r="E33" s="615" t="str">
+        <x:v>src/lib/risk/image-intelligence.ts; check-core.ts</x:v>
+      </x:c>
+      <x:c r="F33" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G33" s="615" t="str">
+        <x:v>AI / Risk</x:v>
+      </x:c>
+      <x:c r="H33" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I33" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
+      </x:c>
+      <x:c r="J33" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K33" s="615" t="str">
+        <x:v>Benign provider category plus phishing URL cannot return Safe without trusted local proof.</x:v>
+      </x:c>
+      <x:c r="L33" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="615" t="str">
+        <x:v>SEC-2026-0712-013</x:v>
+      </x:c>
+      <x:c r="B34" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C34" s="615" t="str">
+        <x:v>Domain identity</x:v>
+      </x:c>
+      <x:c r="D34" s="615" t="str">
+        <x:v>Official-domain skeleton collisions suppress brand detection</x:v>
+      </x:c>
+      <x:c r="E34" s="615" t="str">
+        <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
+      </x:c>
+      <x:c r="F34" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G34" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="H34" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I34" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
+      </x:c>
+      <x:c r="J34" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K34" s="615" t="str">
+        <x:v>Confusable hostname cannot inherit official allowlist membership; controls stay valid.</x:v>
+      </x:c>
+      <x:c r="L34" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="615" t="str">
+        <x:v>SEC-2026-0712-014</x:v>
+      </x:c>
+      <x:c r="B35" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C35" s="615" t="str">
+        <x:v>Domain identity</x:v>
+      </x:c>
+      <x:c r="D35" s="615" t="str">
+        <x:v>News-domain skeleton collisions suppress path-brand warning</x:v>
+      </x:c>
+      <x:c r="E35" s="615" t="str">
+        <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
+      </x:c>
+      <x:c r="F35" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G35" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="H35" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I35" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
+      </x:c>
+      <x:c r="J35" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K35" s="615" t="str">
+        <x:v>sp0t.uz cannot inherit spot.uz suppression; similarity only adds evidence.</x:v>
+      </x:c>
+      <x:c r="L35" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="615" t="str">
+        <x:v>SEC-2026-0712-015</x:v>
+      </x:c>
+      <x:c r="B36" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C36" s="615" t="str">
+        <x:v>Telegram dialogue</x:v>
+      </x:c>
+      <x:c r="D36" s="615" t="str">
+        <x:v>Passport request can be answered as stale Safe follow-up</x:v>
+      </x:c>
+      <x:c r="E36" s="615" t="str">
+        <x:v>src/lib/telegram/check-followup.ts; victim-intent.ts; handlers/check.ts</x:v>
+      </x:c>
+      <x:c r="F36" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G36" s="615" t="str">
+        <x:v>Telegram / Product</x:v>
+      </x:c>
+      <x:c r="H36" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I36" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
+      </x:c>
+      <x:c r="J36" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K36" s="615" t="str">
+        <x:v>Passport/document questions never reuse old results; five legitimate follow-ups still pass.</x:v>
+      </x:c>
+      <x:c r="L36" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
     <x:cfRule type="containsText" dxfId="469" priority="1" operator="containsText" text="Passed"/>
@@ -23627,13 +25842,28 @@
     <x:cfRule type="containsText" dxfId="474" priority="6" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:conditionalFormatting sqref="F2:F36">
+    <x:cfRule type="containsText" dxfId="553" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="554" priority="9" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="555" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="556" priority="11" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="557" priority="12" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="558" priority="13" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="559" priority="14" operator="containsText" text="Deferred"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B21">
       <x:formula1>"P0,P1,P2"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F21">
       <x:formula1>"Open,In Progress,Fixed Local / Awaiting Deploy,Deployed / Awaiting Live Verification,Closed,Accepted Risk"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="B22:B36">
+      <x:formula1>"P0,P1,P2,P3"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F22:F36">
+      <x:formula1>"Open,In Progress,Fixed Local / Awaiting Deploy,Deployed / Awaiting Live Verification,Closed,Accepted Risk"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Fix security revalidation findings (#82)
Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R44f303add1cb497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rce01bdcc5c7f4580"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4cd76356b43849eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd60d1bdc9576485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4964852fc6e4e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R5704deac18cf4975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R2052ccc65c9c442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R9fea1affd62241aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R752edd750c7d439d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf51954a7b3cf43ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R56295e6b3f494817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc509fa81914d474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4b27414a6734dab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra9bec3428dd14783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R9309644b54b4491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0f1c9dc1b572465b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1202,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1221">
+  <x:cellXfs count="1227">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4292,11 +4292,23 @@
     <x:xf numFmtId="0" fontId="1" fillId="203" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="483">
+  <x:dxfs count="567">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -9376,6 +9388,1007 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF92400E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEF3C7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9393,11 +10406,11 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF92400E"/>
+        <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
+          <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9415,6 +10428,50 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
@@ -9426,6 +10483,28 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
@@ -9459,154 +10538,11 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF166534"/>
+        <x:color rgb="FF4B5563"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF92400E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF115E59"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFCCFBF1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF1E40AF"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDBEAFE"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF92400E"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEF3C7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF115E59"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFCCFBF1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF166534"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF991B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF1E40AF"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDBEAFE"/>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9911,13 +10847,13 @@
       </x:c>
       <x:c r="C2" s="1219" t="n">
         <x:f>COUNTA('Current Security Queue'!$A$2:$A$200)</x:f>
-        <x:v>20</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Expand BOT-004 into broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts. Continue the separate Inline visual/client matrix, provider compatibility and resource-soak matrices; close remaining findings and enable leaked-password protection.</x:v>
+        <x:v>All 15 validated findings are fixed locally and the count-only production admin preflight is green. Next: commit and CI, apply the production migration, deploy the exact commit, run targeted trust/privacy/Inline/media/provider/monitor smokes and read-back, complete historical count-only privacy review and close a 72-hour canary. Keep broad real-client RU/UZ/EN bot/Inline evidence separate.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Railway 37a91c7a deployed clean main 4050172 after plan renewal. Health 200, polling-aware monitor and five-action production dispatch smoke passed with cleanup. BOT-001 is Passed; BOT-004 is deployed and automated but remains In Progress until broader real-client transcripts exist.</x:v>
+        <x:v>Local remediation evidence: 4222/4222 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint and original-path PoCs. Production count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Current security rows are In Progress until deployment/read-back; no production state was changed by this verification. Canonical source and evidence copy are synchronized.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -10029,7 +10965,7 @@
       </x:c>
       <x:c r="C11" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A11)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D11" s="629" t="n">
         <x:v>2</x:v>
@@ -10045,7 +10981,7 @@
       </x:c>
       <x:c r="C12" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A12)</x:f>
-        <x:v>5</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D12" s="629" t="n">
         <x:v>3</x:v>
@@ -10061,7 +10997,7 @@
       </x:c>
       <x:c r="C13" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$C$2:$C$200,A13)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D13" s="629" t="n">
         <x:v>4</x:v>
@@ -10108,10 +11044,10 @@
       </x:c>
       <x:c r="B17" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A17)</x:f>
-        <x:v>0</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C17" s="629" t="str">
-        <x:v>Implementation is underway.</x:v>
+        <x:v>Local fixes and regressions pass; deployment/read-back is pending.</x:v>
       </x:c>
       <x:c r="D17" s="629"/>
       <x:c r="E17" s="629"/>
@@ -10184,7 +11120,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -10226,7 +11162,7 @@
       </x:c>
       <x:c r="B26" s="631" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A26)</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C26" s="631" t="str">
         <x:v>Outside the current release scope.</x:v>
@@ -21175,6 +22111,58 @@
         <x:v>BOT-001 is release-passed. Continue BOT-004 with broader real Telegram Desktop/Android/iOS RU/UZ/EN transcripts and keep Inline visual delivery separate because it requires a real client-generated inline_query_id.</x:v>
       </x:c>
     </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>QA-SECURITY-REVALIDATION-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B96" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>Full repository security revalidation</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>388-file inventory; 109 review receipts; 62 raw candidates; 38 independently validated; 24 attack-path candidates; local canonical finalizer and report validator; 4135 tests; TypeScript/lint/build/npm audit; production health/monitor read-only checks</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Completed: 15 final instances (1 High, 9 Medium, 5 Low), 27 reviewed surfaces, 5 explicitly deferred live/product-intent questions.</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>RC-001, OPS-001, SEC-2026-0712-001..015</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>No production data, secrets or repository source changed. Reports, JSON, hardening portfolio and PoCs are in outputs/security_revalidation_2026-07-12.</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>Fix High/P1 first, then nine Medium/P2; keep five Low/P3 tracked. Re-run all original probes, deploy, run targeted smokes and 72-hour canary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>QA-SECURITY-FIX-VERIFICATION-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B97" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Local remediation verification for 15 revalidation findings</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; supabase db reset --local --yes; supabase test db --local; supabase db lint --local --level error --fail-on error; railway run npm run admin-role:preflight; fixed-state and old-assertion PoCs</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Passed locally: 4222/4222 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; fixed-state redaction/QR; old contact/provider/domain/Inline/public-post/moderation/passport/media-order assertions rejected. Production count-only admin preflight passed: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>SEC-2026-0712-001..015, OPS-001, RC-001</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>No production deployment, migration or production-data mutation. The production admin preflight was read-only and logged counts only. One external appeal PoC is excluded by the repository Vitest include pattern; the equivalent real mocked-insert regression is included in the green suite. GitHub action tag SHAs were verified with git ls-remote.</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Commit and run CI; apply the production migration; deploy exact commit; run target smokes/read-back; historical count-only privacy review; 72-hour canary; then reclassify findings.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -22437,7 +23425,7 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H30" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I30" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -22449,13 +23437,13 @@
         <x:v>Telegram / QA</x:v>
       </x:c>
       <x:c r="L30" s="615" t="str">
-        <x:v>Gate 1 Inline deploy</x:v>
+        <x:v>Telegram Desktop/Android/iOS real-client visual and insertion QA</x:v>
       </x:c>
       <x:c r="M30" s="615" t="str">
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>55x3 reason presentations now pass through the real adapter; remaining matrix includes webhook config, faults, prefix/load and stateless follow-ups.</x:v>
+        <x:v>Backend is deployed at 4bd9403. Automated Inline protocol/privacy coverage is green; real-client visual/insertion evidence remains the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -22732,6 +23720,636 @@
       <x:c r="M37" s="615" t="str"/>
       <x:c r="N37" s="615" t="str">
         <x:v>Go requires 0 open P0/P1 and fresh production/security/restore evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="614" t="str">
+        <x:v>SEC-2026-0712-001</x:v>
+      </x:c>
+      <x:c r="B38" s="614" t="str">
+        <x:v>Embedded official contact tokens can mark unrelated attacker content Safe</x:v>
+      </x:c>
+      <x:c r="C38" s="614" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="D38" s="614" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E38" s="614" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F38" s="614" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G38" s="614" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H38" s="614" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I38" s="614" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J38" s="617" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K38" s="614" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="L38" s="614" t="str">
+        <x:v>SEC-2026-0712-001</x:v>
+      </x:c>
+      <x:c r="M38" s="614"/>
+      <x:c r="N38" s="614" t="str">
+        <x:v>High/P1 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="615" t="str">
+        <x:v>SEC-2026-0712-002</x:v>
+      </x:c>
+      <x:c r="B39" s="615" t="str">
+        <x:v>Public reports retain passwords, separated OTPs and recovery phrases</x:v>
+      </x:c>
+      <x:c r="C39" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D39" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E39" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F39" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G39" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H39" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I39" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J39" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K39" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="L39" s="615" t="str">
+        <x:v>SEC-2026-0712-002</x:v>
+      </x:c>
+      <x:c r="M39" s="615"/>
+      <x:c r="N39" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="615" t="str">
+        <x:v>SEC-2026-0712-003</x:v>
+      </x:c>
+      <x:c r="B40" s="615" t="str">
+        <x:v>Appeal reason/contact fields can retain secrets</x:v>
+      </x:c>
+      <x:c r="C40" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D40" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E40" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F40" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G40" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H40" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I40" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J40" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K40" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="L40" s="615" t="str">
+        <x:v>SEC-2026-0712-003</x:v>
+      </x:c>
+      <x:c r="M40" s="615"/>
+      <x:c r="N40" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="615" t="str">
+        <x:v>SEC-2026-0712-004</x:v>
+      </x:c>
+      <x:c r="B41" s="615" t="str">
+        <x:v>Decoded QR credentials can be retained in check records</x:v>
+      </x:c>
+      <x:c r="C41" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D41" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E41" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F41" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G41" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H41" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I41" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J41" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K41" s="615" t="str">
+        <x:v>Media / Privacy</x:v>
+      </x:c>
+      <x:c r="L41" s="615" t="str">
+        <x:v>SEC-2026-0712-004</x:v>
+      </x:c>
+      <x:c r="M41" s="615"/>
+      <x:c r="N41" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="615" t="str">
+        <x:v>SEC-2026-0712-005</x:v>
+      </x:c>
+      <x:c r="B42" s="615" t="str">
+        <x:v>Inline results can republish secrets into selected chats</x:v>
+      </x:c>
+      <x:c r="C42" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D42" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E42" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F42" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G42" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H42" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I42" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J42" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K42" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="L42" s="615" t="str">
+        <x:v>SEC-2026-0712-005</x:v>
+      </x:c>
+      <x:c r="M42" s="615"/>
+      <x:c r="N42" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="615" t="str">
+        <x:v>SEC-2026-0712-006</x:v>
+      </x:c>
+      <x:c r="B43" s="615" t="str">
+        <x:v>Public-post checks can retain passwords and recovery phrases</x:v>
+      </x:c>
+      <x:c r="C43" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D43" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E43" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F43" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G43" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H43" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I43" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J43" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K43" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="L43" s="615" t="str">
+        <x:v>SEC-2026-0712-006</x:v>
+      </x:c>
+      <x:c r="M43" s="615"/>
+      <x:c r="N43" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="615" t="str">
+        <x:v>SEC-2026-0712-007</x:v>
+      </x:c>
+      <x:c r="B44" s="615" t="str">
+        <x:v>Report metadata can forward secrets to moderator Telegram</x:v>
+      </x:c>
+      <x:c r="C44" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D44" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E44" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F44" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G44" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H44" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I44" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J44" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K44" s="615" t="str">
+        <x:v>Telegram / Moderation</x:v>
+      </x:c>
+      <x:c r="L44" s="615" t="str">
+        <x:v>SEC-2026-0712-007</x:v>
+      </x:c>
+      <x:c r="M44" s="615"/>
+      <x:c r="N44" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="615" t="str">
+        <x:v>SEC-2026-0712-008</x:v>
+      </x:c>
+      <x:c r="B45" s="615" t="str">
+        <x:v>Removed admin eligibility is not revoked from durable roles</x:v>
+      </x:c>
+      <x:c r="C45" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D45" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E45" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F45" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G45" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H45" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I45" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J45" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K45" s="615" t="str">
+        <x:v>Data / Security</x:v>
+      </x:c>
+      <x:c r="L45" s="615" t="str">
+        <x:v>SEC-2026-0712-008</x:v>
+      </x:c>
+      <x:c r="M45" s="615"/>
+      <x:c r="N45" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="615" t="str">
+        <x:v>SEC-2026-0712-009</x:v>
+      </x:c>
+      <x:c r="B46" s="615" t="str">
+        <x:v>Embed meta-intents bypass shared limit and append telemetry</x:v>
+      </x:c>
+      <x:c r="C46" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D46" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E46" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F46" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G46" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H46" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I46" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J46" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K46" s="615" t="str">
+        <x:v>Backend / Data</x:v>
+      </x:c>
+      <x:c r="L46" s="615" t="str">
+        <x:v>SEC-2026-0712-009</x:v>
+      </x:c>
+      <x:c r="M46" s="615"/>
+      <x:c r="N46" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="615" t="str">
+        <x:v>SEC-2026-0712-010</x:v>
+      </x:c>
+      <x:c r="B47" s="615" t="str">
+        <x:v>Production-monitor secrets are visible to mutable setup code</x:v>
+      </x:c>
+      <x:c r="C47" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D47" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E47" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F47" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G47" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H47" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I47" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J47" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K47" s="615" t="str">
+        <x:v>DevOps / Security</x:v>
+      </x:c>
+      <x:c r="L47" s="615" t="str">
+        <x:v>SEC-2026-0712-010</x:v>
+      </x:c>
+      <x:c r="M47" s="615"/>
+      <x:c r="N47" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="615" t="str">
+        <x:v>SEC-2026-0712-011</x:v>
+      </x:c>
+      <x:c r="B48" s="615" t="str">
+        <x:v>Report images download before shared media admission</x:v>
+      </x:c>
+      <x:c r="C48" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D48" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E48" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F48" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G48" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H48" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I48" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J48" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K48" s="615" t="str">
+        <x:v>Telegram / Platform</x:v>
+      </x:c>
+      <x:c r="L48" s="615" t="str">
+        <x:v>SEC-2026-0712-011</x:v>
+      </x:c>
+      <x:c r="M48" s="615"/>
+      <x:c r="N48" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="615" t="str">
+        <x:v>SEC-2026-0712-012</x:v>
+      </x:c>
+      <x:c r="B49" s="615" t="str">
+        <x:v>Benign provider evidence can omit phishing URL and return Safe</x:v>
+      </x:c>
+      <x:c r="C49" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="D49" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E49" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F49" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G49" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H49" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I49" s="615" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="J49" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K49" s="615" t="str">
+        <x:v>AI / Risk</x:v>
+      </x:c>
+      <x:c r="L49" s="615" t="str">
+        <x:v>SEC-2026-0712-012</x:v>
+      </x:c>
+      <x:c r="M49" s="615"/>
+      <x:c r="N49" s="615" t="str">
+        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="615" t="str">
+        <x:v>SEC-2026-0712-013</x:v>
+      </x:c>
+      <x:c r="B50" s="615" t="str">
+        <x:v>Official-domain skeleton collisions suppress brand detection</x:v>
+      </x:c>
+      <x:c r="C50" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D50" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E50" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F50" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G50" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H50" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I50" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J50" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K50" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="L50" s="615" t="str">
+        <x:v>SEC-2026-0712-013</x:v>
+      </x:c>
+      <x:c r="M50" s="615"/>
+      <x:c r="N50" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="615" t="str">
+        <x:v>SEC-2026-0712-014</x:v>
+      </x:c>
+      <x:c r="B51" s="615" t="str">
+        <x:v>News-domain skeleton collisions suppress path-brand warning</x:v>
+      </x:c>
+      <x:c r="C51" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D51" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E51" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F51" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G51" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H51" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I51" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J51" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K51" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="L51" s="615" t="str">
+        <x:v>SEC-2026-0712-014</x:v>
+      </x:c>
+      <x:c r="M51" s="615"/>
+      <x:c r="N51" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="615" t="str">
+        <x:v>SEC-2026-0712-015</x:v>
+      </x:c>
+      <x:c r="B52" s="615" t="str">
+        <x:v>Passport request can be answered as stale Safe follow-up</x:v>
+      </x:c>
+      <x:c r="C52" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="D52" s="615" t="str">
+        <x:v>Fixed Local</x:v>
+      </x:c>
+      <x:c r="E52" s="615" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="F52" s="615" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G52" s="615" t="str">
+        <x:v>Passed Local</x:v>
+      </x:c>
+      <x:c r="H52" s="615" t="str">
+        <x:v>Not Deployed</x:v>
+      </x:c>
+      <x:c r="I52" s="615" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="J52" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="K52" s="615" t="str">
+        <x:v>Telegram / Product</x:v>
+      </x:c>
+      <x:c r="L52" s="615" t="str">
+        <x:v>SEC-2026-0712-015</x:v>
+      </x:c>
+      <x:c r="M52" s="615"/>
+      <x:c r="N52" s="615" t="str">
+        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -22753,7 +24371,16 @@
     <x:cfRule type="containsText" dxfId="467" priority="13" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="14">
+  <x:conditionalFormatting sqref="D2:I52">
+    <x:cfRule type="containsText" dxfId="560" priority="15" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="561" priority="16" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="562" priority="17" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="563" priority="18" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="564" priority="19" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="565" priority="20" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="566" priority="21" operator="containsText" text="Deferred"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="C2:C36">
       <x:formula1>"P0,P1,P2,P3"</x:formula1>
     </x:dataValidation>
@@ -22796,6 +24423,24 @@
     <x:dataValidation type="list" sqref="I2:I37">
       <x:formula1>"Blocked,In Progress,Passed,Deferred"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="C38:C52">
+      <x:formula1>"P0,P1,P2,P3"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D38:D52">
+      <x:formula1>"Not Started,In Progress,Fixed Local,Implemented,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E38:F52">
+      <x:formula1>"Pending,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G38:G52">
+      <x:formula1>"Pending,Passed Local,Passed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H38:H52">
+      <x:formula1>"Not Deployed,Pending,Deployed,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I38:I52">
+      <x:formula1>"Blocked,In Progress,Passed,Deferred"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -23617,6 +25262,576 @@
         <x:v>46214</x:v>
       </x:c>
     </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="614" t="str">
+        <x:v>SEC-2026-0712-001</x:v>
+      </x:c>
+      <x:c r="B22" s="614" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C22" s="614" t="str">
+        <x:v>Trust decision</x:v>
+      </x:c>
+      <x:c r="D22" s="614" t="str">
+        <x:v>Embedded official contact tokens can mark unrelated attacker content Safe</x:v>
+      </x:c>
+      <x:c r="E22" s="614" t="str">
+        <x:v>src/lib/risk/check-core.ts:125-143,338-350; src/lib/risk/rules.ts:302-307</x:v>
+      </x:c>
+      <x:c r="F22" s="614" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G22" s="614" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="H22" s="614" t="str">
+        <x:v>Gate 0</x:v>
+      </x:c>
+      <x:c r="I22" s="614" t="str">
+        <x:v>High/P1 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
+      </x:c>
+      <x:c r="J22" s="614" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K22" s="614" t="str">
+        <x:v>Unrelated content cannot become Safe because it merely contains an official token.</x:v>
+      </x:c>
+      <x:c r="L22" s="617" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="615" t="str">
+        <x:v>SEC-2026-0712-002</x:v>
+      </x:c>
+      <x:c r="B23" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C23" s="615" t="str">
+        <x:v>Report privacy</x:v>
+      </x:c>
+      <x:c r="D23" s="615" t="str">
+        <x:v>Public reports retain passwords, separated OTPs and recovery phrases</x:v>
+      </x:c>
+      <x:c r="E23" s="615" t="str">
+        <x:v>src/lib/risk/detect.ts; src/lib/report.functions.ts</x:v>
+      </x:c>
+      <x:c r="F23" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G23" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="H23" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I23" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
+      </x:c>
+      <x:c r="J23" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K23" s="615" t="str">
+        <x:v>Complete reports/entities insert payload contains no supported secret marker.</x:v>
+      </x:c>
+      <x:c r="L23" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="615" t="str">
+        <x:v>SEC-2026-0712-003</x:v>
+      </x:c>
+      <x:c r="B24" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C24" s="615" t="str">
+        <x:v>Appeal privacy</x:v>
+      </x:c>
+      <x:c r="D24" s="615" t="str">
+        <x:v>Appeal reason/contact fields can retain secrets</x:v>
+      </x:c>
+      <x:c r="E24" s="615" t="str">
+        <x:v>src/lib/reputation-appeal.functions.ts; src/lib/risk/detect.ts</x:v>
+      </x:c>
+      <x:c r="F24" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G24" s="615" t="str">
+        <x:v>Privacy / Backend</x:v>
+      </x:c>
+      <x:c r="H24" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I24" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
+      </x:c>
+      <x:c r="J24" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K24" s="615" t="str">
+        <x:v>No secret marker reaches reason or contact_display; generic unsafe contact is rejected.</x:v>
+      </x:c>
+      <x:c r="L24" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="615" t="str">
+        <x:v>SEC-2026-0712-004</x:v>
+      </x:c>
+      <x:c r="B25" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C25" s="615" t="str">
+        <x:v>QR privacy</x:v>
+      </x:c>
+      <x:c r="D25" s="615" t="str">
+        <x:v>Decoded QR credentials can be retained in check records</x:v>
+      </x:c>
+      <x:c r="E25" s="615" t="str">
+        <x:v>src/lib/risk/qr-decoder.ts; image-intelligence.ts; check-core.ts</x:v>
+      </x:c>
+      <x:c r="F25" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G25" s="615" t="str">
+        <x:v>Media / Privacy</x:v>
+      </x:c>
+      <x:c r="H25" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I25" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
+      </x:c>
+      <x:c r="J25" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K25" s="615" t="str">
+        <x:v>Wi-Fi passwords, otpauth secrets and mnemonic candidates never enter redacted_input.</x:v>
+      </x:c>
+      <x:c r="L25" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="615" t="str">
+        <x:v>SEC-2026-0712-005</x:v>
+      </x:c>
+      <x:c r="B26" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C26" s="615" t="str">
+        <x:v>Telegram Inline privacy</x:v>
+      </x:c>
+      <x:c r="D26" s="615" t="str">
+        <x:v>Inline results can republish secrets into selected chats</x:v>
+      </x:c>
+      <x:c r="E26" s="615" t="str">
+        <x:v>src/lib/telegram/handlers/inline.ts; src/lib/risk/detect.ts</x:v>
+      </x:c>
+      <x:c r="F26" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G26" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="H26" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I26" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
+      </x:c>
+      <x:c r="J26" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K26" s="615" t="str">
+        <x:v>No supported secret marker appears in any Inline article field on real clients.</x:v>
+      </x:c>
+      <x:c r="L26" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="615" t="str">
+        <x:v>SEC-2026-0712-006</x:v>
+      </x:c>
+      <x:c r="B27" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C27" s="615" t="str">
+        <x:v>Public-post privacy</x:v>
+      </x:c>
+      <x:c r="D27" s="615" t="str">
+        <x:v>Public-post checks can retain passwords and recovery phrases</x:v>
+      </x:c>
+      <x:c r="E27" s="615" t="str">
+        <x:v>src/lib/telegram/public-post.server.ts; src/lib/risk/check-core.ts</x:v>
+      </x:c>
+      <x:c r="F27" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G27" s="615" t="str">
+        <x:v>Telegram / Privacy</x:v>
+      </x:c>
+      <x:c r="H27" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I27" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
+      </x:c>
+      <x:c r="J27" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K27" s="615" t="str">
+        <x:v>Mocked check insert contains no secret marker from public-post fixtures.</x:v>
+      </x:c>
+      <x:c r="L27" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="615" t="str">
+        <x:v>SEC-2026-0712-007</x:v>
+      </x:c>
+      <x:c r="B28" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C28" s="615" t="str">
+        <x:v>Moderation privacy</x:v>
+      </x:c>
+      <x:c r="D28" s="615" t="str">
+        <x:v>Report metadata can forward secrets to moderator Telegram</x:v>
+      </x:c>
+      <x:c r="E28" s="615" t="str">
+        <x:v>src/lib/report.functions.ts; moderation-notifier.server.ts</x:v>
+      </x:c>
+      <x:c r="F28" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G28" s="615" t="str">
+        <x:v>Telegram / Moderation</x:v>
+      </x:c>
+      <x:c r="H28" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I28" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
+      </x:c>
+      <x:c r="J28" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+      </x:c>
+      <x:c r="K28" s="615" t="str">
+        <x:v>Markdown and plaintext notification payloads contain no secret marker.</x:v>
+      </x:c>
+      <x:c r="L28" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="615" t="str">
+        <x:v>SEC-2026-0712-008</x:v>
+      </x:c>
+      <x:c r="B29" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C29" s="615" t="str">
+        <x:v>Admin authorization</x:v>
+      </x:c>
+      <x:c r="D29" s="615" t="str">
+        <x:v>Removed admin eligibility is not revoked from durable roles</x:v>
+      </x:c>
+      <x:c r="E29" s="615" t="str">
+        <x:v>supabase/migrations/20260629085533_*; src/lib/admin.functions.ts</x:v>
+      </x:c>
+      <x:c r="F29" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G29" s="615" t="str">
+        <x:v>Data / Security</x:v>
+      </x:c>
+      <x:c r="H29" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I29" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+      </x:c>
+      <x:c r="J29" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K29" s="615" t="str">
+        <x:v>Allowlist delete, email drift and confirmation loss immediately deny existing sessions.</x:v>
+      </x:c>
+      <x:c r="L29" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="615" t="str">
+        <x:v>SEC-2026-0712-009</x:v>
+      </x:c>
+      <x:c r="B30" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C30" s="615" t="str">
+        <x:v>Embed availability</x:v>
+      </x:c>
+      <x:c r="D30" s="615" t="str">
+        <x:v>Embed meta-intents bypass shared limit and append telemetry</x:v>
+      </x:c>
+      <x:c r="E30" s="615" t="str">
+        <x:v>src/lib/check.functions.ts; embed-origin-analytics.server.ts</x:v>
+      </x:c>
+      <x:c r="F30" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G30" s="615" t="str">
+        <x:v>Backend / Data</x:v>
+      </x:c>
+      <x:c r="H30" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I30" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
+      </x:c>
+      <x:c r="J30" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K30" s="615" t="str">
+        <x:v>Denied request performs zero analytics inserts; production storage failure fails closed.</x:v>
+      </x:c>
+      <x:c r="L30" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="615" t="str">
+        <x:v>SEC-2026-0712-010</x:v>
+      </x:c>
+      <x:c r="B31" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C31" s="615" t="str">
+        <x:v>CI supply chain</x:v>
+      </x:c>
+      <x:c r="D31" s="615" t="str">
+        <x:v>Production-monitor secrets are visible to mutable setup code</x:v>
+      </x:c>
+      <x:c r="E31" s="615" t="str">
+        <x:v>.github/workflows/prod-monitor.yml</x:v>
+      </x:c>
+      <x:c r="F31" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G31" s="615" t="str">
+        <x:v>DevOps / Security</x:v>
+      </x:c>
+      <x:c r="H31" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I31" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
+      </x:c>
+      <x:c r="J31" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K31" s="615" t="str">
+        <x:v>Policy rejects job-scoped secrets, non-SHA actions and pre-secret install hooks.</x:v>
+      </x:c>
+      <x:c r="L31" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="615" t="str">
+        <x:v>SEC-2026-0712-011</x:v>
+      </x:c>
+      <x:c r="B32" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C32" s="615" t="str">
+        <x:v>Telegram availability</x:v>
+      </x:c>
+      <x:c r="D32" s="615" t="str">
+        <x:v>Report images download before shared media admission</x:v>
+      </x:c>
+      <x:c r="E32" s="615" t="str">
+        <x:v>src/lib/telegram/handlers/report.ts; handlers/check.ts</x:v>
+      </x:c>
+      <x:c r="F32" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G32" s="615" t="str">
+        <x:v>Telegram / Platform</x:v>
+      </x:c>
+      <x:c r="H32" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I32" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
+      </x:c>
+      <x:c r="J32" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K32" s="615" t="str">
+        <x:v>Rate-limited report image makes zero getFile/download calls under concurrency.</x:v>
+      </x:c>
+      <x:c r="L32" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="615" t="str">
+        <x:v>SEC-2026-0712-012</x:v>
+      </x:c>
+      <x:c r="B33" s="615" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="C33" s="615" t="str">
+        <x:v>Image evidence trust</x:v>
+      </x:c>
+      <x:c r="D33" s="615" t="str">
+        <x:v>Benign provider evidence can omit phishing URL and return Safe</x:v>
+      </x:c>
+      <x:c r="E33" s="615" t="str">
+        <x:v>src/lib/risk/image-intelligence.ts; check-core.ts</x:v>
+      </x:c>
+      <x:c r="F33" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G33" s="615" t="str">
+        <x:v>AI / Risk</x:v>
+      </x:c>
+      <x:c r="H33" s="615" t="str">
+        <x:v>Gate 1</x:v>
+      </x:c>
+      <x:c r="I33" s="615" t="str">
+        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
+      </x:c>
+      <x:c r="J33" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K33" s="615" t="str">
+        <x:v>Benign provider category plus phishing URL cannot return Safe without trusted local proof.</x:v>
+      </x:c>
+      <x:c r="L33" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="615" t="str">
+        <x:v>SEC-2026-0712-013</x:v>
+      </x:c>
+      <x:c r="B34" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C34" s="615" t="str">
+        <x:v>Domain identity</x:v>
+      </x:c>
+      <x:c r="D34" s="615" t="str">
+        <x:v>Official-domain skeleton collisions suppress brand detection</x:v>
+      </x:c>
+      <x:c r="E34" s="615" t="str">
+        <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
+      </x:c>
+      <x:c r="F34" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G34" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="H34" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I34" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
+      </x:c>
+      <x:c r="J34" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K34" s="615" t="str">
+        <x:v>Confusable hostname cannot inherit official allowlist membership; controls stay valid.</x:v>
+      </x:c>
+      <x:c r="L34" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="615" t="str">
+        <x:v>SEC-2026-0712-014</x:v>
+      </x:c>
+      <x:c r="B35" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C35" s="615" t="str">
+        <x:v>Domain identity</x:v>
+      </x:c>
+      <x:c r="D35" s="615" t="str">
+        <x:v>News-domain skeleton collisions suppress path-brand warning</x:v>
+      </x:c>
+      <x:c r="E35" s="615" t="str">
+        <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
+      </x:c>
+      <x:c r="F35" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G35" s="615" t="str">
+        <x:v>Risk Engine</x:v>
+      </x:c>
+      <x:c r="H35" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I35" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
+      </x:c>
+      <x:c r="J35" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K35" s="615" t="str">
+        <x:v>sp0t.uz cannot inherit spot.uz suppression; similarity only adds evidence.</x:v>
+      </x:c>
+      <x:c r="L35" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="615" t="str">
+        <x:v>SEC-2026-0712-015</x:v>
+      </x:c>
+      <x:c r="B36" s="615" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="C36" s="615" t="str">
+        <x:v>Telegram dialogue</x:v>
+      </x:c>
+      <x:c r="D36" s="615" t="str">
+        <x:v>Passport request can be answered as stale Safe follow-up</x:v>
+      </x:c>
+      <x:c r="E36" s="615" t="str">
+        <x:v>src/lib/telegram/check-followup.ts; victim-intent.ts; handlers/check.ts</x:v>
+      </x:c>
+      <x:c r="F36" s="615" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="G36" s="615" t="str">
+        <x:v>Telegram / Product</x:v>
+      </x:c>
+      <x:c r="H36" s="615" t="str">
+        <x:v>Post-gate</x:v>
+      </x:c>
+      <x:c r="I36" s="615" t="str">
+        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
+      </x:c>
+      <x:c r="J36" s="615" t="str">
+        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+      </x:c>
+      <x:c r="K36" s="615" t="str">
+        <x:v>Passport/document questions never reuse old results; five legitimate follow-ups still pass.</x:v>
+      </x:c>
+      <x:c r="L36" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:F21">
     <x:cfRule type="containsText" dxfId="469" priority="1" operator="containsText" text="Passed"/>
@@ -23627,13 +25842,28 @@
     <x:cfRule type="containsText" dxfId="474" priority="6" operator="containsText" text="Open"/>
     <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:conditionalFormatting sqref="F2:F36">
+    <x:cfRule type="containsText" dxfId="553" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="554" priority="9" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="555" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="556" priority="11" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="557" priority="12" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="558" priority="13" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="559" priority="14" operator="containsText" text="Deferred"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B21">
       <x:formula1>"P0,P1,P2"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F21">
       <x:formula1>"Open,In Progress,Fixed Local / Awaiting Deploy,Deployed / Awaiting Live Verification,Closed,Accepted Risk"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="B22:B36">
+      <x:formula1>"P0,P1,P2,P3"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F22:F36">
+      <x:formula1>"Open,In Progress,Fixed Local / Awaiting Deploy,Deployed / Awaiting Live Verification,Closed,Accepted Risk"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Expand release readiness gates
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R752edd750c7d439d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf51954a7b3cf43ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R56295e6b3f494817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc509fa81914d474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4b27414a6734dab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra9bec3428dd14783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R9309644b54b4491f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0f1c9dc1b572465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7146198fbd7646de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb18ef2214fdb45e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R368baeb6be9046e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R521ea297fca94fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb26a4ff13bb54aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2c5f1d2c648b4e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R32b6e81362784955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rb5f91f5f2f2a4fbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4308,7 +4308,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="567">
+  <x:dxfs count="581">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -9619,6 +9619,160 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -10850,10 +11004,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>All 15 validated findings are fixed locally and the count-only production admin preflight is green. Next: commit and CI, apply the production migration, deploy the exact commit, run targeted trust/privacy/Inline/media/provider/monitor smokes and read-back, complete historical count-only privacy review and close a 72-hour canary. Keep broad real-client RU/UZ/EN bot/Inline evidence separate.</x:v>
+        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 5c6094add5dee66045adf445fe15e566405c55da and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Next: historical count-only privacy review, real-client RU/UZ/EN Inline evidence, finding-specific acceptance and a 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Local remediation evidence: 4222/4222 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint and original-path PoCs. Production count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Current security rows are In Progress until deployment/read-back; no production state was changed by this verification. Canonical source and evidence copy are synchronized.</x:v>
+        <x:v>Evidence: 4227/4227 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint, PR #83 CI, Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f, app/polling/Inline-boundary/dialogue smokes with cleanup and monitor 29203622435. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Canonical source and evidence copy are synchronized.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11044,10 +11198,10 @@
       </x:c>
       <x:c r="B17" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A17)</x:f>
-        <x:v>15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="629" t="str">
-        <x:v>Local fixes and regressions pass; deployment/read-back is pending.</x:v>
+        <x:v>Fourteen fixes are deployed and await finding-specific live closure; the admin-role migration remains In Progress.</x:v>
       </x:c>
       <x:c r="D17" s="629"/>
       <x:c r="E17" s="629"/>
@@ -11058,7 +11212,7 @@
       </x:c>
       <x:c r="B18" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A18)</x:f>
-        <x:v>16</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C18" s="629" t="str">
         <x:v>Code is in production; targeted real-client or failure-path proof remains.</x:v>
@@ -22145,22 +22299,22 @@
         <x:v>46215</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Local remediation verification for 15 revalidation findings</x:v>
+        <x:v>Deployed remediation verification for 15 revalidation findings</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; supabase db reset --local --yes; supabase test db --local; supabase db lint --local --level error --fail-on error; railway run npm run admin-role:preflight; fixed-state and old-assertion PoCs</x:v>
+        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; CI app + migrations/schema/pgTAP; Railway exact-SHA deploy; prod:smoke; prod:telegram-inline-smoke; prod:telegram-polling-dispatch-smoke; GitHub production monitor; production admin-role count-only preflight</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Passed locally: 4222/4222 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; fixed-state redaction/QR; old contact/provider/domain/Inline/public-post/moderation/passport/media-order assertions rejected. Production count-only admin preflight passed: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+        <x:v>Passed: 4227/4227 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; exact deployment 5c6094a / eb7a6364; app/health/webhook/polling/AI/Inline-boundary/dialogue smokes; monitor 29203622435; cleanup/read-back. Admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
       </x:c>
       <x:c r="F97" t="str">
         <x:v>SEC-2026-0712-001..015, OPS-001, RC-001</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>No production deployment, migration or production-data mutation. The production admin preflight was read-only and logged counts only. One external appeal PoC is excluded by the repository Vitest include pattern; the equivalent real mocked-insert regression is included in the green suite. GitHub action tag SHAs were verified with git ls-remote.</x:v>
+        <x:v>Application code is deployed. The production admin-role migration was not applied because authorized Supabase production access is unavailable. No identifiers, secrets or matched historical values were logged. Real-client Inline rendering, historical privacy review and 72-hour canary remain open.</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>Commit and run CI; apply the production migration; deploy exact commit; run target smokes/read-back; historical count-only privacy review; 72-hour canary; then reclassify findings.</x:v>
+        <x:v>Restore authorized Supabase access and apply/verify the admin migration; complete finding-specific live/read-back, historical count-only privacy review, real-client RU/UZ/EN Inline matrix and 72-hour canary; then close eligible findings.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23443,7 +23597,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend is deployed at 4bd9403. Automated Inline protocol/privacy coverage is green; real-client visual/insertion evidence remains the blocker.</x:v>
+        <x:v>Backend is deployed at 5c6094add5dee66045adf445fe15e566405c55da. Automated Inline protocol/privacy and polling transport-boundary coverage are green; real-client visual/insertion evidence remains the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -23733,7 +23887,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D38" s="614" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E38" s="614" t="str">
         <x:v>Passed</x:v>
@@ -23745,7 +23899,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H38" s="614" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I38" s="614" t="str">
         <x:v>Blocked</x:v>
@@ -23761,7 +23915,7 @@
       </x:c>
       <x:c r="M38" s="614"/>
       <x:c r="N38" s="614" t="str">
-        <x:v>High/P1 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>High/P1 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -23775,7 +23929,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D39" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E39" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23787,7 +23941,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H39" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I39" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23803,7 +23957,7 @@
       </x:c>
       <x:c r="M39" s="615"/>
       <x:c r="N39" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -23817,7 +23971,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D40" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E40" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23829,7 +23983,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H40" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I40" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23845,7 +23999,7 @@
       </x:c>
       <x:c r="M40" s="615"/>
       <x:c r="N40" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -23859,7 +24013,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D41" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E41" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23871,7 +24025,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H41" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I41" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23887,7 +24041,7 @@
       </x:c>
       <x:c r="M41" s="615"/>
       <x:c r="N41" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -23901,7 +24055,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D42" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E42" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23913,7 +24067,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H42" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I42" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23929,7 +24083,7 @@
       </x:c>
       <x:c r="M42" s="615"/>
       <x:c r="N42" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -23943,7 +24097,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D43" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E43" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23955,7 +24109,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H43" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I43" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -23971,7 +24125,7 @@
       </x:c>
       <x:c r="M43" s="615"/>
       <x:c r="N43" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -23985,7 +24139,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D44" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E44" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23997,7 +24151,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H44" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I44" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24013,7 +24167,7 @@
       </x:c>
       <x:c r="M44" s="615"/>
       <x:c r="N44" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -24027,7 +24181,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D45" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E45" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24039,7 +24193,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H45" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="I45" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24055,7 +24209,7 @@
       </x:c>
       <x:c r="M45" s="615"/>
       <x:c r="N45" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 code and regression are deployed, but the production Supabase migration remains unapplied; authorized apply plus grant/revoke read-back is a release blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -24069,7 +24223,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D46" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E46" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24081,7 +24235,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H46" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I46" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24097,7 +24251,7 @@
       </x:c>
       <x:c r="M46" s="615"/>
       <x:c r="N46" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -24111,7 +24265,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D47" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E47" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24123,7 +24277,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H47" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I47" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24139,7 +24293,7 @@
       </x:c>
       <x:c r="M47" s="615"/>
       <x:c r="N47" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -24153,7 +24307,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D48" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E48" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24165,7 +24319,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H48" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I48" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24181,7 +24335,7 @@
       </x:c>
       <x:c r="M48" s="615"/>
       <x:c r="N48" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -24195,7 +24349,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D49" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E49" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24207,7 +24361,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H49" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I49" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24223,7 +24377,7 @@
       </x:c>
       <x:c r="M49" s="615"/>
       <x:c r="N49" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -24237,7 +24391,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D50" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E50" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24249,7 +24403,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H50" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I50" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24265,7 +24419,7 @@
       </x:c>
       <x:c r="M50" s="615"/>
       <x:c r="N50" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -24279,7 +24433,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D51" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E51" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24291,7 +24445,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H51" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I51" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24307,7 +24461,7 @@
       </x:c>
       <x:c r="M51" s="615"/>
       <x:c r="N51" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -24321,7 +24475,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D52" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E52" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24333,7 +24487,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H52" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I52" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24349,7 +24503,7 @@
       </x:c>
       <x:c r="M52" s="615"/>
       <x:c r="N52" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24372,13 +24526,13 @@
     <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I52">
-    <x:cfRule type="containsText" dxfId="560" priority="15" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="561" priority="16" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="562" priority="17" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="563" priority="18" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="564" priority="19" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="565" priority="20" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="566" priority="21" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="574" priority="15" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="575" priority="16" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="576" priority="17" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="577" priority="18" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="578" priority="19" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="579" priority="20" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="580" priority="21" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -25279,7 +25433,7 @@
         <x:v>src/lib/risk/check-core.ts:125-143,338-350; src/lib/risk/rules.ts:302-307</x:v>
       </x:c>
       <x:c r="F22" s="614" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G22" s="614" t="str">
         <x:v>Risk Engine</x:v>
@@ -25288,10 +25442,10 @@
         <x:v>Gate 0</x:v>
       </x:c>
       <x:c r="I22" s="614" t="str">
-        <x:v>High/P1 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
+        <x:v>High/P1 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
       </x:c>
       <x:c r="J22" s="614" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K22" s="614" t="str">
         <x:v>Unrelated content cannot become Safe because it merely contains an official token.</x:v>
@@ -25317,7 +25471,7 @@
         <x:v>src/lib/risk/detect.ts; src/lib/report.functions.ts</x:v>
       </x:c>
       <x:c r="F23" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G23" s="615" t="str">
         <x:v>Privacy / Backend</x:v>
@@ -25326,10 +25480,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I23" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
       </x:c>
       <x:c r="J23" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K23" s="615" t="str">
         <x:v>Complete reports/entities insert payload contains no supported secret marker.</x:v>
@@ -25355,7 +25509,7 @@
         <x:v>src/lib/reputation-appeal.functions.ts; src/lib/risk/detect.ts</x:v>
       </x:c>
       <x:c r="F24" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G24" s="615" t="str">
         <x:v>Privacy / Backend</x:v>
@@ -25364,10 +25518,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I24" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
       </x:c>
       <x:c r="J24" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K24" s="615" t="str">
         <x:v>No secret marker reaches reason or contact_display; generic unsafe contact is rejected.</x:v>
@@ -25393,7 +25547,7 @@
         <x:v>src/lib/risk/qr-decoder.ts; image-intelligence.ts; check-core.ts</x:v>
       </x:c>
       <x:c r="F25" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G25" s="615" t="str">
         <x:v>Media / Privacy</x:v>
@@ -25402,10 +25556,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I25" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
       </x:c>
       <x:c r="J25" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K25" s="615" t="str">
         <x:v>Wi-Fi passwords, otpauth secrets and mnemonic candidates never enter redacted_input.</x:v>
@@ -25431,7 +25585,7 @@
         <x:v>src/lib/telegram/handlers/inline.ts; src/lib/risk/detect.ts</x:v>
       </x:c>
       <x:c r="F26" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G26" s="615" t="str">
         <x:v>Telegram / Privacy</x:v>
@@ -25440,10 +25594,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I26" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
       </x:c>
       <x:c r="J26" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K26" s="615" t="str">
         <x:v>No supported secret marker appears in any Inline article field on real clients.</x:v>
@@ -25469,7 +25623,7 @@
         <x:v>src/lib/telegram/public-post.server.ts; src/lib/risk/check-core.ts</x:v>
       </x:c>
       <x:c r="F27" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
         <x:v>Telegram / Privacy</x:v>
@@ -25478,10 +25632,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
       </x:c>
       <x:c r="J27" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>Mocked check insert contains no secret marker from public-post fixtures.</x:v>
@@ -25507,7 +25661,7 @@
         <x:v>src/lib/report.functions.ts; moderation-notifier.server.ts</x:v>
       </x:c>
       <x:c r="F28" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G28" s="615" t="str">
         <x:v>Telegram / Moderation</x:v>
@@ -25516,10 +25670,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I28" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
       </x:c>
       <x:c r="J28" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K28" s="615" t="str">
         <x:v>Markdown and plaintext notification payloads contain no secret marker.</x:v>
@@ -25554,10 +25708,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I29" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / eb7a6364-f9da-4ca2-a017-1f6102e50c0f, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
       </x:c>
       <x:c r="J29" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Restore authorized production Supabase access; rerun count-only preflight, apply the exact migration, verify migration history and revoke/grant behavior, then collect read-back evidence.</x:v>
       </x:c>
       <x:c r="K29" s="615" t="str">
         <x:v>Allowlist delete, email drift and confirmation loss immediately deny existing sessions.</x:v>
@@ -25583,7 +25737,7 @@
         <x:v>src/lib/check.functions.ts; embed-origin-analytics.server.ts</x:v>
       </x:c>
       <x:c r="F30" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G30" s="615" t="str">
         <x:v>Backend / Data</x:v>
@@ -25592,10 +25746,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I30" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
       </x:c>
       <x:c r="J30" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K30" s="615" t="str">
         <x:v>Denied request performs zero analytics inserts; production storage failure fails closed.</x:v>
@@ -25621,7 +25775,7 @@
         <x:v>.github/workflows/prod-monitor.yml</x:v>
       </x:c>
       <x:c r="F31" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G31" s="615" t="str">
         <x:v>DevOps / Security</x:v>
@@ -25630,10 +25784,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I31" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
       </x:c>
       <x:c r="J31" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K31" s="615" t="str">
         <x:v>Policy rejects job-scoped secrets, non-SHA actions and pre-secret install hooks.</x:v>
@@ -25659,7 +25813,7 @@
         <x:v>src/lib/telegram/handlers/report.ts; handlers/check.ts</x:v>
       </x:c>
       <x:c r="F32" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G32" s="615" t="str">
         <x:v>Telegram / Platform</x:v>
@@ -25668,10 +25822,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I32" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
       </x:c>
       <x:c r="J32" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K32" s="615" t="str">
         <x:v>Rate-limited report image makes zero getFile/download calls under concurrency.</x:v>
@@ -25697,7 +25851,7 @@
         <x:v>src/lib/risk/image-intelligence.ts; check-core.ts</x:v>
       </x:c>
       <x:c r="F33" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G33" s="615" t="str">
         <x:v>AI / Risk</x:v>
@@ -25706,10 +25860,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I33" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
       </x:c>
       <x:c r="J33" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K33" s="615" t="str">
         <x:v>Benign provider category plus phishing URL cannot return Safe without trusted local proof.</x:v>
@@ -25735,7 +25889,7 @@
         <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
       </x:c>
       <x:c r="F34" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G34" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -25744,10 +25898,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I34" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J34" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K34" s="615" t="str">
         <x:v>Confusable hostname cannot inherit official allowlist membership; controls stay valid.</x:v>
@@ -25773,7 +25927,7 @@
         <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
       </x:c>
       <x:c r="F35" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G35" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -25782,10 +25936,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I35" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J35" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K35" s="615" t="str">
         <x:v>sp0t.uz cannot inherit spot.uz suppression; similarity only adds evidence.</x:v>
@@ -25811,7 +25965,7 @@
         <x:v>src/lib/telegram/check-followup.ts; victim-intent.ts; handlers/check.ts</x:v>
       </x:c>
       <x:c r="F36" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G36" s="615" t="str">
         <x:v>Telegram / Product</x:v>
@@ -25820,10 +25974,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I36" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
       </x:c>
       <x:c r="J36" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K36" s="615" t="str">
         <x:v>Passport/document questions never reuse old results; five legitimate follow-ups still pass.</x:v>
@@ -25843,13 +25997,13 @@
     <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F2:F36">
-    <x:cfRule type="containsText" dxfId="553" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="554" priority="9" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="555" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="556" priority="11" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="557" priority="12" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="558" priority="13" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="559" priority="14" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="567" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="568" priority="9" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="569" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="570" priority="11" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="571" priority="12" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="572" priority="13" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="573" priority="14" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
Expand release readiness gates (#84)
* Expand release readiness gates

* Fix release security gate failures

---------

Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R752edd750c7d439d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rf51954a7b3cf43ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R56295e6b3f494817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rc509fa81914d474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Ra4b27414a6734dab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Ra9bec3428dd14783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R9309644b54b4491f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0f1c9dc1b572465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7146198fbd7646de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb18ef2214fdb45e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R368baeb6be9046e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R521ea297fca94fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb26a4ff13bb54aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2c5f1d2c648b4e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R32b6e81362784955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rb5f91f5f2f2a4fbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4308,7 +4308,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="567">
+  <x:dxfs count="581">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -9619,6 +9619,160 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -10850,10 +11004,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>All 15 validated findings are fixed locally and the count-only production admin preflight is green. Next: commit and CI, apply the production migration, deploy the exact commit, run targeted trust/privacy/Inline/media/provider/monitor smokes and read-back, complete historical count-only privacy review and close a 72-hour canary. Keep broad real-client RU/UZ/EN bot/Inline evidence separate.</x:v>
+        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 5c6094add5dee66045adf445fe15e566405c55da and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Next: historical count-only privacy review, real-client RU/UZ/EN Inline evidence, finding-specific acceptance and a 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Local remediation evidence: 4222/4222 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint and original-path PoCs. Production count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Current security rows are In Progress until deployment/read-back; no production state was changed by this verification. Canonical source and evidence copy are synchronized.</x:v>
+        <x:v>Evidence: 4227/4227 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint, PR #83 CI, Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f, app/polling/Inline-boundary/dialogue smokes with cleanup and monitor 29203622435. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Canonical source and evidence copy are synchronized.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11044,10 +11198,10 @@
       </x:c>
       <x:c r="B17" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A17)</x:f>
-        <x:v>15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="629" t="str">
-        <x:v>Local fixes and regressions pass; deployment/read-back is pending.</x:v>
+        <x:v>Fourteen fixes are deployed and await finding-specific live closure; the admin-role migration remains In Progress.</x:v>
       </x:c>
       <x:c r="D17" s="629"/>
       <x:c r="E17" s="629"/>
@@ -11058,7 +11212,7 @@
       </x:c>
       <x:c r="B18" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A18)</x:f>
-        <x:v>16</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C18" s="629" t="str">
         <x:v>Code is in production; targeted real-client or failure-path proof remains.</x:v>
@@ -22145,22 +22299,22 @@
         <x:v>46215</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>Local remediation verification for 15 revalidation findings</x:v>
+        <x:v>Deployed remediation verification for 15 revalidation findings</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; supabase db reset --local --yes; supabase test db --local; supabase db lint --local --level error --fail-on error; railway run npm run admin-role:preflight; fixed-state and old-assertion PoCs</x:v>
+        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; CI app + migrations/schema/pgTAP; Railway exact-SHA deploy; prod:smoke; prod:telegram-inline-smoke; prod:telegram-polling-dispatch-smoke; GitHub production monitor; production admin-role count-only preflight</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Passed locally: 4222/4222 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; fixed-state redaction/QR; old contact/provider/domain/Inline/public-post/moderation/passport/media-order assertions rejected. Production count-only admin preflight passed: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+        <x:v>Passed: 4227/4227 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; exact deployment 5c6094a / eb7a6364; app/health/webhook/polling/AI/Inline-boundary/dialogue smokes; monitor 29203622435; cleanup/read-back. Admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
       </x:c>
       <x:c r="F97" t="str">
         <x:v>SEC-2026-0712-001..015, OPS-001, RC-001</x:v>
       </x:c>
       <x:c r="G97" t="str">
-        <x:v>No production deployment, migration or production-data mutation. The production admin preflight was read-only and logged counts only. One external appeal PoC is excluded by the repository Vitest include pattern; the equivalent real mocked-insert regression is included in the green suite. GitHub action tag SHAs were verified with git ls-remote.</x:v>
+        <x:v>Application code is deployed. The production admin-role migration was not applied because authorized Supabase production access is unavailable. No identifiers, secrets or matched historical values were logged. Real-client Inline rendering, historical privacy review and 72-hour canary remain open.</x:v>
       </x:c>
       <x:c r="H97" t="str">
-        <x:v>Commit and run CI; apply the production migration; deploy exact commit; run target smokes/read-back; historical count-only privacy review; 72-hour canary; then reclassify findings.</x:v>
+        <x:v>Restore authorized Supabase access and apply/verify the admin migration; complete finding-specific live/read-back, historical count-only privacy review, real-client RU/UZ/EN Inline matrix and 72-hour canary; then close eligible findings.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23443,7 +23597,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend is deployed at 4bd9403. Automated Inline protocol/privacy coverage is green; real-client visual/insertion evidence remains the blocker.</x:v>
+        <x:v>Backend is deployed at 5c6094add5dee66045adf445fe15e566405c55da. Automated Inline protocol/privacy and polling transport-boundary coverage are green; real-client visual/insertion evidence remains the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -23733,7 +23887,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D38" s="614" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E38" s="614" t="str">
         <x:v>Passed</x:v>
@@ -23745,7 +23899,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H38" s="614" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I38" s="614" t="str">
         <x:v>Blocked</x:v>
@@ -23761,7 +23915,7 @@
       </x:c>
       <x:c r="M38" s="614"/>
       <x:c r="N38" s="614" t="str">
-        <x:v>High/P1 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>High/P1 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -23775,7 +23929,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D39" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E39" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23787,7 +23941,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H39" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I39" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23803,7 +23957,7 @@
       </x:c>
       <x:c r="M39" s="615"/>
       <x:c r="N39" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -23817,7 +23971,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D40" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E40" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23829,7 +23983,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H40" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I40" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23845,7 +23999,7 @@
       </x:c>
       <x:c r="M40" s="615"/>
       <x:c r="N40" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -23859,7 +24013,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D41" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E41" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23871,7 +24025,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H41" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I41" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23887,7 +24041,7 @@
       </x:c>
       <x:c r="M41" s="615"/>
       <x:c r="N41" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -23901,7 +24055,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D42" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E42" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23913,7 +24067,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H42" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I42" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -23929,7 +24083,7 @@
       </x:c>
       <x:c r="M42" s="615"/>
       <x:c r="N42" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -23943,7 +24097,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D43" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E43" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23955,7 +24109,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H43" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I43" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -23971,7 +24125,7 @@
       </x:c>
       <x:c r="M43" s="615"/>
       <x:c r="N43" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -23985,7 +24139,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D44" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E44" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23997,7 +24151,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H44" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I44" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24013,7 +24167,7 @@
       </x:c>
       <x:c r="M44" s="615"/>
       <x:c r="N44" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -24027,7 +24181,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D45" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E45" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24039,7 +24193,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H45" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Pending</x:v>
       </x:c>
       <x:c r="I45" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24055,7 +24209,7 @@
       </x:c>
       <x:c r="M45" s="615"/>
       <x:c r="N45" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 code and regression are deployed, but the production Supabase migration remains unapplied; authorized apply plus grant/revoke read-back is a release blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -24069,7 +24223,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D46" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E46" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24081,7 +24235,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H46" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I46" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24097,7 +24251,7 @@
       </x:c>
       <x:c r="M46" s="615"/>
       <x:c r="N46" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -24111,7 +24265,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D47" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E47" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24123,7 +24277,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H47" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I47" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24139,7 +24293,7 @@
       </x:c>
       <x:c r="M47" s="615"/>
       <x:c r="N47" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -24153,7 +24307,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D48" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E48" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24165,7 +24319,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H48" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I48" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24181,7 +24335,7 @@
       </x:c>
       <x:c r="M48" s="615"/>
       <x:c r="N48" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -24195,7 +24349,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D49" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E49" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24207,7 +24361,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H49" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I49" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24223,7 +24377,7 @@
       </x:c>
       <x:c r="M49" s="615"/>
       <x:c r="N49" s="615" t="str">
-        <x:v>Medium/P2 fixed locally with regression and original-path proof. Deployment, targeted live/read-back verification and tracker reconciliation remain release blockers.</x:v>
+        <x:v>Medium/P2 fix is deployed with CI, regression and production smoke evidence. Finding-specific live/read-back verification and the 72-hour canary remain release blockers.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -24237,7 +24391,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D50" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E50" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24249,7 +24403,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H50" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I50" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24265,7 +24419,7 @@
       </x:c>
       <x:c r="M50" s="615"/>
       <x:c r="N50" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -24279,7 +24433,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D51" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E51" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24291,7 +24445,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H51" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I51" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24307,7 +24461,7 @@
       </x:c>
       <x:c r="M51" s="615"/>
       <x:c r="N51" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -24321,7 +24475,7 @@
         <x:v>P3</x:v>
       </x:c>
       <x:c r="D52" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E52" s="615" t="str">
         <x:v>Passed</x:v>
@@ -24333,7 +24487,7 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H52" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I52" s="615" t="str">
         <x:v>Deferred</x:v>
@@ -24349,7 +24503,7 @@
       </x:c>
       <x:c r="M52" s="615"/>
       <x:c r="N52" s="615" t="str">
-        <x:v>Low/P3 fixed locally with regression and original-path proof. The item remains post-gate Deferred until the deployment/read-back cycle.</x:v>
+        <x:v>Low/P3 fix is deployed with CI, regression and production smoke evidence. The item remains post-gate Deferred until finding-specific read-back/canary closure.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24372,13 +24526,13 @@
     <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I52">
-    <x:cfRule type="containsText" dxfId="560" priority="15" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="561" priority="16" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="562" priority="17" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="563" priority="18" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="564" priority="19" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="565" priority="20" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="566" priority="21" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="574" priority="15" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="575" priority="16" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="576" priority="17" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="577" priority="18" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="578" priority="19" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="579" priority="20" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="580" priority="21" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -25279,7 +25433,7 @@
         <x:v>src/lib/risk/check-core.ts:125-143,338-350; src/lib/risk/rules.ts:302-307</x:v>
       </x:c>
       <x:c r="F22" s="614" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G22" s="614" t="str">
         <x:v>Risk Engine</x:v>
@@ -25288,10 +25442,10 @@
         <x:v>Gate 0</x:v>
       </x:c>
       <x:c r="I22" s="614" t="str">
-        <x:v>High/P1 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
+        <x:v>High/P1 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
       </x:c>
       <x:c r="J22" s="614" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K22" s="614" t="str">
         <x:v>Unrelated content cannot become Safe because it merely contains an official token.</x:v>
@@ -25317,7 +25471,7 @@
         <x:v>src/lib/risk/detect.ts; src/lib/report.functions.ts</x:v>
       </x:c>
       <x:c r="F23" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G23" s="615" t="str">
         <x:v>Privacy / Backend</x:v>
@@ -25326,10 +25480,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I23" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
       </x:c>
       <x:c r="J23" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K23" s="615" t="str">
         <x:v>Complete reports/entities insert payload contains no supported secret marker.</x:v>
@@ -25355,7 +25509,7 @@
         <x:v>src/lib/reputation-appeal.functions.ts; src/lib/risk/detect.ts</x:v>
       </x:c>
       <x:c r="F24" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G24" s="615" t="str">
         <x:v>Privacy / Backend</x:v>
@@ -25364,10 +25518,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I24" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
       </x:c>
       <x:c r="J24" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K24" s="615" t="str">
         <x:v>No secret marker reaches reason or contact_display; generic unsafe contact is rejected.</x:v>
@@ -25393,7 +25547,7 @@
         <x:v>src/lib/risk/qr-decoder.ts; image-intelligence.ts; check-core.ts</x:v>
       </x:c>
       <x:c r="F25" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G25" s="615" t="str">
         <x:v>Media / Privacy</x:v>
@@ -25402,10 +25556,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I25" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
       </x:c>
       <x:c r="J25" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K25" s="615" t="str">
         <x:v>Wi-Fi passwords, otpauth secrets and mnemonic candidates never enter redacted_input.</x:v>
@@ -25431,7 +25585,7 @@
         <x:v>src/lib/telegram/handlers/inline.ts; src/lib/risk/detect.ts</x:v>
       </x:c>
       <x:c r="F26" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G26" s="615" t="str">
         <x:v>Telegram / Privacy</x:v>
@@ -25440,10 +25594,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I26" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
       </x:c>
       <x:c r="J26" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K26" s="615" t="str">
         <x:v>No supported secret marker appears in any Inline article field on real clients.</x:v>
@@ -25469,7 +25623,7 @@
         <x:v>src/lib/telegram/public-post.server.ts; src/lib/risk/check-core.ts</x:v>
       </x:c>
       <x:c r="F27" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
         <x:v>Telegram / Privacy</x:v>
@@ -25478,10 +25632,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
       </x:c>
       <x:c r="J27" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>Mocked check insert contains no secret marker from public-post fixtures.</x:v>
@@ -25507,7 +25661,7 @@
         <x:v>src/lib/report.functions.ts; moderation-notifier.server.ts</x:v>
       </x:c>
       <x:c r="F28" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G28" s="615" t="str">
         <x:v>Telegram / Moderation</x:v>
@@ -25516,10 +25670,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I28" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
       </x:c>
       <x:c r="J28" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed. Run a count-only historical privacy review without logging matched values.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
       </x:c>
       <x:c r="K28" s="615" t="str">
         <x:v>Markdown and plaintext notification payloads contain no secret marker.</x:v>
@@ -25554,10 +25708,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I29" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / eb7a6364-f9da-4ca2-a017-1f6102e50c0f, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
       </x:c>
       <x:c r="J29" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Restore authorized production Supabase access; rerun count-only preflight, apply the exact migration, verify migration history and revoke/grant behavior, then collect read-back evidence.</x:v>
       </x:c>
       <x:c r="K29" s="615" t="str">
         <x:v>Allowlist delete, email drift and confirmation loss immediately deny existing sessions.</x:v>
@@ -25583,7 +25737,7 @@
         <x:v>src/lib/check.functions.ts; embed-origin-analytics.server.ts</x:v>
       </x:c>
       <x:c r="F30" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G30" s="615" t="str">
         <x:v>Backend / Data</x:v>
@@ -25592,10 +25746,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I30" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
       </x:c>
       <x:c r="J30" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K30" s="615" t="str">
         <x:v>Denied request performs zero analytics inserts; production storage failure fails closed.</x:v>
@@ -25621,7 +25775,7 @@
         <x:v>.github/workflows/prod-monitor.yml</x:v>
       </x:c>
       <x:c r="F31" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G31" s="615" t="str">
         <x:v>DevOps / Security</x:v>
@@ -25630,10 +25784,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I31" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
       </x:c>
       <x:c r="J31" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K31" s="615" t="str">
         <x:v>Policy rejects job-scoped secrets, non-SHA actions and pre-secret install hooks.</x:v>
@@ -25659,7 +25813,7 @@
         <x:v>src/lib/telegram/handlers/report.ts; handlers/check.ts</x:v>
       </x:c>
       <x:c r="F32" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G32" s="615" t="str">
         <x:v>Telegram / Platform</x:v>
@@ -25668,10 +25822,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I32" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
       </x:c>
       <x:c r="J32" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K32" s="615" t="str">
         <x:v>Rate-limited report image makes zero getFile/download calls under concurrency.</x:v>
@@ -25697,7 +25851,7 @@
         <x:v>src/lib/risk/image-intelligence.ts; check-core.ts</x:v>
       </x:c>
       <x:c r="F33" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G33" s="615" t="str">
         <x:v>AI / Risk</x:v>
@@ -25706,10 +25860,10 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I33" s="615" t="str">
-        <x:v>Medium/P2 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
+        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
       </x:c>
       <x:c r="J33" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K33" s="615" t="str">
         <x:v>Benign provider category plus phishing URL cannot return Safe without trusted local proof.</x:v>
@@ -25735,7 +25889,7 @@
         <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
       </x:c>
       <x:c r="F34" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G34" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -25744,10 +25898,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I34" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J34" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K34" s="615" t="str">
         <x:v>Confusable hostname cannot inherit official allowlist membership; controls stay valid.</x:v>
@@ -25773,7 +25927,7 @@
         <x:v>src/lib/risk/domain-normalizer.ts; brand-matcher.ts</x:v>
       </x:c>
       <x:c r="F35" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G35" s="615" t="str">
         <x:v>Risk Engine</x:v>
@@ -25782,10 +25936,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I35" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J35" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K35" s="615" t="str">
         <x:v>sp0t.uz cannot inherit spot.uz suppression; similarity only adds evidence.</x:v>
@@ -25811,7 +25965,7 @@
         <x:v>src/lib/telegram/check-followup.ts; victim-intent.ts; handlers/check.ts</x:v>
       </x:c>
       <x:c r="F36" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deployed / Awaiting Live Verification</x:v>
       </x:c>
       <x:c r="G36" s="615" t="str">
         <x:v>Telegram / Product</x:v>
@@ -25820,10 +25974,10 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I36" s="615" t="str">
-        <x:v>Low/P3 fixed locally on codex/security-revalidation-fixes-20260712. Integration: 4222/4222 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38, schema lint; original safe PoC or realistic boundary regression no longer reproduces. Count-only production admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
+        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
       </x:c>
       <x:c r="J36" s="615" t="str">
-        <x:v>Commit/CI/deploy the exact patch, run the stated targeted acceptance and collect read-back evidence before changing to Deployed/Closed.</x:v>
+        <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
       </x:c>
       <x:c r="K36" s="615" t="str">
         <x:v>Passport/document questions never reuse old results; five legitimate follow-ups still pass.</x:v>
@@ -25843,13 +25997,13 @@
     <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F2:F36">
-    <x:cfRule type="containsText" dxfId="553" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="554" priority="9" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="555" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="556" priority="11" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="557" priority="12" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="558" priority="13" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="559" priority="14" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="567" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="568" priority="9" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="569" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="570" priority="11" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="571" priority="12" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="572" priority="13" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="573" priority="14" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
Record release gate deployment evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7146198fbd7646de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb18ef2214fdb45e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R368baeb6be9046e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R521ea297fca94fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb26a4ff13bb54aed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2c5f1d2c648b4e3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R32b6e81362784955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rb5f91f5f2f2a4fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfaf73d77a0554f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra04dbe72a96a4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R508f37af59404867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R12e49900df5343a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R00f0f9b68d5144f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R32085d1aaa2c4dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R69d39cd45eef4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd199101e62144eb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4308,7 +4308,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="581">
+  <x:dxfs count="623">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -9619,6 +9619,468 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -10991,7 +11453,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="72" customHeight="1">
+    <x:row r="2" ht="108" customHeight="1">
       <x:c r="A2" s="1218" t="n">
         <x:v>46215</x:v>
       </x:c>
@@ -11004,10 +11466,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 5c6094add5dee66045adf445fe15e566405c55da and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Next: historical count-only privacy review, real-client RU/UZ/EN Inline evidence, finding-specific acceptance and a 72-hour canary.</x:v>
+        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Automated release gates, the 1872-row bot corpus and production smokes are green. Next: real-client RU/UZ/EN + Inline evidence, authorized data drills, legal approval and a 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Evidence: 4227/4227 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint, PR #83 CI, Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f, app/polling/Inline-boundary/dialogue smokes with cleanup and monitor 29203622435. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Canonical source and evidence copy are synchronized.</x:v>
+        <x:v>Evidence: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CodeQL; Gitleaks; Trivy 0 fixed High/Critical; CycloneDX 1.6 SBOM; 28 migrations; pgTAP 38/38; schema lint; CI 29204994706/29204994736; Railway be7d6f8d-f06d-459b-b438-ef8924454c4e; app/polling/Inline-boundary/dialogue smokes with cleanup; monitor 29205158630. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11274,7 +11736,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -11288,7 +11750,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -11302,7 +11764,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -22302,10 +22764,10 @@
         <x:v>Deployed remediation verification for 15 revalidation findings</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; CI app + migrations/schema/pgTAP; Railway exact-SHA deploy; prod:smoke; prod:telegram-inline-smoke; prod:telegram-polling-dispatch-smoke; GitHub production monitor; production admin-role count-only preflight</x:v>
+        <x:v>npm run test:run; coverage thresholds; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; CodeQL; Gitleaks; Trivy; CycloneDX; migrations/schema/pgTAP; Railway exact-SHA deploy; production smokes and monitor; production admin-role count-only preflight</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Passed: 4227/4227 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; exact deployment 5c6094a / eb7a6364; app/health/webhook/polling/AI/Inline-boundary/dialogue smokes; monitor 29203622435; cleanup/read-back. Admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+        <x:v>Passed: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CodeQL; Gitleaks; Trivy 0 fixed High/Critical; CycloneDX 1.6; 28 migrations; pgTAP 38/38; schema lint; exact deployment 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e; monitor 29205158630; cleanup/read-back. Admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
       </x:c>
       <x:c r="F97" t="str">
         <x:v>SEC-2026-0712-001..015, OPS-001, RC-001</x:v>
@@ -22315,6 +22777,32 @@
       </x:c>
       <x:c r="H97" t="str">
         <x:v>Restore authorized Supabase access and apply/verify the admin migration; complete finding-specific live/read-back, historical count-only privacy review, real-client RU/UZ/EN Inline matrix and 72-hour canary; then close eligible findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>QA-RELEASE-GATES-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B98" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Release-gate expansion, supply-chain gates and production revalidation</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>4867-test suite; coverage thresholds; TypeScript; lint; build; npm audit; CodeQL; Gitleaks; Trivy; CycloneDX SBOM; Supabase migrations/schema/pgTAP; exact Railway deploy; production app/Inline/polling-dialogue smokes; GitHub monitor</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Passed: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; npm audit 0; CI 29204994706; security 29204994736; CycloneDX 1.6 / 91 components; Trivy 0 fixed High/Critical; Railway 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e; monitor 29205158630; test data cleanup read-back.</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>BOT-004, INL-001, OPS-001, OPS-002, OPS-004, DR-001, RC-001</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>No broad real-client Inline/RU-UZ-EN transcript matrix, real 60-minute polling/resource soak, restore/key-rotation drill, external legal approval, production Supabase migration apply or 72-hour canary is claimed.</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>Execute the external/live gates in order: real clients; authorized Supabase apply; isolated restore/rotation; 60-minute soak; legal approval; freeze RC and complete 144 canary observations.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23470,10 +23958,12 @@
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
       </x:c>
-      <x:c r="L27" s="615" t="str"/>
+      <x:c r="L27" s="615" t="str">
+        <x:v>Real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
+      </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>Deterministic DSL covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. PR #79 / b4cabb9 is deployed via Railway 37a91c7a; polling monitor and the five-action production dispatch smoke passed. Broader real Telegram-client RU/UZ/EN transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
+        <x:v>The deterministic DSL now covers 13 actions x 3 languages x 6 reviewed surface variants x 8 contexts = 1872 unique rows. All 78 normalized reply-to-bot/typo phrases have exhaustive handler tests forbidding cold checks, session writes and trusted-contact side effects. PR #84 CI 29204994706, Railway be7d6f8d-f06d-459b-b438-ef8924454c4e, polling dispatch and cleanup passed. Broad real-client RU/UZ/EN transcripts remain required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -23567,16 +24057,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D30" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E30" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F30" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G30" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H30" s="615" t="str">
         <x:v>Deployed</x:v>
@@ -23585,7 +24075,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J30" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K30" s="615" t="str">
         <x:v>Telegram / QA</x:v>
@@ -23597,7 +24087,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend is deployed at 5c6094add5dee66045adf445fe15e566405c55da. Automated Inline protocol/privacy and polling transport-boundary coverage are green; real-client visual/insertion evidence remains the blocker.</x:v>
+        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -23651,33 +24141,33 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D32" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E32" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F32" s="615" t="str">
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="G32" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H32" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="I32" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J32" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K32" s="615" t="str">
         <x:v>DevOps / Security</x:v>
       </x:c>
-      <x:c r="L32" s="615" t="str"/>
+      <x:c r="L32" s="615"/>
       <x:c r="M32" s="615" t="str"/>
       <x:c r="N32" s="615" t="str">
-        <x:v>Full lint now passes with 0 errors/8 warnings; typecheck, 2863x2 tests, npm audits and build pass. Coverage/SAST/secret/container gates still require CI evidence; High/Critical blocks release or has an expiry-bound exception.</x:v>
+        <x:v>Mandatory format/lint/type/test/build/coverage, CodeQL, Gitleaks, dependency audit and release-container Trivy gates passed in CI 29204994706/29204994736. Coverage: 82.85% statements, 76.99% branches, 89.29% functions, 84.71% lines. Trivy reported 0 fixed High/Critical.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -23691,31 +24181,35 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D33" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E33" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F33" s="615" t="str">
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="G33" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H33" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="I33" s="615" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="J33" s="618"/>
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="J33" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K33" s="615" t="str">
         <x:v>DevOps / Security</x:v>
       </x:c>
-      <x:c r="L33" s="615" t="str"/>
+      <x:c r="L33" s="615" t="str">
+        <x:v>Artifact signing / verifiable build provenance</x:v>
+      </x:c>
       <x:c r="M33" s="615" t="str"/>
       <x:c r="N33" s="615" t="str">
-        <x:v>Release artifact is bound to commit and immutable dependencies.</x:v>
+        <x:v>All GitHub actions and tool versions are immutable-pinned. Security run 29204994736 uploaded a valid CycloneDX 1.6 SBOM with 91 components before the blocking container scan. Artifact signing and verifiable provenance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -23767,33 +24261,35 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D35" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E35" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F35" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G35" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H35" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I35" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J35" s="618"/>
+      <x:c r="J35" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K35" s="615" t="str">
         <x:v>Product / Legal</x:v>
       </x:c>
       <x:c r="L35" s="615" t="str">
-        <x:v>External legal review</x:v>
+        <x:v>External legal/privacy approval and final appeal retention decision</x:v>
       </x:c>
       <x:c r="M35" s="615" t="str"/>
       <x:c r="N35" s="615" t="str">
-        <x:v>One current approved privacy spec and truthful public copy.</x:v>
+        <x:v>RU/UZ/EN public privacy copy now states raw screenshot disposal, actual retention periods and /appeal guidance; privacy contract tests pass and 190c82a2a0d7db8f1583c57265afe353e97f3f22 is live. Independent legal approval, partner governance and the final appeal-retention decision remain external gates.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -23807,7 +24303,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D36" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E36" s="615" t="str">
         <x:v>Pending</x:v>
@@ -23819,21 +24315,23 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H36" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="I36" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J36" s="618"/>
+      <x:c r="J36" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K36" s="615" t="str">
         <x:v>DevOps / Data</x:v>
       </x:c>
       <x:c r="L36" s="615" t="str">
-        <x:v>Production access</x:v>
+        <x:v>Authorized isolated restore and production key-rotation windows</x:v>
       </x:c>
       <x:c r="M36" s="615" t="str"/>
       <x:c r="N36" s="615" t="str">
-        <x:v>Restore/rollback/key rotation evidence exists and is current.</x:v>
+        <x:v>RECOVERY_AND_KEY_ROTATION.md defines isolated restore, rollback, RPO/RTO evidence and safe rotation order. No real restore or key-rotation drill is claimed; HASH_PEPPER_SECRET requires a versioned dual-read/new-write design before rotation.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -23847,33 +24345,35 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D37" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E37" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F37" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G37" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H37" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I37" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J37" s="618"/>
+      <x:c r="J37" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K37" s="615" t="str">
         <x:v>Release Team</x:v>
       </x:c>
       <x:c r="L37" s="615" t="str">
-        <x:v>All P0/P1 gates</x:v>
+        <x:v>All remaining P0/P1 live gates plus uninterrupted 72-hour canary</x:v>
       </x:c>
       <x:c r="M37" s="615" t="str"/>
       <x:c r="N37" s="615" t="str">
-        <x:v>Go requires 0 open P0/P1 and fresh production/security/restore evidence.</x:v>
+        <x:v>Fresh CI/security gates, SBOM, exact Railway deployment be7d6f8d-f06d-459b-b438-ef8924454c4e, production smokes and monitor 29205158630 are green. CANARY_72H.md defines 144 eligible half-hour observations; the clock has not started and no 72-hour completion is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -24526,13 +25026,13 @@
     <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I52">
-    <x:cfRule type="containsText" dxfId="574" priority="15" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="575" priority="16" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="576" priority="17" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="577" priority="18" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="578" priority="19" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="579" priority="20" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="580" priority="21" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="616" priority="15" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="617" priority="16" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="618" priority="17" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="619" priority="18" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="620" priority="19" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="621" priority="20" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="622" priority="21" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -25442,7 +25942,7 @@
         <x:v>Gate 0</x:v>
       </x:c>
       <x:c r="I22" s="614" t="str">
-        <x:v>High/P1 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
+        <x:v>High/P1 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
       </x:c>
       <x:c r="J22" s="614" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25480,7 +25980,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I23" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
       </x:c>
       <x:c r="J23" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25518,7 +26018,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I24" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
       </x:c>
       <x:c r="J24" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25556,7 +26056,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I25" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
       </x:c>
       <x:c r="J25" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25594,7 +26094,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I26" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
       </x:c>
       <x:c r="J26" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25632,7 +26132,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
       </x:c>
       <x:c r="J27" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25670,7 +26170,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I28" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
       </x:c>
       <x:c r="J28" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25708,7 +26208,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I29" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / eb7a6364-f9da-4ca2-a017-1f6102e50c0f, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
       </x:c>
       <x:c r="J29" s="615" t="str">
         <x:v>Restore authorized production Supabase access; rerun count-only preflight, apply the exact migration, verify migration history and revoke/grant behavior, then collect read-back evidence.</x:v>
@@ -25746,7 +26246,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I30" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
       </x:c>
       <x:c r="J30" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25784,7 +26284,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I31" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
       </x:c>
       <x:c r="J31" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25822,7 +26322,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I32" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
       </x:c>
       <x:c r="J32" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25860,7 +26360,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I33" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
       </x:c>
       <x:c r="J33" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25898,7 +26398,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I34" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J34" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25936,7 +26436,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I35" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J35" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25974,7 +26474,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I36" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
       </x:c>
       <x:c r="J36" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25997,13 +26497,13 @@
     <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F2:F36">
-    <x:cfRule type="containsText" dxfId="567" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="568" priority="9" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="569" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="570" priority="11" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="571" priority="12" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="572" priority="13" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="573" priority="14" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="609" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="610" priority="9" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="611" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="612" priority="11" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="613" priority="12" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="614" priority="13" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="615" priority="14" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
Record release gate deployment evidence (#85)
Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R7146198fbd7646de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rb18ef2214fdb45e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R368baeb6be9046e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R521ea297fca94fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rb26a4ff13bb54aed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2c5f1d2c648b4e3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R32b6e81362784955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rb5f91f5f2f2a4fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfaf73d77a0554f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra04dbe72a96a4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R508f37af59404867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R12e49900df5343a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R00f0f9b68d5144f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R32085d1aaa2c4dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R69d39cd45eef4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd199101e62144eb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4308,7 +4308,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="581">
+  <x:dxfs count="623">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -9619,6 +9619,468 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF115E59"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFCCFBF1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF991B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF1E40AF"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDBEAFE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF4B5563"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -10991,7 +11453,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="72" customHeight="1">
+    <x:row r="2" ht="108" customHeight="1">
       <x:c r="A2" s="1218" t="n">
         <x:v>46215</x:v>
       </x:c>
@@ -11004,10 +11466,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 5c6094add5dee66045adf445fe15e566405c55da and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Next: historical count-only privacy review, real-client RU/UZ/EN Inline evidence, finding-specific acceptance and a 72-hour canary.</x:v>
+        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Automated release gates, the 1872-row bot corpus and production smokes are green. Next: real-client RU/UZ/EN + Inline evidence, authorized data drills, legal approval and a 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Evidence: 4227/4227 tests, TypeScript, lint (0 errors/8 existing warnings), production build, npm audit 0, 28-migration reset, pgTAP 38/38, schema lint, PR #83 CI, Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f, app/polling/Inline-boundary/dialogue smokes with cleanup and monitor 29203622435. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0. Canonical source and evidence copy are synchronized.</x:v>
+        <x:v>Evidence: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CodeQL; Gitleaks; Trivy 0 fixed High/Critical; CycloneDX 1.6 SBOM; 28 migrations; pgTAP 38/38; schema lint; CI 29204994706/29204994736; Railway be7d6f8d-f06d-459b-b438-ef8924454c4e; app/polling/Inline-boundary/dialogue smokes with cleanup; monitor 29205158630. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11274,7 +11736,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -11288,7 +11750,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -11302,7 +11764,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -22302,10 +22764,10 @@
         <x:v>Deployed remediation verification for 15 revalidation findings</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; CI app + migrations/schema/pgTAP; Railway exact-SHA deploy; prod:smoke; prod:telegram-inline-smoke; prod:telegram-polling-dispatch-smoke; GitHub production monitor; production admin-role count-only preflight</x:v>
+        <x:v>npm run test:run; coverage thresholds; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; CodeQL; Gitleaks; Trivy; CycloneDX; migrations/schema/pgTAP; Railway exact-SHA deploy; production smokes and monitor; production admin-role count-only preflight</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>Passed: 4227/4227 tests; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; 28 migrations; pgTAP 38/38; schema lint; exact deployment 5c6094a / eb7a6364; app/health/webhook/polling/AI/Inline-boundary/dialogue smokes; monitor 29203622435; cleanup/read-back. Admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+        <x:v>Passed: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CodeQL; Gitleaks; Trivy 0 fixed High/Critical; CycloneDX 1.6; 28 migrations; pgTAP 38/38; schema lint; exact deployment 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e; monitor 29205158630; cleanup/read-back. Admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
       </x:c>
       <x:c r="F97" t="str">
         <x:v>SEC-2026-0712-001..015, OPS-001, RC-001</x:v>
@@ -22315,6 +22777,32 @@
       </x:c>
       <x:c r="H97" t="str">
         <x:v>Restore authorized Supabase access and apply/verify the admin migration; complete finding-specific live/read-back, historical count-only privacy review, real-client RU/UZ/EN Inline matrix and 72-hour canary; then close eligible findings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>QA-RELEASE-GATES-2026-07-12</x:v>
+      </x:c>
+      <x:c r="B98" s="1097" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Release-gate expansion, supply-chain gates and production revalidation</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>4867-test suite; coverage thresholds; TypeScript; lint; build; npm audit; CodeQL; Gitleaks; Trivy; CycloneDX SBOM; Supabase migrations/schema/pgTAP; exact Railway deploy; production app/Inline/polling-dialogue smokes; GitHub monitor</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Passed: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; npm audit 0; CI 29204994706; security 29204994736; CycloneDX 1.6 / 91 components; Trivy 0 fixed High/Critical; Railway 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e; monitor 29205158630; test data cleanup read-back.</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>BOT-004, INL-001, OPS-001, OPS-002, OPS-004, DR-001, RC-001</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>No broad real-client Inline/RU-UZ-EN transcript matrix, real 60-minute polling/resource soak, restore/key-rotation drill, external legal approval, production Supabase migration apply or 72-hour canary is claimed.</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>Execute the external/live gates in order: real clients; authorized Supabase apply; isolated restore/rotation; 60-minute soak; legal approval; freeze RC and complete 144 canary observations.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23470,10 +23958,12 @@
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
       </x:c>
-      <x:c r="L27" s="615" t="str"/>
+      <x:c r="L27" s="615" t="str">
+        <x:v>Real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
+      </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>Deterministic DSL covers 13 follow-up actions x 3 languages x 4 surface variants x 8 contexts = 1248 unique rows; all 238 actual legacy live-matrix rows map to canonical contracts. PR #79 / b4cabb9 is deployed via Railway 37a91c7a; polling monitor and the five-action production dispatch smoke passed. Broader real Telegram-client RU/UZ/EN transcripts remain required; generated rows are not claimed as independent live conversations.</x:v>
+        <x:v>The deterministic DSL now covers 13 actions x 3 languages x 6 reviewed surface variants x 8 contexts = 1872 unique rows. All 78 normalized reply-to-bot/typo phrases have exhaustive handler tests forbidding cold checks, session writes and trusted-contact side effects. PR #84 CI 29204994706, Railway be7d6f8d-f06d-459b-b438-ef8924454c4e, polling dispatch and cleanup passed. Broad real-client RU/UZ/EN transcripts remain required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -23567,16 +24057,16 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D30" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E30" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F30" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G30" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H30" s="615" t="str">
         <x:v>Deployed</x:v>
@@ -23585,7 +24075,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J30" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K30" s="615" t="str">
         <x:v>Telegram / QA</x:v>
@@ -23597,7 +24087,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend is deployed at 5c6094add5dee66045adf445fe15e566405c55da. Automated Inline protocol/privacy and polling transport-boundary coverage are green; real-client visual/insertion evidence remains the blocker.</x:v>
+        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -23651,33 +24141,33 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D32" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E32" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F32" s="615" t="str">
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="G32" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H32" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="I32" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J32" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46215</x:v>
       </x:c>
       <x:c r="K32" s="615" t="str">
         <x:v>DevOps / Security</x:v>
       </x:c>
-      <x:c r="L32" s="615" t="str"/>
+      <x:c r="L32" s="615"/>
       <x:c r="M32" s="615" t="str"/>
       <x:c r="N32" s="615" t="str">
-        <x:v>Full lint now passes with 0 errors/8 warnings; typecheck, 2863x2 tests, npm audits and build pass. Coverage/SAST/secret/container gates still require CI evidence; High/Critical blocks release or has an expiry-bound exception.</x:v>
+        <x:v>Mandatory format/lint/type/test/build/coverage, CodeQL, Gitleaks, dependency audit and release-container Trivy gates passed in CI 29204994706/29204994736. Coverage: 82.85% statements, 76.99% branches, 89.29% functions, 84.71% lines. Trivy reported 0 fixed High/Critical.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -23691,31 +24181,35 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D33" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E33" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F33" s="615" t="str">
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="G33" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H33" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="I33" s="615" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="J33" s="618"/>
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="J33" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K33" s="615" t="str">
         <x:v>DevOps / Security</x:v>
       </x:c>
-      <x:c r="L33" s="615" t="str"/>
+      <x:c r="L33" s="615" t="str">
+        <x:v>Artifact signing / verifiable build provenance</x:v>
+      </x:c>
       <x:c r="M33" s="615" t="str"/>
       <x:c r="N33" s="615" t="str">
-        <x:v>Release artifact is bound to commit and immutable dependencies.</x:v>
+        <x:v>All GitHub actions and tool versions are immutable-pinned. Security run 29204994736 uploaded a valid CycloneDX 1.6 SBOM with 91 components before the blocking container scan. Artifact signing and verifiable provenance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -23767,33 +24261,35 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D35" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E35" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F35" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G35" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H35" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I35" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J35" s="618"/>
+      <x:c r="J35" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K35" s="615" t="str">
         <x:v>Product / Legal</x:v>
       </x:c>
       <x:c r="L35" s="615" t="str">
-        <x:v>External legal review</x:v>
+        <x:v>External legal/privacy approval and final appeal retention decision</x:v>
       </x:c>
       <x:c r="M35" s="615" t="str"/>
       <x:c r="N35" s="615" t="str">
-        <x:v>One current approved privacy spec and truthful public copy.</x:v>
+        <x:v>RU/UZ/EN public privacy copy now states raw screenshot disposal, actual retention periods and /appeal guidance; privacy contract tests pass and 190c82a2a0d7db8f1583c57265afe353e97f3f22 is live. Independent legal approval, partner governance and the final appeal-retention decision remain external gates.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -23807,7 +24303,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="D36" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E36" s="615" t="str">
         <x:v>Pending</x:v>
@@ -23819,21 +24315,23 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H36" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="I36" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J36" s="618"/>
+      <x:c r="J36" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K36" s="615" t="str">
         <x:v>DevOps / Data</x:v>
       </x:c>
       <x:c r="L36" s="615" t="str">
-        <x:v>Production access</x:v>
+        <x:v>Authorized isolated restore and production key-rotation windows</x:v>
       </x:c>
       <x:c r="M36" s="615" t="str"/>
       <x:c r="N36" s="615" t="str">
-        <x:v>Restore/rollback/key rotation evidence exists and is current.</x:v>
+        <x:v>RECOVERY_AND_KEY_ROTATION.md defines isolated restore, rollback, RPO/RTO evidence and safe rotation order. No real restore or key-rotation drill is claimed; HASH_PEPPER_SECRET requires a versioned dual-read/new-write design before rotation.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -23847,33 +24345,35 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D37" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E37" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="F37" s="615" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G37" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H37" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I37" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J37" s="618"/>
+      <x:c r="J37" s="618" t="n">
+        <x:v>46215</x:v>
+      </x:c>
       <x:c r="K37" s="615" t="str">
         <x:v>Release Team</x:v>
       </x:c>
       <x:c r="L37" s="615" t="str">
-        <x:v>All P0/P1 gates</x:v>
+        <x:v>All remaining P0/P1 live gates plus uninterrupted 72-hour canary</x:v>
       </x:c>
       <x:c r="M37" s="615" t="str"/>
       <x:c r="N37" s="615" t="str">
-        <x:v>Go requires 0 open P0/P1 and fresh production/security/restore evidence.</x:v>
+        <x:v>Fresh CI/security gates, SBOM, exact Railway deployment be7d6f8d-f06d-459b-b438-ef8924454c4e, production smokes and monitor 29205158630 are green. CANARY_72H.md defines 144 eligible half-hour observations; the clock has not started and no 72-hour completion is claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -24526,13 +25026,13 @@
     <x:cfRule type="containsText" dxfId="468" priority="14" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D2:I52">
-    <x:cfRule type="containsText" dxfId="574" priority="15" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="575" priority="16" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="576" priority="17" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="577" priority="18" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="578" priority="19" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="579" priority="20" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="580" priority="21" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="616" priority="15" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="617" priority="16" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="618" priority="17" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="619" priority="18" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="620" priority="19" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="621" priority="20" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="622" priority="21" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="20">
     <x:dataValidation type="list" sqref="C2:C36">
@@ -25442,7 +25942,7 @@
         <x:v>Gate 0</x:v>
       </x:c>
       <x:c r="I22" s="614" t="str">
-        <x:v>High/P1 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
+        <x:v>High/P1 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/verified-contact-risk-override.</x:v>
       </x:c>
       <x:c r="J22" s="614" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25480,7 +25980,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I23" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/shared-redaction-secret-leak.</x:v>
       </x:c>
       <x:c r="J23" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25518,7 +26018,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I24" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/appeal-secret-persistence.</x:v>
       </x:c>
       <x:c r="J24" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25556,7 +26056,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I25" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/qr-secret-check-persistence.</x:v>
       </x:c>
       <x:c r="J25" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25594,7 +26094,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I26" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-inline-secret-republication.</x:v>
       </x:c>
       <x:c r="J26" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25632,7 +26132,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/public-post-secret-persistence.</x:v>
       </x:c>
       <x:c r="J27" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25670,7 +26170,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I28" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/moderation-notifier-secret-delivery.</x:v>
       </x:c>
       <x:c r="J28" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed. Run a count-only historical privacy review without logging matched values.</x:v>
@@ -25708,7 +26208,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I29" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / eb7a6364-f9da-4ca2-a017-1f6102e50c0f, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
       </x:c>
       <x:c r="J29" s="615" t="str">
         <x:v>Restore authorized production Supabase access; rerun count-only preflight, apply the exact migration, verify migration history and revoke/grant behavior, then collect read-back evidence.</x:v>
@@ -25746,7 +26246,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I30" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/embed-meta-intent-telemetry-amplification.</x:v>
       </x:c>
       <x:c r="J30" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25784,7 +26284,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I31" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/production-monitor-secret-scope.</x:v>
       </x:c>
       <x:c r="J31" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25822,7 +26322,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I32" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-report-image-prelimit-download.</x:v>
       </x:c>
       <x:c r="J32" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25860,7 +26360,7 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I33" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
+        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/provider-benign-image-url-omission.</x:v>
       </x:c>
       <x:c r="J33" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25898,7 +26398,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I34" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/official-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J34" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25936,7 +26436,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I35" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/news-domain-skeleton-collision.</x:v>
       </x:c>
       <x:c r="J35" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25974,7 +26474,7 @@
         <x:v>Post-gate</x:v>
       </x:c>
       <x:c r="I36" s="615" t="str">
-        <x:v>Low/P3 remediation verified: 4227/4227 tests, TypeScript, lint 0 errors, build, npm audit 0, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 5c6094add5dee66045adf445fe15e566405c55da / Railway eb7a6364-f9da-4ca2-a017-1f6102e50c0f. PR #83 CI passed both jobs; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29203622435 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
+        <x:v>Low/P3 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Fixed application code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / Railway be7d6f8d-f06d-459b-b438-ef8924454c4e. PR #84 CI 29204994706 and security gates 29204994736 passed; production app/polling/Inline-boundary/dialogue smokes and GitHub monitor 29205158630 passed with cleanup/read-back. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/telegram-passport-followup-misrouting.</x:v>
       </x:c>
       <x:c r="J36" s="615" t="str">
         <x:v>Complete the finding-specific live/read-back acceptance and 72-hour canary before changing to Closed.</x:v>
@@ -25997,13 +26497,13 @@
     <x:cfRule type="containsText" dxfId="475" priority="7" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F2:F36">
-    <x:cfRule type="containsText" dxfId="567" priority="8" operator="containsText" text="Passed"/>
-    <x:cfRule type="containsText" dxfId="568" priority="9" operator="containsText" text="Closed"/>
-    <x:cfRule type="containsText" dxfId="569" priority="10" operator="containsText" text="Deployed"/>
-    <x:cfRule type="containsText" dxfId="570" priority="11" operator="containsText" text="Blocked"/>
-    <x:cfRule type="containsText" dxfId="571" priority="12" operator="containsText" text="Open"/>
-    <x:cfRule type="containsText" dxfId="572" priority="13" operator="containsText" text="In Progress"/>
-    <x:cfRule type="containsText" dxfId="573" priority="14" operator="containsText" text="Deferred"/>
+    <x:cfRule type="containsText" dxfId="609" priority="8" operator="containsText" text="Passed"/>
+    <x:cfRule type="containsText" dxfId="610" priority="9" operator="containsText" text="Closed"/>
+    <x:cfRule type="containsText" dxfId="611" priority="10" operator="containsText" text="Deployed"/>
+    <x:cfRule type="containsText" dxfId="612" priority="11" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="613" priority="12" operator="containsText" text="Open"/>
+    <x:cfRule type="containsText" dxfId="614" priority="13" operator="containsText" text="In Progress"/>
+    <x:cfRule type="containsText" dxfId="615" priority="14" operator="containsText" text="Deferred"/>
   </x:conditionalFormatting>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B2:B21">

</xml_diff>

<commit_message>
Expand Telegram dialogue QA and clause-local routing
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfaf73d77a0554f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra04dbe72a96a4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R508f37af59404867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R12e49900df5343a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R00f0f9b68d5144f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R32085d1aaa2c4dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R69d39cd45eef4cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd199101e62144eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R48b3f0dfd7e0416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R34d0fb01804d4a38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd93aeb3768984a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re3db89d978944bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R3b9a361518b14b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2054a321a3d64a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd6df23b0134d4194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R6f6f373b049847fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1202,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1227">
+  <x:cellXfs count="1228">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4304,6 +4304,9 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11014,7 +11017,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11025,7 +11028,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11036,7 +11039,7 @@
         <x:color rgb="FF115E59"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFCCFBF1"/>
         </x:patternFill>
       </x:fill>
@@ -11047,7 +11050,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11058,7 +11061,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11069,7 +11072,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -11080,7 +11083,7 @@
         <x:color rgb="FF4B5563"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
@@ -11091,7 +11094,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11102,7 +11105,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11113,7 +11116,7 @@
         <x:color rgb="FF115E59"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFCCFBF1"/>
         </x:patternFill>
       </x:fill>
@@ -11124,7 +11127,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11135,7 +11138,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11146,7 +11149,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -11157,7 +11160,7 @@
         <x:color rgb="FF4B5563"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
@@ -11454,8 +11457,8 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="108" customHeight="1">
-      <x:c r="A2" s="1218" t="n">
-        <x:v>46215</x:v>
+      <x:c r="A2" s="1227" t="n">
+        <x:v>46216</x:v>
       </x:c>
       <x:c r="B2" s="1219" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
@@ -11466,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Automated release gates, the 1872-row bot corpus and production smokes are green. Next: real-client RU/UZ/EN + Inline evidence, authorized data drills, legal approval and a 72-hour canary.</x:v>
+        <x:v>Review, merge and deploy the local BOT-004 conversational-perimeter change, then capture real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot evidence. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Evidence: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CodeQL; Gitleaks; Trivy 0 fixed High/Critical; CycloneDX 1.6 SBOM; 28 migrations; pgTAP 38/38; schema lint; CI 29204994706/29204994736; Railway be7d6f8d-f06d-459b-b438-ef8924454c4e; app/polling/Inline-boundary/dialogue smokes with cleanup; monitor 29205158630. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+        <x:v>Local 2026-07-13 evidence: 8583/8583 tests in 134 files with global unmocked-network denial; 1008 RU/UZ/EN context cases; exactly 1000 synthetic multi-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause adversarial messages; independent conversational/risk review 2438/2438; 17 benign end-to-end controls and 33/33 paired direct-danger probes; TypeScript; changed-file Prettier; lint 0 errors/8 existing warnings; production build; npm audit 0. Final review found and fixed a working-tree-only whole-message exemption: door/entrance, postal, dress and source-code clauses can no longer hide a later banking/login-code request; 28 focused RU/UZ/EN regressions pass and genuine physical-access codes remain neutral. The screenshot phrase asks for the actual link instead of starting an empty check. No AI provider, Telegram, database or production call was made by this QA. This is deterministic testing, not model training or live-client evidence; prior deployed release/security evidence remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -12092,10 +12095,8 @@
           <x:t xml:space="preserve">Commands/callbacks/scenarios win first; meta questions route to safe explanatory copy; scam-context override still checks risky input.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/lib/telegram/meta-intent.ts; src/lib/telegram/router.ts; src/lib/telegram/bot-i18n.ts</x:t>
-        </x:is>
+      <x:c r="F5" s="8" t="str">
+        <x:v>src/lib/meta-intent.ts; src/lib/telegram/conversation-wrapper.ts; src/lib/telegram/router.ts; src/lib/telegram/bot-i18n.ts</x:v>
       </x:c>
       <x:c r="G5" s="8" t="inlineStr">
         <x:is>
@@ -12107,25 +12108,19 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit/property tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Add broader conversational layer for questions about the last check.</x:t>
-        </x:is>
+      <x:c r="I5" s="8" t="str">
+        <x:v>Unit/property/router integration; 1008 offline RU/UZ/EN context cases; 1000 unique multi-turn dialogues / 2500 user turns; 540 everyday dialogues / 1080 turns / 102 follow-ups; 363 mixed-clause cases; independent 2438/2438; 28 clause-local code-context regressions; full suite 8583/8583 on 2026-07-13</x:v>
+      </x:c>
+      <x:c r="J5" s="8" t="str">
+        <x:v>Local change fixes the observed empty-check phrase and adds bounded greeting/off-topic/capability routing. Review/merge/deploy and real Telegram Desktop/Android/iOS RU/UZ/EN evidence remain required.</x:v>
       </x:c>
       <x:c r="K5" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P2</x:t>
         </x:is>
       </x:c>
-      <x:c r="L5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Answers must not reveal system prompts or internal scoring thresholds beyond approved language.</x:t>
-        </x:is>
+      <x:c r="L5" s="8" t="str">
+        <x:v>Reply-only meta contracts forbid persistence and trusted-contact effects. Concrete artifacts/forwarded content and mixed unsafe clauses bypass meta routing. Door/entrance, postal, dress and source-code exceptions are clause-local and cannot suppress a later banking/login-code request. Global Vitest and corpus guards deny unmocked network access. Verified locally 2026-07-13; the affected helpers were never deployed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12169,25 +12164,19 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit tests + live production smoke</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RU/UZ/EN acknowledgement and confirmation-request follow-ups passed live smoke; extend phrase list only from real transcripts.</x:t>
-        </x:is>
+      <x:c r="I6" s="8" t="str">
+        <x:v>Unit/integration plus context, multi-turn and everyday corpora; actual production-derived last-check snapshots; 17 benign end-to-end controls; 33/33 direct-danger probes; recent-result methodology/fresh-domain separation; full suite 8583/8583 on 2026-07-13</x:v>
+      </x:c>
+      <x:c r="J6" s="8" t="str">
+        <x:v>Saved provenance now wins for short or wrapped methodology questions; a new concrete domain remains a fresh check. Real-client RU/UZ/EN reply/restart/language matrix is still open.</x:v>
       </x:c>
       <x:c r="K6" s="12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P1</x:t>
         </x:is>
       </x:c>
-      <x:c r="L6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups. 2026-06-30: .claude QA feedback rechecked in focused suite: acknowledgement replies, confirmation-request follow-ups and word-boundary voice transcript previews are covered; `npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/check-followup.test.ts` passed 4 files / 127 tests. 2026-06-30 production pass: prod:telegram-user-story-smoke verified thanks/confirmation follow-ups after a last delivery check did not create checks in RU/UZ/EN sessions.</x:t>
-        </x:is>
+      <x:c r="L6" s="8" t="str">
+        <x:v>Follow-ups use production-bounded stored reasons/levels, explain visible evidence and limitations, never claim an unperformed recheck, and create no check/contact side effects. Verified locally with network blocked on 2026-07-13.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -22803,6 +22792,32 @@
       </x:c>
       <x:c r="H98" t="str">
         <x:v>Execute the external/live gates in order: real clients; authorized Supabase apply; isolated restore/rotation; 60-minute soak; legal approval; freeze RC and complete 144 canary observations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>QA-HUMAN-DIALOGUE-OFFLINE-2026-07-13</x:v>
+      </x:c>
+      <x:c r="B99" s="1097" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>Offline RU/UZ/EN human-style conversational perimeter and observed Telegram phrase regression</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>npm run test:run with global unmocked-network denial; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; changed-file Prettier; corpus hard fetch guards; independent conversational/risk review</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>Passed: 134 files / 8583 tests; 1008 context utterances; exactly 1000 unique 2/3-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause messages; independent 2438/2438; 17 benign controls; 33/33 direct-danger probes; 28 clause-local code-context regressions; actual production-derived follow-up snapshots; screenshot link-capability phrase asks for the real link; 0 AI/provider/Telegram calls.</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>BOT-004, TG-004, TG-005</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Reply-only contracts forbid check persistence and trusted-contact effects. Concrete artifacts, forwarded messages and mixed unsafe clauses remain risk checks. Final review fixed a working-tree-only whole-message exemption so neutral/physical code context cannot suppress a later banking/login-code request; genuine physical-access codes remain neutral. This is deterministic offline QA, not model training and not 1000 live Telegram chats. No production, Telegram Bot API, database or external-provider call occurred.</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>Review/merge/deploy the local change, then capture the real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix before marking BOT-004 Passed. Inline remains a separate client gate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23935,7 +23950,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D27" s="615" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>Fixed Local</x:v>
       </x:c>
       <x:c r="E27" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23944,26 +23959,26 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
-        <x:v>Deployed</x:v>
+        <x:v>Not Deployed</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J27" s="618" t="n">
-        <x:v>46215</x:v>
+        <x:v>46216</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
       </x:c>
       <x:c r="L27" s="615" t="str">
-        <x:v>Real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
+        <x:v>Review/merge/deploy current local change + real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>The deterministic DSL now covers 13 actions x 3 languages x 6 reviewed surface variants x 8 contexts = 1872 unique rows. All 78 normalized reply-to-bot/typo phrases have exhaustive handler tests forbidding cold checks, session writes and trusted-contact side effects. PR #84 CI 29204994706, Railway be7d6f8d-f06d-459b-b438-ef8924454c4e, polling dispatch and cleanup passed. Broad real-client RU/UZ/EN transcripts remain required.</x:v>
+        <x:v>The deployed 1872-row follow-up DSL remains green. Local evidence adds 1008 RU/UZ/EN context cases; exactly 1000 unique 2/3-turn dialogues (2500 user turns: 620 risk, 930 follow-up, 950 meta/ordinary); 540 everyday two-turn dialogues (1080 user turns, 102 unique follow-ups); and 363 mixed-clause adversarial messages. All 36 already-happened rows use aftercare, 17 benign end-to-end controls stay clean and 33/33 paired direct-danger probes remain detected. Independent conversational/risk review: 2438/2438. Final review fixed a working-tree-only whole-message code-context exemption; 28 focused RU/UZ/EN regressions prove door/entrance, postal, dress and source-code clauses cannot hide a later banking/login-code request while genuine physical-access codes remain neutral. Full suite: 8583/8583 in 134 files, TypeScript, changed-file Prettier, lint 0 errors, build, npm audit 0; global tests deny unmocked network. These are deterministic synthetic cases, not model training or live chats. Local changes are not deployed; broad real-client evidence remains required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
Expand Telegram dialogue QA and clause-local routing (#86)
Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfaf73d77a0554f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Ra04dbe72a96a4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R508f37af59404867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R12e49900df5343a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R00f0f9b68d5144f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R32085d1aaa2c4dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R69d39cd45eef4cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd199101e62144eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R48b3f0dfd7e0416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R34d0fb01804d4a38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd93aeb3768984a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re3db89d978944bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R3b9a361518b14b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2054a321a3d64a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd6df23b0134d4194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R6f6f373b049847fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1202,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1227">
+  <x:cellXfs count="1228">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4304,6 +4304,9 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11014,7 +11017,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11025,7 +11028,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11036,7 +11039,7 @@
         <x:color rgb="FF115E59"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFCCFBF1"/>
         </x:patternFill>
       </x:fill>
@@ -11047,7 +11050,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11058,7 +11061,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11069,7 +11072,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -11080,7 +11083,7 @@
         <x:color rgb="FF4B5563"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
@@ -11091,7 +11094,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11102,7 +11105,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -11113,7 +11116,7 @@
         <x:color rgb="FF115E59"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFCCFBF1"/>
         </x:patternFill>
       </x:fill>
@@ -11124,7 +11127,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11135,7 +11138,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -11146,7 +11149,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -11157,7 +11160,7 @@
         <x:color rgb="FF4B5563"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3F4F6"/>
         </x:patternFill>
       </x:fill>
@@ -11454,8 +11457,8 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="108" customHeight="1">
-      <x:c r="A2" s="1218" t="n">
-        <x:v>46215</x:v>
+      <x:c r="A2" s="1227" t="n">
+        <x:v>46216</x:v>
       </x:c>
       <x:c r="B2" s="1219" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
@@ -11466,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>All 15 validated findings are fixed in code. Fourteen are deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 and remain Deployed / Awaiting Live Verification; SEC-2026-0712-008 remains In Progress until the production Supabase migration is authorized, applied and read back. Automated release gates, the 1872-row bot corpus and production smokes are green. Next: real-client RU/UZ/EN + Inline evidence, authorized data drills, legal approval and a 72-hour canary.</x:v>
+        <x:v>Review, merge and deploy the local BOT-004 conversational-perimeter change, then capture real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot evidence. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Evidence: 4867/4867 tests; coverage 82.85/76.99/89.29/84.71; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CodeQL; Gitleaks; Trivy 0 fixed High/Critical; CycloneDX 1.6 SBOM; 28 migrations; pgTAP 38/38; schema lint; CI 29204994706/29204994736; Railway be7d6f8d-f06d-459b-b438-ef8924454c4e; app/polling/Inline-boundary/dialogue smokes with cleanup; monitor 29205158630. Count-only admin preflight: Auth 1, admins 1, eligible 1, stale 0, missing 0.</x:v>
+        <x:v>Local 2026-07-13 evidence: 8583/8583 tests in 134 files with global unmocked-network denial; 1008 RU/UZ/EN context cases; exactly 1000 synthetic multi-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause adversarial messages; independent conversational/risk review 2438/2438; 17 benign end-to-end controls and 33/33 paired direct-danger probes; TypeScript; changed-file Prettier; lint 0 errors/8 existing warnings; production build; npm audit 0. Final review found and fixed a working-tree-only whole-message exemption: door/entrance, postal, dress and source-code clauses can no longer hide a later banking/login-code request; 28 focused RU/UZ/EN regressions pass and genuine physical-access codes remain neutral. The screenshot phrase asks for the actual link instead of starting an empty check. No AI provider, Telegram, database or production call was made by this QA. This is deterministic testing, not model training or live-client evidence; prior deployed release/security evidence remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -12092,10 +12095,8 @@
           <x:t xml:space="preserve">Commands/callbacks/scenarios win first; meta questions route to safe explanatory copy; scam-context override still checks risky input.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/lib/telegram/meta-intent.ts; src/lib/telegram/router.ts; src/lib/telegram/bot-i18n.ts</x:t>
-        </x:is>
+      <x:c r="F5" s="8" t="str">
+        <x:v>src/lib/meta-intent.ts; src/lib/telegram/conversation-wrapper.ts; src/lib/telegram/router.ts; src/lib/telegram/bot-i18n.ts</x:v>
       </x:c>
       <x:c r="G5" s="8" t="inlineStr">
         <x:is>
@@ -12107,25 +12108,19 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit/property tests</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Add broader conversational layer for questions about the last check.</x:t>
-        </x:is>
+      <x:c r="I5" s="8" t="str">
+        <x:v>Unit/property/router integration; 1008 offline RU/UZ/EN context cases; 1000 unique multi-turn dialogues / 2500 user turns; 540 everyday dialogues / 1080 turns / 102 follow-ups; 363 mixed-clause cases; independent 2438/2438; 28 clause-local code-context regressions; full suite 8583/8583 on 2026-07-13</x:v>
+      </x:c>
+      <x:c r="J5" s="8" t="str">
+        <x:v>Local change fixes the observed empty-check phrase and adds bounded greeting/off-topic/capability routing. Review/merge/deploy and real Telegram Desktop/Android/iOS RU/UZ/EN evidence remain required.</x:v>
       </x:c>
       <x:c r="K5" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P2</x:t>
         </x:is>
       </x:c>
-      <x:c r="L5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Answers must not reveal system prompts or internal scoring thresholds beyond approved language.</x:t>
-        </x:is>
+      <x:c r="L5" s="8" t="str">
+        <x:v>Reply-only meta contracts forbid persistence and trusted-contact effects. Concrete artifacts/forwarded content and mixed unsafe clauses bypass meta routing. Door/entrance, postal, dress and source-code exceptions are clause-local and cannot suppress a later banking/login-code request. Global Vitest and corpus guards deny unmocked network access. Verified locally 2026-07-13; the affected helpers were never deployed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12169,25 +12164,19 @@
           <x:t xml:space="preserve">Implemented</x:t>
         </x:is>
       </x:c>
-      <x:c r="I6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unit tests + live production smoke</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RU/UZ/EN acknowledgement and confirmation-request follow-ups passed live smoke; extend phrase list only from real transcripts.</x:t>
-        </x:is>
+      <x:c r="I6" s="8" t="str">
+        <x:v>Unit/integration plus context, multi-turn and everyday corpora; actual production-derived last-check snapshots; 17 benign end-to-end controls; 33/33 direct-danger probes; recent-result methodology/fresh-domain separation; full suite 8583/8583 on 2026-07-13</x:v>
+      </x:c>
+      <x:c r="J6" s="8" t="str">
+        <x:v>Saved provenance now wins for short or wrapped methodology questions; a new concrete domain remains a fresh check. Real-client RU/UZ/EN reply/restart/language matrix is still open.</x:v>
       </x:c>
       <x:c r="K6" s="12" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P1</x:t>
         </x:is>
       </x:c>
-      <x:c r="L6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-30: TG-005 implemented/verified. Last-check follow-ups cover confidence, next steps, contacts, explanations, and AI-origin questions; orphan follow-ups get safe guidance; stale/panic contexts are guarded; fresh URL/phone/username/payment/APK/secret-code payloads bypass follow-up routing and go through the risk pipeline. Added regression for Uzbek SMS kod and English verification-code follow-ups. 2026-06-30: .claude QA feedback rechecked in focused suite: acknowledgement replies, confirmation-request follow-ups and word-boundary voice transcript previews are covered; `npm run test:run -- src/lib/telegram/webhook.integration.test.ts src/lib/telegram/handlers/check.followup-routing.test.ts src/lib/telegram/handlers/check.voice.test.ts src/lib/telegram/check-followup.test.ts` passed 4 files / 127 tests. 2026-06-30 production pass: prod:telegram-user-story-smoke verified thanks/confirmation follow-ups after a last delivery check did not create checks in RU/UZ/EN sessions.</x:t>
-        </x:is>
+      <x:c r="L6" s="8" t="str">
+        <x:v>Follow-ups use production-bounded stored reasons/levels, explain visible evidence and limitations, never claim an unperformed recheck, and create no check/contact side effects. Verified locally with network blocked on 2026-07-13.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -22803,6 +22792,32 @@
       </x:c>
       <x:c r="H98" t="str">
         <x:v>Execute the external/live gates in order: real clients; authorized Supabase apply; isolated restore/rotation; 60-minute soak; legal approval; freeze RC and complete 144 canary observations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>QA-HUMAN-DIALOGUE-OFFLINE-2026-07-13</x:v>
+      </x:c>
+      <x:c r="B99" s="1097" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>Offline RU/UZ/EN human-style conversational perimeter and observed Telegram phrase regression</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>npm run test:run with global unmocked-network denial; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; changed-file Prettier; corpus hard fetch guards; independent conversational/risk review</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>Passed: 134 files / 8583 tests; 1008 context utterances; exactly 1000 unique 2/3-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause messages; independent 2438/2438; 17 benign controls; 33/33 direct-danger probes; 28 clause-local code-context regressions; actual production-derived follow-up snapshots; screenshot link-capability phrase asks for the real link; 0 AI/provider/Telegram calls.</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>BOT-004, TG-004, TG-005</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Reply-only contracts forbid check persistence and trusted-contact effects. Concrete artifacts, forwarded messages and mixed unsafe clauses remain risk checks. Final review fixed a working-tree-only whole-message exemption so neutral/physical code context cannot suppress a later banking/login-code request; genuine physical-access codes remain neutral. This is deterministic offline QA, not model training and not 1000 live Telegram chats. No production, Telegram Bot API, database or external-provider call occurred.</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>Review/merge/deploy the local change, then capture the real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix before marking BOT-004 Passed. Inline remains a separate client gate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23935,7 +23950,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D27" s="615" t="str">
-        <x:v>Implemented</x:v>
+        <x:v>Fixed Local</x:v>
       </x:c>
       <x:c r="E27" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23944,26 +23959,26 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
-        <x:v>Deployed</x:v>
+        <x:v>Not Deployed</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J27" s="618" t="n">
-        <x:v>46215</x:v>
+        <x:v>46216</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
       </x:c>
       <x:c r="L27" s="615" t="str">
-        <x:v>Real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
+        <x:v>Review/merge/deploy current local change + real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>The deterministic DSL now covers 13 actions x 3 languages x 6 reviewed surface variants x 8 contexts = 1872 unique rows. All 78 normalized reply-to-bot/typo phrases have exhaustive handler tests forbidding cold checks, session writes and trusted-contact side effects. PR #84 CI 29204994706, Railway be7d6f8d-f06d-459b-b438-ef8924454c4e, polling dispatch and cleanup passed. Broad real-client RU/UZ/EN transcripts remain required.</x:v>
+        <x:v>The deployed 1872-row follow-up DSL remains green. Local evidence adds 1008 RU/UZ/EN context cases; exactly 1000 unique 2/3-turn dialogues (2500 user turns: 620 risk, 930 follow-up, 950 meta/ordinary); 540 everyday two-turn dialogues (1080 user turns, 102 unique follow-ups); and 363 mixed-clause adversarial messages. All 36 already-happened rows use aftercare, 17 benign end-to-end controls stay clean and 33/33 paired direct-danger probes remain detected. Independent conversational/risk review: 2438/2438. Final review fixed a working-tree-only whole-message code-context exemption; 28 focused RU/UZ/EN regressions prove door/entrance, postal, dress and source-code clauses cannot hide a later banking/login-code request while genuine physical-access codes remain neutral. Full suite: 8583/8583 in 134 files, TypeScript, changed-file Prettier, lint 0 errors, build, npm audit 0; global tests deny unmocked network. These are deterministic synthetic cases, not model training or live chats. Local changes are not deployed; broad real-client evidence remains required.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
Record deployed dialogue QA evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R48b3f0dfd7e0416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R34d0fb01804d4a38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd93aeb3768984a73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re3db89d978944bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R3b9a361518b14b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2054a321a3d64a4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd6df23b0134d4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R6f6f373b049847fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R626d1b21ba17415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3e1729ab9e644f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae736bed545d450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R74b9742c358a473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0eaf8d162f7b4e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7a01d4712b0242eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R47c840ee1609445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0d343a26d47a4c99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11469,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Review, merge and deploy the local BOT-004 conversational-perimeter change, then capture real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot evidence. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
+        <x:v>Capture real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence evidence for BOT-004. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Local 2026-07-13 evidence: 8583/8583 tests in 134 files with global unmocked-network denial; 1008 RU/UZ/EN context cases; exactly 1000 synthetic multi-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause adversarial messages; independent conversational/risk review 2438/2438; 17 benign end-to-end controls and 33/33 paired direct-danger probes; TypeScript; changed-file Prettier; lint 0 errors/8 existing warnings; production build; npm audit 0. Final review found and fixed a working-tree-only whole-message exemption: door/entrance, postal, dress and source-code clauses can no longer hide a later banking/login-code request; 28 focused RU/UZ/EN regressions pass and genuine physical-access codes remain neutral. The screenshot phrase asks for the actual link instead of starting an empty check. No AI provider, Telegram, database or production call was made by this QA. This is deterministic testing, not model training or live-client evidence; prior deployed release/security evidence remains unchanged.</x:v>
+        <x:v>2026-07-13 evidence: PR #86 deployed the deterministic RU/UZ/EN conversational perimeter; PR #87 deployed corrected high-risk confidence copy that separates an organization callback through an official channel/number from calling a known person on a previously saved number. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. Full suite 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; production build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM, migrations/schema/pgTAP passed. Production app/health, polling leader, queue, getMe, AI provider and RLS/security smokes passed. The bounded polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, then deleted its Bot API replies and synthetic DB rows. The 540 everyday dialogues, 1000 synthetic dialogues and 363 mixed-clause cases remain offline deterministic QA, not model training or live-client evidence. Broad Telegram Desktop/Android/iOS RU/UZ/EN and real-client Inline acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -12109,10 +12109,10 @@
         </x:is>
       </x:c>
       <x:c r="I5" s="8" t="str">
-        <x:v>Unit/property/router integration; 1008 offline RU/UZ/EN context cases; 1000 unique multi-turn dialogues / 2500 user turns; 540 everyday dialogues / 1080 turns / 102 follow-ups; 363 mixed-clause cases; independent 2438/2438; 28 clause-local code-context regressions; full suite 8583/8583 on 2026-07-13</x:v>
+        <x:v>Unit/property/router integration; 1008 offline RU/UZ/EN context cases; 1000 unique multi-turn dialogues / 2500 user turns; 540 everyday dialogues / 1080 turns / 102 follow-ups; 363 mixed-clause cases; independent 2438/2438; 28 clause-local code-context regressions; full suite 8584/8584; PR #86 deployed on 2026-07-13</x:v>
       </x:c>
       <x:c r="J5" s="8" t="str">
-        <x:v>Local change fixes the observed empty-check phrase and adds bounded greeting/off-topic/capability routing. Review/merge/deploy and real Telegram Desktop/Android/iOS RU/UZ/EN evidence remain required.</x:v>
+        <x:v>Implementation is deployed. Capture the real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix; keep Inline as a separate client gate.</x:v>
       </x:c>
       <x:c r="K5" s="13" t="inlineStr">
         <x:is>
@@ -12120,7 +12120,7 @@
         </x:is>
       </x:c>
       <x:c r="L5" s="8" t="str">
-        <x:v>Reply-only meta contracts forbid persistence and trusted-contact effects. Concrete artifacts/forwarded content and mixed unsafe clauses bypass meta routing. Door/entrance, postal, dress and source-code exceptions are clause-local and cannot suppress a later banking/login-code request. Global Vitest and corpus guards deny unmocked network access. Verified locally 2026-07-13; the affected helpers were never deployed.</x:v>
+        <x:v>Reply-only meta contracts forbid persistence and trusted-contact effects. Concrete artifacts/forwarded content and mixed unsafe clauses bypass meta routing. Door/entrance, postal, dress and source-code exceptions are clause-local and cannot suppress a later banking/login-code request. Global Vitest and corpus guards deny unmocked network access. PR #86 is deployed; exact production SHA 5ceb9eaa includes the PR #87 confidence-copy correction. Production polling-dispatch cleanup read-back passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12165,7 +12165,7 @@
         </x:is>
       </x:c>
       <x:c r="I6" s="8" t="str">
-        <x:v>Unit/integration plus context, multi-turn and everyday corpora; actual production-derived last-check snapshots; 17 benign end-to-end controls; 33/33 direct-danger probes; recent-result methodology/fresh-domain separation; full suite 8583/8583 on 2026-07-13</x:v>
+        <x:v>Unit/integration plus context, multi-turn and everyday corpora; actual production-derived last-check snapshots; 17 benign end-to-end controls; 33/33 direct-danger probes; recent-result methodology/fresh-domain separation; full suite 8584/8584; production polling-dispatch confidence/methodology/action flows passed on 2026-07-13</x:v>
       </x:c>
       <x:c r="J6" s="8" t="str">
         <x:v>Saved provenance now wins for short or wrapped methodology questions; a new concrete domain remains a fresh check. Real-client RU/UZ/EN reply/restart/language matrix is still open.</x:v>
@@ -12176,7 +12176,7 @@
         </x:is>
       </x:c>
       <x:c r="L6" s="8" t="str">
-        <x:v>Follow-ups use production-bounded stored reasons/levels, explain visible evidence and limitations, never claim an unperformed recheck, and create no check/contact side effects. Verified locally with network blocked on 2026-07-13.</x:v>
+        <x:v>Follow-ups use retained reasons/levels, explain visible evidence and limitations, never claim an unperformed recheck, and create no check/contact side effects. PR #87 distinguishes official organization callbacks from saved-number callbacks for known people in RU/UZ/EN. Deployed at 5ceb9eaa; bounded production dispatch and cleanup read-back passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -22808,7 +22808,7 @@
         <x:v>npm run test:run with global unmocked-network denial; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; changed-file Prettier; corpus hard fetch guards; independent conversational/risk review</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Passed: 134 files / 8583 tests; 1008 context utterances; exactly 1000 unique 2/3-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause messages; independent 2438/2438; 17 benign controls; 33/33 direct-danger probes; 28 clause-local code-context regressions; actual production-derived follow-up snapshots; screenshot link-capability phrase asks for the real link; 0 AI/provider/Telegram calls.</x:v>
+        <x:v>Passed offline: 134 files / 8583 tests before production follow-up correction; 1008 context utterances; exactly 1000 unique 2/3-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause messages; independent 2438/2438; 17 benign controls; 33/33 direct-danger probes; 28 clause-local code-context regressions; actual production-derived follow-up snapshots; screenshot link-capability phrase asks for the real link; 0 AI/provider/Telegram calls in this offline run.</x:v>
       </x:c>
       <x:c r="F99" t="str">
         <x:v>BOT-004, TG-004, TG-005</x:v>
@@ -22817,7 +22817,33 @@
         <x:v>Reply-only contracts forbid check persistence and trusted-contact effects. Concrete artifacts, forwarded messages and mixed unsafe clauses remain risk checks. Final review fixed a working-tree-only whole-message exemption so neutral/physical code context cannot suppress a later banking/login-code request; genuine physical-access codes remain neutral. This is deterministic offline QA, not model training and not 1000 live Telegram chats. No production, Telegram Bot API, database or external-provider call occurred.</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>Review/merge/deploy the local change, then capture the real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix before marking BOT-004 Passed. Inline remains a separate client gate.</x:v>
+        <x:v>Promoted through PR #86 and production-corrected through PR #87; see QA-HUMAN-DIALOGUE-PROD-2026-07-13. Remaining gate is real Telegram Desktop/Android/iOS RU/UZ/EN acceptance; Inline remains separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>QA-HUMAN-DIALOGUE-PROD-2026-07-13</x:v>
+      </x:c>
+      <x:c r="B100" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>Deployed human-dialogue perimeter and bounded production Telegram follow-up verification</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>PR #86 / f5e86cb; PR #87 / 5ceb9eaa; GitHub CI 29251154053 and security 29251154008; Railway deployment 8c76285e; prod:smoke; monitor:prod; prod:security-smoke; prod:telegram-polling-dispatch-smoke</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>Passed: exact SHA 5ceb9eaa deployed; 8584/8584 tests; CI/security/database gates green; home/health 200; polling leader healthy; queue 0; getMe and AI provider 200; RLS/security smoke passed; confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows passed; Bot API replies and synthetic DB rows cleaned up.</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>BOT-004, TG-004, TG-005</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>The first bounded production run exposed missing official-callback wording; PR #87 fixed and deployed it in RU/UZ/EN. A stale domain-methodology smoke expectation was aligned to the already-tested retained-provenance contract without weakening evidence/limitation checks. The final harness acquired no polling lease, allowed replies only to TELEGRAM_QA_CHAT_ID and completed cleanup read-back.</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>Capture real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence evidence before marking BOT-004 Passed. Inline rendering/insertion remains a separate real-client gate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23950,7 +23976,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D27" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E27" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23959,10 +23985,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
         <x:v>In Progress</x:v>
@@ -23974,11 +24000,11 @@
         <x:v>QA Automation</x:v>
       </x:c>
       <x:c r="L27" s="615" t="str">
-        <x:v>Review/merge/deploy current local change + real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
+        <x:v>Real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix</x:v>
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>The deployed 1872-row follow-up DSL remains green. Local evidence adds 1008 RU/UZ/EN context cases; exactly 1000 unique 2/3-turn dialogues (2500 user turns: 620 risk, 930 follow-up, 950 meta/ordinary); 540 everyday two-turn dialogues (1080 user turns, 102 unique follow-ups); and 363 mixed-clause adversarial messages. All 36 already-happened rows use aftercare, 17 benign end-to-end controls stay clean and 33/33 paired direct-danger probes remain detected. Independent conversational/risk review: 2438/2438. Final review fixed a working-tree-only whole-message code-context exemption; 28 focused RU/UZ/EN regressions prove door/entrance, postal, dress and source-code clauses cannot hide a later banking/login-code request while genuine physical-access codes remain neutral. Full suite: 8583/8583 in 134 files, TypeScript, changed-file Prettier, lint 0 errors, build, npm audit 0; global tests deny unmocked network. These are deterministic synthetic cases, not model training or live chats. Local changes are not deployed; broad real-client evidence remains required.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
Record deployed dialogue QA evidence (#88)
Co-authored-by: Web-pixel-creator <190506225+Web-pixel-creator@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R48b3f0dfd7e0416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R34d0fb01804d4a38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rd93aeb3768984a73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Re3db89d978944bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R3b9a361518b14b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2054a321a3d64a4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rd6df23b0134d4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R6f6f373b049847fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R626d1b21ba17415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3e1729ab9e644f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae736bed545d450f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R74b9742c358a473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0eaf8d162f7b4e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7a01d4712b0242eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R47c840ee1609445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0d343a26d47a4c99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11469,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Review, merge and deploy the local BOT-004 conversational-perimeter change, then capture real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot evidence. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
+        <x:v>Capture real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence evidence for BOT-004. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>Local 2026-07-13 evidence: 8583/8583 tests in 134 files with global unmocked-network denial; 1008 RU/UZ/EN context cases; exactly 1000 synthetic multi-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause adversarial messages; independent conversational/risk review 2438/2438; 17 benign end-to-end controls and 33/33 paired direct-danger probes; TypeScript; changed-file Prettier; lint 0 errors/8 existing warnings; production build; npm audit 0. Final review found and fixed a working-tree-only whole-message exemption: door/entrance, postal, dress and source-code clauses can no longer hide a later banking/login-code request; 28 focused RU/UZ/EN regressions pass and genuine physical-access codes remain neutral. The screenshot phrase asks for the actual link instead of starting an empty check. No AI provider, Telegram, database or production call was made by this QA. This is deterministic testing, not model training or live-client evidence; prior deployed release/security evidence remains unchanged.</x:v>
+        <x:v>2026-07-13 evidence: PR #86 deployed the deterministic RU/UZ/EN conversational perimeter; PR #87 deployed corrected high-risk confidence copy that separates an organization callback through an official channel/number from calling a known person on a previously saved number. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. Full suite 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; production build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM, migrations/schema/pgTAP passed. Production app/health, polling leader, queue, getMe, AI provider and RLS/security smokes passed. The bounded polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, then deleted its Bot API replies and synthetic DB rows. The 540 everyday dialogues, 1000 synthetic dialogues and 363 mixed-clause cases remain offline deterministic QA, not model training or live-client evidence. Broad Telegram Desktop/Android/iOS RU/UZ/EN and real-client Inline acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -12109,10 +12109,10 @@
         </x:is>
       </x:c>
       <x:c r="I5" s="8" t="str">
-        <x:v>Unit/property/router integration; 1008 offline RU/UZ/EN context cases; 1000 unique multi-turn dialogues / 2500 user turns; 540 everyday dialogues / 1080 turns / 102 follow-ups; 363 mixed-clause cases; independent 2438/2438; 28 clause-local code-context regressions; full suite 8583/8583 on 2026-07-13</x:v>
+        <x:v>Unit/property/router integration; 1008 offline RU/UZ/EN context cases; 1000 unique multi-turn dialogues / 2500 user turns; 540 everyday dialogues / 1080 turns / 102 follow-ups; 363 mixed-clause cases; independent 2438/2438; 28 clause-local code-context regressions; full suite 8584/8584; PR #86 deployed on 2026-07-13</x:v>
       </x:c>
       <x:c r="J5" s="8" t="str">
-        <x:v>Local change fixes the observed empty-check phrase and adds bounded greeting/off-topic/capability routing. Review/merge/deploy and real Telegram Desktop/Android/iOS RU/UZ/EN evidence remain required.</x:v>
+        <x:v>Implementation is deployed. Capture the real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix; keep Inline as a separate client gate.</x:v>
       </x:c>
       <x:c r="K5" s="13" t="inlineStr">
         <x:is>
@@ -12120,7 +12120,7 @@
         </x:is>
       </x:c>
       <x:c r="L5" s="8" t="str">
-        <x:v>Reply-only meta contracts forbid persistence and trusted-contact effects. Concrete artifacts/forwarded content and mixed unsafe clauses bypass meta routing. Door/entrance, postal, dress and source-code exceptions are clause-local and cannot suppress a later banking/login-code request. Global Vitest and corpus guards deny unmocked network access. Verified locally 2026-07-13; the affected helpers were never deployed.</x:v>
+        <x:v>Reply-only meta contracts forbid persistence and trusted-contact effects. Concrete artifacts/forwarded content and mixed unsafe clauses bypass meta routing. Door/entrance, postal, dress and source-code exceptions are clause-local and cannot suppress a later banking/login-code request. Global Vitest and corpus guards deny unmocked network access. PR #86 is deployed; exact production SHA 5ceb9eaa includes the PR #87 confidence-copy correction. Production polling-dispatch cleanup read-back passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12165,7 +12165,7 @@
         </x:is>
       </x:c>
       <x:c r="I6" s="8" t="str">
-        <x:v>Unit/integration plus context, multi-turn and everyday corpora; actual production-derived last-check snapshots; 17 benign end-to-end controls; 33/33 direct-danger probes; recent-result methodology/fresh-domain separation; full suite 8583/8583 on 2026-07-13</x:v>
+        <x:v>Unit/integration plus context, multi-turn and everyday corpora; actual production-derived last-check snapshots; 17 benign end-to-end controls; 33/33 direct-danger probes; recent-result methodology/fresh-domain separation; full suite 8584/8584; production polling-dispatch confidence/methodology/action flows passed on 2026-07-13</x:v>
       </x:c>
       <x:c r="J6" s="8" t="str">
         <x:v>Saved provenance now wins for short or wrapped methodology questions; a new concrete domain remains a fresh check. Real-client RU/UZ/EN reply/restart/language matrix is still open.</x:v>
@@ -12176,7 +12176,7 @@
         </x:is>
       </x:c>
       <x:c r="L6" s="8" t="str">
-        <x:v>Follow-ups use production-bounded stored reasons/levels, explain visible evidence and limitations, never claim an unperformed recheck, and create no check/contact side effects. Verified locally with network blocked on 2026-07-13.</x:v>
+        <x:v>Follow-ups use retained reasons/levels, explain visible evidence and limitations, never claim an unperformed recheck, and create no check/contact side effects. PR #87 distinguishes official organization callbacks from saved-number callbacks for known people in RU/UZ/EN. Deployed at 5ceb9eaa; bounded production dispatch and cleanup read-back passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -22808,7 +22808,7 @@
         <x:v>npm run test:run with global unmocked-network denial; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=low; changed-file Prettier; corpus hard fetch guards; independent conversational/risk review</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>Passed: 134 files / 8583 tests; 1008 context utterances; exactly 1000 unique 2/3-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause messages; independent 2438/2438; 17 benign controls; 33/33 direct-danger probes; 28 clause-local code-context regressions; actual production-derived follow-up snapshots; screenshot link-capability phrase asks for the real link; 0 AI/provider/Telegram calls.</x:v>
+        <x:v>Passed offline: 134 files / 8583 tests before production follow-up correction; 1008 context utterances; exactly 1000 unique 2/3-turn dialogues / 2500 user turns; 540 everyday two-turn dialogues / 1080 user turns / 102 unique follow-ups; 363 mixed-clause messages; independent 2438/2438; 17 benign controls; 33/33 direct-danger probes; 28 clause-local code-context regressions; actual production-derived follow-up snapshots; screenshot link-capability phrase asks for the real link; 0 AI/provider/Telegram calls in this offline run.</x:v>
       </x:c>
       <x:c r="F99" t="str">
         <x:v>BOT-004, TG-004, TG-005</x:v>
@@ -22817,7 +22817,33 @@
         <x:v>Reply-only contracts forbid check persistence and trusted-contact effects. Concrete artifacts, forwarded messages and mixed unsafe clauses remain risk checks. Final review fixed a working-tree-only whole-message exemption so neutral/physical code context cannot suppress a later banking/login-code request; genuine physical-access codes remain neutral. This is deterministic offline QA, not model training and not 1000 live Telegram chats. No production, Telegram Bot API, database or external-provider call occurred.</x:v>
       </x:c>
       <x:c r="H99" t="str">
-        <x:v>Review/merge/deploy the local change, then capture the real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix before marking BOT-004 Passed. Inline remains a separate client gate.</x:v>
+        <x:v>Promoted through PR #86 and production-corrected through PR #87; see QA-HUMAN-DIALOGUE-PROD-2026-07-13. Remaining gate is real Telegram Desktop/Android/iOS RU/UZ/EN acceptance; Inline remains separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>QA-HUMAN-DIALOGUE-PROD-2026-07-13</x:v>
+      </x:c>
+      <x:c r="B100" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>Deployed human-dialogue perimeter and bounded production Telegram follow-up verification</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>PR #86 / f5e86cb; PR #87 / 5ceb9eaa; GitHub CI 29251154053 and security 29251154008; Railway deployment 8c76285e; prod:smoke; monitor:prod; prod:security-smoke; prod:telegram-polling-dispatch-smoke</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>Passed: exact SHA 5ceb9eaa deployed; 8584/8584 tests; CI/security/database gates green; home/health 200; polling leader healthy; queue 0; getMe and AI provider 200; RLS/security smoke passed; confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows passed; Bot API replies and synthetic DB rows cleaned up.</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>BOT-004, TG-004, TG-005</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>The first bounded production run exposed missing official-callback wording; PR #87 fixed and deployed it in RU/UZ/EN. A stale domain-methodology smoke expectation was aligned to the already-tested retained-provenance contract without weakening evidence/limitation checks. The final harness acquired no polling lease, allowed replies only to TELEGRAM_QA_CHAT_ID and completed cleanup read-back.</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>Capture real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence evidence before marking BOT-004 Passed. Inline rendering/insertion remains a separate real-client gate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23950,7 +23976,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D27" s="615" t="str">
-        <x:v>Fixed Local</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E27" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23959,10 +23985,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="G27" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H27" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I27" s="615" t="str">
         <x:v>In Progress</x:v>
@@ -23974,11 +24000,11 @@
         <x:v>QA Automation</x:v>
       </x:c>
       <x:c r="L27" s="615" t="str">
-        <x:v>Review/merge/deploy current local change + real Telegram Desktop/Android/iOS RU/UZ/EN reply-to-bot matrix</x:v>
+        <x:v>Real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence matrix</x:v>
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>The deployed 1872-row follow-up DSL remains green. Local evidence adds 1008 RU/UZ/EN context cases; exactly 1000 unique 2/3-turn dialogues (2500 user turns: 620 risk, 930 follow-up, 950 meta/ordinary); 540 everyday two-turn dialogues (1080 user turns, 102 unique follow-ups); and 363 mixed-clause adversarial messages. All 36 already-happened rows use aftercare, 17 benign end-to-end controls stay clean and 33/33 paired direct-danger probes remain detected. Independent conversational/risk review: 2438/2438. Final review fixed a working-tree-only whole-message code-context exemption; 28 focused RU/UZ/EN regressions prove door/entrance, postal, dress and source-code clauses cannot hide a later banking/login-code request while genuine physical-access codes remain neutral. Full suite: 8583/8583 in 134 files, TypeScript, changed-file Prettier, lint 0 errors, build, npm audit 0; global tests deny unmocked network. These are deterministic synthetic cases, not model training or live chats. Local changes are not deployed; broad real-client evidence remains required.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
Fix production QR worker runtime
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R626d1b21ba17415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R3e1729ab9e644f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rae736bed545d450f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R74b9742c358a473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R0eaf8d162f7b4e02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R7a01d4712b0242eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R47c840ee1609445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0d343a26d47a4c99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfbc02b4bfa9e4ce8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2e9ecf01420048b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R89a8c5e7fd694d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra108761b51a94ede"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R4cc1724e63a544ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2b4789c196a348a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra0fe6c34417f4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R14225d14208f49ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11458,7 +11458,7 @@
     </x:row>
     <x:row r="2" ht="108" customHeight="1">
       <x:c r="A2" s="1227" t="n">
-        <x:v>46216</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="B2" s="1219" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
@@ -11469,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Capture real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence evidence for BOT-004. Keep Inline real-client rendering/insertion, authorized data drills, legal approval and the 72-hour canary as separate open gates.</x:v>
+        <x:v>Complete the physical Railway restart/polling-leader re-election with one approved QA update, then run the legitimate QR-worker corpus/crash-restart profile. Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, legal approval and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-13 evidence: PR #86 deployed the deterministic RU/UZ/EN conversational perimeter; PR #87 deployed corrected high-risk confidence copy that separates an organization callback through an official channel/number from calling a known person on a previously saved number. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. Full suite 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; production build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM, migrations/schema/pgTAP passed. Production app/health, polling leader, queue, getMe, AI provider and RLS/security smokes passed. The bounded polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, then deleted its Bot API replies and synthetic DB rows. The 540 everyday dialogues, 1000 synthetic dialogues and 363 mixed-clause cases remain offline deterministic QA, not model training or live-client evidence. Broad Telegram Desktop/Android/iOS RU/UZ/EN and real-client Inline acceptance remain open.</x:v>
+        <x:v>2026-07-14 evidence: PR #89 deployed exact main 868eb18d as Railway 24b9cb4a. The uninterrupted 60-minute in-container polling/resource soak passed 36,000/36,000 with zero lost updates/duplicate modeled effects, max queue 35, max RSS 101.41 MiB, event-loop p99 21.84 ms and update-latency p99 2.57 ms. The runner made no Telegram, Supabase, AI/reputation call or persistent write; production remained 200 ok after cleanup. RES-004 advances to In Progress, not Passed: a physical Railway restart/leader re-election and the dedicated QR-worker corpus/crash-restart profile remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11739,7 +11739,7 @@
       </x:c>
       <x:c r="B23" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A23)</x:f>
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C23" s="629" t="str">
         <x:v>Required evidence or work is missing.</x:v>
@@ -11753,7 +11753,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -22846,6 +22846,32 @@
         <x:v>Capture real Telegram Desktop/Android/iOS RU/UZ/EN reply, typo, new-object, restart and language-persistence evidence before marking BOT-004 Passed. Inline rendering/insertion remains a separate real-client gate.</x:v>
       </x:c>
     </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>QA-POLLING-RESOURCE-SOAK-PROD-2026-07-14</x:v>
+      </x:c>
+      <x:c r="B101" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>60-minute production-image polling/resource soak</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>PR #89 / exact main 868eb18d410f2616030a92b410a36b6bc3784c4e; Railway deployment 24b9cb4a-aefe-4807-9d2b-84fc6f931f3b; node dist/ops/polling-resource-soak.mjs --duration-minutes=60; public /healthz before and after</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>Passed: SOAK_FINAL.passed=true; 36,000/36,000 completed/effects; lost=0; duplicates=0; retries=3; max queue=35; final/max RSS=98.00/101.41 MiB; event-loop p99/max=21.84/41.45 ms; update latency p95/p99/max=1.13/2.57/3314.39 ms; 180/180 media-admission fixtures accepted.</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>RES-004</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Controlled updates and media buffers remained inside the runner. No Telegram, Supabase, AI/reputation-provider request, user data or synthetic persistence. Stale-leader rejection, process-offset loss replay, pre-effect failure and acknowledgement-loss recovery passed. The isolated tmux session was deleted; production health remained 200 ok.</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>Run an approved physical Railway restart/leader re-election with one real QA update and prove no duplicate reply. Separately run the legitimate QR corpus and QR-worker crash/restart resource profile; this soak did not execute QR decoding.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -23732,7 +23758,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="D21" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="E21" s="615" t="str">
         <x:v>Passed</x:v>
@@ -23744,25 +23770,25 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H21" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I21" s="615" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J21" s="618" t="n">
-        <x:v>46213</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="K21" s="615" t="str">
         <x:v>QA / Platform</x:v>
       </x:c>
       <x:c r="L21" s="615" t="str">
-        <x:v>Railway deploy + 60-minute soak/crash-restart run</x:v>
+        <x:v>Actual Railway restart/leader re-election with one approved QA update; legitimate QR-worker corpus and crash/restart profile</x:v>
       </x:c>
       <x:c r="M21" s="615" t="str">
         <x:v>RES-001..003</x:v>
       </x:c>
       <x:c r="N21" s="615" t="str">
-        <x:v>Local four-job 3.6 MP burst completed in 91 ms with about 11 ms max event-loop lag; production soak remains.</x:v>
+        <x:v>PR #89 / exact main 868eb18d deployed as Railway 24b9cb4a. Uninterrupted in-container soak passed: 36,000/36,000 completed, zero lost updates or duplicate modeled effects, final/max queue 0/35, final/max RSS 98.00/101.41 MiB, event-loop p99 21.84 ms, update-latency p99 2.57 ms, retries 3. Stale-leader rejection, process-offset replay, pre-effect failure and acknowledgement-loss recovery passed. No Telegram, Supabase, AI/reputation provider call or persistence. This runner admits large media data URLs but does not execute QR decode or physically restart the Railway instance.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">

</xml_diff>

<commit_message>
Record production QR runtime evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rfbc02b4bfa9e4ce8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R2e9ecf01420048b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R89a8c5e7fd694d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra108761b51a94ede"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R4cc1724e63a544ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2b4789c196a348a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Ra0fe6c34417f4c78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R14225d14208f49ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9165dbf5cc8d40d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R78e7f083ffcb4e37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R885ba381d8054033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb194947a385d4a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rbd723065841345a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R04c3fa97fda34c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rb6b64bd60c534824"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0882278d53494c1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11469,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Complete the physical Railway restart/polling-leader re-election with one approved QA update, then run the legitimate QR-worker corpus/crash-restart profile. Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, legal approval and the fixed-RC 72-hour canary.</x:v>
+        <x:v>Complete the physical Railway restart/polling-leader re-election with one approved QA update. Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, legal approval and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14 evidence: PR #89 deployed exact main 868eb18d as Railway 24b9cb4a. The uninterrupted 60-minute in-container polling/resource soak passed 36,000/36,000 with zero lost updates/duplicate modeled effects, max queue 35, max RSS 101.41 MiB, event-loop p99 21.84 ms and update-latency p99 2.57 ms. The runner made no Telegram, Supabase, AI/reputation call or persistent write; production remained 200 ok after cleanup. RES-004 advances to In Progress, not Passed: a physical Railway restart/leader re-election and the dedicated QR-worker corpus/crash-restart profile remain.</x:v>
+        <x:v>2026-07-14 evidence: the 60-minute Railway polling/resource soak passed 36,000/36,000 with zero loss/duplicate modeled effects. PR #94 then fixed missing QR decoder packages in the production image; exact main f1ddf349 deployed as Railway 09f984bd / image sha256:abbba9cf. The live module probe and detached 10-minute QR worker profile passed 5,055 cases with zero failures, PNG/JPEG coverage, queue 4/1, forced fail-closed interruption and successful recovery; max RSS 234.60 MiB and event-loop p99 21.04 ms. Post-load production smoke is green. Both isolated runners made no Telegram, Supabase, AI/reputation call or persistent write. RES-001 and RES-002 are Passed. RES-004 remains In Progress only for the approved physical Railway restart/leader re-election with one QA update.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11753,7 +11753,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -11767,7 +11767,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -22872,6 +22872,32 @@
         <x:v>Run an approved physical Railway restart/leader re-election with one real QA update and prove no duplicate reply. Separately run the legitimate QR corpus and QR-worker crash/restart resource profile; this soak did not execute QR decoding.</x:v>
       </x:c>
     </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>QA-QR-WORKER-RESOURCE-SOAK-PROD-2026-07-14</x:v>
+      </x:c>
+      <x:c r="B102" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>10-minute production-image QR worker corpus/resource/crash profile</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>PR #94 / exact main f1ddf3490573e667907beed2a027e468298f954d; Railway deployment 09f984bd-1930-4a2b-a04a-4f4ef46e2058; image sha256:abbba9cf1cb45f7ca4e4e6c5a40a6d78d37ef1c5672aab6def2dbba641a038e5; live require of jsqr/jpeg-js/pngjs; node dist/ops/qr-worker-resource-soak.mjs --duration-minutes=10 --progress-seconds=60; post-load prod:smoke</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>Passed: QR_SOAK_FINAL.passed=true; 5,055 processed; failures=0; PNG=2,087; JPEG=693; expected empty passes=2,274; queue accepted/rejected=4/1; crash observed=true; interrupted job failed closed=true; worker recovery=true; final/max RSS=165.88/234.60 MiB; RSS growth=110.08 MiB; event-loop p99/max=21.04/28.26 ms; decode latency p95/p99/max=50.09/225.53/279.47 ms.</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>RES-001, RES-002, RES-004</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Generated safe/suspicious/text QR, JPEG QR, non-QR, malformed, oversized and high-resolution fixtures remained in the isolated runner. No Telegram, Supabase, AI/reputation-provider call, user data or persistent write. A first direct SSH attempt was transport-interrupted after 360 seconds with 3,002 cases and zero failures; the required full run was repeated in a detached tmux session and passed. The session was deleted and production smoke remained green: home/health 200, webhook 503 in polling mode, pending updates 0, polling leader 200 and AI provider 200.</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>RES-001/RES-002 QR runtime evidence is complete. Keep RES-004 In Progress until an approved physical Railway restart/leader re-election with one QA update proves health, empty pending queue and no duplicate reply.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -23638,29 +23664,27 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F18" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G18" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H18" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I18" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J18" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="K18" s="615" t="str">
         <x:v>Media / Security</x:v>
       </x:c>
-      <x:c r="L18" s="615" t="str">
-        <x:v>Railway deploy + legitimate corpus smoke</x:v>
-      </x:c>
+      <x:c r="L18" s="615"/>
       <x:c r="M18" s="615" t="str"/>
       <x:c r="N18" s="615" t="str">
-        <x:v>4 MiB/4 MP decode cap; 1.5 MP, 5-attempt and 350 ms QR scan budgets; PNG/JPEG QR regressions pass. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
+        <x:v>Production boundary passed 2026-07-14 at exact main f1ddf349 / Railway 09f984bd / image sha256:abbba9cf. Live runtime resolved jsqr/jpeg-js/pngjs. The generated 10-minute corpus exercised PNG/JPEG QR, non-QR, malformed, oversized and high-resolution inputs under the 4 MiB/4 MP, 1.5 MP, five-attempt and 350 ms scan budgets: 5,055 processed, zero failures, PNG 2,087 and JPEG 693; decode p95/p99/max 50.09/225.53/279.47 ms. No external calls or writes.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -23680,29 +23704,27 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F19" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G19" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H19" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I19" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J19" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="K19" s="615" t="str">
         <x:v>Backend / Platform</x:v>
       </x:c>
-      <x:c r="L19" s="615" t="str">
-        <x:v>Railway deploy + runtime CPU/RAM profile</x:v>
-      </x:c>
+      <x:c r="L19" s="615"/>
       <x:c r="M19" s="615" t="str"/>
       <x:c r="N19" s="615" t="str">
-        <x:v>Single isolated worker, four-job total backlog, 900 ms deadline and 128 MiB old-generation cap keep untrusted decode off the Node event loop. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
+        <x:v>Production boundary passed 2026-07-14 at exact main f1ddf349 / Railway 09f984bd / image sha256:abbba9cf. The detached 10-minute worker profile proved one isolated worker with a four-job bound: queue accepted/rejected 4/1, forced in-flight termination observed, interrupted job failed closed and the next QR decoded after worker recreation. Final/max RSS 165.88/234.60 MiB, RSS growth 110.08 MiB, event-loop p99/max 21.04/28.26 ms; zero failures. Post-load production smoke passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -23782,13 +23804,13 @@
         <x:v>QA / Platform</x:v>
       </x:c>
       <x:c r="L21" s="615" t="str">
-        <x:v>Actual Railway restart/leader re-election with one approved QA update; legitimate QR-worker corpus and crash/restart profile</x:v>
+        <x:v>Actual Railway restart/leader re-election with one approved QA update</x:v>
       </x:c>
       <x:c r="M21" s="615" t="str">
         <x:v>RES-001..003</x:v>
       </x:c>
       <x:c r="N21" s="615" t="str">
-        <x:v>PR #89 / exact main 868eb18d deployed as Railway 24b9cb4a. Uninterrupted in-container soak passed: 36,000/36,000 completed, zero lost updates or duplicate modeled effects, final/max queue 0/35, final/max RSS 98.00/101.41 MiB, event-loop p99 21.84 ms, update-latency p99 2.57 ms, retries 3. Stale-leader rejection, process-offset replay, pre-effect failure and acknowledgement-loss recovery passed. No Telegram, Supabase, AI/reputation provider call or persistence. This runner admits large media data URLs but does not execute QR decode or physically restart the Railway instance.</x:v>
+        <x:v>Polling subgate: PR #89 / exact main 868eb18d / Railway 24b9cb4a; uninterrupted 60-minute in-container soak passed 36,000/36,000 with zero lost updates or duplicate modeled effects, max queue 35, max RSS 101.41 MiB, event-loop p99 21.84 ms and update-latency p99 2.57 ms. QR subgate: PR #94 / exact main f1ddf349 / Railway 09f984bd / image sha256:abbba9cf; live module require passed and the detached 10-minute QR worker profile passed 5,055 cases with zero failures, PNG 2,087, JPEG 693, queue 4 accepted/1 rejected, forced interruption fail-closed and worker recovery true, max RSS 234.60 MiB, RSS growth 110.08 MiB, event-loop p99 21.04 ms and decode p99/max 225.53/279.47 ms. Both runners used generated in-memory data and made no Telegram, Supabase, AI/reputation-provider call or persistent write. Production smoke after QR load passed. Only the approved physical Railway restart/leader re-election proof remains; neither runner claims it.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">

</xml_diff>

<commit_message>
Record shared rate-limit production evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9165dbf5cc8d40d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R78e7f083ffcb4e37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R885ba381d8054033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rb194947a385d4a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rbd723065841345a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R04c3fa97fda34c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rb6b64bd60c534824"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R0882278d53494c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb0581c4b8a234f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R6d919cdc2a854dc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8c8355dd3c5641c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R416f1e153493490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re081f16e835d4857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R6844d165763d4723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R23a53582c11440dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R93d55bea6e8247ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11472,7 +11472,7 @@
         <x:v>Complete the physical Railway restart/polling-leader re-election with one approved QA update. Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, legal approval and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14 evidence: the 60-minute Railway polling/resource soak passed 36,000/36,000 with zero loss/duplicate modeled effects. PR #94 then fixed missing QR decoder packages in the production image; exact main f1ddf349 deployed as Railway 09f984bd / image sha256:abbba9cf. The live module probe and detached 10-minute QR worker profile passed 5,055 cases with zero failures, PNG/JPEG coverage, queue 4/1, forced fail-closed interruption and successful recovery; max RSS 234.60 MiB and event-loop p99 21.04 ms. Post-load production smoke is green. Both isolated runners made no Telegram, Supabase, AI/reputation call or persistent write. RES-001 and RES-002 are Passed. RES-004 remains In Progress only for the approved physical Railway restart/leader re-election with one QA update.</x:v>
+        <x:v>2026-07-14: the 60-minute Railway polling soak passed 36,000/36,000 with zero loss/duplicate modeled effects. The deployed QR worker passed 5,055 PNG/JPEG/corpus/crash-recovery cases with zero failures; RES-001/RES-002 are Passed. Exact main 00f3b11d / Railway 6a8ec5f6 then passed the isolated six-case shared-limiter failure matrix with real-consumer 429 before sinks, zero external calls/writes, green production smoke and zero total/live/expired buckets; RES-003 and SG-P0-005 are closed. RES-004 still needs one approved real Telegram update after restart.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11677,7 +11677,7 @@
       </x:c>
       <x:c r="B18" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A18)</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C18" s="629" t="str">
         <x:v>Code is in production; targeted real-client or failure-path proof remains.</x:v>
@@ -11691,7 +11691,7 @@
       </x:c>
       <x:c r="B19" s="629" t="n">
         <x:f>COUNTIF('Current Security Queue'!$F$2:$F$200,A19)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C19" s="629" t="str">
         <x:v>Original path revalidated after deployment.</x:v>
@@ -11753,7 +11753,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -11767,7 +11767,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -22898,6 +22898,32 @@
         <x:v>RES-001/RES-002 QR runtime evidence is complete. Keep RES-004 In Progress until an approved physical Railway restart/leader re-election with one QA update proves health, empty pending queue and no duplicate reply.</x:v>
       </x:c>
     </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>QA-SHARED-RATE-LIMIT-FAILURE-PROD-2026-07-14</x:v>
+      </x:c>
+      <x:c r="B103" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>Production-image shared rate-limit forced-failure and sink-ordering smoke</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>PRs #96/#97; exact main 00f3b11ddaeabecaed1412238edec23861e35c5d; Railway 6a8ec5f6-e758-4574-8d15-34eb1206ca43; image sha256:b4cc9f1138528cb698ca5d26cec136b8ab1bf5c2d7ec7e111371c358564741b9; node dist/ops/shared-rate-limit-failure-smoke.mjs; post-probe prod:smoke; count-only rate_limit_buckets observation</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>Passed: missing_config, hash_error, rpc_error, invalid_shape, transport_error and consumer_429_before_sinks; productionPolicy=true; externalNetworkCalls=0; databaseWrites=0; unexpectedSinkCalls=0. Home/health 200, polling leader 200, pending updates 0 and AI provider 200 after probe. Buckets total/live/expired=0/0/0.</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>RES-003, SG-P0-005</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>The short-lived operator bundle used only synthetic process-local values and a strict fetch interceptor; it exposed no application endpoint and opened no external connection. WebCrypto was restored in finally. Count-only DB observation read no row content and printed no secret or identifier.</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>Release gate and finding closed. Keep degraded-429 and bucket-volume monitoring; consider another shared store only if later latency/volume evidence exceeds the agreed Postgres budget.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -23744,29 +23770,27 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F20" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G20" s="615" t="str">
-        <x:v>Passed Local</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H20" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I20" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J20" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="K20" s="615" t="str">
         <x:v>Backend / Data</x:v>
       </x:c>
-      <x:c r="L20" s="615" t="str">
-        <x:v>Railway deploy + forced shared-RPC failure smoke</x:v>
-      </x:c>
+      <x:c r="L20" s="615"/>
       <x:c r="M20" s="615" t="str"/>
       <x:c r="N20" s="615" t="str">
-        <x:v>Production/Railway fails closed on missing config, hash/RPC error or invalid shape; dev/test fallback caps 4096 TTL/LRU keys and denies overflow. Production release: PR #71 / 6fb71ec8; migrations, polling cutover, restart and smoke evidence recorded 2026-07-11.</x:v>
+        <x:v>Production runtime passed 2026-07-14 at PRs #96/#97, exact main 00f3b11ddaeabecaed1412238edec23861e35c5d, Railway 6a8ec5f6-e758-4574-8d15-34eb1206ca43, image sha256:b4cc9f1138528cb698ca5d26cec136b8ab1bf5c2d7ec7e111371c358564741b9. The isolated in-container probe denied missing config, hash/WebCrypto exception, RPC error, invalid response shape and transport exception, and the real runCheck consumer returned rate_limited/429 before AI, persistence or another sink. Summary: passed=true, externalNetworkCalls=0, databaseWrites=0, unexpectedSinkCalls=0. Non-production fallback cap/TTL/LRU/overflow tests remain green. Post-probe production smoke passed; count-only rate_limit_buckets observation returned total/live/expired=0/0/0.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -25414,7 +25438,7 @@
         <x:v>src/lib/risk/shared-rate-limit.server.ts; src/lib/risk/rate-limit.ts</x:v>
       </x:c>
       <x:c r="F6" s="615" t="str">
-        <x:v>Deployed / Awaiting Live Verification</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="G6" s="615" t="str">
         <x:v>Backend / Data</x:v>
@@ -25423,16 +25447,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I6" s="615" t="str">
-        <x:v>5-failure reproducer + 13 focus + 534 owning-suite + 2652 full tests. Prod 6fb71ec8 + QA 74066f1: migrations, no-drop polling cutover and restart passed; polling-compatible response harness verified all five post-check actions with Bot API delivery and cleanup read-back; monitor/CI green.</x:v>
+        <x:v>Local reproducer/fallback cap and owning suites plus production PRs #96/#97. Exact main 00f3b11d / Railway 6a8ec5f6 / image sha256:b4cc9f11 passed the six-case in-container config/hash/RPC/shape/transport/consumer-429 probe with zero external calls, writes or unexpected sinks. Post-probe production smoke passed and count-only buckets were total/live/expired 0/0/0.</x:v>
       </x:c>
       <x:c r="J6" s="615" t="str">
-        <x:v>Run remaining targeted force shared config/hash/RPC/shape failures and verify 429/no sink work</x:v>
+        <x:v>Closed after exact-image forced-failure verification. Continue degraded-429 and bucket-volume monitoring as an operational watch.</x:v>
       </x:c>
       <x:c r="K6" s="615" t="str">
         <x:v>Production shared-control failure grants no local allowance; fallback state stays &lt;=4096 keys with bounded cleanup</x:v>
       </x:c>
       <x:c r="L6" s="618" t="n">
-        <x:v>46214</x:v>
+        <x:v>46217</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Record real Telegram restart QA evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb0581c4b8a234f95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R6d919cdc2a854dc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R8c8355dd3c5641c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R416f1e153493490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Re081f16e835d4857"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R6844d165763d4723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R23a53582c11440dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R93d55bea6e8247ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Ra57bab9d37934da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R8bb6360890c946e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4e301106445b4796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd35d5aba412c4d38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R9c1e821ec5e148ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc1339265f6e94c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R07618c75434c46df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd4742280588b4817"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11469,10 +11469,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Complete the physical Railway restart/polling-leader re-election with one approved QA update. Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, legal approval and the fixed-RC 72-hour canary.</x:v>
+        <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14: the 60-minute Railway polling soak passed 36,000/36,000 with zero loss/duplicate modeled effects. The deployed QR worker passed 5,055 PNG/JPEG/corpus/crash-recovery cases with zero failures; RES-001/RES-002 are Passed. Exact main 00f3b11d / Railway 6a8ec5f6 then passed the isolated six-case shared-limiter failure matrix with real-consumer 429 before sinks, zero external calls/writes, green production smoke and zero total/live/expired buckets; RES-003 and SG-P0-005 are closed. RES-004 still needs one approved real Telegram update after restart.</x:v>
+        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11753,7 +11753,7 @@
       </x:c>
       <x:c r="B24" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A24)</x:f>
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C24" s="629" t="str">
         <x:v>Work started but gate is not complete.</x:v>
@@ -11767,7 +11767,7 @@
       </x:c>
       <x:c r="B25" s="629" t="n">
         <x:f>COUNTIF('Release Gates'!$I$2:$I$200,A25)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C25" s="629" t="str">
         <x:v>All required evidence for the row is present.</x:v>
@@ -22924,6 +22924,32 @@
         <x:v>Release gate and finding closed. Keep degraded-429 and bucket-volume monitoring; consider another shared store only if later latency/volume evidence exceeds the agreed Postgres budget.</x:v>
       </x:c>
     </x:row>
+    <x:row r="104" ht="135" customHeight="1">
+      <x:c r="A104" s="596" t="str">
+        <x:v>QA-TELEGRAM-RESTART-REAL-UPDATE-PROD-2026-07-14</x:v>
+      </x:c>
+      <x:c r="B104" s="596" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C104" s="596" t="str">
+        <x:v>Real Telegram update after Railway instance replacement and polling-leader re-election</x:v>
+      </x:c>
+      <x:c r="D104" s="596" t="str">
+        <x:v>Railway c2b98732 / main 128e27d2; user-approved real client greeting; two metadata-only lifecycle aggregate read-backs about 30 seconds apart; post-update prod:smoke</x:v>
+      </x:c>
+      <x:c r="E104" s="596" t="str">
+        <x:v>Passed: client showed one deterministic greeting reply; both read-backs observed one completed row, zero processing rows, retries or failure-stage rows, and max attempt count 1. Pending updates 0, polling leader 200, public/health 200 and AI provider health 200.</x:v>
+      </x:c>
+      <x:c r="F104" s="596" t="str">
+        <x:v>RES-004</x:v>
+      </x:c>
+      <x:c r="G104" s="596" t="str">
+        <x:v>The client screenshot is the visible single-reply evidence. Server verification retained only aggregate lifecycle counts; no chat/user/update ID, message text, token or secret was printed. The greeting is deterministic and did not invoke the AI provider. This is no-duplicate evidence for this run, not an exactly-once guarantee.</x:v>
+      </x:c>
+      <x:c r="H104" s="596" t="str">
+        <x:v>RES-004 closed. Continue the broader real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance matrix, authorized Supabase/data drills, legal review and fixed-RC 72-hour canary.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -23810,16 +23836,16 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F21" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G21" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H21" s="615" t="str">
         <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I21" s="615" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J21" s="618" t="n">
         <x:v>46217</x:v>
@@ -23827,14 +23853,12 @@
       <x:c r="K21" s="615" t="str">
         <x:v>QA / Platform</x:v>
       </x:c>
-      <x:c r="L21" s="615" t="str">
-        <x:v>Actual Railway restart/leader re-election with one approved QA update</x:v>
-      </x:c>
+      <x:c r="L21" s="615"/>
       <x:c r="M21" s="615" t="str">
         <x:v>RES-001..003</x:v>
       </x:c>
       <x:c r="N21" s="615" t="str">
-        <x:v>Polling subgate: PR #89 / exact main 868eb18d / Railway 24b9cb4a; uninterrupted 60-minute in-container soak passed 36,000/36,000 with zero lost updates or duplicate modeled effects, max queue 35, max RSS 101.41 MiB, event-loop p99 21.84 ms and update-latency p99 2.57 ms. QR subgate: PR #94 / exact main f1ddf349 / Railway 09f984bd / image sha256:abbba9cf; live module require passed and the detached 10-minute QR worker profile passed 5,055 cases with zero failures, PNG 2,087, JPEG 693, queue 4 accepted/1 rejected, forced interruption fail-closed and worker recovery true, max RSS 234.60 MiB, RSS growth 110.08 MiB, event-loop p99 21.04 ms and decode p99/max 225.53/279.47 ms. Both runners used generated in-memory data and made no Telegram, Supabase, AI/reputation-provider call or persistent write. Production smoke after QR load passed. Only the approved physical Railway restart/leader re-election proof remains; neither runner claims it.</x:v>
+        <x:v>Polling subgate: PR #89 / exact main 868eb18d / Railway 24b9cb4a; 60-minute in-container soak passed 36,000/36,000 with zero lost updates or duplicate modeled effects, max queue 35, max RSS 101.41 MiB, event-loop p99 21.84 ms and update-latency p99 2.57 ms. QR subgate: PR #94 / exact main f1ddf349 / Railway 09f984bd; 10-minute worker profile passed 5,055 cases with zero failures, queue 4 accepted/1 rejected, forced interruption fail-closed and worker recovery true, max RSS 234.60 MiB and decode p99/max 225.53/279.47 ms. Restart closure: main 128e27d2 / Railway c2b98732 replaced the application instance using image sha256:b4cc9f11; health and polling leader were 200, webhook URL empty and pending updates 0. The user sent the approved real greeting at 15:00 +05:00 and the client showed exactly one reply. Two metadata-only read-backs about 30 seconds apart each found one completed row, zero processing/retries/failure and maximum attempt count 1. Post-update production smoke passed. No exactly-once claim; delivery remains at-least-once with bounded idempotent handling.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">

</xml_diff>

<commit_message>
Adapt 1,000-dialogue corpus to Telegram Inline
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Ra57bab9d37934da3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R8bb6360890c946e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R4e301106445b4796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd35d5aba412c4d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R9c1e821ec5e148ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rc1339265f6e94c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R07618c75434c46df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rd4742280588b4817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R128c433cff164df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9648412070b54a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ra5e4f5386eb94caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R35ad5fb2c0a94ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R09627668905442e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R213efb2a1254422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R340ae5ebc6a44fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R87daf8f24b8c41a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11456,7 +11456,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="108" customHeight="1">
+    <x:row r="2" ht="135" customHeight="1">
       <x:c r="A2" s="1227" t="n">
         <x:v>46217</x:v>
       </x:c>
@@ -11472,7 +11472,7 @@
         <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once.</x:v>
+        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once. 2026-07-14 local Inline evidence: 3,805 source cases / 2,140 unique RU/UZ/EN queries passed through the real handler with Telegram/Supabase mocked, fetch 0, DB mutations 0 and no paid API usage. Live Desktop/Android/iOS preview/insertion remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -12787,30 +12787,20 @@
           <x:t xml:space="preserve">Inline mode accepts short queries and returns compact risk cards without forcing the user to leave the chat.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F17" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">src/lib/telegram/inline.ts; src/lib/telegram/bot.ts</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G17" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">.kiro/specs/telegram-inline-check-v1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H17" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implemented</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I17" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manual BotFather + smoke test</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J17" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Add start-menu hint that inline mode exists.</x:t>
-        </x:is>
+      <x:c r="F17" s="8" t="str">
+        <x:v>src/lib/telegram/handlers/inline.ts; src/lib/telegram/inline-adapted-dialogue-corpus.ts; src/lib/telegram/router.ts; src/lib/telegram/bot-i18n.ts; src/lib/risk/sensitive-text.ts</x:v>
+      </x:c>
+      <x:c r="G17" s="8" t="str">
+        <x:v>.kiro/specs/telegram-inline-check-v1; ai_docs/TELEGRAM_INLINE_QA.md; ai_docs/TELEGRAM_INLINE_PHRASE_CORPUS.md; ai_docs/TELEGRAM_INLINE_OFFLINE_QA_2026-07-14.md</x:v>
+      </x:c>
+      <x:c r="H17" s="11" t="str">
+        <x:v>Implemented</x:v>
+      </x:c>
+      <x:c r="I17" s="8" t="str">
+        <x:v>Real-handler offline corpus: 3,805 source cases / 2,140 unique RU/UZ/EN queries with strict no-network/no-write guards; focused Inline/privacy regressions and synthetic production smoke; real-client checklist remains open.</x:v>
+      </x:c>
+      <x:c r="J17" s="8" t="str">
+        <x:v>Complete Telegram Desktop/Android/iOS RU/UZ/EN preview + insert QA: 0/1/255/256/257 characters, Markdown/plaintext retry, timeout/error UX, privacy and language.</x:v>
       </x:c>
       <x:c r="K17" s="14" t="inlineStr">
         <x:is>
@@ -22948,6 +22938,32 @@
       </x:c>
       <x:c r="H104" s="596" t="str">
         <x:v>RES-004 closed. Continue the broader real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance matrix, authorized Supabase/data drills, legal review and fixed-RC 72-hour canary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="135" customHeight="1">
+      <x:c r="A105" t="str">
+        <x:v>QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14</x:v>
+      </x:c>
+      <x:c r="B105" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>Local RU/UZ/EN Inline adaptation of the 1,000-dialogue perimeter</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>npx vitest run src/lib/telegram/inline-adapted-dialogue-corpus.test.ts src/lib/risk/sensitive-text.test.ts src/lib/telegram/handlers/inline.test.ts; npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=moderate</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>Passed locally: 3,805 source cases / 2,140 unique queries; RU 1,270, UZ 1,269, EN 1,266. Sources: 2,500 raw turns from all 1,000 dialogues, 930 stateless contextual follow-ups, 363 mixed-clause adversarial queries and 12 synthetic credential-boundary fixtures. The real Inline handler returned one bounded MarkdownV2 article per case. Full suite: 137 files / 8,647 tests.</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>BOT-004, INL-001, TG-016</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Telegram answerInlineQuery and Supabase were mocked; global fetch remained unused; DB mutations were zero. Every runCheck call used channel=telegram, skipAi=true, skipUrlReputation=true and persist=false. Forward/reverse OTP/PIN/CVV punctuation, partial-secret oracle and password-request scoring regressions passed. No user data or paid API usage.</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>Deploy the candidate, then complete INL-002 on real Telegram Desktop/Android/iOS. This run does not prove Bot API acceptance, result-list rendering, insertion, client truncation, timeout UX or plaintext retry.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24090,7 +24106,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J27" s="618" t="n">
-        <x:v>46216</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
@@ -24100,7 +24116,7 @@
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -24212,7 +24228,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J30" s="618" t="n">
-        <x:v>46215</x:v>
+        <x:v>46217</x:v>
       </x:c>
       <x:c r="K30" s="615" t="str">
         <x:v>Telegram / QA</x:v>
@@ -24224,7 +24240,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker.</x:v>
+        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker. The local real-handler Inline sub-gate passed 3,805 source cases / 2,140 unique RU/UZ/EN queries with bounded MarkdownV2 articles, external fetch denied, Telegram/Supabase mocked, zero DB mutations and runCheck fixed to skipAi=true, skipUrlReputation=true, persist=false. Real-client preview, insertion, truncation, retry, timeout and rendering evidence remains blocking.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -24264,7 +24280,7 @@
       </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients.</x:v>
+        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients. The offline corpus is a prerequisite only; it does not prove Telegram Desktop/Android/iOS result-list rendering or insertion.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>

<commit_message>
Record Inline corpus deployment evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R128c433cff164df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R9648412070b54a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ra5e4f5386eb94caf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R35ad5fb2c0a94ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R09627668905442e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R213efb2a1254422c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R340ae5ebc6a44fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R87daf8f24b8c41a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9bea1ac9e16747a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R867b14a18e494dfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ra440ead78cb5479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbd1e4ba4a0644085"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1960bea7e35a46ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2cee0c792d46466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re1bea48aec9b4f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R1c8f6c693f5e42f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11456,7 +11456,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="135" customHeight="1">
+    <x:row r="2" ht="180" customHeight="1">
       <x:c r="A2" s="1227" t="n">
         <x:v>46217</x:v>
       </x:c>
@@ -11472,7 +11472,7 @@
         <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once. 2026-07-14 local Inline evidence: 3,805 source cases / 2,140 unique RU/UZ/EN queries passed through the real handler with Telegram/Supabase mocked, fetch 0, DB mutations 0 and no paid API usage. Live Desktop/Android/iOS preview/insertion remains open.</x:v>
+        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once. 2026-07-14 local Inline evidence: 3,805 source cases / 2,140 unique RU/UZ/EN queries passed through the real handler with Telegram/Supabase mocked, fetch 0, DB mutations 0 and no paid API usage. Live Desktop/Android/iOS preview/insertion remains open. PR #100 / main 87c5ff5 deployed successfully as Railway 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432; /healthz and polling leader returned 200; no mass Inline or AI production calls were made.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -12797,7 +12797,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="I17" s="8" t="str">
-        <x:v>Real-handler offline corpus: 3,805 source cases / 2,140 unique RU/UZ/EN queries with strict no-network/no-write guards; focused Inline/privacy regressions and synthetic production smoke; real-client checklist remains open.</x:v>
+        <x:v>Real-handler offline corpus: 3,805 source cases / 2,140 unique RU/UZ/EN queries with strict no-network/no-write guards; PR #100 / main 87c5ff5 deployed successfully on Railway; health and polling leader returned 200; real-client checklist remains open.</x:v>
       </x:c>
       <x:c r="J17" s="8" t="str">
         <x:v>Complete Telegram Desktop/Android/iOS RU/UZ/EN preview + insert QA: 0/1/255/256/257 characters, Markdown/plaintext retry, timeout/error UX, privacy and language.</x:v>
@@ -22940,7 +22940,7 @@
         <x:v>RES-004 closed. Continue the broader real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance matrix, authorized Supabase/data drills, legal review and fixed-RC 72-hour canary.</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="135" customHeight="1">
+    <x:row r="105" ht="185" customHeight="1">
       <x:c r="A105" t="str">
         <x:v>QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14</x:v>
       </x:c>
@@ -22954,7 +22954,7 @@
         <x:v>npx vitest run src/lib/telegram/inline-adapted-dialogue-corpus.test.ts src/lib/risk/sensitive-text.test.ts src/lib/telegram/handlers/inline.test.ts; npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit --audit-level=moderate</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>Passed locally: 3,805 source cases / 2,140 unique queries; RU 1,270, UZ 1,269, EN 1,266. Sources: 2,500 raw turns from all 1,000 dialogues, 930 stateless contextual follow-ups, 363 mixed-clause adversarial queries and 12 synthetic credential-boundary fixtures. The real Inline handler returned one bounded MarkdownV2 article per case. Full suite: 137 files / 8,647 tests.</x:v>
+        <x:v>Passed locally: 3,805 source cases / 2,140 unique queries; RU 1,270, UZ 1,269, EN 1,266. Sources: 2,500 raw turns from all 1,000 dialogues, 930 stateless contextual follow-ups, 363 mixed-clause adversarial queries and 12 synthetic credential-boundary fixtures. The real Inline handler returned one bounded MarkdownV2 article per case. Full suite: 137 files / 8,647 tests. PR #100 merged as main 87c5ff5; Railway deployment 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432 reached SUCCESS; health and polling leader returned 200.</x:v>
       </x:c>
       <x:c r="F105" t="str">
         <x:v>BOT-004, INL-001, TG-016</x:v>
@@ -22963,7 +22963,7 @@
         <x:v>Telegram answerInlineQuery and Supabase were mocked; global fetch remained unused; DB mutations were zero. Every runCheck call used channel=telegram, skipAi=true, skipUrlReputation=true and persist=false. Forward/reverse OTP/PIN/CVV punctuation, partial-secret oracle and password-request scoring regressions passed. No user data or paid API usage.</x:v>
       </x:c>
       <x:c r="H105" t="str">
-        <x:v>Deploy the candidate, then complete INL-002 on real Telegram Desktop/Android/iOS. This run does not prove Bot API acceptance, result-list rendering, insertion, client truncation, timeout UX or plaintext retry.</x:v>
+        <x:v>Complete INL-002 on real Telegram Desktop/Android/iOS. Deployment health does not prove Bot API acceptance, result-list rendering, insertion, client truncation, timeout UX or plaintext retry.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24240,7 +24240,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker. The local real-handler Inline sub-gate passed 3,805 source cases / 2,140 unique RU/UZ/EN queries with bounded MarkdownV2 articles, external fetch denied, Telegram/Supabase mocked, zero DB mutations and runCheck fixed to skipAi=true, skipUrlReputation=true, persist=false. Real-client preview, insertion, truncation, retry, timeout and rendering evidence remains blocking.</x:v>
+        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker. The local real-handler Inline sub-gate passed 3,805 source cases / 2,140 unique RU/UZ/EN queries with bounded MarkdownV2 articles, external fetch denied, Telegram/Supabase mocked, zero DB mutations and runCheck fixed to skipAi=true, skipUrlReputation=true, persist=false. Real-client preview, insertion, truncation, retry, timeout and rendering evidence remains blocking. PR #100 merged as main 87c5ff5 and Railway deployment 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432 reached SUCCESS; /healthz and the protected polling-leader endpoint returned 200. No mass Inline or AI production calls were made.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">

</xml_diff>

<commit_message>
Record Inline Unicode deployment evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R9bea1ac9e16747a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R867b14a18e494dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Ra440ead78cb5479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rbd1e4ba4a0644085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R1960bea7e35a46ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R2cee0c792d46466c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re1bea48aec9b4f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R1c8f6c693f5e42f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re3f8c2fc4c3846cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R7be692b34cef48ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R443828f4116242fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd1a7af66d23f4a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2ee21759df3d4547"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re3487a9d328c43a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R55cca13bd3cd442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R5c59ee3ff1834cec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11456,7 +11456,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="180" customHeight="1">
+    <x:row r="2" ht="195" customHeight="1">
       <x:c r="A2" s="1227" t="n">
         <x:v>46217</x:v>
       </x:c>
@@ -11472,7 +11472,7 @@
         <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once. 2026-07-14 local Inline evidence: 3,805 source cases / 2,140 unique RU/UZ/EN queries passed through the real handler with Telegram/Supabase mocked, fetch 0, DB mutations 0 and no paid API usage. Live Desktop/Android/iOS preview/insertion remains open. PR #100 / main 87c5ff5 deployed successfully as Railway 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432; /healthz and polling leader returned 200; no mass Inline or AI production calls were made.</x:v>
+        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once. 2026-07-14 local Inline evidence: 3,805 source cases / 2,140 unique RU/UZ/EN queries passed through the real handler with Telegram/Supabase mocked, fetch 0, DB mutations 0 and no paid API usage. Live Desktop/Android/iOS preview/insertion remains open. PR #100 / main 87c5ff5 deployed successfully as Railway 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432; /healthz and polling leader returned 200; no mass Inline or AI production calls were made. 2026-07-14 Inline Unicode boundary fix is deployed at main f26eece / Railway 90962188; the exact 51-row Desktop/Android/iOS client pack is ready without API use, while all real-client rows remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -22576,6 +22576,32 @@
         <x:v>Next: continue residual live UX QA: 15-20 manual direct/inline phrases, UZ voice spot-checks when STT budget resets, and image provider routine spot-checks.</x:v>
       </x:c>
     </x:row>
+    <x:row r="84" ht="185" customHeight="1">
+      <x:c r="A84" t="str">
+        <x:v>QA-TELEGRAM-INLINE-UNICODE-GATE-2026-07-14</x:v>
+      </x:c>
+      <x:c r="B84" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>Inline Unicode boundary fix, evidence taxonomy and deployed client-matrix preflight</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>npx vitest run inline/API/privacy slice; npm run test:run; npx tsc --noEmit; npm run lint; npm run build; npm audit; qa:telegram-inline-client-matrix; GitHub PR #102 CI/security; Railway deploy; health/polling probes; polling-aware prod:telegram-inline-smoke</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>Passed: 222/222 focused tests and 8,650/8,650 full tests; TypeScript/build; lint 0 errors/8 existing warnings; npm audit 0; 17 cases per client / 51 required real-client rows / maximum 256 Unicode code points / generator network calls 0. PR #102 merged as main f26eece; all seven CI/security jobs passed. Railway 90962188 is SUCCESS, image sha256:5c5e4e70b5bb08a1c14510976cabba9f7c99709c5077951930fb27371d2f26ab; health and polling leader returned 200.</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>BOT-004, INL-001, INL-002, TG-016</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>No mass Telegram messages and no AI/reputation call. The polling transport smoke used synthetic ids, observed the expected webhook 503, created no checks/session rows and completed cleanup. A normal client is not used to force 257-character, timeout, ok:false or parse failures.</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>Run all 17 fixtures on each of Telegram Desktop, Android and iOS, capture sanitized preview/insertion evidence and read back zero persistence before closing BOT-004/INL-001/INL-002.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
         <x:v>QA-2026-07-09-010</x:v>
@@ -24116,7 +24142,7 @@
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -24240,7 +24266,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker. The local real-handler Inline sub-gate passed 3,805 source cases / 2,140 unique RU/UZ/EN queries with bounded MarkdownV2 articles, external fetch denied, Telegram/Supabase mocked, zero DB mutations and runCheck fixed to skipAi=true, skipUrlReputation=true, persist=false. Real-client preview, insertion, truncation, retry, timeout and rendering evidence remains blocking. PR #100 merged as main 87c5ff5 and Railway deployment 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432 reached SUCCESS; /healthz and the protected polling-leader endpoint returned 200. No mass Inline or AI production calls were made.</x:v>
+        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker. The local real-handler Inline sub-gate passed 3,805 source cases / 2,140 unique RU/UZ/EN queries with bounded MarkdownV2 articles, external fetch denied, Telegram/Supabase mocked, zero DB mutations and runCheck fixed to skipAi=true, skipUrlReputation=true, persist=false. Real-client preview, insertion, truncation, retry, timeout and rendering evidence remains blocking. PR #100 merged as main 87c5ff5 and Railway deployment 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432 reached SUCCESS; /healthz and the protected polling-leader endpoint returned 200. No mass Inline or AI production calls were made. PR #102 / main f26eece fixed the 256-character boundary to count Unicode code points and passed 8,650/8,650 tests. Railway 90962188 / image sha256:5c5e4e70 is SUCCESS; health and polling leader are 200; the polling Inline transport smoke returned the expected authenticated webhook 503 and persisted no checks/session rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -24254,7 +24280,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="D31" s="615" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E31" s="615" t="str">
         <x:v>Pending</x:v>
@@ -24271,16 +24297,18 @@
       <x:c r="I31" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
-      <x:c r="J31" s="618"/>
+      <x:c r="J31" s="618" t="n">
+        <x:v>46217</x:v>
+      </x:c>
       <x:c r="K31" s="615" t="str">
         <x:v>QA / Product</x:v>
       </x:c>
       <x:c r="L31" s="615" t="str">
-        <x:v>Devices + staging deploy</x:v>
+        <x:v>Real Telegram Desktop/Android/iOS access and sanitized before/after screenshots</x:v>
       </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients. The offline corpus is a prerequisite only; it does not prove Telegram Desktop/Android/iOS result-list rendering or insertion.</x:v>
+        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients. The offline corpus is a prerequisite only; it does not prove Telegram Desktop/Android/iOS result-list rendering or insertion. The zero-network qa:telegram-inline-client-matrix generator now defines 17 cases per client / 51 Desktop-Android-iOS rows: RU/UZ/EN high/suspicious/low, empty/1/255/256 and four synthetic privacy cases. The real-client rows remain pending. 257-character rejection, timeout, ok:false and Markdown parse retry are automated-only evidence and must not be forced by damaging production.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>

<commit_message>
docs: record inline release evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Re3f8c2fc4c3846cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R7be692b34cef48ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R443828f4116242fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd1a7af66d23f4a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R2ee21759df3d4547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Re3487a9d328c43a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R55cca13bd3cd442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R5c59ee3ff1834cec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R93921726fa7d4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbd9c64c235b0413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R17281f74b5d24515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R10bcfb6fc8584593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raf3b3a8232064092"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb79ff2c0666e44aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rb76fb651cf784455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R460c821a79c546f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11458,7 +11458,7 @@
     </x:row>
     <x:row r="2" ht="195" customHeight="1">
       <x:c r="A2" s="1227" t="n">
-        <x:v>46217</x:v>
+        <x:v>46218</x:v>
       </x:c>
       <x:c r="B2" s="1219" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$200)</x:f>
@@ -11472,7 +11472,7 @@
         <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-14: polling passed 36,000/36,000 with zero lost updates or duplicate modeled effects; the QR worker passed 5,055 cases with zero failures; the exact production shared-limiter failure matrix passed with zero external calls/writes. Railway c2b98732 then replaced the app instance. One approved real Telegram greeting produced one reply; two stable metadata-only read-backs found one completed attempt with no retry or failure, pending updates 0 and leader 200. RES-001..004 are Passed; SG-P0-005 is Closed. Delivery remains at-least-once, not exactly-once. 2026-07-14 local Inline evidence: 3,805 source cases / 2,140 unique RU/UZ/EN queries passed through the real handler with Telegram/Supabase mocked, fetch 0, DB mutations 0 and no paid API usage. Live Desktop/Android/iOS preview/insertion remains open. PR #100 / main 87c5ff5 deployed successfully as Railway 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432; /healthz and polling leader returned 200; no mass Inline or AI production calls were made. 2026-07-14 Inline Unicode boundary fix is deployed at main f26eece / Railway 90962188; the exact 51-row Desktop/Android/iOS client pack is ready without API use, while all real-client rows remain open.</x:v>
+        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -11666,7 +11666,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="629" t="str">
-        <x:v>Fourteen fixes are deployed and await finding-specific live closure; the admin-role migration remains In Progress.</x:v>
+        <x:v>One admin-role finding remains In Progress: remote history records the migration and count-only entitlement drift is zero; direct live catalog/grant and revocation-event verification remains.</x:v>
       </x:c>
       <x:c r="D17" s="629"/>
       <x:c r="E17" s="629"/>
@@ -24266,7 +24266,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Backend/protocol/privacy/polling-boundary automation is green at 190c82a2a0d7db8f1583c57265afe353e97f3f22; synthetic Inline smokes persist no checks or sessions. Real-client rendering, insert-result, length, error and timeout evidence remains the blocker. The local real-handler Inline sub-gate passed 3,805 source cases / 2,140 unique RU/UZ/EN queries with bounded MarkdownV2 articles, external fetch denied, Telegram/Supabase mocked, zero DB mutations and runCheck fixed to skipAi=true, skipUrlReputation=true, persist=false. Real-client preview, insertion, truncation, retry, timeout and rendering evidence remains blocking. PR #100 merged as main 87c5ff5 and Railway deployment 78dc6e9b-2464-4e3c-a6ed-c7b0f71cc432 reached SUCCESS; /healthz and the protected polling-leader endpoint returned 200. No mass Inline or AI production calls were made. PR #102 / main f26eece fixed the 256-character boundary to count Unicode code points and passed 8,650/8,650 tests. Railway 90962188 / image sha256:5c5e4e70 is SUCCESS; health and polling leader are 200; the polling Inline transport smoke returned the expected authenticated webhook 503 and persisted no checks/session rows.</x:v>
+        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -24308,7 +24308,7 @@
       </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>Screenshots before/after insert; critical privacy/language/high-risk cases on all three clients. The offline corpus is a prerequisite only; it does not prove Telegram Desktop/Android/iOS result-list rendering or insertion. The zero-network qa:telegram-inline-client-matrix generator now defines 17 cases per client / 51 Desktop-Android-iOS rows: RU/UZ/EN high/suspicious/low, empty/1/255/256 and four synthetic privacy cases. The real-client rows remain pending. 257-character rejection, timeout, ok:false and Markdown parse retry are automated-only evidence and must not be forced by damaging production.</x:v>
+        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -24874,23 +24874,23 @@
         <x:v>Passed Local</x:v>
       </x:c>
       <x:c r="H45" s="615" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I45" s="615" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J45" s="618" t="n">
-        <x:v>46215</x:v>
+        <x:v>46218</x:v>
       </x:c>
       <x:c r="K45" s="615" t="str">
         <x:v>Data / Security</x:v>
       </x:c>
       <x:c r="L45" s="615" t="str">
-        <x:v>SEC-2026-0712-008</x:v>
+        <x:v>Direct live catalog/grant read-back + controlled revocation-event drill</x:v>
       </x:c>
       <x:c r="M45" s="615"/>
       <x:c r="N45" s="615" t="str">
-        <x:v>Medium/P2 code and regression are deployed, but the production Supabase migration remains unapplied; authorized apply plus grant/revoke read-back is a release blocker.</x:v>
+        <x:v>Medium/P2 remediation remains green across 4867 tests, coverage, TypeScript, lint, build, npm audit 0, CodeQL, Gitleaks, Trivy, CycloneDX, clean-database migrations, pgTAP 38/38 and schema lint. Remote migration history records 20260712142514 on 2026-07-15; linked dry-run has no pending migration and remote schema lint reports no error. Stable count-only preflight is Auth 1, current admins 1, eligible admins 1, stale 0, missing 0, with no identifier emitted. Direct live catalog trigger/function-owner/search_path/EXECUTE-grant read-back and a controlled allowlist-delete, email-drift and confirmation-loss revocation drill remain blocking.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -26389,16 +26389,16 @@
         <x:v>Gate 1</x:v>
       </x:c>
       <x:c r="I29" s="615" t="str">
-        <x:v>Medium/P2 remediation verified: 4867/4867 tests, coverage thresholds, TypeScript, lint 0 errors, build, npm audit 0, CodeQL, Gitleaks, Trivy 0 fixed High/Critical, CycloneDX SBOM, 28 migrations, pgTAP 38/38 and schema lint. Application reconciliation code is deployed at 190c82a2a0d7db8f1583c57265afe353e97f3f22 / be7d6f8d-f06d-459b-b438-ef8924454c4e, but the production Supabase migration is not applied because no authorized production CLI/database credential is available. Count-only production preflight remains green: Auth 1, admins 1, eligible 1, stale 0, missing 0. Detailed evidence: outputs/security_revalidation_2026-07-12/findings/stale-admin-role-entitlement.</x:v>
+        <x:v>Medium/P2 remediation remains green across 4867 tests, coverage, TypeScript, lint, build, npm audit 0, CodeQL, Gitleaks, Trivy, CycloneDX, clean-database migrations, pgTAP 38/38 and schema lint. Remote migration history records 20260712142514_reconcile_admin_role_lifecycle.sql on 2026-07-15. Linked local/remote history matches, dry-run reports no pending migration and remote schema lint reports no error. Stable count-only production preflight: Auth 1, current admins 1, eligible admins 1, stale 0, missing 0; no identifier was emitted. Direct live catalog trigger/function-owner/search_path/grant read-back and a controlled revocation-event drill remain open.</x:v>
       </x:c>
       <x:c r="J29" s="615" t="str">
-        <x:v>Restore authorized production Supabase access; rerun count-only preflight, apply the exact migration, verify migration history and revoke/grant behavior, then collect read-back evidence.</x:v>
+        <x:v>Use an authenticated production SQL channel to read back trigger, function owner/search_path and EXECUTE grants. Then run a controlled synthetic allowlist-delete, email-drift and confirmation-loss revocation drill with count-only evidence. Keep In Progress until both checks pass.</x:v>
       </x:c>
       <x:c r="K29" s="615" t="str">
         <x:v>Allowlist delete, email drift and confirmation loss immediately deny existing sessions.</x:v>
       </x:c>
       <x:c r="L29" s="618" t="n">
-        <x:v>46215</x:v>
+        <x:v>46218</x:v>
       </x:c>
     </x:row>
     <x:row r="30">

</xml_diff>

<commit_message>
fix(telegram): recover edited inline context
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R93921726fa7d4258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rbd9c64c235b0413d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R17281f74b5d24515"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="R10bcfb6fc8584593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Raf3b3a8232064092"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb79ff2c0666e44aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rb76fb651cf784455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R460c821a79c546f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb153be9965614fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc199f2a72c7b4e36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb16742265b5b400e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf0d8e3398b01464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R27a1261015194180"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R19fbb347b4c54a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re793de878f6c42cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R36611c6ca69140e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11456,7 +11456,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="195" customHeight="1">
+    <x:row r="2" ht="245" customHeight="1">
       <x:c r="A2" s="1227" t="n">
         <x:v>46218</x:v>
       </x:c>
@@ -11472,7 +11472,7 @@
         <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once.</x:v>
+        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once. 2026-07-15 second Desktop Inline remediation is locally green: 30 additional pre-fix screenshots, 1,175/1,175 new context cases, 10,131/10,131 total tests, coverage above repository thresholds, TypeScript/build/lint 0 errors and npm audit 0. The branch is not yet deployment or real-client evidence; Desktop replay and all Android/iOS rows remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -22992,6 +22992,32 @@
         <x:v>Complete INL-002 on real Telegram Desktop/Android/iOS. Deployment health does not prove Bot API acceptance, result-list rendering, insertion, client truncation, timeout UX or plaintext retry.</x:v>
       </x:c>
     </x:row>
+    <x:row r="106" ht="195" customHeight="1">
+      <x:c r="A106" t="str">
+        <x:v>QA-TELEGRAM-INLINE-CONTEXT-RECOVERY-2026-07-15</x:v>
+      </x:c>
+      <x:c r="B106" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>Second Telegram Desktop screenshot-driven Inline context recovery</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>1,175-case real-handler context corpus; complete vitest run; repository coverage gate; TypeScript; ESLint; production build; npm audit; manual diff/security review</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>Passed locally: 1,175/1,175 context cases and 10,131/10,131 complete-project tests across 475 files. Coverage passed: statements 84.76%, branches 78.91%, functions 90.89%, lines 86.82%. TypeScript, build and npm audit 0 passed; ESLint had 0 errors and 8 existing Fast Refresh warnings.</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>BOT-004, INL-001, INL-002, TG-016</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>Thirty owner-supplied Desktop screenshots are pre-fix evidence. The new corpus uses the real handleInlineQuery path with Telegram/Supabase mocked, global fetch denied, zero DB mutations, skipAi=true, skipUrlReputation=true and persist=false. It checks edited-query ids, multiline danger priority, 120/256/4096 limits, MarkdownV2 and OTP/PIN/CVV redaction without paid API use.</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>Publish and deploy the reviewed branch, verify exact deployment health, then replay the affected Desktop cases and the 17-case Android/iOS matrices. Keep INL-001/INL-002 blocked and BOT-004 In Progress until real-client evidence passes.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -24132,7 +24158,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J27" s="618" t="n">
-        <x:v>46217</x:v>
+        <x:v>46218</x:v>
       </x:c>
       <x:c r="K27" s="615" t="str">
         <x:v>QA Automation</x:v>
@@ -24142,7 +24168,7 @@
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix. 2026-07-15 second Desktop remediation evidence: 30 additional pre-fix screenshots were converted into a 1,175-case local RU/UZ/EN Inline context suite. All 1,175 pass, including 1,152 dialogue mutations plus safe-control, redaction and result-id contracts. The complete project passes 10,131/10,131 tests and coverage 84.76/78.91/90.89/86.82. This remains deterministic offline evidence and does not replace the real Desktop/Android/iOS BOT-004 matrix.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -24254,7 +24280,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J30" s="618" t="n">
-        <x:v>46217</x:v>
+        <x:v>46218</x:v>
       </x:c>
       <x:c r="K30" s="615" t="str">
         <x:v>Telegram / QA</x:v>
@@ -24266,7 +24292,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking.</x:v>
+        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking. The screenshot-driven branch fixes changed-query result identity, concrete second-line priority, truncated/repetitive suspicious previews, RU/UZ/EN authority/SIM/investment context and false urgency from user safety questions. The 1,175-case handler suite denies external fetch and DB mutations; each check uses skipAi=true, skipUrlReputation=true and persist=false. Full local verification is 10,131/10,131 with coverage above all thresholds, TypeScript, lint 0 errors, build and npm audit 0. Deployment and real-client rendering/insertion remain blocking.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -24298,7 +24324,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="J31" s="618" t="n">
-        <x:v>46217</x:v>
+        <x:v>46218</x:v>
       </x:c>
       <x:c r="K31" s="615" t="str">
         <x:v>QA / Product</x:v>
@@ -24308,7 +24334,7 @@
       </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production.</x:v>
+        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production. A second batch of 30 Telegram Desktop screenshots reproduces unchanged or missing edited-query results and truncated generic preview copy. They are pre-fix evidence only. Post-deploy Desktop replay plus the complete 17-case Android and iOS matrices remain required; no real-client pass is inferred from the local 1,175-case corpus.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>

<commit_message>
docs(qa): record inline context deployment evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="Rb153be9965614fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc199f2a72c7b4e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb16742265b5b400e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rf0d8e3398b01464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R27a1261015194180"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="R19fbb347b4c54a53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Re793de878f6c42cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="R36611c6ca69140e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6ffd92cfff924920"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R5c391322a4dd4395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb300f540469349e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra2ca5852fe3d42a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R468eb7be48d741cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb567a345c32e432c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rdbad337f32fe47a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Ree5a290ef7e74a66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11456,7 +11456,7 @@
         <x:v>Owner note</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="245" customHeight="1">
+    <x:row r="2" ht="270" customHeight="1">
       <x:c r="A2" s="1227" t="n">
         <x:v>46218</x:v>
       </x:c>
@@ -11472,7 +11472,7 @@
         <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once. 2026-07-15 second Desktop Inline remediation is locally green: 30 additional pre-fix screenshots, 1,175/1,175 new context cases, 10,131/10,131 total tests, coverage above repository thresholds, TypeScript/build/lint 0 errors and npm audit 0. The branch is not yet deployment or real-client evidence; Desktop replay and all Android/iOS rows remain open.</x:v>
+        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once. 2026-07-15 second Desktop Inline remediation is locally green: 30 additional pre-fix screenshots, 1,175/1,175 new context cases, 10,131/10,131 total tests, coverage above repository thresholds, TypeScript/build/lint 0 errors and npm audit 0. The branch is not yet deployment or real-client evidence; Desktop replay and all Android/iOS rows remain open. 2026-07-15 PR #108 and exact Railway deployment da4c0a2/a1c6eab5 are green. Bounded production verification passed home/health, expected polling webhook policy, getMe, pending 0 and leader 200 with AI/alerts disabled. Deployment is closed; real Desktop/Android/iOS acceptance remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -23018,6 +23018,32 @@
         <x:v>Publish and deploy the reviewed branch, verify exact deployment health, then replay the affected Desktop cases and the 17-case Android/iOS matrices. Keep INL-001/INL-002 blocked and BOT-004 In Progress until real-client evidence passes.</x:v>
       </x:c>
     </x:row>
+    <x:row r="107" ht="195" customHeight="1">
+      <x:c r="A107" t="str">
+        <x:v>QA-TELEGRAM-INLINE-CONTEXT-DEPLOYMENT-2026-07-15</x:v>
+      </x:c>
+      <x:c r="B107" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>PR #108 CI, exact Railway deployment and bounded production runtime verification</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>GitHub application/security/database CI; Railway deployment identity and image; no-AI/no-alert production monitor</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>Passed: PR #108 merged as da4c0a2; deployment a1c6eab5 reached SUCCESS; home/health 200; webhook missing-secret 401 and polling-mode valid-secret 503; getMe valid; polling pending 0; leader 200; no paid AI call or Telegram alert.</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>BOT-004, INL-001, INL-002, PLAT-002</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>Read-only deployment evidence. Runtime code equals the reviewed merge. No Telegram user message, synthetic update, database mutation, provider reputation request or model call was made.</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>Replay affected post-fix Desktop cases, then complete the bounded 17-case Android and iOS matrices. Keep INL-001/INL-002 outside Passed and BOT-004 In Progress until client evidence is captured.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -24168,7 +24194,7 @@
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix. 2026-07-15 second Desktop remediation evidence: 30 additional pre-fix screenshots were converted into a 1,175-case local RU/UZ/EN Inline context suite. All 1,175 pass, including 1,152 dialogue mutations plus safe-control, redaction and result-id contracts. The complete project passes 10,131/10,131 tests and coverage 84.76/78.91/90.89/86.82. This remains deterministic offline evidence and does not replace the real Desktop/Android/iOS BOT-004 matrix.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix. 2026-07-15 second Desktop remediation evidence: 30 additional pre-fix screenshots were converted into a 1,175-case local RU/UZ/EN Inline context suite. All 1,175 pass, including 1,152 dialogue mutations plus safe-control, redaction and result-id contracts. The complete project passes 10,131/10,131 tests and coverage 84.76/78.91/90.89/86.82. This remains deterministic offline evidence and does not replace the real Desktop/Android/iOS BOT-004 matrix. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. BOT-004 remains In Progress until the wider RU/UZ/EN direct-bot real-client matrix passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -24292,7 +24318,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking. The screenshot-driven branch fixes changed-query result identity, concrete second-line priority, truncated/repetitive suspicious previews, RU/UZ/EN authority/SIM/investment context and false urgency from user safety questions. The 1,175-case handler suite denies external fetch and DB mutations; each check uses skipAi=true, skipUrlReputation=true and persist=false. Full local verification is 10,131/10,131 with coverage above all thresholds, TypeScript, lint 0 errors, build and npm audit 0. Deployment and real-client rendering/insertion remain blocking.</x:v>
+        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking. The screenshot-driven branch fixes changed-query result identity, concrete second-line priority, truncated/repetitive suspicious previews, RU/UZ/EN authority/SIM/investment context and false urgency from user safety questions. The 1,175-case handler suite denies external fetch and DB mutations; each check uses skipAi=true, skipUrlReputation=true and persist=false. Full local verification is 10,131/10,131 with coverage above all thresholds, TypeScript, lint 0 errors, build and npm audit 0. Deployment and real-client rendering/insertion remain blocking. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. Deployment/runtime preconditions are closed, but real Telegram Desktop preview/insertion replay is still required.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -24334,7 +24360,7 @@
       </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production. A second batch of 30 Telegram Desktop screenshots reproduces unchanged or missing edited-query results and truncated generic preview copy. They are pre-fix evidence only. Post-deploy Desktop replay plus the complete 17-case Android and iOS matrices remain required; no real-client pass is inferred from the local 1,175-case corpus.</x:v>
+        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production. A second batch of 30 Telegram Desktop screenshots reproduces unchanged or missing edited-query results and truncated generic preview copy. They are pre-fix evidence only. Post-deploy Desktop replay plus the complete 17-case Android and iOS matrices remain required; no real-client pass is inferred from the local 1,175-case corpus. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. Android and iOS 17-case matrices remain blocking; no pre-fix screenshot is counted as post-fix evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>

<commit_message>
Record Inline follow-up deployment evidence
</commit_message>
<xml_diff>
--- a/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
+++ b/ai_docs/FEATURE_USER_STORY_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R6ffd92cfff924920"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="R5c391322a4dd4395"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="Rb300f540469349e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Ra2ca5852fe3d42a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="R468eb7be48d741cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rb567a345c32e432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="Rdbad337f32fe47a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Ree5a290ef7e74a66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="1" r:id="R11bc31ae5749466b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="2" r:id="Rc05f73fd94bb4bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Findings" sheetId="3" r:id="R36793f3862194fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Queue" sheetId="4" r:id="Rd390b2d335644470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Errors" sheetId="5" r:id="Rc18c3c62a7474327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Runs" sheetId="6" r:id="Rff0125652ba54f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="7" r:id="R5ac209d30d3c4aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Security Queue" sheetId="8" r:id="Rfb8aca8626a54419"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1202,7 +1202,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1228">
+  <x:cellXfs count="1231">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -4306,6 +4306,15 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -11469,10 +11478,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="D2" s="1219" t="str">
-        <x:v>Continue real Telegram Desktop/Android/iOS RU/UZ/EN and Inline acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
+        <x:v>Replay the seven affected Telegram Desktop Inline edits, then complete the 17-case Android and iOS matrices. Continue broad direct-bot RU/UZ/EN acceptance, authorized Supabase/data drills, finding-specific live closure, legal/privacy approval, backup/restore/rollback/key-rotation drills and the fixed-RC 72-hour canary.</x:v>
       </x:c>
       <x:c r="E2" s="1219" t="str">
-        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once. 2026-07-15 second Desktop Inline remediation is locally green: 30 additional pre-fix screenshots, 1,175/1,175 new context cases, 10,131/10,131 total tests, coverage above repository thresholds, TypeScript/build/lint 0 errors and npm audit 0. The branch is not yet deployment or real-client evidence; Desktop replay and all Android/iOS rows remain open. 2026-07-15 PR #108 and exact Railway deployment da4c0a2/a1c6eab5 are green. Bounded production verification passed home/health, expected polling webhook policy, getMe, pending 0 and leader 200 with AI/alerts disabled. Deployment is closed; real Desktop/Android/iOS acceptance remains open.</x:v>
+        <x:v>2026-07-15: PR #106 merged as 87bf181b4d4df92e438e768f83ab4c02883f1d9f and Railway deployment 39cf9f6d-294d-410a-9cef-972e41829561 reached SUCCESS. Remote migration history records Supabase migrations 20260712142514 and 20260715040836; linked history matches, dry-run has no pending migration and schema lint is clean. Direct live catalog grant/trigger read-back remains open. A bounded no-AI/no-alert monitor passed home/health 200, webhook 401/503, mode=polling, pending=0 and leader 200. A one-minute local in-memory soak passed 600/600 with no duplicate or loss. The 41 Desktop screenshots remain pre-fix; post-fix Desktop and all Android/iOS acceptance rows remain open. Delivery remains at-least-once, not exactly-once. 2026-07-15 second Desktop Inline remediation is locally green: 30 additional pre-fix screenshots, 1,175/1,175 new context cases, 10,131/10,131 total tests, coverage above repository thresholds, TypeScript/build/lint 0 errors and npm audit 0. The branch is not yet deployment or real-client evidence; Desktop replay and all Android/iOS rows remain open. 2026-07-15 PR #108 and exact Railway deployment da4c0a2/a1c6eab5 are green. Bounded production verification passed home/health, expected polling webhook policy, getMe, pending 0 and leader 200 with AI/alerts disabled. Deployment is closed; real Desktop/Android/iOS acceptance remains open. 2026-07-15 third Desktop Inline follow-up remediation: seven owner-supplied Telegram Desktop screenshots showed that the first-line card rendered but edited second-line questions usually kept the stale preview; passport aftercare was the visible control that changed. PR #110 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as 581e71536e729253b73012baf5086241caf68e13. Exact Railway deployment f5915159-ccaa-46bc-9e42-be8c521010be reached SUCCESS with image sha256:b094e4592d2492bece73f64a21eeb802792b7ec32996370800b2fa0efbe84ddb. Focused verification passed 2,002/2,002 and the complete project passed 10,172/10,172 tests; coverage was 84.87% statements, 79.06% branches, 90.91% functions and 86.92% lines; TypeScript, production build, lint with 0 errors/8 existing warnings and npm audit 0 passed. A bounded read-only no-AI/no-alert monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200. These screenshots remain pre-fix evidence: the same seven Desktop cases must be replayed post-fix and the Android/iOS matrices remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -19821,7 +19830,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="50" t="inlineStr">
+      <x:c r="B2" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -19863,7 +19872,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-002</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="50" t="inlineStr">
+      <x:c r="B3" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -19905,7 +19914,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-003</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="50" t="inlineStr">
+      <x:c r="B4" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -19947,7 +19956,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-004</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="50" t="inlineStr">
+      <x:c r="B5" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -19989,7 +19998,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-005</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="50" t="inlineStr">
+      <x:c r="B6" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -20031,7 +20040,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-006</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="50" t="inlineStr">
+      <x:c r="B7" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -20073,7 +20082,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-007</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="50" t="inlineStr">
+      <x:c r="B8" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -20115,7 +20124,7 @@
           <x:t xml:space="preserve">QA-2026-06-29-008</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="50" t="inlineStr">
+      <x:c r="B9" s="1228" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-29</x:t>
         </x:is>
@@ -20157,7 +20166,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="6" t="inlineStr">
+      <x:c r="B10" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20199,7 +20208,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-002</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="6" t="inlineStr">
+      <x:c r="B11" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20241,7 +20250,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-003</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" s="6" t="inlineStr">
+      <x:c r="B12" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20283,7 +20292,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-004</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" s="6" t="inlineStr">
+      <x:c r="B13" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20325,7 +20334,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-005</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="6" t="inlineStr">
+      <x:c r="B14" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20367,7 +20376,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-006</x:t>
         </x:is>
       </x:c>
-      <x:c r="B15" s="6" t="inlineStr">
+      <x:c r="B15" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20409,7 +20418,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-007</x:t>
         </x:is>
       </x:c>
-      <x:c r="B16" s="6" t="inlineStr">
+      <x:c r="B16" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20451,7 +20460,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-008</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" s="6" t="inlineStr">
+      <x:c r="B17" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20493,7 +20502,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-009</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" s="6" t="inlineStr">
+      <x:c r="B18" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20535,7 +20544,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-010</x:t>
         </x:is>
       </x:c>
-      <x:c r="B19" s="6" t="inlineStr">
+      <x:c r="B19" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20577,7 +20586,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-011</x:t>
         </x:is>
       </x:c>
-      <x:c r="B20" s="6" t="inlineStr">
+      <x:c r="B20" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20619,7 +20628,7 @@
           <x:t xml:space="preserve">QA-2026-06-30-012</x:t>
         </x:is>
       </x:c>
-      <x:c r="B21" s="6" t="inlineStr">
+      <x:c r="B21" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-06-30</x:t>
         </x:is>
@@ -20661,7 +20670,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="B22" s="6" t="inlineStr">
+      <x:c r="B22" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20703,7 +20712,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-002</x:t>
         </x:is>
       </x:c>
-      <x:c r="B23" s="6" t="inlineStr">
+      <x:c r="B23" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20745,7 +20754,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-003</x:t>
         </x:is>
       </x:c>
-      <x:c r="B24" s="6" t="inlineStr">
+      <x:c r="B24" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20787,7 +20796,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-004</x:t>
         </x:is>
       </x:c>
-      <x:c r="B25" s="6" t="inlineStr">
+      <x:c r="B25" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20829,7 +20838,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-005</x:t>
         </x:is>
       </x:c>
-      <x:c r="B26" s="6" t="inlineStr">
+      <x:c r="B26" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20871,7 +20880,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-006</x:t>
         </x:is>
       </x:c>
-      <x:c r="B27" s="6" t="inlineStr">
+      <x:c r="B27" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20913,7 +20922,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-007</x:t>
         </x:is>
       </x:c>
-      <x:c r="B28" s="6" t="inlineStr">
+      <x:c r="B28" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20955,7 +20964,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-008</x:t>
         </x:is>
       </x:c>
-      <x:c r="B29" s="6" t="inlineStr">
+      <x:c r="B29" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -20997,7 +21006,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-009</x:t>
         </x:is>
       </x:c>
-      <x:c r="B30" s="6" t="inlineStr">
+      <x:c r="B30" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21039,7 +21048,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-010</x:t>
         </x:is>
       </x:c>
-      <x:c r="B31" s="6" t="inlineStr">
+      <x:c r="B31" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21081,7 +21090,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-011</x:t>
         </x:is>
       </x:c>
-      <x:c r="B32" s="6" t="inlineStr">
+      <x:c r="B32" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21123,7 +21132,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-012</x:t>
         </x:is>
       </x:c>
-      <x:c r="B33" s="6" t="inlineStr">
+      <x:c r="B33" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21165,7 +21174,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-013</x:t>
         </x:is>
       </x:c>
-      <x:c r="B34" s="6" t="inlineStr">
+      <x:c r="B34" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21207,7 +21216,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-014</x:t>
         </x:is>
       </x:c>
-      <x:c r="B35" s="6" t="inlineStr">
+      <x:c r="B35" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21249,7 +21258,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-015</x:t>
         </x:is>
       </x:c>
-      <x:c r="B36" s="6" t="inlineStr">
+      <x:c r="B36" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21291,7 +21300,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-016</x:t>
         </x:is>
       </x:c>
-      <x:c r="B37" s="6" t="inlineStr">
+      <x:c r="B37" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21333,7 +21342,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-017</x:t>
         </x:is>
       </x:c>
-      <x:c r="B38" s="6" t="inlineStr">
+      <x:c r="B38" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21375,7 +21384,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-018</x:t>
         </x:is>
       </x:c>
-      <x:c r="B39" s="6" t="inlineStr">
+      <x:c r="B39" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21417,7 +21426,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-019</x:t>
         </x:is>
       </x:c>
-      <x:c r="B40" s="6" t="inlineStr">
+      <x:c r="B40" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21459,7 +21468,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-020</x:t>
         </x:is>
       </x:c>
-      <x:c r="B41" s="6" t="inlineStr">
+      <x:c r="B41" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21501,7 +21510,7 @@
           <x:t xml:space="preserve">QA-2026-07-01-021</x:t>
         </x:is>
       </x:c>
-      <x:c r="B42" s="6" t="inlineStr">
+      <x:c r="B42" s="1229" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-07-01</x:t>
         </x:is>
@@ -21541,7 +21550,7 @@
       <x:c r="A43" t="str">
         <x:v>QA-2026-07-01-022</x:v>
       </x:c>
-      <x:c r="B43" t="str">
+      <x:c r="B43" s="1097" t="str">
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C43" t="str">
@@ -21567,7 +21576,7 @@
       <x:c r="A44" t="str">
         <x:v>QA-2026-07-01-023</x:v>
       </x:c>
-      <x:c r="B44" t="str">
+      <x:c r="B44" s="1097" t="str">
         <x:v>2026-07-01</x:v>
       </x:c>
       <x:c r="C44" t="str">
@@ -21593,7 +21602,7 @@
       <x:c r="A45" t="str">
         <x:v>QA-2026-07-02-001</x:v>
       </x:c>
-      <x:c r="B45" t="str">
+      <x:c r="B45" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C45" t="str">
@@ -21619,7 +21628,7 @@
       <x:c r="A46" t="str">
         <x:v>QA-2026-07-02-002</x:v>
       </x:c>
-      <x:c r="B46" t="str">
+      <x:c r="B46" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C46" t="str">
@@ -21645,7 +21654,7 @@
       <x:c r="A47" t="str">
         <x:v>QA-2026-07-02-003</x:v>
       </x:c>
-      <x:c r="B47" t="str">
+      <x:c r="B47" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C47" t="str">
@@ -21671,7 +21680,7 @@
       <x:c r="A48" t="str">
         <x:v>QA-2026-07-02-004</x:v>
       </x:c>
-      <x:c r="B48" t="str">
+      <x:c r="B48" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C48" t="str">
@@ -21697,7 +21706,7 @@
       <x:c r="A49" s="595" t="str">
         <x:v>QA-2026-07-02-005</x:v>
       </x:c>
-      <x:c r="B49" s="595" t="str">
+      <x:c r="B49" s="1230" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C49" s="595" t="str">
@@ -21723,7 +21732,7 @@
       <x:c r="A50" s="595" t="str">
         <x:v>QA-2026-07-02-006</x:v>
       </x:c>
-      <x:c r="B50" s="595" t="str">
+      <x:c r="B50" s="1230" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C50" s="595" t="str">
@@ -21749,7 +21758,7 @@
       <x:c r="A51" s="596" t="str">
         <x:v>QA-2026-07-02-007</x:v>
       </x:c>
-      <x:c r="B51" s="596" t="str">
+      <x:c r="B51" s="1229" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C51" s="596" t="str">
@@ -21775,7 +21784,7 @@
       <x:c r="A52" t="str">
         <x:v>QA-2026-07-02-008</x:v>
       </x:c>
-      <x:c r="B52" t="str">
+      <x:c r="B52" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C52" t="str">
@@ -21801,7 +21810,7 @@
       <x:c r="A53" t="str">
         <x:v>QA-2026-07-02-009</x:v>
       </x:c>
-      <x:c r="B53" t="str">
+      <x:c r="B53" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C53" t="str">
@@ -21827,7 +21836,7 @@
       <x:c r="A54" s="596" t="str">
         <x:v>QA-2026-07-02-010</x:v>
       </x:c>
-      <x:c r="B54" s="596" t="str">
+      <x:c r="B54" s="1229" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C54" s="596" t="str">
@@ -21853,7 +21862,7 @@
       <x:c r="A55" s="596" t="str">
         <x:v>QA-2026-07-02-011</x:v>
       </x:c>
-      <x:c r="B55" s="596" t="str">
+      <x:c r="B55" s="1229" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C55" s="596" t="str">
@@ -21879,7 +21888,7 @@
       <x:c r="A56" s="595" t="str">
         <x:v>QA-2026-07-02-012</x:v>
       </x:c>
-      <x:c r="B56" s="595" t="str">
+      <x:c r="B56" s="1230" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C56" s="595" t="str">
@@ -21905,7 +21914,7 @@
       <x:c r="A57" s="595" t="str">
         <x:v>QA-2026-07-02-013</x:v>
       </x:c>
-      <x:c r="B57" s="595" t="str">
+      <x:c r="B57" s="1230" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C57" s="595" t="str">
@@ -21931,7 +21940,7 @@
       <x:c r="A58" s="595" t="str">
         <x:v>QA-2026-07-02-014</x:v>
       </x:c>
-      <x:c r="B58" s="595" t="str">
+      <x:c r="B58" s="1230" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C58" s="595" t="str">
@@ -21957,7 +21966,7 @@
       <x:c r="A59" s="595" t="str">
         <x:v>QA-2026-07-02-015</x:v>
       </x:c>
-      <x:c r="B59" s="595" t="str">
+      <x:c r="B59" s="1230" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C59" s="595" t="str">
@@ -21983,7 +21992,7 @@
       <x:c r="A60" t="str">
         <x:v>QA-2026-07-02-016</x:v>
       </x:c>
-      <x:c r="B60" t="str">
+      <x:c r="B60" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C60" t="str">
@@ -22009,7 +22018,7 @@
       <x:c r="A61" t="str">
         <x:v>QA-2026-07-02-017</x:v>
       </x:c>
-      <x:c r="B61" t="str">
+      <x:c r="B61" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C61" t="str">
@@ -22035,7 +22044,7 @@
       <x:c r="A62" t="str">
         <x:v>QA-2026-07-02-018</x:v>
       </x:c>
-      <x:c r="B62" t="str">
+      <x:c r="B62" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C62" t="str">
@@ -22061,7 +22070,7 @@
       <x:c r="A63" t="str">
         <x:v>QA-2026-07-02-019</x:v>
       </x:c>
-      <x:c r="B63" t="str">
+      <x:c r="B63" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C63" t="str">
@@ -22087,7 +22096,7 @@
       <x:c r="A64" t="str">
         <x:v>QA-2026-07-02-020</x:v>
       </x:c>
-      <x:c r="B64" t="str">
+      <x:c r="B64" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C64" t="str">
@@ -22113,7 +22122,7 @@
       <x:c r="A65" t="str">
         <x:v>QA-2026-07-02-021</x:v>
       </x:c>
-      <x:c r="B65" t="str">
+      <x:c r="B65" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C65" t="str">
@@ -22139,7 +22148,7 @@
       <x:c r="A66" t="str">
         <x:v>QA-2026-07-02-022</x:v>
       </x:c>
-      <x:c r="B66" t="str">
+      <x:c r="B66" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C66" t="str">
@@ -22165,7 +22174,7 @@
       <x:c r="A67" t="str">
         <x:v>QA-2026-07-02-023</x:v>
       </x:c>
-      <x:c r="B67" t="str">
+      <x:c r="B67" s="1097" t="str">
         <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="C67" t="str">
@@ -22191,7 +22200,7 @@
       <x:c r="A68" t="str">
         <x:v>QA-2026-07-04-001</x:v>
       </x:c>
-      <x:c r="B68" t="str">
+      <x:c r="B68" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C68" t="str">
@@ -22217,7 +22226,7 @@
       <x:c r="A69" t="str">
         <x:v>QA-2026-07-04-002</x:v>
       </x:c>
-      <x:c r="B69" t="str">
+      <x:c r="B69" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C69" t="str">
@@ -22243,7 +22252,7 @@
       <x:c r="A70" t="str">
         <x:v>QA-2026-07-04-003</x:v>
       </x:c>
-      <x:c r="B70" t="str">
+      <x:c r="B70" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C70" t="str">
@@ -22269,7 +22278,7 @@
       <x:c r="A71" t="str">
         <x:v>QA-2026-07-04-004</x:v>
       </x:c>
-      <x:c r="B71" t="str">
+      <x:c r="B71" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C71" t="str">
@@ -22295,7 +22304,7 @@
       <x:c r="A72" t="str">
         <x:v>QA-2026-07-04-005</x:v>
       </x:c>
-      <x:c r="B72" t="str">
+      <x:c r="B72" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C72" t="str">
@@ -22321,7 +22330,7 @@
       <x:c r="A73" t="str">
         <x:v>QA-2026-07-04-006</x:v>
       </x:c>
-      <x:c r="B73" t="str">
+      <x:c r="B73" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C73" t="str">
@@ -22347,7 +22356,7 @@
       <x:c r="A74" t="str">
         <x:v>QA-2026-07-04-007</x:v>
       </x:c>
-      <x:c r="B74" t="str">
+      <x:c r="B74" s="1097" t="str">
         <x:v>2026-07-04</x:v>
       </x:c>
       <x:c r="C74" t="str">
@@ -22373,7 +22382,7 @@
       <x:c r="A75" t="str">
         <x:v>QA-2026-07-08-001</x:v>
       </x:c>
-      <x:c r="B75" t="str">
+      <x:c r="B75" s="1097" t="str">
         <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C75" t="str">
@@ -22399,7 +22408,7 @@
       <x:c r="A76" t="str">
         <x:v>QA-2026-07-08-002</x:v>
       </x:c>
-      <x:c r="B76" t="str">
+      <x:c r="B76" s="1097" t="str">
         <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C76" t="str">
@@ -22425,7 +22434,7 @@
       <x:c r="A77" t="str">
         <x:v>QA-2026-07-08-003</x:v>
       </x:c>
-      <x:c r="B77" t="str">
+      <x:c r="B77" s="1097" t="str">
         <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="C77" t="str">
@@ -22451,7 +22460,7 @@
       <x:c r="A78" t="str">
         <x:v>QA-2026-07-09-002</x:v>
       </x:c>
-      <x:c r="B78" t="str">
+      <x:c r="B78" s="1097" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="C78" t="str">
@@ -22477,7 +22486,7 @@
       <x:c r="A79" t="str">
         <x:v>QA-2026-07-09-003</x:v>
       </x:c>
-      <x:c r="B79" t="str">
+      <x:c r="B79" s="1097" t="str">
         <x:v>Live Telegram image QA partial</x:v>
       </x:c>
       <x:c r="C79" t="str">
@@ -22494,7 +22503,7 @@
       <x:c r="A80" t="str">
         <x:v>QA-2026-07-09-004</x:v>
       </x:c>
-      <x:c r="B80" t="str">
+      <x:c r="B80" s="1097" t="str">
         <x:v>MIME-spoofing router guard regression</x:v>
       </x:c>
       <x:c r="C80" t="str">
@@ -22511,7 +22520,7 @@
       <x:c r="A81" t="str">
         <x:v>QA-2026-07-09-005</x:v>
       </x:c>
-      <x:c r="B81" t="str">
+      <x:c r="B81" s="1097" t="str">
         <x:v>Quality Gate residual direct phrase regression</x:v>
       </x:c>
       <x:c r="C81" t="str">
@@ -22528,7 +22537,7 @@
       <x:c r="A82" t="str">
         <x:v>QA-2026-07-09-006</x:v>
       </x:c>
-      <x:c r="B82" t="str">
+      <x:c r="B82" s="1097" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="C82" t="str">
@@ -22554,7 +22563,7 @@
       <x:c r="A83" t="str">
         <x:v>QA-2026-07-09-007</x:v>
       </x:c>
-      <x:c r="B83" t="str">
+      <x:c r="B83" s="1097" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="C83" t="str">
@@ -22580,7 +22589,7 @@
       <x:c r="A84" t="str">
         <x:v>QA-TELEGRAM-INLINE-UNICODE-GATE-2026-07-14</x:v>
       </x:c>
-      <x:c r="B84" t="n">
+      <x:c r="B84" s="1097" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="C84" t="str">
@@ -22601,12 +22610,30 @@
       <x:c r="H84" t="str">
         <x:v>Run all 17 fixtures on each of Telegram Desktop, Android and iOS, capture sanitized preview/insertion evidence and read back zero persistence before closing BOT-004/INL-001/INL-002.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="B85" s="1097"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="B86" s="1097"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="B87" s="1097"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="B88" s="1097"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="B89" s="1097"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="B90" s="1097"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
         <x:v>QA-2026-07-09-010</x:v>
       </x:c>
-      <x:c r="B91" t="str">
+      <x:c r="B91" s="1097" t="str">
         <x:v>2026-07-09</x:v>
       </x:c>
       <x:c r="C91" t="str">
@@ -22840,7 +22867,7 @@
       <x:c r="A100" t="str">
         <x:v>QA-HUMAN-DIALOGUE-PROD-2026-07-13</x:v>
       </x:c>
-      <x:c r="B100" t="n">
+      <x:c r="B100" s="1097" t="n">
         <x:v>46216</x:v>
       </x:c>
       <x:c r="C100" t="str">
@@ -22866,7 +22893,7 @@
       <x:c r="A101" t="str">
         <x:v>QA-POLLING-RESOURCE-SOAK-PROD-2026-07-14</x:v>
       </x:c>
-      <x:c r="B101" t="n">
+      <x:c r="B101" s="1097" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="C101" t="str">
@@ -22892,7 +22919,7 @@
       <x:c r="A102" t="str">
         <x:v>QA-QR-WORKER-RESOURCE-SOAK-PROD-2026-07-14</x:v>
       </x:c>
-      <x:c r="B102" t="n">
+      <x:c r="B102" s="1097" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="C102" t="str">
@@ -22918,7 +22945,7 @@
       <x:c r="A103" t="str">
         <x:v>QA-SHARED-RATE-LIMIT-FAILURE-PROD-2026-07-14</x:v>
       </x:c>
-      <x:c r="B103" t="n">
+      <x:c r="B103" s="1097" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="C103" t="str">
@@ -22944,7 +22971,7 @@
       <x:c r="A104" s="596" t="str">
         <x:v>QA-TELEGRAM-RESTART-REAL-UPDATE-PROD-2026-07-14</x:v>
       </x:c>
-      <x:c r="B104" s="596" t="n">
+      <x:c r="B104" s="1229" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="C104" s="596" t="str">
@@ -22970,7 +22997,7 @@
       <x:c r="A105" t="str">
         <x:v>QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14</x:v>
       </x:c>
-      <x:c r="B105" t="n">
+      <x:c r="B105" s="1097" t="n">
         <x:v>46217</x:v>
       </x:c>
       <x:c r="C105" t="str">
@@ -22996,7 +23023,7 @@
       <x:c r="A106" t="str">
         <x:v>QA-TELEGRAM-INLINE-CONTEXT-RECOVERY-2026-07-15</x:v>
       </x:c>
-      <x:c r="B106" t="n">
+      <x:c r="B106" s="1097" t="n">
         <x:v>46218</x:v>
       </x:c>
       <x:c r="C106" t="str">
@@ -23022,7 +23049,7 @@
       <x:c r="A107" t="str">
         <x:v>QA-TELEGRAM-INLINE-CONTEXT-DEPLOYMENT-2026-07-15</x:v>
       </x:c>
-      <x:c r="B107" t="n">
+      <x:c r="B107" s="1097" t="n">
         <x:v>46218</x:v>
       </x:c>
       <x:c r="C107" t="str">
@@ -23042,6 +23069,32 @@
       </x:c>
       <x:c r="H107" t="str">
         <x:v>Replay affected post-fix Desktop cases, then complete the bounded 17-case Android and iOS matrices. Keep INL-001/INL-002 outside Passed and BOT-004 In Progress until client evidence is captured.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>QA-TELEGRAM-INLINE-FOLLOWUP-DEPLOY-2026-07-15</x:v>
+      </x:c>
+      <x:c r="B108" s="1097" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>Third Telegram Desktop Inline follow-up visibility remediation and exact production deployment</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>PR #110 application/coverage/security/database CI; focused and full lockfile-pinned tests; Railway deployment identity/image; bounded no-AI/no-alert production monitor</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>Passed: PR #110 merged as 581e71536e729253b73012baf5086241caf68e13; Railway f5915159-ccaa-46bc-9e42-be8c521010be SUCCESS; focused 2,002/2,002; full 10,172/10,172; coverage 84.87/79.06/90.91/86.92; TypeScript/build/lint 0 errors/npm audit 0; all GitHub checks green; home/health 200, webhook 401/503, getMe, pending 0 and leader 200.</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>BOT-004, INL-001, INL-002, TG-016, PLAT-002</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>Seven owner-supplied Desktop screenshots are pre-fix evidence. The deployed code makes trust, scam-confirmation, bank-chat-number, link-verification, reason and next-action follow-ups visibly change the card, adds blackmail guidance, keeps concrete danger above broad meta copy, and retains stateless privacy boundaries: skipAi=true, skipUrlReputation=true and persist=false. No paid AI/provider call, Telegram test message or database mutation was used by this verification.</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>Replay the same seven Desktop cases against deployment f5915159, capture sanitized preview/insertion screenshots, then complete the bounded 17-case Android and iOS matrices. Keep BOT-004 In Progress and INL-001/INL-002 Blocked until client evidence passes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24194,7 +24247,7 @@
       </x:c>
       <x:c r="M27" s="615" t="str"/>
       <x:c r="N27" s="615" t="str">
-        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix. 2026-07-15 second Desktop remediation evidence: 30 additional pre-fix screenshots were converted into a 1,175-case local RU/UZ/EN Inline context suite. All 1,175 pass, including 1,152 dialogue mutations plus safe-control, redaction and result-id contracts. The complete project passes 10,131/10,131 tests and coverage 84.76/78.91/90.89/86.82. This remains deterministic offline evidence and does not replace the real Desktop/Android/iOS BOT-004 matrix. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. BOT-004 remains In Progress until the wider RU/UZ/EN direct-bot real-client matrix passes.</x:v>
+        <x:v>PR #86 deployed the human-style routing/corpus change; PR #87 corrected RU/UZ/EN high-risk confidence guidance after the first production harness exposed an ambiguous organization/person callback sentence. Railway exact SHA 5ceb9eaa2ed447e0072a7cee4b25e16eae673b03 / deployment 8c76285e-51c0-4539-b305-d2d1d3301227 is SUCCESS. The final polling-dispatch harness passed confidence, trusted-person, recheck, disagreement, domain-methodology and passport flows, and deleted its Bot API replies plus synthetic DB rows. Full suite: 8584/8584 in 134 files; TypeScript; lint 0 errors/8 existing warnings; build; npm audit 0; CI, CodeQL, Gitleaks, container/SBOM and migrations/schema/pgTAP passed. Offline evidence remains 1008 context cases, exactly 1000 unique 2/3-turn dialogues / 2500 user turns, 540 everyday dialogues / 1080 turns / 102 follow-ups, 363 mixed-clause messages, independent 2438/2438, 17 benign controls, 33/33 direct-danger probes and 28 clause-local code-context regressions. These are deterministic cases, not model training or live chats. Broad real-client RU/UZ/EN evidence remains required before BOT-004 can pass. 2026-07-14 local Inline reuse: QA-TELEGRAM-INLINE-OFFLINE-CORPUS-2026-07-14 passed 3,805 source cases / 2,140 unique queries through the real Inline handler with external sinks denied. This is local corpus evidence only and does not replace the real Telegram Desktop/Android/iOS RU/UZ/EN BOT-004 matrix. PR #102 / main f26eece deployed as Railway 90962188 with image sha256:5c5e4e70; health and polling leader returned 200. The Inline Unicode fix and client fixture pack do not replace the broad direct-bot real-client RU/UZ/EN matrix. 2026-07-15 second Desktop remediation evidence: 30 additional pre-fix screenshots were converted into a 1,175-case local RU/UZ/EN Inline context suite. All 1,175 pass, including 1,152 dialogue mutations plus safe-control, redaction and result-id contracts. The complete project passes 10,131/10,131 tests and coverage 84.76/78.91/90.89/86.82. This remains deterministic offline evidence and does not replace the real Desktop/Android/iOS BOT-004 matrix. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. BOT-004 remains In Progress until the wider RU/UZ/EN direct-bot real-client matrix passes. 2026-07-15 third Desktop Inline follow-up remediation: seven owner-supplied Telegram Desktop screenshots showed that the first-line card rendered but edited second-line questions usually kept the stale preview; passport aftercare was the visible control that changed. PR #110 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as 581e71536e729253b73012baf5086241caf68e13. Exact Railway deployment f5915159-ccaa-46bc-9e42-be8c521010be reached SUCCESS with image sha256:b094e4592d2492bece73f64a21eeb802792b7ec32996370800b2fa0efbe84ddb. Focused verification passed 2,002/2,002 and the complete project passed 10,172/10,172 tests; coverage was 84.87% statements, 79.06% branches, 90.91% functions and 86.92% lines; TypeScript, production build, lint with 0 errors/8 existing warnings and npm audit 0 passed. A bounded read-only no-AI/no-alert monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200. These screenshots remain pre-fix evidence: the same seven Desktop cases must be replayed post-fix and the Android/iOS matrices remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -24318,7 +24371,7 @@
         <x:v>INL-P0-01..04</x:v>
       </x:c>
       <x:c r="N30" s="615" t="str">
-        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking. The screenshot-driven branch fixes changed-query result identity, concrete second-line priority, truncated/repetitive suspicious previews, RU/UZ/EN authority/SIM/investment context and false urgency from user safety questions. The 1,175-case handler suite denies external fetch and DB mutations; each check uses skipAi=true, skipUrlReputation=true and persist=false. Full local verification is 10,131/10,131 with coverage above all thresholds, TypeScript, lint 0 errors, build and npm audit 0. Deployment and real-client rendering/insertion remain blocking. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. Deployment/runtime preconditions are closed, but real Telegram Desktop preview/insertion replay is still required.</x:v>
+        <x:v>Automated backend/protocol/privacy evidence remains Passed: 3,805 source cases / 2,140 unique RU/UZ/EN queries are rules-only and non-persistent, and the full release suite passes 8,882/8,882. PR #106 final application, coverage, clean-database migration/schema/35-pgTAP, CodeQL, Gitleaks and container/SBOM jobs passed; historical Railway deployment 39cf9f6d of merge 87bf181b reached SUCCESS. Supabase migration history matches local, dry-run is no-op and remote schema lint is clean. The bounded no-AI/no-alert monitor passed health, expected polling webhook behavior, pending=0 and leader 200; the one-minute local in-memory soak passed 600/600 with zero duplicate/loss. The 41 screenshots are pre-fix evidence only. Real Desktop/Android/iOS rendering, insertion and recovery evidence remains blocking. The screenshot-driven branch fixes changed-query result identity, concrete second-line priority, truncated/repetitive suspicious previews, RU/UZ/EN authority/SIM/investment context and false urgency from user safety questions. The 1,175-case handler suite denies external fetch and DB mutations; each check uses skipAi=true, skipUrlReputation=true and persist=false. Full local verification is 10,131/10,131 with coverage above all thresholds, TypeScript, lint 0 errors, build and npm audit 0. Deployment and real-client rendering/insertion remain blocking. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. Deployment/runtime preconditions are closed, but real Telegram Desktop preview/insertion replay is still required. 2026-07-15 third Desktop Inline follow-up remediation: seven owner-supplied Telegram Desktop screenshots showed that the first-line card rendered but edited second-line questions usually kept the stale preview; passport aftercare was the visible control that changed. PR #110 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as 581e71536e729253b73012baf5086241caf68e13. Exact Railway deployment f5915159-ccaa-46bc-9e42-be8c521010be reached SUCCESS with image sha256:b094e4592d2492bece73f64a21eeb802792b7ec32996370800b2fa0efbe84ddb. Focused verification passed 2,002/2,002 and the complete project passed 10,172/10,172 tests; coverage was 84.87% statements, 79.06% branches, 90.91% functions and 86.92% lines; TypeScript, production build, lint with 0 errors/8 existing warnings and npm audit 0 passed. A bounded read-only no-AI/no-alert monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200. These screenshots remain pre-fix evidence: the same seven Desktop cases must be replayed post-fix and the Android/iOS matrices remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -24344,7 +24397,7 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H31" s="615" t="str">
-        <x:v>Not Deployed</x:v>
+        <x:v>Deployed</x:v>
       </x:c>
       <x:c r="I31" s="615" t="str">
         <x:v>Blocked</x:v>
@@ -24360,7 +24413,7 @@
       </x:c>
       <x:c r="M31" s="615" t="str"/>
       <x:c r="N31" s="615" t="str">
-        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production. A second batch of 30 Telegram Desktop screenshots reproduces unchanged or missing edited-query results and truncated generic preview copy. They are pre-fix evidence only. Post-deploy Desktop replay plus the complete 17-case Android and iOS matrices remain required; no real-client pass is inferred from the local 1,175-case corpus. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. Android and iOS 17-case matrices remain blocking; no pre-fix screenshot is counted as post-fix evidence.</x:v>
+        <x:v>The zero-network client generator defines 17 cases per client / 51 Desktop-Android-iOS rows. Forty-one 2026-07-15 Desktop screenshots reproduced pre-fix job-fee, multiline-link, passport, ambiguous-number, phone/privacy, rate-limit and stale/missing-result defects. Historical Railway deployment 39cf9f6d of PR #106 merge 87bf181b reached SUCCESS, but no post-fix row is inferred from those screenshots. Counted progress remains 1/17 Desktop from the 2026-07-14 passing pair and 0/17 on Android and iOS. The 257-character, timeout, ok:false and parse-retry branches remain automated-only and must not be forced in production. A second batch of 30 Telegram Desktop screenshots reproduces unchanged or missing edited-query results and truncated generic preview copy. They are pre-fix evidence only. Post-deploy Desktop replay plus the complete 17-case Android and iOS matrices remain required; no real-client pass is inferred from the local 1,175-case corpus. PR #108 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as da4c0a259a228d864432a77ccb1b3291468c52cf. Exact Railway deployment a1c6eab5-a8da-4341-a7ff-387212cd3784 reached SUCCESS with image sha256:9cc2da03c7e57eb29f53fadb332596a48e154ff9be372620349943eeae1155e9. A bounded read-only monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200 with AI and alerts disabled. Android and iOS 17-case matrices remain blocking; no pre-fix screenshot is counted as post-fix evidence. 2026-07-15 third Desktop Inline follow-up remediation: seven owner-supplied Telegram Desktop screenshots showed that the first-line card rendered but edited second-line questions usually kept the stale preview; passport aftercare was the visible control that changed. PR #110 passed application, coverage, Supabase/schema/pgTAP, CodeQL, Gitleaks and container/SBOM gates and merged as 581e71536e729253b73012baf5086241caf68e13. Exact Railway deployment f5915159-ccaa-46bc-9e42-be8c521010be reached SUCCESS with image sha256:b094e4592d2492bece73f64a21eeb802792b7ec32996370800b2fa0efbe84ddb. Focused verification passed 2,002/2,002 and the complete project passed 10,172/10,172 tests; coverage was 84.87% statements, 79.06% branches, 90.91% functions and 86.92% lines; TypeScript, production build, lint with 0 errors/8 existing warnings and npm audit 0 passed. A bounded read-only no-AI/no-alert monitor passed home/health 200, webhook 401/expected polling 503, getMe, pending 0 and polling leader 200. These screenshots remain pre-fix evidence: the same seven Desktop cases must be replayed post-fix and the Android/iOS matrices remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>